<commit_message>
Refresh dashboard Tue 06/23/2026  6:46
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -706,7 +706,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 19 Jun 2026 16:27</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 23 Jun 2026 06:46</t>
         </is>
       </c>
     </row>
@@ -6549,7 +6549,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 19 Jun 2026 16:27 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 23 Jun 2026 06:46 (in IDR Million)</t>
         </is>
       </c>
     </row>
@@ -14074,16 +14074,16 @@
         <v>1555978395.440002</v>
       </c>
       <c r="E6" s="9" t="n">
-        <v>-1257887353</v>
+        <v>-871753665</v>
       </c>
       <c r="F6" s="9" t="n">
-        <v>298091042.4400024</v>
+        <v>684224730.4400024</v>
       </c>
       <c r="G6" s="21" t="n">
-        <v>17534.76720235308</v>
+        <v>40248.51355529426</v>
       </c>
       <c r="H6" s="21" t="n">
-        <v>1577201.282751336</v>
+        <v>3620236.668994722</v>
       </c>
     </row>
     <row r="7">
@@ -14106,16 +14106,16 @@
         <v>186144708</v>
       </c>
       <c r="E7" s="11" t="n">
-        <v>-42174061</v>
+        <v>-41903061</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>143970647</v>
+        <v>144241647</v>
       </c>
       <c r="G7" s="22" t="n">
-        <v>8468.861588235293</v>
+        <v>8484.802764705883</v>
       </c>
       <c r="H7" s="22" t="n">
-        <v>761749.455026455</v>
+        <v>763183.3174603175</v>
       </c>
     </row>
     <row r="8">
@@ -14289,13 +14289,13 @@
       <c r="D13" s="24" t="n"/>
       <c r="E13" s="24" t="n"/>
       <c r="F13" s="25" t="n">
-        <v>3445289718.370002</v>
+        <v>3831694406.370002</v>
       </c>
       <c r="G13" s="26" t="n">
-        <v>202664.1010805884</v>
+        <v>225393.7886100001</v>
       </c>
       <c r="H13" s="26" t="n">
-        <v>18229046.12894181</v>
+        <v>20273515.37761906</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh dashboard Wed 06/24/2026 16:26
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -706,7 +706,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 23 Jun 2026 06:46</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 24 Jun 2026 16:26</t>
         </is>
       </c>
     </row>
@@ -6549,7 +6549,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 23 Jun 2026 06:46 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 24 Jun 2026 16:26 (in IDR Million)</t>
         </is>
       </c>
     </row>
@@ -14074,16 +14074,16 @@
         <v>1555978395.440002</v>
       </c>
       <c r="E6" s="9" t="n">
-        <v>-871753665</v>
+        <v>-666187365</v>
       </c>
       <c r="F6" s="9" t="n">
-        <v>684224730.4400024</v>
+        <v>889791030.4400024</v>
       </c>
       <c r="G6" s="21" t="n">
-        <v>40248.51355529426</v>
+        <v>52340.64884941191</v>
       </c>
       <c r="H6" s="21" t="n">
-        <v>3620236.668994722</v>
+        <v>4707889.049947103</v>
       </c>
     </row>
     <row r="7">
@@ -14289,13 +14289,13 @@
       <c r="D13" s="24" t="n"/>
       <c r="E13" s="24" t="n"/>
       <c r="F13" s="25" t="n">
-        <v>3831694406.370002</v>
+        <v>4037260706.370002</v>
       </c>
       <c r="G13" s="26" t="n">
-        <v>225393.7886100001</v>
+        <v>237485.9239041178</v>
       </c>
       <c r="H13" s="26" t="n">
-        <v>20273515.37761906</v>
+        <v>21361167.75857144</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh dashboard Mon 06/29/2026 16:48
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -671,7 +671,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:T123"/>
+  <dimension ref="B1:T124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -706,7 +706,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 26 Jun 2026 16:39</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 29 Jun 2026 16:48</t>
         </is>
       </c>
     </row>
@@ -5827,18 +5827,12 @@
     <row r="111">
       <c r="B111" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">        Bank Guarantee SBLC Pertagas</t>
-        </is>
-      </c>
-      <c r="C111" s="9" t="n">
-        <v>-8425000</v>
-      </c>
-      <c r="D111" s="9" t="n">
-        <v>-495.5882352941176</v>
-      </c>
-      <c r="E111" s="9" t="n">
-        <v>-44576.71957671957</v>
-      </c>
+          <t xml:space="preserve">        Bank Guarantee PGN</t>
+        </is>
+      </c>
+      <c r="C111" s="9" t="n"/>
+      <c r="D111" s="9" t="n"/>
+      <c r="E111" s="9" t="n"/>
       <c r="F111" s="9" t="n"/>
       <c r="G111" s="9" t="n"/>
       <c r="H111" s="9" t="n"/>
@@ -5851,667 +5845,698 @@
       <c r="O111" s="9" t="n"/>
       <c r="P111" s="9" t="n"/>
       <c r="Q111" s="9" t="n"/>
-      <c r="R111" s="9" t="n">
+      <c r="R111" s="9" t="n"/>
+      <c r="S111" s="9" t="n"/>
+      <c r="T111" s="9" t="n"/>
+    </row>
+    <row r="112">
+      <c r="B112" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        Bank Guarantee SBLC Pertagas</t>
+        </is>
+      </c>
+      <c r="C112" s="11" t="n">
         <v>-8425000</v>
       </c>
-      <c r="S111" s="9" t="n">
+      <c r="D112" s="11" t="n">
         <v>-495.5882352941176</v>
       </c>
-      <c r="T111" s="9" t="n">
+      <c r="E112" s="11" t="n">
         <v>-44576.71957671957</v>
       </c>
-    </row>
-    <row r="112">
-      <c r="B112" s="12" t="inlineStr">
+      <c r="F112" s="11" t="n"/>
+      <c r="G112" s="11" t="n"/>
+      <c r="H112" s="11" t="n"/>
+      <c r="I112" s="11" t="n"/>
+      <c r="J112" s="11" t="n"/>
+      <c r="K112" s="11" t="n"/>
+      <c r="L112" s="11" t="n"/>
+      <c r="M112" s="11" t="n"/>
+      <c r="N112" s="11" t="n"/>
+      <c r="O112" s="11" t="n"/>
+      <c r="P112" s="11" t="n"/>
+      <c r="Q112" s="11" t="n"/>
+      <c r="R112" s="11" t="n">
+        <v>-8425000</v>
+      </c>
+      <c r="S112" s="11" t="n">
+        <v>-495.5882352941176</v>
+      </c>
+      <c r="T112" s="11" t="n">
+        <v>-44576.71957671957</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="B113" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">    TOTAL OTHERS</t>
         </is>
       </c>
-      <c r="C112" s="13" t="n">
+      <c r="C113" s="13" t="n">
         <v>-79485890</v>
       </c>
-      <c r="D112" s="13" t="n">
+      <c r="D113" s="13" t="n">
         <v>-4675.640588235294</v>
       </c>
-      <c r="E112" s="13" t="n">
+      <c r="E113" s="13" t="n">
         <v>-420560.2645502646</v>
       </c>
-      <c r="F112" s="13" t="n">
+      <c r="F113" s="13" t="n">
         <v>-44305279</v>
       </c>
-      <c r="G112" s="13" t="n">
+      <c r="G113" s="13" t="n">
         <v>-2606.192882352941</v>
       </c>
-      <c r="H112" s="13" t="n">
+      <c r="H113" s="13" t="n">
         <v>-234419.4656084656</v>
       </c>
-      <c r="I112" s="13" t="n">
+      <c r="I113" s="13" t="n">
         <v>-145625200</v>
       </c>
-      <c r="J112" s="13" t="n">
+      <c r="J113" s="13" t="n">
         <v>-8566.188235294117</v>
       </c>
-      <c r="K112" s="13" t="n">
+      <c r="K113" s="13" t="n">
         <v>-770503.7037037037</v>
       </c>
-      <c r="L112" s="13" t="n">
+      <c r="L113" s="13" t="n">
         <v>-274058059</v>
       </c>
-      <c r="M112" s="13" t="n">
+      <c r="M113" s="13" t="n">
         <v>-16121.06229411765</v>
       </c>
-      <c r="N112" s="13" t="n">
+      <c r="N113" s="13" t="n">
         <v>-1450042.64021164</v>
       </c>
-      <c r="O112" s="13" t="n">
+      <c r="O113" s="13" t="n">
         <v>-82243464</v>
       </c>
-      <c r="P112" s="13" t="n">
+      <c r="P113" s="13" t="n">
         <v>-4837.850823529412</v>
       </c>
-      <c r="Q112" s="13" t="n">
+      <c r="Q113" s="13" t="n">
         <v>-435150.6031746032</v>
       </c>
-      <c r="R112" s="13" t="n">
+      <c r="R113" s="13" t="n">
         <v>-625717892</v>
       </c>
-      <c r="S112" s="13" t="n">
+      <c r="S113" s="13" t="n">
         <v>-36806.93482352941</v>
       </c>
-      <c r="T112" s="13" t="n">
+      <c r="T113" s="13" t="n">
         <v>-3310676.677248677</v>
       </c>
     </row>
-    <row r="113">
-      <c r="B113" s="14" t="inlineStr">
+    <row r="114">
+      <c r="B114" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">    FINANCE COST</t>
         </is>
       </c>
-      <c r="C113" s="15" t="n"/>
-      <c r="D113" s="15" t="n"/>
-      <c r="E113" s="15" t="n"/>
-      <c r="F113" s="15" t="n"/>
-      <c r="G113" s="15" t="n"/>
-      <c r="H113" s="15" t="n"/>
-      <c r="I113" s="15" t="n"/>
-      <c r="J113" s="15" t="n"/>
-      <c r="K113" s="15" t="n"/>
-      <c r="L113" s="15" t="n"/>
-      <c r="M113" s="15" t="n"/>
-      <c r="N113" s="15" t="n"/>
-      <c r="O113" s="15" t="n"/>
-      <c r="P113" s="15" t="n"/>
-      <c r="Q113" s="15" t="n"/>
-      <c r="R113" s="15" t="n"/>
-      <c r="S113" s="15" t="n"/>
-      <c r="T113" s="15" t="n"/>
-    </row>
-    <row r="114">
-      <c r="B114" s="8" t="inlineStr">
+      <c r="C114" s="15" t="n"/>
+      <c r="D114" s="15" t="n"/>
+      <c r="E114" s="15" t="n"/>
+      <c r="F114" s="15" t="n"/>
+      <c r="G114" s="15" t="n"/>
+      <c r="H114" s="15" t="n"/>
+      <c r="I114" s="15" t="n"/>
+      <c r="J114" s="15" t="n"/>
+      <c r="K114" s="15" t="n"/>
+      <c r="L114" s="15" t="n"/>
+      <c r="M114" s="15" t="n"/>
+      <c r="N114" s="15" t="n"/>
+      <c r="O114" s="15" t="n"/>
+      <c r="P114" s="15" t="n"/>
+      <c r="Q114" s="15" t="n"/>
+      <c r="R114" s="15" t="n"/>
+      <c r="S114" s="15" t="n"/>
+      <c r="T114" s="15" t="n"/>
+    </row>
+    <row r="115">
+      <c r="B115" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">        Bank Charges</t>
         </is>
       </c>
-      <c r="C114" s="9" t="n">
+      <c r="C115" s="9" t="n">
         <v>-4093500.68</v>
       </c>
-      <c r="D114" s="9" t="n">
+      <c r="D115" s="9" t="n">
         <v>-240.7941576470588</v>
       </c>
-      <c r="E114" s="9" t="n">
+      <c r="E115" s="9" t="n">
         <v>-21658.73375661375</v>
       </c>
-      <c r="F114" s="9" t="n">
+      <c r="F115" s="9" t="n">
         <v>-924700</v>
       </c>
-      <c r="G114" s="9" t="n">
+      <c r="G115" s="9" t="n">
         <v>-54.39411764705882</v>
       </c>
-      <c r="H114" s="9" t="n">
+      <c r="H115" s="9" t="n">
         <v>-4892.592592592592</v>
       </c>
-      <c r="I114" s="9" t="n">
+      <c r="I115" s="9" t="n">
         <v>-3564540</v>
       </c>
-      <c r="J114" s="9" t="n">
+      <c r="J115" s="9" t="n">
         <v>-209.6788235294118</v>
       </c>
-      <c r="K114" s="9" t="n">
+      <c r="K115" s="9" t="n">
         <v>-18860</v>
       </c>
-      <c r="L114" s="9" t="n">
+      <c r="L115" s="9" t="n">
         <v>-1559098</v>
       </c>
-      <c r="M114" s="9" t="n">
+      <c r="M115" s="9" t="n">
         <v>-91.71164705882353</v>
       </c>
-      <c r="N114" s="9" t="n">
+      <c r="N115" s="9" t="n">
         <v>-8249.195767195768</v>
       </c>
-      <c r="O114" s="9" t="n">
+      <c r="O115" s="9" t="n">
         <v>-2578416</v>
       </c>
-      <c r="P114" s="9" t="n">
+      <c r="P115" s="9" t="n">
         <v>-151.6715294117647</v>
       </c>
-      <c r="Q114" s="9" t="n">
+      <c r="Q115" s="9" t="n">
         <v>-13642.4126984127</v>
       </c>
-      <c r="R114" s="9" t="n">
+      <c r="R115" s="9" t="n">
         <v>-12720254.68</v>
       </c>
-      <c r="S114" s="9" t="n">
+      <c r="S115" s="9" t="n">
         <v>-748.2502752941176</v>
       </c>
-      <c r="T114" s="9" t="n">
+      <c r="T115" s="9" t="n">
         <v>-67302.9348148148</v>
       </c>
     </row>
-    <row r="115">
-      <c r="B115" s="10" t="inlineStr">
+    <row r="116">
+      <c r="B116" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">        Forex</t>
         </is>
       </c>
-      <c r="C115" s="11" t="n">
+      <c r="C116" s="11" t="n">
         <v>-502398.6</v>
       </c>
-      <c r="D115" s="11" t="n">
+      <c r="D116" s="11" t="n">
         <v>-29.55285882352941</v>
       </c>
-      <c r="E115" s="11" t="n">
+      <c r="E116" s="11" t="n">
         <v>-2658.193650793651</v>
       </c>
-      <c r="F115" s="11" t="n"/>
-      <c r="G115" s="11" t="n"/>
-      <c r="H115" s="11" t="n"/>
-      <c r="I115" s="11" t="n">
+      <c r="F116" s="11" t="n"/>
+      <c r="G116" s="11" t="n"/>
+      <c r="H116" s="11" t="n"/>
+      <c r="I116" s="11" t="n">
         <v>-217171.16</v>
       </c>
-      <c r="J115" s="11" t="n">
+      <c r="J116" s="11" t="n">
         <v>-12.77477411764706</v>
       </c>
-      <c r="K115" s="11" t="n">
+      <c r="K116" s="11" t="n">
         <v>-1149.053756613757</v>
       </c>
-      <c r="L115" s="11" t="n"/>
-      <c r="M115" s="11" t="n"/>
-      <c r="N115" s="11" t="n"/>
-      <c r="O115" s="11" t="n">
+      <c r="L116" s="11" t="n"/>
+      <c r="M116" s="11" t="n"/>
+      <c r="N116" s="11" t="n"/>
+      <c r="O116" s="11" t="n">
         <v>-476000</v>
       </c>
-      <c r="P115" s="11" t="n">
+      <c r="P116" s="11" t="n">
         <v>-28</v>
       </c>
-      <c r="Q115" s="11" t="n">
+      <c r="Q116" s="11" t="n">
         <v>-2518.518518518519</v>
       </c>
-      <c r="R115" s="11" t="n">
+      <c r="R116" s="11" t="n">
         <v>-1195569.76</v>
       </c>
-      <c r="S115" s="11" t="n">
+      <c r="S116" s="11" t="n">
         <v>-70.32763294117646</v>
       </c>
-      <c r="T115" s="11" t="n">
+      <c r="T116" s="11" t="n">
         <v>-6325.765925925925</v>
       </c>
     </row>
-    <row r="116">
-      <c r="B116" s="8" t="inlineStr">
+    <row r="117">
+      <c r="B117" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">        Interest on Bank Term Loans</t>
         </is>
       </c>
-      <c r="C116" s="9" t="n">
+      <c r="C117" s="9" t="n">
         <v>-304089642.44</v>
       </c>
-      <c r="D116" s="9" t="n">
+      <c r="D117" s="9" t="n">
         <v>-17887.62602588235</v>
       </c>
-      <c r="E116" s="9" t="n">
+      <c r="E117" s="9" t="n">
         <v>-1608939.907089947</v>
       </c>
-      <c r="F116" s="9" t="n">
+      <c r="F117" s="9" t="n">
         <v>-192548915.91</v>
       </c>
-      <c r="G116" s="9" t="n">
+      <c r="G117" s="9" t="n">
         <v>-11326.40681823529</v>
       </c>
-      <c r="H116" s="9" t="n">
+      <c r="H117" s="9" t="n">
         <v>-1018777.332857143</v>
       </c>
-      <c r="I116" s="9" t="n">
+      <c r="I117" s="9" t="n">
         <v>-154772188.99</v>
       </c>
-      <c r="J116" s="9" t="n">
+      <c r="J117" s="9" t="n">
         <v>-9104.246411176471</v>
       </c>
-      <c r="K116" s="9" t="n">
+      <c r="K117" s="9" t="n">
         <v>-818900.4708465609</v>
       </c>
-      <c r="L116" s="9" t="n">
+      <c r="L117" s="9" t="n">
         <v>-185501545.14</v>
       </c>
-      <c r="M116" s="9" t="n">
+      <c r="M117" s="9" t="n">
         <v>-10911.85559647059</v>
       </c>
-      <c r="N116" s="9" t="n">
+      <c r="N117" s="9" t="n">
         <v>-981489.6568253967</v>
       </c>
-      <c r="O116" s="9" t="n">
+      <c r="O117" s="9" t="n">
         <v>-2857131528.42</v>
       </c>
-      <c r="P116" s="9" t="n">
+      <c r="P117" s="9" t="n">
         <v>-168066.5604952941</v>
       </c>
-      <c r="Q116" s="9" t="n">
+      <c r="Q117" s="9" t="n">
         <v>-15117098.03396825</v>
       </c>
-      <c r="R116" s="9" t="n">
+      <c r="R117" s="9" t="n">
         <v>-3694043820.9</v>
       </c>
-      <c r="S116" s="9" t="n">
+      <c r="S117" s="9" t="n">
         <v>-217296.6953470588</v>
       </c>
-      <c r="T116" s="9" t="n">
+      <c r="T117" s="9" t="n">
         <v>-19545205.4015873</v>
       </c>
     </row>
-    <row r="117">
-      <c r="B117" s="10" t="inlineStr">
+    <row r="118">
+      <c r="B118" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">        Interest on Bank Working Capital Loans</t>
         </is>
       </c>
-      <c r="C117" s="11" t="n"/>
-      <c r="D117" s="11" t="n"/>
-      <c r="E117" s="11" t="n"/>
-      <c r="F117" s="11" t="n"/>
-      <c r="G117" s="11" t="n"/>
-      <c r="H117" s="11" t="n"/>
-      <c r="I117" s="11" t="n">
+      <c r="C118" s="11" t="n"/>
+      <c r="D118" s="11" t="n"/>
+      <c r="E118" s="11" t="n"/>
+      <c r="F118" s="11" t="n"/>
+      <c r="G118" s="11" t="n"/>
+      <c r="H118" s="11" t="n"/>
+      <c r="I118" s="11" t="n">
         <v>-268756578</v>
       </c>
-      <c r="J117" s="11" t="n">
+      <c r="J118" s="11" t="n">
         <v>-15809.21047058824</v>
       </c>
-      <c r="K117" s="11" t="n">
+      <c r="K118" s="11" t="n">
         <v>-1421992.476190476</v>
       </c>
-      <c r="L117" s="11" t="n">
+      <c r="L118" s="11" t="n">
         <v>-171119871</v>
       </c>
-      <c r="M117" s="11" t="n">
+      <c r="M118" s="11" t="n">
         <v>-10065.87476470588</v>
       </c>
-      <c r="N117" s="11" t="n">
+      <c r="N118" s="11" t="n">
         <v>-905396.1428571428</v>
       </c>
-      <c r="O117" s="11" t="n">
+      <c r="O118" s="11" t="n">
         <v>-96386746</v>
       </c>
-      <c r="P117" s="11" t="n">
+      <c r="P118" s="11" t="n">
         <v>-5669.808588235294</v>
       </c>
-      <c r="Q117" s="11" t="n">
+      <c r="Q118" s="11" t="n">
         <v>-509982.7830687831</v>
       </c>
-      <c r="R117" s="11" t="n">
+      <c r="R118" s="11" t="n">
         <v>-536263195</v>
       </c>
-      <c r="S117" s="11" t="n">
+      <c r="S118" s="11" t="n">
         <v>-31544.89382352941</v>
       </c>
-      <c r="T117" s="11" t="n">
+      <c r="T118" s="11" t="n">
         <v>-2837371.402116402</v>
       </c>
     </row>
-    <row r="118">
-      <c r="B118" s="8" t="inlineStr">
+    <row r="119">
+      <c r="B119" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">        Loan Related Charges</t>
         </is>
       </c>
-      <c r="C118" s="9" t="n"/>
-      <c r="D118" s="9" t="n"/>
-      <c r="E118" s="9" t="n"/>
-      <c r="F118" s="9" t="n">
+      <c r="C119" s="9" t="n"/>
+      <c r="D119" s="9" t="n"/>
+      <c r="E119" s="9" t="n"/>
+      <c r="F119" s="9" t="n">
         <v>-773891532</v>
       </c>
-      <c r="G118" s="9" t="n">
+      <c r="G119" s="9" t="n">
         <v>-45523.03129411765</v>
       </c>
-      <c r="H118" s="9" t="n">
+      <c r="H119" s="9" t="n">
         <v>-4094664.19047619</v>
       </c>
-      <c r="I118" s="9" t="n">
+      <c r="I119" s="9" t="n">
         <v>-19344233</v>
       </c>
-      <c r="J118" s="9" t="n">
+      <c r="J119" s="9" t="n">
         <v>-1137.896058823529</v>
       </c>
-      <c r="K118" s="9" t="n">
+      <c r="K119" s="9" t="n">
         <v>-102350.4391534391</v>
       </c>
-      <c r="L118" s="9" t="n"/>
-      <c r="M118" s="9" t="n"/>
-      <c r="N118" s="9" t="n"/>
-      <c r="O118" s="9" t="n"/>
-      <c r="P118" s="9" t="n"/>
-      <c r="Q118" s="9" t="n"/>
-      <c r="R118" s="9" t="n">
+      <c r="L119" s="9" t="n"/>
+      <c r="M119" s="9" t="n"/>
+      <c r="N119" s="9" t="n"/>
+      <c r="O119" s="9" t="n"/>
+      <c r="P119" s="9" t="n"/>
+      <c r="Q119" s="9" t="n"/>
+      <c r="R119" s="9" t="n">
         <v>-793235765</v>
       </c>
-      <c r="S118" s="9" t="n">
+      <c r="S119" s="9" t="n">
         <v>-46660.92735294117</v>
       </c>
-      <c r="T118" s="9" t="n">
+      <c r="T119" s="9" t="n">
         <v>-4197014.62962963</v>
       </c>
     </row>
-    <row r="119">
-      <c r="B119" s="12" t="inlineStr">
+    <row r="120">
+      <c r="B120" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">    TOTAL FINANCE COST</t>
         </is>
       </c>
-      <c r="C119" s="13" t="n">
+      <c r="C120" s="13" t="n">
         <v>-308685541.72</v>
       </c>
-      <c r="D119" s="13" t="n">
+      <c r="D120" s="13" t="n">
         <v>-18157.97304235294</v>
       </c>
-      <c r="E119" s="13" t="n">
+      <c r="E120" s="13" t="n">
         <v>-1633256.834497354</v>
       </c>
-      <c r="F119" s="13" t="n">
+      <c r="F120" s="13" t="n">
         <v>-967365147.9100001</v>
       </c>
-      <c r="G119" s="13" t="n">
+      <c r="G120" s="13" t="n">
         <v>-56903.83223000001</v>
       </c>
-      <c r="H119" s="13" t="n">
+      <c r="H120" s="13" t="n">
         <v>-5118334.115925927</v>
       </c>
-      <c r="I119" s="13" t="n">
+      <c r="I120" s="13" t="n">
         <v>-446654711.15</v>
       </c>
-      <c r="J119" s="13" t="n">
+      <c r="J120" s="13" t="n">
         <v>-26273.8065382353</v>
       </c>
-      <c r="K119" s="13" t="n">
+      <c r="K120" s="13" t="n">
         <v>-2363252.43994709</v>
       </c>
-      <c r="L119" s="13" t="n">
+      <c r="L120" s="13" t="n">
         <v>-358180514.14</v>
       </c>
-      <c r="M119" s="13" t="n">
+      <c r="M120" s="13" t="n">
         <v>-21069.44200823529</v>
       </c>
-      <c r="N119" s="13" t="n">
+      <c r="N120" s="13" t="n">
         <v>-1895134.995449735</v>
       </c>
-      <c r="O119" s="13" t="n">
+      <c r="O120" s="13" t="n">
         <v>-2956572690.42</v>
       </c>
-      <c r="P119" s="13" t="n">
+      <c r="P120" s="13" t="n">
         <v>-173916.0406129412</v>
       </c>
-      <c r="Q119" s="13" t="n">
+      <c r="Q120" s="13" t="n">
         <v>-15643241.74825397</v>
       </c>
-      <c r="R119" s="13" t="n">
+      <c r="R120" s="13" t="n">
         <v>-5037458605.34</v>
       </c>
-      <c r="S119" s="13" t="n">
+      <c r="S120" s="13" t="n">
         <v>-296321.0944317647</v>
       </c>
-      <c r="T119" s="13" t="n">
+      <c r="T120" s="13" t="n">
         <v>-26653220.13407408</v>
-      </c>
-    </row>
-    <row r="120">
-      <c r="B120" s="16" t="inlineStr">
-        <is>
-          <t>TOTAL OUTFLOW</t>
-        </is>
-      </c>
-      <c r="C120" s="17" t="n">
-        <v>-44493158195.03</v>
-      </c>
-      <c r="D120" s="17" t="n">
-        <v>-2617244.599707647</v>
-      </c>
-      <c r="E120" s="17" t="n">
-        <v>-235413535.4234391</v>
-      </c>
-      <c r="F120" s="17" t="n">
-        <v>-87290805698.13</v>
-      </c>
-      <c r="G120" s="17" t="n">
-        <v>-5134753.276360588</v>
-      </c>
-      <c r="H120" s="17" t="n">
-        <v>-461856114.8049207</v>
-      </c>
-      <c r="I120" s="17" t="n">
-        <v>-56595899794.15</v>
-      </c>
-      <c r="J120" s="17" t="n">
-        <v>-3329170.576126471</v>
-      </c>
-      <c r="K120" s="17" t="n">
-        <v>-299449205.2600529</v>
-      </c>
-      <c r="L120" s="17" t="n">
-        <v>-47009379649.2</v>
-      </c>
-      <c r="M120" s="17" t="n">
-        <v>-2765257.626423529</v>
-      </c>
-      <c r="N120" s="17" t="n">
-        <v>-248726876.4507936</v>
-      </c>
-      <c r="O120" s="17" t="n">
-        <v>-27914586083.82</v>
-      </c>
-      <c r="P120" s="17" t="n">
-        <v>-1642034.475518824</v>
-      </c>
-      <c r="Q120" s="17" t="n">
-        <v>-147696222.6657143</v>
-      </c>
-      <c r="R120" s="17" t="n">
-        <v>-263303829420.33</v>
-      </c>
-      <c r="S120" s="17" t="n">
-        <v>-15488460.55413706</v>
-      </c>
-      <c r="T120" s="17" t="n">
-        <v>-1393141954.604921</v>
       </c>
     </row>
     <row r="121">
       <c r="B121" s="16" t="inlineStr">
         <is>
+          <t>TOTAL OUTFLOW</t>
+        </is>
+      </c>
+      <c r="C121" s="17" t="n">
+        <v>-44493158195.03</v>
+      </c>
+      <c r="D121" s="17" t="n">
+        <v>-2617244.599707647</v>
+      </c>
+      <c r="E121" s="17" t="n">
+        <v>-235413535.4234391</v>
+      </c>
+      <c r="F121" s="17" t="n">
+        <v>-87290805698.13</v>
+      </c>
+      <c r="G121" s="17" t="n">
+        <v>-5134753.276360588</v>
+      </c>
+      <c r="H121" s="17" t="n">
+        <v>-461856114.8049207</v>
+      </c>
+      <c r="I121" s="17" t="n">
+        <v>-56595899794.15</v>
+      </c>
+      <c r="J121" s="17" t="n">
+        <v>-3329170.576126471</v>
+      </c>
+      <c r="K121" s="17" t="n">
+        <v>-299449205.2600529</v>
+      </c>
+      <c r="L121" s="17" t="n">
+        <v>-47009379649.2</v>
+      </c>
+      <c r="M121" s="17" t="n">
+        <v>-2765257.626423529</v>
+      </c>
+      <c r="N121" s="17" t="n">
+        <v>-248726876.4507936</v>
+      </c>
+      <c r="O121" s="17" t="n">
+        <v>-27914586083.82</v>
+      </c>
+      <c r="P121" s="17" t="n">
+        <v>-1642034.475518824</v>
+      </c>
+      <c r="Q121" s="17" t="n">
+        <v>-147696222.6657143</v>
+      </c>
+      <c r="R121" s="17" t="n">
+        <v>-263303829420.33</v>
+      </c>
+      <c r="S121" s="17" t="n">
+        <v>-15488460.55413706</v>
+      </c>
+      <c r="T121" s="17" t="n">
+        <v>-1393141954.604921</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="B122" s="16" t="inlineStr">
+        <is>
           <t>NET CASH SURPLUS (LOSS)</t>
         </is>
       </c>
-      <c r="C121" s="17" t="n">
+      <c r="C122" s="17" t="n">
         <v>11812902160.24</v>
       </c>
-      <c r="D121" s="17" t="n">
+      <c r="D122" s="17" t="n">
         <v>694876.5976611763</v>
       </c>
-      <c r="E121" s="17" t="n">
+      <c r="E122" s="17" t="n">
         <v>62502127.83195766</v>
       </c>
-      <c r="F121" s="17" t="n">
+      <c r="F122" s="17" t="n">
         <v>-75526959730.20001</v>
       </c>
-      <c r="G121" s="17" t="n">
+      <c r="G122" s="17" t="n">
         <v>-4442762.337070589</v>
       </c>
-      <c r="H121" s="17" t="n">
+      <c r="H122" s="17" t="n">
         <v>-399613543.5460318</v>
       </c>
-      <c r="I121" s="17" t="n">
+      <c r="I122" s="17" t="n">
         <v>2573810161.360001</v>
       </c>
-      <c r="J121" s="17" t="n">
+      <c r="J122" s="17" t="n">
         <v>151400.5977270589</v>
       </c>
-      <c r="K121" s="17" t="n">
+      <c r="K122" s="17" t="n">
         <v>13618043.18179894</v>
       </c>
-      <c r="L121" s="17" t="n">
+      <c r="L122" s="17" t="n">
         <v>11041904011.41</v>
       </c>
-      <c r="M121" s="17" t="n">
+      <c r="M122" s="17" t="n">
         <v>649523.765377059</v>
       </c>
-      <c r="N121" s="17" t="n">
+      <c r="N122" s="17" t="n">
         <v>58422772.54714288</v>
       </c>
-      <c r="O121" s="17" t="n">
+      <c r="O122" s="17" t="n">
         <v>-15435413590.8</v>
       </c>
-      <c r="P121" s="17" t="n">
+      <c r="P122" s="17" t="n">
         <v>-907965.5053411764</v>
       </c>
-      <c r="Q121" s="17" t="n">
+      <c r="Q122" s="17" t="n">
         <v>-81668854.97777778</v>
       </c>
-      <c r="R121" s="17" t="n">
+      <c r="R122" s="17" t="n">
         <v>-65533756987.99001</v>
       </c>
-      <c r="S121" s="17" t="n">
+      <c r="S122" s="17" t="n">
         <v>-3854926.881646471</v>
       </c>
-      <c r="T121" s="17" t="n">
+      <c r="T122" s="17" t="n">
         <v>-346739454.9629102</v>
       </c>
     </row>
-    <row r="122">
-      <c r="B122" s="14" t="inlineStr">
+    <row r="123">
+      <c r="B123" s="14" t="inlineStr">
         <is>
           <t>BEGINNING BALANCE</t>
         </is>
       </c>
-      <c r="C122" s="15" t="n">
+      <c r="C123" s="15" t="n">
         <v>67473660826.36001</v>
       </c>
-      <c r="D122" s="15" t="n">
+      <c r="D123" s="15" t="n">
         <v>3969038.872138824</v>
       </c>
-      <c r="E122" s="15" t="n">
+      <c r="E123" s="15" t="n">
         <v>357003496.4357672</v>
       </c>
-      <c r="F122" s="15" t="n">
+      <c r="F123" s="15" t="n">
         <v>79286562986.60001</v>
       </c>
-      <c r="G122" s="15" t="n">
+      <c r="G123" s="15" t="n">
         <v>4663915.4698</v>
       </c>
-      <c r="H122" s="15" t="n">
+      <c r="H123" s="15" t="n">
         <v>419505624.2677249</v>
       </c>
-      <c r="I122" s="15" t="n">
+      <c r="I123" s="15" t="n">
         <v>3759603256.400002</v>
       </c>
-      <c r="J122" s="15" t="n">
+      <c r="J123" s="15" t="n">
         <v>221153.1327294119</v>
       </c>
-      <c r="K122" s="15" t="n">
+      <c r="K123" s="15" t="n">
         <v>19892080.72169314</v>
       </c>
-      <c r="L122" s="15" t="n">
+      <c r="L123" s="15" t="n">
         <v>6333413418.760002</v>
       </c>
-      <c r="M122" s="15" t="n">
+      <c r="M123" s="15" t="n">
         <v>372553.7305152942</v>
       </c>
-      <c r="N122" s="15" t="n">
+      <c r="N123" s="15" t="n">
         <v>33510123.90878308</v>
       </c>
-      <c r="O122" s="15" t="n">
+      <c r="O123" s="15" t="n">
         <v>17375317430.17</v>
       </c>
-      <c r="P122" s="15" t="n">
+      <c r="P123" s="15" t="n">
         <v>1022077.495892353</v>
       </c>
-      <c r="Q122" s="15" t="n">
+      <c r="Q123" s="15" t="n">
         <v>91932896.45592594</v>
       </c>
-      <c r="R122" s="15" t="n">
+      <c r="R123" s="15" t="n">
         <v>67473660826.36001</v>
       </c>
-      <c r="S122" s="15" t="n">
+      <c r="S123" s="15" t="n">
         <v>3969038.872138824</v>
       </c>
-      <c r="T122" s="15" t="n">
+      <c r="T123" s="15" t="n">
         <v>357003496.4357672</v>
       </c>
     </row>
-    <row r="123">
-      <c r="B123" s="16" t="inlineStr">
+    <row r="124">
+      <c r="B124" s="16" t="inlineStr">
         <is>
           <t>ENDING BALANCE</t>
         </is>
       </c>
-      <c r="C123" s="17" t="n">
+      <c r="C124" s="17" t="n">
         <v>79286562986.60001</v>
       </c>
-      <c r="D123" s="17" t="n">
+      <c r="D124" s="17" t="n">
         <v>4663915.4698</v>
       </c>
-      <c r="E123" s="17" t="n">
+      <c r="E124" s="17" t="n">
         <v>419505624.2677249</v>
       </c>
-      <c r="F123" s="17" t="n">
+      <c r="F124" s="17" t="n">
         <v>3759603256.399994</v>
       </c>
-      <c r="G123" s="17" t="n">
+      <c r="G124" s="17" t="n">
         <v>221153.1327294114</v>
       </c>
-      <c r="H123" s="17" t="n">
+      <c r="H124" s="17" t="n">
         <v>19892080.72169309</v>
       </c>
-      <c r="I123" s="17" t="n">
+      <c r="I124" s="17" t="n">
         <v>6333413417.760003</v>
       </c>
-      <c r="J123" s="17" t="n">
+      <c r="J124" s="17" t="n">
         <v>372553.7304564707</v>
       </c>
-      <c r="K123" s="17" t="n">
+      <c r="K124" s="17" t="n">
         <v>33510123.90349208</v>
       </c>
-      <c r="L123" s="17" t="n">
+      <c r="L124" s="17" t="n">
         <v>17375317430.17001</v>
       </c>
-      <c r="M123" s="17" t="n">
+      <c r="M124" s="17" t="n">
         <v>1022077.495892353</v>
       </c>
-      <c r="N123" s="17" t="n">
+      <c r="N124" s="17" t="n">
         <v>91932896.45592596</v>
       </c>
-      <c r="O123" s="17" t="n">
+      <c r="O124" s="17" t="n">
         <v>1939903839.370003</v>
       </c>
-      <c r="P123" s="17" t="n">
+      <c r="P124" s="17" t="n">
         <v>114111.9905511766</v>
       </c>
-      <c r="Q123" s="17" t="n">
+      <c r="Q124" s="17" t="n">
         <v>10264041.47814816</v>
       </c>
-      <c r="R123" s="17" t="n">
+      <c r="R124" s="17" t="n">
         <v>1939903839.370003</v>
       </c>
-      <c r="S123" s="17" t="n">
+      <c r="S124" s="17" t="n">
         <v>114111.9905511766</v>
       </c>
-      <c r="T123" s="17" t="n">
+      <c r="T124" s="17" t="n">
         <v>10264041.47814816</v>
       </c>
     </row>
@@ -6539,7 +6564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:T123"/>
+  <dimension ref="B1:T124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -6574,7 +6599,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 26 Jun 2026 16:39 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 29 Jun 2026 16:48 (in IDR Million)</t>
         </is>
       </c>
     </row>
@@ -11695,18 +11720,12 @@
     <row r="111">
       <c r="B111" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">        Bank Guarantee SBLC Pertagas</t>
-        </is>
-      </c>
-      <c r="C111" s="9" t="n">
-        <v>-8.425000000000001</v>
-      </c>
-      <c r="D111" s="9" t="n">
-        <v>-0.0004955882352941177</v>
-      </c>
-      <c r="E111" s="9" t="n">
-        <v>-0.04457671957671958</v>
-      </c>
+          <t xml:space="preserve">        Bank Guarantee PGN</t>
+        </is>
+      </c>
+      <c r="C111" s="9" t="n"/>
+      <c r="D111" s="9" t="n"/>
+      <c r="E111" s="9" t="n"/>
       <c r="F111" s="9" t="n"/>
       <c r="G111" s="9" t="n"/>
       <c r="H111" s="9" t="n"/>
@@ -11719,667 +11738,698 @@
       <c r="O111" s="9" t="n"/>
       <c r="P111" s="9" t="n"/>
       <c r="Q111" s="9" t="n"/>
-      <c r="R111" s="9" t="n">
+      <c r="R111" s="9" t="n"/>
+      <c r="S111" s="9" t="n"/>
+      <c r="T111" s="9" t="n"/>
+    </row>
+    <row r="112">
+      <c r="B112" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        Bank Guarantee SBLC Pertagas</t>
+        </is>
+      </c>
+      <c r="C112" s="11" t="n">
         <v>-8.425000000000001</v>
       </c>
-      <c r="S111" s="9" t="n">
+      <c r="D112" s="11" t="n">
         <v>-0.0004955882352941177</v>
       </c>
-      <c r="T111" s="9" t="n">
+      <c r="E112" s="11" t="n">
         <v>-0.04457671957671958</v>
       </c>
-    </row>
-    <row r="112">
-      <c r="B112" s="12" t="inlineStr">
+      <c r="F112" s="11" t="n"/>
+      <c r="G112" s="11" t="n"/>
+      <c r="H112" s="11" t="n"/>
+      <c r="I112" s="11" t="n"/>
+      <c r="J112" s="11" t="n"/>
+      <c r="K112" s="11" t="n"/>
+      <c r="L112" s="11" t="n"/>
+      <c r="M112" s="11" t="n"/>
+      <c r="N112" s="11" t="n"/>
+      <c r="O112" s="11" t="n"/>
+      <c r="P112" s="11" t="n"/>
+      <c r="Q112" s="11" t="n"/>
+      <c r="R112" s="11" t="n">
+        <v>-8.425000000000001</v>
+      </c>
+      <c r="S112" s="11" t="n">
+        <v>-0.0004955882352941177</v>
+      </c>
+      <c r="T112" s="11" t="n">
+        <v>-0.04457671957671958</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="B113" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">    TOTAL OTHERS</t>
         </is>
       </c>
-      <c r="C112" s="13" t="n">
+      <c r="C113" s="13" t="n">
         <v>-79.48589</v>
       </c>
-      <c r="D112" s="13" t="n">
+      <c r="D113" s="13" t="n">
         <v>-0.004675640588235294</v>
       </c>
-      <c r="E112" s="13" t="n">
+      <c r="E113" s="13" t="n">
         <v>-0.4205602645502645</v>
       </c>
-      <c r="F112" s="13" t="n">
+      <c r="F113" s="13" t="n">
         <v>-44.305279</v>
       </c>
-      <c r="G112" s="13" t="n">
+      <c r="G113" s="13" t="n">
         <v>-0.002606192882352941</v>
       </c>
-      <c r="H112" s="13" t="n">
+      <c r="H113" s="13" t="n">
         <v>-0.2344194656084656</v>
       </c>
-      <c r="I112" s="13" t="n">
+      <c r="I113" s="13" t="n">
         <v>-145.6252</v>
       </c>
-      <c r="J112" s="13" t="n">
+      <c r="J113" s="13" t="n">
         <v>-0.008566188235294118</v>
       </c>
-      <c r="K112" s="13" t="n">
+      <c r="K113" s="13" t="n">
         <v>-0.7705037037037037</v>
       </c>
-      <c r="L112" s="13" t="n">
+      <c r="L113" s="13" t="n">
         <v>-274.058059</v>
       </c>
-      <c r="M112" s="13" t="n">
+      <c r="M113" s="13" t="n">
         <v>-0.01612106229411765</v>
       </c>
-      <c r="N112" s="13" t="n">
+      <c r="N113" s="13" t="n">
         <v>-1.45004264021164</v>
       </c>
-      <c r="O112" s="13" t="n">
+      <c r="O113" s="13" t="n">
         <v>-82.243464</v>
       </c>
-      <c r="P112" s="13" t="n">
+      <c r="P113" s="13" t="n">
         <v>-0.004837850823529412</v>
       </c>
-      <c r="Q112" s="13" t="n">
+      <c r="Q113" s="13" t="n">
         <v>-0.4351506031746032</v>
       </c>
-      <c r="R112" s="13" t="n">
+      <c r="R113" s="13" t="n">
         <v>-625.717892</v>
       </c>
-      <c r="S112" s="13" t="n">
+      <c r="S113" s="13" t="n">
         <v>-0.03680693482352941</v>
       </c>
-      <c r="T112" s="13" t="n">
+      <c r="T113" s="13" t="n">
         <v>-3.310676677248677</v>
       </c>
     </row>
-    <row r="113">
-      <c r="B113" s="14" t="inlineStr">
+    <row r="114">
+      <c r="B114" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">    FINANCE COST</t>
         </is>
       </c>
-      <c r="C113" s="15" t="n"/>
-      <c r="D113" s="15" t="n"/>
-      <c r="E113" s="15" t="n"/>
-      <c r="F113" s="15" t="n"/>
-      <c r="G113" s="15" t="n"/>
-      <c r="H113" s="15" t="n"/>
-      <c r="I113" s="15" t="n"/>
-      <c r="J113" s="15" t="n"/>
-      <c r="K113" s="15" t="n"/>
-      <c r="L113" s="15" t="n"/>
-      <c r="M113" s="15" t="n"/>
-      <c r="N113" s="15" t="n"/>
-      <c r="O113" s="15" t="n"/>
-      <c r="P113" s="15" t="n"/>
-      <c r="Q113" s="15" t="n"/>
-      <c r="R113" s="15" t="n"/>
-      <c r="S113" s="15" t="n"/>
-      <c r="T113" s="15" t="n"/>
-    </row>
-    <row r="114">
-      <c r="B114" s="8" t="inlineStr">
+      <c r="C114" s="15" t="n"/>
+      <c r="D114" s="15" t="n"/>
+      <c r="E114" s="15" t="n"/>
+      <c r="F114" s="15" t="n"/>
+      <c r="G114" s="15" t="n"/>
+      <c r="H114" s="15" t="n"/>
+      <c r="I114" s="15" t="n"/>
+      <c r="J114" s="15" t="n"/>
+      <c r="K114" s="15" t="n"/>
+      <c r="L114" s="15" t="n"/>
+      <c r="M114" s="15" t="n"/>
+      <c r="N114" s="15" t="n"/>
+      <c r="O114" s="15" t="n"/>
+      <c r="P114" s="15" t="n"/>
+      <c r="Q114" s="15" t="n"/>
+      <c r="R114" s="15" t="n"/>
+      <c r="S114" s="15" t="n"/>
+      <c r="T114" s="15" t="n"/>
+    </row>
+    <row r="115">
+      <c r="B115" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">        Bank Charges</t>
         </is>
       </c>
-      <c r="C114" s="9" t="n">
+      <c r="C115" s="9" t="n">
         <v>-4.09350068</v>
       </c>
-      <c r="D114" s="9" t="n">
+      <c r="D115" s="9" t="n">
         <v>-0.0002407941576470588</v>
       </c>
-      <c r="E114" s="9" t="n">
+      <c r="E115" s="9" t="n">
         <v>-0.02165873375661376</v>
       </c>
-      <c r="F114" s="9" t="n">
+      <c r="F115" s="9" t="n">
         <v>-0.9247</v>
       </c>
-      <c r="G114" s="9" t="n">
+      <c r="G115" s="9" t="n">
         <v>-5.439411764705882e-05</v>
       </c>
-      <c r="H114" s="9" t="n">
+      <c r="H115" s="9" t="n">
         <v>-0.004892592592592592</v>
       </c>
-      <c r="I114" s="9" t="n">
+      <c r="I115" s="9" t="n">
         <v>-3.56454</v>
       </c>
-      <c r="J114" s="9" t="n">
+      <c r="J115" s="9" t="n">
         <v>-0.0002096788235294118</v>
       </c>
-      <c r="K114" s="9" t="n">
+      <c r="K115" s="9" t="n">
         <v>-0.01886</v>
       </c>
-      <c r="L114" s="9" t="n">
+      <c r="L115" s="9" t="n">
         <v>-1.559098</v>
       </c>
-      <c r="M114" s="9" t="n">
+      <c r="M115" s="9" t="n">
         <v>-9.171164705882353e-05</v>
       </c>
-      <c r="N114" s="9" t="n">
+      <c r="N115" s="9" t="n">
         <v>-0.008249195767195768</v>
       </c>
-      <c r="O114" s="9" t="n">
+      <c r="O115" s="9" t="n">
         <v>-2.578416</v>
       </c>
-      <c r="P114" s="9" t="n">
+      <c r="P115" s="9" t="n">
         <v>-0.0001516715294117647</v>
       </c>
-      <c r="Q114" s="9" t="n">
+      <c r="Q115" s="9" t="n">
         <v>-0.0136424126984127</v>
       </c>
-      <c r="R114" s="9" t="n">
+      <c r="R115" s="9" t="n">
         <v>-12.72025468</v>
       </c>
-      <c r="S114" s="9" t="n">
+      <c r="S115" s="9" t="n">
         <v>-0.0007482502752941177</v>
       </c>
-      <c r="T114" s="9" t="n">
+      <c r="T115" s="9" t="n">
         <v>-0.06730293481481482</v>
       </c>
     </row>
-    <row r="115">
-      <c r="B115" s="10" t="inlineStr">
+    <row r="116">
+      <c r="B116" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">        Forex</t>
         </is>
       </c>
-      <c r="C115" s="11" t="n">
+      <c r="C116" s="11" t="n">
         <v>-0.5023986</v>
       </c>
-      <c r="D115" s="11" t="n">
+      <c r="D116" s="11" t="n">
         <v>-2.955285882352941e-05</v>
       </c>
-      <c r="E115" s="11" t="n">
+      <c r="E116" s="11" t="n">
         <v>-0.002658193650793651</v>
       </c>
-      <c r="F115" s="11" t="n"/>
-      <c r="G115" s="11" t="n"/>
-      <c r="H115" s="11" t="n"/>
-      <c r="I115" s="11" t="n">
+      <c r="F116" s="11" t="n"/>
+      <c r="G116" s="11" t="n"/>
+      <c r="H116" s="11" t="n"/>
+      <c r="I116" s="11" t="n">
         <v>-0.21717116</v>
       </c>
-      <c r="J115" s="11" t="n">
+      <c r="J116" s="11" t="n">
         <v>-1.277477411764706e-05</v>
       </c>
-      <c r="K115" s="11" t="n">
+      <c r="K116" s="11" t="n">
         <v>-0.001149053756613757</v>
       </c>
-      <c r="L115" s="11" t="n"/>
-      <c r="M115" s="11" t="n"/>
-      <c r="N115" s="11" t="n"/>
-      <c r="O115" s="11" t="n">
+      <c r="L116" s="11" t="n"/>
+      <c r="M116" s="11" t="n"/>
+      <c r="N116" s="11" t="n"/>
+      <c r="O116" s="11" t="n">
         <v>-0.476</v>
       </c>
-      <c r="P115" s="11" t="n">
+      <c r="P116" s="11" t="n">
         <v>-2.8e-05</v>
       </c>
-      <c r="Q115" s="11" t="n">
+      <c r="Q116" s="11" t="n">
         <v>-0.002518518518518518</v>
       </c>
-      <c r="R115" s="11" t="n">
+      <c r="R116" s="11" t="n">
         <v>-1.19556976</v>
       </c>
-      <c r="S115" s="11" t="n">
+      <c r="S116" s="11" t="n">
         <v>-7.032763294117647e-05</v>
       </c>
-      <c r="T115" s="11" t="n">
+      <c r="T116" s="11" t="n">
         <v>-0.006325765925925926</v>
       </c>
     </row>
-    <row r="116">
-      <c r="B116" s="8" t="inlineStr">
+    <row r="117">
+      <c r="B117" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">        Interest on Bank Term Loans</t>
         </is>
       </c>
-      <c r="C116" s="9" t="n">
+      <c r="C117" s="9" t="n">
         <v>-304.08964244</v>
       </c>
-      <c r="D116" s="9" t="n">
+      <c r="D117" s="9" t="n">
         <v>-0.01788762602588235</v>
       </c>
-      <c r="E116" s="9" t="n">
+      <c r="E117" s="9" t="n">
         <v>-1.608939907089947</v>
       </c>
-      <c r="F116" s="9" t="n">
+      <c r="F117" s="9" t="n">
         <v>-192.54891591</v>
       </c>
-      <c r="G116" s="9" t="n">
+      <c r="G117" s="9" t="n">
         <v>-0.01132640681823529</v>
       </c>
-      <c r="H116" s="9" t="n">
+      <c r="H117" s="9" t="n">
         <v>-1.018777332857143</v>
       </c>
-      <c r="I116" s="9" t="n">
+      <c r="I117" s="9" t="n">
         <v>-154.77218899</v>
       </c>
-      <c r="J116" s="9" t="n">
+      <c r="J117" s="9" t="n">
         <v>-0.009104246411176471</v>
       </c>
-      <c r="K116" s="9" t="n">
+      <c r="K117" s="9" t="n">
         <v>-0.8189004708465609</v>
       </c>
-      <c r="L116" s="9" t="n">
+      <c r="L117" s="9" t="n">
         <v>-185.50154514</v>
       </c>
-      <c r="M116" s="9" t="n">
+      <c r="M117" s="9" t="n">
         <v>-0.01091185559647059</v>
       </c>
-      <c r="N116" s="9" t="n">
+      <c r="N117" s="9" t="n">
         <v>-0.9814896568253968</v>
       </c>
-      <c r="O116" s="9" t="n">
+      <c r="O117" s="9" t="n">
         <v>-2857.13152842</v>
       </c>
-      <c r="P116" s="9" t="n">
+      <c r="P117" s="9" t="n">
         <v>-0.1680665604952941</v>
       </c>
-      <c r="Q116" s="9" t="n">
+      <c r="Q117" s="9" t="n">
         <v>-15.11709803396825</v>
       </c>
-      <c r="R116" s="9" t="n">
+      <c r="R117" s="9" t="n">
         <v>-3694.0438209</v>
       </c>
-      <c r="S116" s="9" t="n">
+      <c r="S117" s="9" t="n">
         <v>-0.2172966953470588</v>
       </c>
-      <c r="T116" s="9" t="n">
+      <c r="T117" s="9" t="n">
         <v>-19.5452054015873</v>
       </c>
     </row>
-    <row r="117">
-      <c r="B117" s="10" t="inlineStr">
+    <row r="118">
+      <c r="B118" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">        Interest on Bank Working Capital Loans</t>
         </is>
       </c>
-      <c r="C117" s="11" t="n"/>
-      <c r="D117" s="11" t="n"/>
-      <c r="E117" s="11" t="n"/>
-      <c r="F117" s="11" t="n"/>
-      <c r="G117" s="11" t="n"/>
-      <c r="H117" s="11" t="n"/>
-      <c r="I117" s="11" t="n">
+      <c r="C118" s="11" t="n"/>
+      <c r="D118" s="11" t="n"/>
+      <c r="E118" s="11" t="n"/>
+      <c r="F118" s="11" t="n"/>
+      <c r="G118" s="11" t="n"/>
+      <c r="H118" s="11" t="n"/>
+      <c r="I118" s="11" t="n">
         <v>-268.756578</v>
       </c>
-      <c r="J117" s="11" t="n">
+      <c r="J118" s="11" t="n">
         <v>-0.01580921047058824</v>
       </c>
-      <c r="K117" s="11" t="n">
+      <c r="K118" s="11" t="n">
         <v>-1.421992476190476</v>
       </c>
-      <c r="L117" s="11" t="n">
+      <c r="L118" s="11" t="n">
         <v>-171.119871</v>
       </c>
-      <c r="M117" s="11" t="n">
+      <c r="M118" s="11" t="n">
         <v>-0.01006587476470588</v>
       </c>
-      <c r="N117" s="11" t="n">
+      <c r="N118" s="11" t="n">
         <v>-0.9053961428571428</v>
       </c>
-      <c r="O117" s="11" t="n">
+      <c r="O118" s="11" t="n">
         <v>-96.386746</v>
       </c>
-      <c r="P117" s="11" t="n">
+      <c r="P118" s="11" t="n">
         <v>-0.005669808588235294</v>
       </c>
-      <c r="Q117" s="11" t="n">
+      <c r="Q118" s="11" t="n">
         <v>-0.5099827830687831</v>
       </c>
-      <c r="R117" s="11" t="n">
+      <c r="R118" s="11" t="n">
         <v>-536.263195</v>
       </c>
-      <c r="S117" s="11" t="n">
+      <c r="S118" s="11" t="n">
         <v>-0.03154489382352941</v>
       </c>
-      <c r="T117" s="11" t="n">
+      <c r="T118" s="11" t="n">
         <v>-2.837371402116402</v>
       </c>
     </row>
-    <row r="118">
-      <c r="B118" s="8" t="inlineStr">
+    <row r="119">
+      <c r="B119" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">        Loan Related Charges</t>
         </is>
       </c>
-      <c r="C118" s="9" t="n"/>
-      <c r="D118" s="9" t="n"/>
-      <c r="E118" s="9" t="n"/>
-      <c r="F118" s="9" t="n">
+      <c r="C119" s="9" t="n"/>
+      <c r="D119" s="9" t="n"/>
+      <c r="E119" s="9" t="n"/>
+      <c r="F119" s="9" t="n">
         <v>-773.891532</v>
       </c>
-      <c r="G118" s="9" t="n">
+      <c r="G119" s="9" t="n">
         <v>-0.04552303129411765</v>
       </c>
-      <c r="H118" s="9" t="n">
+      <c r="H119" s="9" t="n">
         <v>-4.09466419047619</v>
       </c>
-      <c r="I118" s="9" t="n">
+      <c r="I119" s="9" t="n">
         <v>-19.344233</v>
       </c>
-      <c r="J118" s="9" t="n">
+      <c r="J119" s="9" t="n">
         <v>-0.001137896058823529</v>
       </c>
-      <c r="K118" s="9" t="n">
+      <c r="K119" s="9" t="n">
         <v>-0.1023504391534392</v>
       </c>
-      <c r="L118" s="9" t="n"/>
-      <c r="M118" s="9" t="n"/>
-      <c r="N118" s="9" t="n"/>
-      <c r="O118" s="9" t="n"/>
-      <c r="P118" s="9" t="n"/>
-      <c r="Q118" s="9" t="n"/>
-      <c r="R118" s="9" t="n">
+      <c r="L119" s="9" t="n"/>
+      <c r="M119" s="9" t="n"/>
+      <c r="N119" s="9" t="n"/>
+      <c r="O119" s="9" t="n"/>
+      <c r="P119" s="9" t="n"/>
+      <c r="Q119" s="9" t="n"/>
+      <c r="R119" s="9" t="n">
         <v>-793.235765</v>
       </c>
-      <c r="S118" s="9" t="n">
+      <c r="S119" s="9" t="n">
         <v>-0.04666092735294117</v>
       </c>
-      <c r="T118" s="9" t="n">
+      <c r="T119" s="9" t="n">
         <v>-4.19701462962963</v>
       </c>
     </row>
-    <row r="119">
-      <c r="B119" s="12" t="inlineStr">
+    <row r="120">
+      <c r="B120" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">    TOTAL FINANCE COST</t>
         </is>
       </c>
-      <c r="C119" s="13" t="n">
+      <c r="C120" s="13" t="n">
         <v>-308.6855417199999</v>
       </c>
-      <c r="D119" s="13" t="n">
+      <c r="D120" s="13" t="n">
         <v>-0.01815797304235294</v>
       </c>
-      <c r="E119" s="13" t="n">
+      <c r="E120" s="13" t="n">
         <v>-1.633256834497354</v>
       </c>
-      <c r="F119" s="13" t="n">
+      <c r="F120" s="13" t="n">
         <v>-967.3651479100001</v>
       </c>
-      <c r="G119" s="13" t="n">
+      <c r="G120" s="13" t="n">
         <v>-0.05690383223000001</v>
       </c>
-      <c r="H119" s="13" t="n">
+      <c r="H120" s="13" t="n">
         <v>-5.118334115925927</v>
       </c>
-      <c r="I119" s="13" t="n">
+      <c r="I120" s="13" t="n">
         <v>-446.65471115</v>
       </c>
-      <c r="J119" s="13" t="n">
+      <c r="J120" s="13" t="n">
         <v>-0.0262738065382353</v>
       </c>
-      <c r="K119" s="13" t="n">
+      <c r="K120" s="13" t="n">
         <v>-2.36325243994709</v>
       </c>
-      <c r="L119" s="13" t="n">
+      <c r="L120" s="13" t="n">
         <v>-358.18051414</v>
       </c>
-      <c r="M119" s="13" t="n">
+      <c r="M120" s="13" t="n">
         <v>-0.0210694420082353</v>
       </c>
-      <c r="N119" s="13" t="n">
+      <c r="N120" s="13" t="n">
         <v>-1.895134995449736</v>
       </c>
-      <c r="O119" s="13" t="n">
+      <c r="O120" s="13" t="n">
         <v>-2956.57269042</v>
       </c>
-      <c r="P119" s="13" t="n">
+      <c r="P120" s="13" t="n">
         <v>-0.1739160406129412</v>
       </c>
-      <c r="Q119" s="13" t="n">
+      <c r="Q120" s="13" t="n">
         <v>-15.64324174825397</v>
       </c>
-      <c r="R119" s="13" t="n">
+      <c r="R120" s="13" t="n">
         <v>-5037.45860534</v>
       </c>
-      <c r="S119" s="13" t="n">
+      <c r="S120" s="13" t="n">
         <v>-0.2963210944317647</v>
       </c>
-      <c r="T119" s="13" t="n">
+      <c r="T120" s="13" t="n">
         <v>-26.65322013407408</v>
-      </c>
-    </row>
-    <row r="120">
-      <c r="B120" s="16" t="inlineStr">
-        <is>
-          <t>TOTAL OUTFLOW</t>
-        </is>
-      </c>
-      <c r="C120" s="17" t="n">
-        <v>-44493.15819503</v>
-      </c>
-      <c r="D120" s="17" t="n">
-        <v>-2.617244599707647</v>
-      </c>
-      <c r="E120" s="17" t="n">
-        <v>-235.4135354234392</v>
-      </c>
-      <c r="F120" s="17" t="n">
-        <v>-87290.80569813</v>
-      </c>
-      <c r="G120" s="17" t="n">
-        <v>-5.134753276360589</v>
-      </c>
-      <c r="H120" s="17" t="n">
-        <v>-461.8561148049207</v>
-      </c>
-      <c r="I120" s="17" t="n">
-        <v>-56595.89979415</v>
-      </c>
-      <c r="J120" s="17" t="n">
-        <v>-3.32917057612647</v>
-      </c>
-      <c r="K120" s="17" t="n">
-        <v>-299.4492052600529</v>
-      </c>
-      <c r="L120" s="17" t="n">
-        <v>-47009.3796492</v>
-      </c>
-      <c r="M120" s="17" t="n">
-        <v>-2.765257626423529</v>
-      </c>
-      <c r="N120" s="17" t="n">
-        <v>-248.7268764507936</v>
-      </c>
-      <c r="O120" s="17" t="n">
-        <v>-27914.58608382</v>
-      </c>
-      <c r="P120" s="17" t="n">
-        <v>-1.642034475518823</v>
-      </c>
-      <c r="Q120" s="17" t="n">
-        <v>-147.6962226657143</v>
-      </c>
-      <c r="R120" s="17" t="n">
-        <v>-263303.8294203299</v>
-      </c>
-      <c r="S120" s="17" t="n">
-        <v>-15.48846055413706</v>
-      </c>
-      <c r="T120" s="17" t="n">
-        <v>-1393.141954604921</v>
       </c>
     </row>
     <row r="121">
       <c r="B121" s="16" t="inlineStr">
         <is>
+          <t>TOTAL OUTFLOW</t>
+        </is>
+      </c>
+      <c r="C121" s="17" t="n">
+        <v>-44493.15819503</v>
+      </c>
+      <c r="D121" s="17" t="n">
+        <v>-2.617244599707647</v>
+      </c>
+      <c r="E121" s="17" t="n">
+        <v>-235.4135354234392</v>
+      </c>
+      <c r="F121" s="17" t="n">
+        <v>-87290.80569813</v>
+      </c>
+      <c r="G121" s="17" t="n">
+        <v>-5.134753276360589</v>
+      </c>
+      <c r="H121" s="17" t="n">
+        <v>-461.8561148049207</v>
+      </c>
+      <c r="I121" s="17" t="n">
+        <v>-56595.89979415</v>
+      </c>
+      <c r="J121" s="17" t="n">
+        <v>-3.32917057612647</v>
+      </c>
+      <c r="K121" s="17" t="n">
+        <v>-299.4492052600529</v>
+      </c>
+      <c r="L121" s="17" t="n">
+        <v>-47009.3796492</v>
+      </c>
+      <c r="M121" s="17" t="n">
+        <v>-2.765257626423529</v>
+      </c>
+      <c r="N121" s="17" t="n">
+        <v>-248.7268764507936</v>
+      </c>
+      <c r="O121" s="17" t="n">
+        <v>-27914.58608382</v>
+      </c>
+      <c r="P121" s="17" t="n">
+        <v>-1.642034475518823</v>
+      </c>
+      <c r="Q121" s="17" t="n">
+        <v>-147.6962226657143</v>
+      </c>
+      <c r="R121" s="17" t="n">
+        <v>-263303.8294203299</v>
+      </c>
+      <c r="S121" s="17" t="n">
+        <v>-15.48846055413706</v>
+      </c>
+      <c r="T121" s="17" t="n">
+        <v>-1393.141954604921</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="B122" s="16" t="inlineStr">
+        <is>
           <t>NET CASH SURPLUS (LOSS)</t>
         </is>
       </c>
-      <c r="C121" s="17" t="n">
+      <c r="C122" s="17" t="n">
         <v>11812.90216024</v>
       </c>
-      <c r="D121" s="17" t="n">
+      <c r="D122" s="17" t="n">
         <v>0.6948765976611763</v>
       </c>
-      <c r="E121" s="17" t="n">
+      <c r="E122" s="17" t="n">
         <v>62.50212783195766</v>
       </c>
-      <c r="F121" s="17" t="n">
+      <c r="F122" s="17" t="n">
         <v>-75526.95973020002</v>
       </c>
-      <c r="G121" s="17" t="n">
+      <c r="G122" s="17" t="n">
         <v>-4.442762337070589</v>
       </c>
-      <c r="H121" s="17" t="n">
+      <c r="H122" s="17" t="n">
         <v>-399.6135435460318</v>
       </c>
-      <c r="I121" s="17" t="n">
+      <c r="I122" s="17" t="n">
         <v>2573.810161360001</v>
       </c>
-      <c r="J121" s="17" t="n">
+      <c r="J122" s="17" t="n">
         <v>0.1514005977270589</v>
       </c>
-      <c r="K121" s="17" t="n">
+      <c r="K122" s="17" t="n">
         <v>13.61804318179895</v>
       </c>
-      <c r="L121" s="17" t="n">
+      <c r="L122" s="17" t="n">
         <v>11041.90401141</v>
       </c>
-      <c r="M121" s="17" t="n">
+      <c r="M122" s="17" t="n">
         <v>0.6495237653770591</v>
       </c>
-      <c r="N121" s="17" t="n">
+      <c r="N122" s="17" t="n">
         <v>58.42277254714288</v>
       </c>
-      <c r="O121" s="17" t="n">
+      <c r="O122" s="17" t="n">
         <v>-15435.4135908</v>
       </c>
-      <c r="P121" s="17" t="n">
+      <c r="P122" s="17" t="n">
         <v>-0.9079655053411764</v>
       </c>
-      <c r="Q121" s="17" t="n">
+      <c r="Q122" s="17" t="n">
         <v>-81.66885497777777</v>
       </c>
-      <c r="R121" s="17" t="n">
+      <c r="R122" s="17" t="n">
         <v>-65533.75698799001</v>
       </c>
-      <c r="S121" s="17" t="n">
+      <c r="S122" s="17" t="n">
         <v>-3.854926881646472</v>
       </c>
-      <c r="T121" s="17" t="n">
+      <c r="T122" s="17" t="n">
         <v>-346.7394549629101</v>
       </c>
     </row>
-    <row r="122">
-      <c r="B122" s="14" t="inlineStr">
+    <row r="123">
+      <c r="B123" s="14" t="inlineStr">
         <is>
           <t>BEGINNING BALANCE</t>
         </is>
       </c>
-      <c r="C122" s="15" t="n">
+      <c r="C123" s="15" t="n">
         <v>67473.66082636001</v>
       </c>
-      <c r="D122" s="15" t="n">
+      <c r="D123" s="15" t="n">
         <v>3.969038872138824</v>
       </c>
-      <c r="E122" s="15" t="n">
+      <c r="E123" s="15" t="n">
         <v>357.0034964357672</v>
       </c>
-      <c r="F122" s="15" t="n">
+      <c r="F123" s="15" t="n">
         <v>79286.56298660001</v>
       </c>
-      <c r="G122" s="15" t="n">
+      <c r="G123" s="15" t="n">
         <v>4.663915469800001</v>
       </c>
-      <c r="H122" s="15" t="n">
+      <c r="H123" s="15" t="n">
         <v>419.5056242677249</v>
       </c>
-      <c r="I122" s="15" t="n">
+      <c r="I123" s="15" t="n">
         <v>3759.603256400002</v>
       </c>
-      <c r="J122" s="15" t="n">
+      <c r="J123" s="15" t="n">
         <v>0.2211531327294119</v>
       </c>
-      <c r="K122" s="15" t="n">
+      <c r="K123" s="15" t="n">
         <v>19.89208072169313</v>
       </c>
-      <c r="L122" s="15" t="n">
+      <c r="L123" s="15" t="n">
         <v>6333.413418760002</v>
       </c>
-      <c r="M122" s="15" t="n">
+      <c r="M123" s="15" t="n">
         <v>0.3725537305152942</v>
       </c>
-      <c r="N122" s="15" t="n">
+      <c r="N123" s="15" t="n">
         <v>33.51012390878308</v>
       </c>
-      <c r="O122" s="15" t="n">
+      <c r="O123" s="15" t="n">
         <v>17375.31743017</v>
       </c>
-      <c r="P122" s="15" t="n">
+      <c r="P123" s="15" t="n">
         <v>1.022077495892353</v>
       </c>
-      <c r="Q122" s="15" t="n">
+      <c r="Q123" s="15" t="n">
         <v>91.93289645592594</v>
       </c>
-      <c r="R122" s="15" t="n">
+      <c r="R123" s="15" t="n">
         <v>67473.66082636001</v>
       </c>
-      <c r="S122" s="15" t="n">
+      <c r="S123" s="15" t="n">
         <v>3.969038872138824</v>
       </c>
-      <c r="T122" s="15" t="n">
+      <c r="T123" s="15" t="n">
         <v>357.0034964357672</v>
       </c>
     </row>
-    <row r="123">
-      <c r="B123" s="16" t="inlineStr">
+    <row r="124">
+      <c r="B124" s="16" t="inlineStr">
         <is>
           <t>ENDING BALANCE</t>
         </is>
       </c>
-      <c r="C123" s="17" t="n">
+      <c r="C124" s="17" t="n">
         <v>79286.56298660001</v>
       </c>
-      <c r="D123" s="17" t="n">
+      <c r="D124" s="17" t="n">
         <v>4.663915469800001</v>
       </c>
-      <c r="E123" s="17" t="n">
+      <c r="E124" s="17" t="n">
         <v>419.5056242677249</v>
       </c>
-      <c r="F123" s="17" t="n">
+      <c r="F124" s="17" t="n">
         <v>3759.603256399994</v>
       </c>
-      <c r="G123" s="17" t="n">
+      <c r="G124" s="17" t="n">
         <v>0.2211531327294114</v>
       </c>
-      <c r="H123" s="17" t="n">
+      <c r="H124" s="17" t="n">
         <v>19.89208072169309</v>
       </c>
-      <c r="I123" s="17" t="n">
+      <c r="I124" s="17" t="n">
         <v>6333.413417760004</v>
       </c>
-      <c r="J123" s="17" t="n">
+      <c r="J124" s="17" t="n">
         <v>0.3725537304564708</v>
       </c>
-      <c r="K123" s="17" t="n">
+      <c r="K124" s="17" t="n">
         <v>33.51012390349208</v>
       </c>
-      <c r="L123" s="17" t="n">
+      <c r="L124" s="17" t="n">
         <v>17375.31743017001</v>
       </c>
-      <c r="M123" s="17" t="n">
+      <c r="M124" s="17" t="n">
         <v>1.022077495892353</v>
       </c>
-      <c r="N123" s="17" t="n">
+      <c r="N124" s="17" t="n">
         <v>91.93289645592596</v>
       </c>
-      <c r="O123" s="17" t="n">
+      <c r="O124" s="17" t="n">
         <v>1939.903839370003</v>
       </c>
-      <c r="P123" s="17" t="n">
+      <c r="P124" s="17" t="n">
         <v>0.1141119905511766</v>
       </c>
-      <c r="Q123" s="17" t="n">
+      <c r="Q124" s="17" t="n">
         <v>10.26404147814816</v>
       </c>
-      <c r="R123" s="17" t="n">
+      <c r="R124" s="17" t="n">
         <v>1939.903839370003</v>
       </c>
-      <c r="S123" s="17" t="n">
+      <c r="S124" s="17" t="n">
         <v>0.1141119905511766</v>
       </c>
-      <c r="T123" s="17" t="n">
+      <c r="T124" s="17" t="n">
         <v>10.26404147814816</v>
       </c>
     </row>
@@ -14124,16 +14174,16 @@
         <v>1555978395.440002</v>
       </c>
       <c r="E6" s="9" t="n">
-        <v>-1107171401.44</v>
+        <v>-817865913.4400001</v>
       </c>
       <c r="F6" s="9" t="n">
-        <v>448806994.0000024</v>
+        <v>738112482.0000024</v>
       </c>
       <c r="G6" s="21" t="n">
-        <v>26400.41141176485</v>
+        <v>43418.38129411779</v>
       </c>
       <c r="H6" s="21" t="n">
-        <v>2374640.179894193</v>
+        <v>3905357.04761906</v>
       </c>
     </row>
     <row r="7">
@@ -14156,16 +14206,16 @@
         <v>186144708</v>
       </c>
       <c r="E7" s="11" t="n">
-        <v>-41903061</v>
+        <v>127831780</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>144241647</v>
+        <v>313976488</v>
       </c>
       <c r="G7" s="22" t="n">
-        <v>8484.802764705883</v>
+        <v>18469.20517647059</v>
       </c>
       <c r="H7" s="22" t="n">
-        <v>763183.3174603175</v>
+        <v>1661251.259259259</v>
       </c>
     </row>
     <row r="8">
@@ -14220,16 +14270,16 @@
         <v>74014769.52</v>
       </c>
       <c r="E9" s="11" t="n">
-        <v>1852176625</v>
+        <v>235680125</v>
       </c>
       <c r="F9" s="11" t="n">
-        <v>1926191394.52</v>
+        <v>309694894.52</v>
       </c>
       <c r="G9" s="22" t="n">
-        <v>113305.3761482353</v>
+        <v>18217.34673647059</v>
       </c>
       <c r="H9" s="22" t="n">
-        <v>10191488.85989418</v>
+        <v>1638597.325502645</v>
       </c>
     </row>
     <row r="10">
@@ -14252,16 +14302,16 @@
         <v>8627665</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>0</v>
+        <v>1574933000</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>8627665</v>
+        <v>1583560665</v>
       </c>
       <c r="G10" s="21" t="n">
-        <v>507.5097058823529</v>
+        <v>93150.62735294117</v>
       </c>
       <c r="H10" s="21" t="n">
-        <v>45649.02116402116</v>
+        <v>8378627.857142857</v>
       </c>
     </row>
     <row r="11">
@@ -14339,13 +14389,13 @@
       <c r="D13" s="24" t="n"/>
       <c r="E13" s="24" t="n"/>
       <c r="F13" s="25" t="n">
-        <v>3078942466.930002</v>
+        <v>3496419295.930002</v>
       </c>
       <c r="G13" s="26" t="n">
-        <v>181114.2627605884</v>
+        <v>205671.7232900001</v>
       </c>
       <c r="H13" s="26" t="n">
-        <v>16290700.88322753</v>
+        <v>18499572.99433864</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh dashboard Thu 07/02/2026  9:11
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -710,7 +710,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 01 Jul 2026 16:59</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 02 Jul 2026 09:11</t>
         </is>
       </c>
     </row>
@@ -7531,7 +7531,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 01 Jul 2026 16:59 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 02 Jul 2026 09:11 (in IDR Million)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh dashboard Thu 07/02/2026  9:15
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -710,7 +710,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 02 Jul 2026 09:11</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 02 Jul 2026 09:15</t>
         </is>
       </c>
     </row>
@@ -7531,7 +7531,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 02 Jul 2026 09:11 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 02 Jul 2026 09:15 (in IDR Million)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh dashboard Thu 07/02/2026  9:25
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -710,7 +710,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 02 Jul 2026 09:15</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 02 Jul 2026 09:25</t>
         </is>
       </c>
     </row>
@@ -7531,7 +7531,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 02 Jul 2026 09:15 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 02 Jul 2026 09:25 (in IDR Million)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh dashboard Thu 07/09/2026 16:26
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -710,7 +710,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 07 Jul 2026 10:11</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 09 Jul 2026 16:26</t>
         </is>
       </c>
     </row>
@@ -7607,7 +7607,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 07 Jul 2026 10:11 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 09 Jul 2026 16:26 (in IDR Million)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh dashboard Fri 07/10/2026 17:26
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -710,7 +710,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 10 Jul 2026 13:32</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 10 Jul 2026 17:25</t>
         </is>
       </c>
     </row>
@@ -7663,7 +7663,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 10 Jul 2026 13:32 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 10 Jul 2026 17:25 (in IDR Million)</t>
         </is>
       </c>
     </row>
@@ -16728,16 +16728,16 @@
         <v>310487173.9</v>
       </c>
       <c r="E9" s="11" t="n">
-        <v>-105442103</v>
+        <v>-176279413</v>
       </c>
       <c r="F9" s="11" t="n">
-        <v>205045070.9</v>
+        <v>134207760.9</v>
       </c>
       <c r="G9" s="22" t="n">
-        <v>12061.47475882353</v>
+        <v>7894.574170588234</v>
       </c>
       <c r="H9" s="22" t="n">
-        <v>1084894.555026455</v>
+        <v>710093.9730158729</v>
       </c>
     </row>
     <row r="10">
@@ -16847,13 +16847,13 @@
       <c r="D13" s="24" t="n"/>
       <c r="E13" s="24" t="n"/>
       <c r="F13" s="25" t="n">
-        <v>2740055973.24</v>
+        <v>2669218663.24</v>
       </c>
       <c r="G13" s="26" t="n">
-        <v>161179.7631317647</v>
+        <v>157012.8625435294</v>
       </c>
       <c r="H13" s="26" t="n">
-        <v>14497650.65206349</v>
+        <v>14122850.07005291</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh dashboard Tue 07/14/2026 16:59
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -710,7 +710,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 10 Jul 2026 17:25</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 14 Jul 2026 16:59</t>
         </is>
       </c>
     </row>
@@ -7663,7 +7663,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 10 Jul 2026 17:25 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 14 Jul 2026 16:59 (in IDR Million)</t>
         </is>
       </c>
     </row>
@@ -16632,16 +16632,16 @@
         <v>631754694</v>
       </c>
       <c r="E6" s="9" t="n">
-        <v>1052064654</v>
+        <v>1781614297</v>
       </c>
       <c r="F6" s="9" t="n">
-        <v>1683819348</v>
+        <v>2413368991</v>
       </c>
       <c r="G6" s="21" t="n">
-        <v>99048.19694117647</v>
+        <v>141962.8818235294</v>
       </c>
       <c r="H6" s="21" t="n">
-        <v>8909097.07936508</v>
+        <v>12769148.1005291</v>
       </c>
     </row>
     <row r="7">
@@ -16664,16 +16664,16 @@
         <v>313976489</v>
       </c>
       <c r="E7" s="11" t="n">
-        <v>-32146596</v>
+        <v>-53068183</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>281829893</v>
+        <v>260908306</v>
       </c>
       <c r="G7" s="22" t="n">
-        <v>16578.229</v>
+        <v>15347.54741176471</v>
       </c>
       <c r="H7" s="22" t="n">
-        <v>1491163.455026455</v>
+        <v>1380467.227513228</v>
       </c>
     </row>
     <row r="8">
@@ -16728,16 +16728,16 @@
         <v>310487173.9</v>
       </c>
       <c r="E9" s="11" t="n">
-        <v>-176279413</v>
+        <v>-242111942</v>
       </c>
       <c r="F9" s="11" t="n">
-        <v>134207760.9</v>
+        <v>68375231.89999998</v>
       </c>
       <c r="G9" s="22" t="n">
-        <v>7894.574170588234</v>
+        <v>4022.072464705881</v>
       </c>
       <c r="H9" s="22" t="n">
-        <v>710093.9730158729</v>
+        <v>361773.7137566136</v>
       </c>
     </row>
     <row r="10">
@@ -16847,13 +16847,13 @@
       <c r="D13" s="24" t="n"/>
       <c r="E13" s="24" t="n"/>
       <c r="F13" s="25" t="n">
-        <v>2669218663.24</v>
+        <v>3312014190.24</v>
       </c>
       <c r="G13" s="26" t="n">
-        <v>157012.8625435294</v>
+        <v>194824.3641317647</v>
       </c>
       <c r="H13" s="26" t="n">
-        <v>14122850.07005291</v>
+        <v>17523884.60444444</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh dashboard Mon 07/20/2026  8:52
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -710,7 +710,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 17 Jul 2026 05:14</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 20 Jul 2026 08:52</t>
         </is>
       </c>
     </row>
@@ -7803,7 +7803,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 17 Jul 2026 05:14 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 20 Jul 2026 08:52 (in IDR Million)</t>
         </is>
       </c>
     </row>
@@ -16912,16 +16912,16 @@
         <v>631754694</v>
       </c>
       <c r="E6" s="9" t="n">
-        <v>138807184</v>
+        <v>1072209407</v>
       </c>
       <c r="F6" s="9" t="n">
-        <v>770561878</v>
+        <v>1703964101</v>
       </c>
       <c r="G6" s="21" t="n">
-        <v>45327.16929411764</v>
+        <v>100233.1824117647</v>
       </c>
       <c r="H6" s="21" t="n">
-        <v>4077046.973544973</v>
+        <v>9015683.074074075</v>
       </c>
     </row>
     <row r="7">
@@ -17127,13 +17127,13 @@
       <c r="D13" s="24" t="n"/>
       <c r="E13" s="24" t="n"/>
       <c r="F13" s="25" t="n">
-        <v>1172072263.24</v>
+        <v>2105474486.24</v>
       </c>
       <c r="G13" s="26" t="n">
-        <v>68945.42724941176</v>
+        <v>123851.4403670588</v>
       </c>
       <c r="H13" s="26" t="n">
-        <v>6201440.546243386</v>
+        <v>11140076.64677249</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh dashboard Tue 07/21/2026 16:19
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -710,7 +710,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 20 Jul 2026 08:52</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 21 Jul 2026 16:19</t>
         </is>
       </c>
     </row>
@@ -7803,7 +7803,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 20 Jul 2026 08:52 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 21 Jul 2026 16:19 (in IDR Million)</t>
         </is>
       </c>
     </row>
@@ -16912,16 +16912,16 @@
         <v>631754694</v>
       </c>
       <c r="E6" s="9" t="n">
-        <v>1072209407</v>
+        <v>1091514499</v>
       </c>
       <c r="F6" s="9" t="n">
-        <v>1703964101</v>
+        <v>1723269193</v>
       </c>
       <c r="G6" s="21" t="n">
-        <v>100233.1824117647</v>
+        <v>101368.7760588235</v>
       </c>
       <c r="H6" s="21" t="n">
-        <v>9015683.074074075</v>
+        <v>9117826.417989418</v>
       </c>
     </row>
     <row r="7">
@@ -17008,16 +17008,16 @@
         <v>310487173.9</v>
       </c>
       <c r="E9" s="11" t="n">
-        <v>-228876342</v>
+        <v>-292651908</v>
       </c>
       <c r="F9" s="11" t="n">
-        <v>81610831.89999998</v>
+        <v>17835265.89999998</v>
       </c>
       <c r="G9" s="22" t="n">
-        <v>4800.637170588234</v>
+        <v>1049.133288235293</v>
       </c>
       <c r="H9" s="22" t="n">
-        <v>431803.3433862433</v>
+        <v>94366.48624338611</v>
       </c>
     </row>
     <row r="10">
@@ -17127,13 +17127,13 @@
       <c r="D13" s="24" t="n"/>
       <c r="E13" s="24" t="n"/>
       <c r="F13" s="25" t="n">
-        <v>2105474486.24</v>
+        <v>2061004012.24</v>
       </c>
       <c r="G13" s="26" t="n">
-        <v>123851.4403670588</v>
+        <v>121235.5301317647</v>
       </c>
       <c r="H13" s="26" t="n">
-        <v>11140076.64677249</v>
+        <v>10904783.13354497</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh dashboard Mon 07/27/2026  9:41
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -710,7 +710,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 24 Jul 2026 16:01</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 27 Jul 2026 09:41</t>
         </is>
       </c>
     </row>
@@ -7819,7 +7819,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 24 Jul 2026 16:01 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 27 Jul 2026 09:41 (in IDR Million)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh dashboard Tue 07/28/2026 16:03
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -710,7 +710,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 28 Jul 2026 13:47</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 28 Jul 2026 16:03</t>
         </is>
       </c>
     </row>
@@ -8637,7 +8637,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 28 Jul 2026 13:47 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 28 Jul 2026 16:03 (in IDR Million)</t>
         </is>
       </c>
     </row>
@@ -18676,16 +18676,16 @@
         <v>310487173.9</v>
       </c>
       <c r="E9" s="11" t="n">
-        <v>-303086275</v>
+        <v>-302049275</v>
       </c>
       <c r="F9" s="11" t="n">
-        <v>7400898.899999976</v>
+        <v>8437898.899999976</v>
       </c>
       <c r="G9" s="22" t="n">
-        <v>435.3469941176456</v>
+        <v>496.3469941176456</v>
       </c>
       <c r="H9" s="22" t="n">
-        <v>39158.19523809511</v>
+        <v>44644.9677248676</v>
       </c>
     </row>
     <row r="10">
@@ -18795,13 +18795,13 @@
       <c r="D13" s="24" t="n"/>
       <c r="E13" s="24" t="n"/>
       <c r="F13" s="25" t="n">
-        <v>1423601280.24</v>
+        <v>1424638280.24</v>
       </c>
       <c r="G13" s="26" t="n">
-        <v>83741.25177882353</v>
+        <v>83802.25177882353</v>
       </c>
       <c r="H13" s="26" t="n">
-        <v>7532281.906031746</v>
+        <v>7537768.678518519</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh dashboard Tue 07/28/2026 16:28
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -672,7 +672,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:W152"/>
+  <dimension ref="B1:Z152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -698,6 +698,9 @@
     <col width="16" customWidth="1" min="21" max="21"/>
     <col width="16" customWidth="1" min="22" max="22"/>
     <col width="16" customWidth="1" min="23" max="23"/>
+    <col width="16" customWidth="1" min="24" max="24"/>
+    <col width="16" customWidth="1" min="25" max="25"/>
+    <col width="16" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -710,7 +713,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 28 Jul 2026 16:03</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 28 Jul 2026 16:28</t>
         </is>
       </c>
     </row>
@@ -769,6 +772,13 @@
       </c>
       <c r="V3" s="4" t="n"/>
       <c r="W3" s="4" t="n"/>
+      <c r="X3" s="3" t="inlineStr">
+        <is>
+          <t>YTD as of 28 Jul 2026</t>
+        </is>
+      </c>
+      <c r="Y3" s="4" t="n"/>
+      <c r="Z3" s="4" t="n"/>
     </row>
     <row r="4" ht="18" customHeight="1">
       <c r="B4" s="5" t="n"/>
@@ -873,6 +883,21 @@
         </is>
       </c>
       <c r="W4" s="3" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="X4" s="3" t="inlineStr">
+        <is>
+          <t>IDR</t>
+        </is>
+      </c>
+      <c r="Y4" s="3" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Z4" s="3" t="inlineStr">
         <is>
           <t>INR</t>
         </is>
@@ -905,6 +930,9 @@
       <c r="U5" s="7" t="n"/>
       <c r="V5" s="7" t="n"/>
       <c r="W5" s="7" t="n"/>
+      <c r="X5" s="7" t="n"/>
+      <c r="Y5" s="7" t="n"/>
+      <c r="Z5" s="7" t="n"/>
     </row>
     <row r="6">
       <c r="B6" s="8" t="inlineStr">
@@ -974,6 +1002,15 @@
       </c>
       <c r="W6" s="9" t="n">
         <v>822520524.1798942</v>
+      </c>
+      <c r="X6" s="9" t="n">
+        <v>162351695487</v>
+      </c>
+      <c r="Y6" s="9" t="n">
+        <v>9550099.734529411</v>
+      </c>
+      <c r="Z6" s="9" t="n">
+        <v>859003679.8253969</v>
       </c>
     </row>
     <row r="7">
@@ -1027,6 +1064,15 @@
       <c r="W7" s="11" t="n">
         <v>483844930.0899471</v>
       </c>
+      <c r="X7" s="11" t="n">
+        <v>91465996879</v>
+      </c>
+      <c r="Y7" s="11" t="n">
+        <v>5380352.757588236</v>
+      </c>
+      <c r="Z7" s="11" t="n">
+        <v>483947073.4338624</v>
+      </c>
     </row>
     <row r="8">
       <c r="B8" s="8" t="inlineStr">
@@ -1096,6 +1142,15 @@
       </c>
       <c r="W8" s="9" t="n">
         <v>154675211.6666667</v>
+      </c>
+      <c r="X8" s="9" t="n">
+        <v>32823856519</v>
+      </c>
+      <c r="Y8" s="9" t="n">
+        <v>1930815.089352941</v>
+      </c>
+      <c r="Z8" s="9" t="n">
+        <v>173671198.5132275</v>
       </c>
     </row>
     <row r="9">
@@ -1161,6 +1216,15 @@
       <c r="W9" s="11" t="n">
         <v>142676871.7566138</v>
       </c>
+      <c r="X9" s="11" t="n">
+        <v>29263769826</v>
+      </c>
+      <c r="Y9" s="11" t="n">
+        <v>1721398.225058824</v>
+      </c>
+      <c r="Z9" s="11" t="n">
+        <v>154834760.984127</v>
+      </c>
     </row>
     <row r="10">
       <c r="B10" s="8" t="inlineStr">
@@ -1225,6 +1289,15 @@
       <c r="W10" s="9" t="n">
         <v>34982738.17989418</v>
       </c>
+      <c r="X10" s="9" t="n">
+        <v>7187586263</v>
+      </c>
+      <c r="Y10" s="9" t="n">
+        <v>422799.1919411765</v>
+      </c>
+      <c r="Z10" s="9" t="n">
+        <v>38029556.94708995</v>
+      </c>
     </row>
     <row r="11">
       <c r="B11" s="10" t="inlineStr">
@@ -1282,6 +1355,15 @@
       </c>
       <c r="W11" s="11" t="n">
         <v>5450793.650793651</v>
+      </c>
+      <c r="X11" s="11" t="n">
+        <v>1442280000</v>
+      </c>
+      <c r="Y11" s="11" t="n">
+        <v>84840</v>
+      </c>
+      <c r="Z11" s="11" t="n">
+        <v>7631111.111111112</v>
       </c>
     </row>
     <row r="12">
@@ -1323,6 +1405,15 @@
       <c r="W12" s="9" t="n">
         <v>740835.9788359788</v>
       </c>
+      <c r="X12" s="9" t="n">
+        <v>140018000</v>
+      </c>
+      <c r="Y12" s="9" t="n">
+        <v>8236.35294117647</v>
+      </c>
+      <c r="Z12" s="9" t="n">
+        <v>740835.9788359788</v>
+      </c>
     </row>
     <row r="13">
       <c r="B13" s="10" t="inlineStr">
@@ -1363,6 +1454,15 @@
       <c r="W13" s="11" t="n">
         <v>149142.8571428571</v>
       </c>
+      <c r="X13" s="11" t="n">
+        <v>28188000</v>
+      </c>
+      <c r="Y13" s="11" t="n">
+        <v>1658.117647058823</v>
+      </c>
+      <c r="Z13" s="11" t="n">
+        <v>149142.8571428571</v>
+      </c>
     </row>
     <row r="14">
       <c r="B14" s="8" t="inlineStr">
@@ -1403,6 +1503,15 @@
       <c r="W14" s="9" t="n">
         <v>262412698.4126984</v>
       </c>
+      <c r="X14" s="9" t="n">
+        <v>49596000000</v>
+      </c>
+      <c r="Y14" s="9" t="n">
+        <v>2917411.764705882</v>
+      </c>
+      <c r="Z14" s="9" t="n">
+        <v>262412698.4126984</v>
+      </c>
     </row>
     <row r="15">
       <c r="B15" s="10" t="inlineStr">
@@ -1443,6 +1552,15 @@
       <c r="W15" s="11" t="n">
         <v>262412698.4126984</v>
       </c>
+      <c r="X15" s="11" t="n">
+        <v>49596000000</v>
+      </c>
+      <c r="Y15" s="11" t="n">
+        <v>2917411.764705882</v>
+      </c>
+      <c r="Z15" s="11" t="n">
+        <v>262412698.4126984</v>
+      </c>
     </row>
     <row r="16">
       <c r="B16" s="8" t="inlineStr">
@@ -1513,6 +1631,15 @@
       <c r="W16" s="9" t="n">
         <v>1910739.122063492</v>
       </c>
+      <c r="X16" s="9" t="n">
+        <v>391421744.07</v>
+      </c>
+      <c r="Y16" s="9" t="n">
+        <v>23024.80847470588</v>
+      </c>
+      <c r="Z16" s="9" t="n">
+        <v>2071014.518888889</v>
+      </c>
     </row>
     <row r="17">
       <c r="B17" s="10" t="inlineStr">
@@ -1581,6 +1708,15 @@
         <v>7469.042321176472</v>
       </c>
       <c r="W17" s="11" t="n">
+        <v>671818.6214814816</v>
+      </c>
+      <c r="X17" s="11" t="n">
+        <v>126973719.46</v>
+      </c>
+      <c r="Y17" s="11" t="n">
+        <v>7469.042321176472</v>
+      </c>
+      <c r="Z17" s="11" t="n">
         <v>671818.6214814816</v>
       </c>
     </row>
@@ -1623,6 +1759,15 @@
       <c r="W18" s="9" t="n">
         <v>657985.1851851852</v>
       </c>
+      <c r="X18" s="9" t="n">
+        <v>124359200</v>
+      </c>
+      <c r="Y18" s="9" t="n">
+        <v>7315.247058823529</v>
+      </c>
+      <c r="Z18" s="9" t="n">
+        <v>657985.1851851852</v>
+      </c>
     </row>
     <row r="19">
       <c r="B19" s="10" t="inlineStr">
@@ -1663,6 +1808,15 @@
       <c r="W19" s="11" t="n">
         <v>123121.6931216931</v>
       </c>
+      <c r="X19" s="11" t="n">
+        <v>23270000</v>
+      </c>
+      <c r="Y19" s="11" t="n">
+        <v>1368.823529411765</v>
+      </c>
+      <c r="Z19" s="11" t="n">
+        <v>123121.6931216931</v>
+      </c>
     </row>
     <row r="20">
       <c r="B20" s="8" t="inlineStr">
@@ -1720,6 +1874,15 @@
       </c>
       <c r="W20" s="9" t="n">
         <v>97701.0582010582</v>
+      </c>
+      <c r="X20" s="9" t="n">
+        <v>22480000</v>
+      </c>
+      <c r="Y20" s="9" t="n">
+        <v>1322.35294117647</v>
+      </c>
+      <c r="Z20" s="9" t="n">
+        <v>118941.7989417989</v>
       </c>
     </row>
     <row r="21">
@@ -1765,6 +1928,15 @@
         <v>1188.532352941176</v>
       </c>
       <c r="W21" s="11" t="n">
+        <v>106905.0264550265</v>
+      </c>
+      <c r="X21" s="11" t="n">
+        <v>20205050</v>
+      </c>
+      <c r="Y21" s="11" t="n">
+        <v>1188.532352941176</v>
+      </c>
+      <c r="Z21" s="11" t="n">
         <v>106905.0264550265</v>
       </c>
     </row>
@@ -1795,6 +1967,15 @@
       <c r="U22" s="9" t="n"/>
       <c r="V22" s="9" t="n"/>
       <c r="W22" s="9" t="n"/>
+      <c r="X22" s="9" t="n">
+        <v>17865000</v>
+      </c>
+      <c r="Y22" s="9" t="n">
+        <v>1050.882352941177</v>
+      </c>
+      <c r="Z22" s="9" t="n">
+        <v>94523.80952380953</v>
+      </c>
     </row>
     <row r="23">
       <c r="B23" s="10" t="inlineStr">
@@ -1835,6 +2016,15 @@
       <c r="W23" s="11" t="n">
         <v>74473.01587301587</v>
       </c>
+      <c r="X23" s="11" t="n">
+        <v>14075400</v>
+      </c>
+      <c r="Y23" s="11" t="n">
+        <v>827.964705882353</v>
+      </c>
+      <c r="Z23" s="11" t="n">
+        <v>74473.01587301587</v>
+      </c>
     </row>
     <row r="24">
       <c r="B24" s="8" t="inlineStr">
@@ -1892,6 +2082,15 @@
       </c>
       <c r="W24" s="9" t="n">
         <v>41382.97354497355</v>
+      </c>
+      <c r="X24" s="9" t="n">
+        <v>11858382</v>
+      </c>
+      <c r="Y24" s="9" t="n">
+        <v>697.5518823529411</v>
+      </c>
+      <c r="Z24" s="9" t="n">
+        <v>62742.76190476191</v>
       </c>
     </row>
     <row r="25">
@@ -1933,6 +2132,15 @@
       <c r="W25" s="11" t="n">
         <v>39765.75132275133</v>
       </c>
+      <c r="X25" s="11" t="n">
+        <v>7515727</v>
+      </c>
+      <c r="Y25" s="11" t="n">
+        <v>442.1015882352941</v>
+      </c>
+      <c r="Z25" s="11" t="n">
+        <v>39765.75132275133</v>
+      </c>
     </row>
     <row r="26">
       <c r="B26" s="8" t="inlineStr">
@@ -1979,6 +2187,15 @@
       <c r="W26" s="9" t="n">
         <v>31746.03174603175</v>
       </c>
+      <c r="X26" s="9" t="n">
+        <v>6000000</v>
+      </c>
+      <c r="Y26" s="9" t="n">
+        <v>352.9411764705882</v>
+      </c>
+      <c r="Z26" s="9" t="n">
+        <v>31746.03174603175</v>
+      </c>
     </row>
     <row r="27">
       <c r="B27" s="10" t="inlineStr">
@@ -2024,6 +2241,15 @@
       </c>
       <c r="W27" s="11" t="n">
         <v>21873.1746031746</v>
+      </c>
+      <c r="X27" s="11" t="n">
+        <v>4484030</v>
+      </c>
+      <c r="Y27" s="11" t="n">
+        <v>263.7664705882353</v>
+      </c>
+      <c r="Z27" s="11" t="n">
+        <v>23725.02645502645</v>
       </c>
     </row>
     <row r="28">
@@ -2065,6 +2291,15 @@
       <c r="W28" s="9" t="n">
         <v>20227.7671957672</v>
       </c>
+      <c r="X28" s="9" t="n">
+        <v>3823048</v>
+      </c>
+      <c r="Y28" s="9" t="n">
+        <v>224.8851764705882</v>
+      </c>
+      <c r="Z28" s="9" t="n">
+        <v>20227.7671957672</v>
+      </c>
     </row>
     <row r="29">
       <c r="B29" s="10" t="inlineStr">
@@ -2105,6 +2340,15 @@
       <c r="W29" s="11" t="n">
         <v>556.6137566137567</v>
       </c>
+      <c r="X29" s="11" t="n">
+        <v>2700450</v>
+      </c>
+      <c r="Y29" s="11" t="n">
+        <v>158.85</v>
+      </c>
+      <c r="Z29" s="11" t="n">
+        <v>14288.09523809524</v>
+      </c>
     </row>
     <row r="30">
       <c r="B30" s="8" t="inlineStr">
@@ -2155,6 +2399,15 @@
         <v>103.1552123529412</v>
       </c>
       <c r="W30" s="9" t="n">
+        <v>9278.511164021163</v>
+      </c>
+      <c r="X30" s="9" t="n">
+        <v>1753638.61</v>
+      </c>
+      <c r="Y30" s="9" t="n">
+        <v>103.1552123529412</v>
+      </c>
+      <c r="Z30" s="9" t="n">
         <v>9278.511164021163</v>
       </c>
     </row>
@@ -2197,6 +2450,15 @@
       <c r="W31" s="11" t="n">
         <v>1502.603174603175</v>
       </c>
+      <c r="X31" s="11" t="n">
+        <v>1644292</v>
+      </c>
+      <c r="Y31" s="11" t="n">
+        <v>96.72305882352941</v>
+      </c>
+      <c r="Z31" s="11" t="n">
+        <v>8699.957671957673</v>
+      </c>
     </row>
     <row r="32">
       <c r="B32" s="8" t="inlineStr">
@@ -2237,6 +2499,15 @@
       <c r="W32" s="9" t="n">
         <v>5291.005291005291</v>
       </c>
+      <c r="X32" s="9" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="Y32" s="9" t="n">
+        <v>58.8235294117647</v>
+      </c>
+      <c r="Z32" s="9" t="n">
+        <v>5291.005291005291</v>
+      </c>
     </row>
     <row r="33">
       <c r="B33" s="10" t="inlineStr">
@@ -2287,6 +2558,15 @@
         <v>43.48235294117647</v>
       </c>
       <c r="W33" s="11" t="n">
+        <v>3911.111111111111</v>
+      </c>
+      <c r="X33" s="11" t="n">
+        <v>739200</v>
+      </c>
+      <c r="Y33" s="11" t="n">
+        <v>43.48235294117647</v>
+      </c>
+      <c r="Z33" s="11" t="n">
         <v>3911.111111111111</v>
       </c>
     </row>
@@ -2335,6 +2615,15 @@
       <c r="W34" s="9" t="n">
         <v>2648.703703703704</v>
       </c>
+      <c r="X34" s="9" t="n">
+        <v>500605</v>
+      </c>
+      <c r="Y34" s="9" t="n">
+        <v>29.44735294117647</v>
+      </c>
+      <c r="Z34" s="9" t="n">
+        <v>2648.703703703704</v>
+      </c>
     </row>
     <row r="35">
       <c r="B35" s="10" t="inlineStr">
@@ -2375,6 +2664,15 @@
       <c r="W35" s="11" t="n">
         <v>529.1111111111111</v>
       </c>
+      <c r="X35" s="11" t="n">
+        <v>170002</v>
+      </c>
+      <c r="Y35" s="11" t="n">
+        <v>10.00011764705882</v>
+      </c>
+      <c r="Z35" s="11" t="n">
+        <v>899.4814814814815</v>
+      </c>
     </row>
     <row r="36">
       <c r="B36" s="8" t="inlineStr">
@@ -2415,6 +2713,15 @@
       <c r="W36" s="9" t="n">
         <v>21.16402116402116</v>
       </c>
+      <c r="X36" s="9" t="n">
+        <v>4000</v>
+      </c>
+      <c r="Y36" s="9" t="n">
+        <v>0.2352941176470588</v>
+      </c>
+      <c r="Z36" s="9" t="n">
+        <v>21.16402116402116</v>
+      </c>
     </row>
     <row r="37">
       <c r="B37" s="10" t="inlineStr">
@@ -2455,6 +2762,15 @@
       <c r="W37" s="11" t="n">
         <v>1164021.164021164</v>
       </c>
+      <c r="X37" s="11" t="n">
+        <v>220000000</v>
+      </c>
+      <c r="Y37" s="11" t="n">
+        <v>12941.17647058824</v>
+      </c>
+      <c r="Z37" s="11" t="n">
+        <v>1164021.164021164</v>
+      </c>
     </row>
     <row r="38">
       <c r="B38" s="12" t="inlineStr">
@@ -2524,6 +2840,15 @@
       </c>
       <c r="W38" s="13" t="n">
         <v>1088007982.878677</v>
+      </c>
+      <c r="X38" s="13" t="n">
+        <v>212559117231.07</v>
+      </c>
+      <c r="Y38" s="13" t="n">
+        <v>12503477.48418059</v>
+      </c>
+      <c r="Z38" s="13" t="n">
+        <v>1124651413.921005</v>
       </c>
     </row>
     <row r="39">
@@ -2553,6 +2878,9 @@
       <c r="U39" s="7" t="n"/>
       <c r="V39" s="7" t="n"/>
       <c r="W39" s="7" t="n"/>
+      <c r="X39" s="7" t="n"/>
+      <c r="Y39" s="7" t="n"/>
+      <c r="Z39" s="7" t="n"/>
     </row>
     <row r="40">
       <c r="B40" s="14" t="inlineStr">
@@ -2581,6 +2909,9 @@
       <c r="U40" s="15" t="n"/>
       <c r="V40" s="15" t="n"/>
       <c r="W40" s="15" t="n"/>
+      <c r="X40" s="15" t="n"/>
+      <c r="Y40" s="15" t="n"/>
+      <c r="Z40" s="15" t="n"/>
     </row>
     <row r="41">
       <c r="B41" s="8" t="inlineStr">
@@ -2650,6 +2981,15 @@
       </c>
       <c r="W41" s="9" t="n">
         <v>-24773249.62962963</v>
+      </c>
+      <c r="X41" s="9" t="n">
+        <v>-4688969180</v>
+      </c>
+      <c r="Y41" s="9" t="n">
+        <v>-275821.7164705882</v>
+      </c>
+      <c r="Z41" s="9" t="n">
+        <v>-24809360.74074074</v>
       </c>
     </row>
     <row r="42">
@@ -2695,6 +3035,15 @@
         <v>-9178.077352941176</v>
       </c>
       <c r="W42" s="11" t="n">
+        <v>-825541.3492063492</v>
+      </c>
+      <c r="X42" s="11" t="n">
+        <v>-156027315</v>
+      </c>
+      <c r="Y42" s="11" t="n">
+        <v>-9178.077352941176</v>
+      </c>
+      <c r="Z42" s="11" t="n">
         <v>-825541.3492063492</v>
       </c>
     </row>
@@ -2725,6 +3074,15 @@
       <c r="U43" s="9" t="n"/>
       <c r="V43" s="9" t="n"/>
       <c r="W43" s="9" t="n"/>
+      <c r="X43" s="9" t="n">
+        <v>-172443500</v>
+      </c>
+      <c r="Y43" s="9" t="n">
+        <v>-10143.73529411765</v>
+      </c>
+      <c r="Z43" s="9" t="n">
+        <v>-912399.4708994708</v>
+      </c>
     </row>
     <row r="44">
       <c r="B44" s="10" t="inlineStr">
@@ -2783,6 +3141,15 @@
       <c r="W44" s="11" t="n">
         <v>-5654963.767195767</v>
       </c>
+      <c r="X44" s="11" t="n">
+        <v>-1268268418</v>
+      </c>
+      <c r="Y44" s="11" t="n">
+        <v>-74604.02458823529</v>
+      </c>
+      <c r="Z44" s="11" t="n">
+        <v>-6710414.91005291</v>
+      </c>
     </row>
     <row r="45">
       <c r="B45" s="8" t="inlineStr">
@@ -2828,6 +3195,15 @@
       </c>
       <c r="W45" s="9" t="n">
         <v>-442737.3015873016</v>
+      </c>
+      <c r="X45" s="9" t="n">
+        <v>-134989875</v>
+      </c>
+      <c r="Y45" s="9" t="n">
+        <v>-7940.580882352942</v>
+      </c>
+      <c r="Z45" s="9" t="n">
+        <v>-714232.1428571428</v>
       </c>
     </row>
     <row r="46">
@@ -2857,6 +3233,15 @@
       <c r="U46" s="11" t="n"/>
       <c r="V46" s="11" t="n"/>
       <c r="W46" s="11" t="n"/>
+      <c r="X46" s="11" t="n">
+        <v>-29400000</v>
+      </c>
+      <c r="Y46" s="11" t="n">
+        <v>-1729.411764705882</v>
+      </c>
+      <c r="Z46" s="11" t="n">
+        <v>-155555.5555555556</v>
+      </c>
     </row>
     <row r="47">
       <c r="B47" s="8" t="inlineStr">
@@ -2897,6 +3282,15 @@
       <c r="W47" s="9" t="n">
         <v>-184444.4444444444</v>
       </c>
+      <c r="X47" s="9" t="n">
+        <v>-47578550</v>
+      </c>
+      <c r="Y47" s="9" t="n">
+        <v>-2798.738235294118</v>
+      </c>
+      <c r="Z47" s="9" t="n">
+        <v>-251738.3597883598</v>
+      </c>
     </row>
     <row r="48">
       <c r="B48" s="10" t="inlineStr">
@@ -2955,6 +3349,15 @@
       <c r="W48" s="11" t="n">
         <v>-3673993.804232804</v>
       </c>
+      <c r="X48" s="11" t="n">
+        <v>-1005168514</v>
+      </c>
+      <c r="Y48" s="11" t="n">
+        <v>-59127.55964705883</v>
+      </c>
+      <c r="Z48" s="11" t="n">
+        <v>-5318351.925925925</v>
+      </c>
     </row>
     <row r="49">
       <c r="B49" s="8" t="inlineStr">
@@ -3005,6 +3408,15 @@
         <v>-5460.122647058824</v>
       </c>
       <c r="W49" s="9" t="n">
+        <v>-491122.1428571428</v>
+      </c>
+      <c r="X49" s="9" t="n">
+        <v>-92822085</v>
+      </c>
+      <c r="Y49" s="9" t="n">
+        <v>-5460.122647058824</v>
+      </c>
+      <c r="Z49" s="9" t="n">
         <v>-491122.1428571428</v>
       </c>
     </row>
@@ -3058,6 +3470,15 @@
       </c>
       <c r="W50" s="11" t="n">
         <v>-6807835.645502645</v>
+      </c>
+      <c r="X50" s="11" t="n">
+        <v>-1328241875</v>
+      </c>
+      <c r="Y50" s="11" t="n">
+        <v>-78131.875</v>
+      </c>
+      <c r="Z50" s="11" t="n">
+        <v>-7027734.788359787</v>
       </c>
     </row>
     <row r="51">
@@ -3099,6 +3520,15 @@
       <c r="W51" s="9" t="n">
         <v>-10041970.37037037</v>
       </c>
+      <c r="X51" s="9" t="n">
+        <v>-1897932400</v>
+      </c>
+      <c r="Y51" s="9" t="n">
+        <v>-111643.0823529412</v>
+      </c>
+      <c r="Z51" s="9" t="n">
+        <v>-10041970.37037037</v>
+      </c>
     </row>
     <row r="52">
       <c r="B52" s="10" t="inlineStr">
@@ -3168,6 +3598,15 @@
       </c>
       <c r="W52" s="11" t="n">
         <v>-726268.4444444445</v>
+      </c>
+      <c r="X52" s="11" t="n">
+        <v>-154499829</v>
+      </c>
+      <c r="Y52" s="11" t="n">
+        <v>-9088.225235294118</v>
+      </c>
+      <c r="Z52" s="11" t="n">
+        <v>-817459.4126984128</v>
       </c>
     </row>
     <row r="53">
@@ -3197,6 +3636,15 @@
       <c r="U53" s="9" t="n"/>
       <c r="V53" s="9" t="n"/>
       <c r="W53" s="9" t="n"/>
+      <c r="X53" s="9" t="n">
+        <v>-30945000</v>
+      </c>
+      <c r="Y53" s="9" t="n">
+        <v>-1820.294117647059</v>
+      </c>
+      <c r="Z53" s="9" t="n">
+        <v>-163730.1587301587</v>
+      </c>
     </row>
     <row r="54">
       <c r="B54" s="10" t="inlineStr">
@@ -3266,6 +3714,15 @@
       </c>
       <c r="W54" s="11" t="n">
         <v>-7334781.486137566</v>
+      </c>
+      <c r="X54" s="11" t="n">
+        <v>-1408985750.88</v>
+      </c>
+      <c r="Y54" s="11" t="n">
+        <v>-82881.51475764706</v>
+      </c>
+      <c r="Z54" s="11" t="n">
+        <v>-7454951.062857143</v>
       </c>
     </row>
     <row r="55">
@@ -3305,6 +3762,15 @@
         <v>-101247.6705882353</v>
       </c>
       <c r="W55" s="9" t="n">
+        <v>-9106933.333333334</v>
+      </c>
+      <c r="X55" s="9" t="n">
+        <v>-1721210400</v>
+      </c>
+      <c r="Y55" s="9" t="n">
+        <v>-101247.6705882353</v>
+      </c>
+      <c r="Z55" s="9" t="n">
         <v>-9106933.333333334</v>
       </c>
     </row>
@@ -3335,6 +3801,15 @@
       <c r="U56" s="11" t="n"/>
       <c r="V56" s="11" t="n"/>
       <c r="W56" s="11" t="n"/>
+      <c r="X56" s="11" t="n">
+        <v>-2000000</v>
+      </c>
+      <c r="Y56" s="11" t="n">
+        <v>-117.6470588235294</v>
+      </c>
+      <c r="Z56" s="11" t="n">
+        <v>-10582.01058201058</v>
+      </c>
     </row>
     <row r="57">
       <c r="B57" s="8" t="inlineStr">
@@ -3399,6 +3874,15 @@
       <c r="W57" s="9" t="n">
         <v>-587301.5873015873</v>
       </c>
+      <c r="X57" s="9" t="n">
+        <v>-129500000</v>
+      </c>
+      <c r="Y57" s="9" t="n">
+        <v>-7617.64705882353</v>
+      </c>
+      <c r="Z57" s="9" t="n">
+        <v>-685185.1851851852</v>
+      </c>
     </row>
     <row r="58">
       <c r="B58" s="12" t="inlineStr">
@@ -3468,6 +3952,15 @@
       </c>
       <c r="W58" s="13" t="n">
         <v>-70651143.30624339</v>
+      </c>
+      <c r="X58" s="13" t="n">
+        <v>-14268982691.88</v>
+      </c>
+      <c r="Y58" s="13" t="n">
+        <v>-839351.9230517646</v>
+      </c>
+      <c r="Z58" s="13" t="n">
+        <v>-75497262.92</v>
       </c>
     </row>
     <row r="59">
@@ -3497,6 +3990,9 @@
       <c r="U59" s="15" t="n"/>
       <c r="V59" s="15" t="n"/>
       <c r="W59" s="15" t="n"/>
+      <c r="X59" s="15" t="n"/>
+      <c r="Y59" s="15" t="n"/>
+      <c r="Z59" s="15" t="n"/>
     </row>
     <row r="60">
       <c r="B60" s="8" t="inlineStr">
@@ -3537,6 +4033,15 @@
       <c r="W60" s="9" t="n">
         <v>-19170479.17460318</v>
       </c>
+      <c r="X60" s="9" t="n">
+        <v>-3623220564</v>
+      </c>
+      <c r="Y60" s="9" t="n">
+        <v>-213130.6214117647</v>
+      </c>
+      <c r="Z60" s="9" t="n">
+        <v>-19170479.17460318</v>
+      </c>
     </row>
     <row r="61">
       <c r="B61" s="10" t="inlineStr">
@@ -3577,6 +4082,15 @@
       <c r="W61" s="11" t="n">
         <v>-19170479.17460318</v>
       </c>
+      <c r="X61" s="11" t="n">
+        <v>-3623220564</v>
+      </c>
+      <c r="Y61" s="11" t="n">
+        <v>-213130.6214117647</v>
+      </c>
+      <c r="Z61" s="11" t="n">
+        <v>-19170479.17460318</v>
+      </c>
     </row>
     <row r="62">
       <c r="B62" s="8" t="inlineStr">
@@ -3623,6 +4137,15 @@
       <c r="W62" s="9" t="n">
         <v>-535387394.05291</v>
       </c>
+      <c r="X62" s="9" t="n">
+        <v>-101188217476</v>
+      </c>
+      <c r="Y62" s="9" t="n">
+        <v>-5952248.086823529</v>
+      </c>
+      <c r="Z62" s="9" t="n">
+        <v>-535387394.05291</v>
+      </c>
     </row>
     <row r="63">
       <c r="B63" s="10" t="inlineStr">
@@ -3667,6 +4190,15 @@
         <v>-5952248.086823529</v>
       </c>
       <c r="W63" s="11" t="n">
+        <v>-535387394.05291</v>
+      </c>
+      <c r="X63" s="11" t="n">
+        <v>-101188217476</v>
+      </c>
+      <c r="Y63" s="11" t="n">
+        <v>-5952248.086823529</v>
+      </c>
+      <c r="Z63" s="11" t="n">
         <v>-535387394.05291</v>
       </c>
     </row>
@@ -3709,6 +4241,15 @@
       <c r="W64" s="9" t="n">
         <v>-55908663.44444445</v>
       </c>
+      <c r="X64" s="9" t="n">
+        <v>-10566737391</v>
+      </c>
+      <c r="Y64" s="9" t="n">
+        <v>-621572.7877058823</v>
+      </c>
+      <c r="Z64" s="9" t="n">
+        <v>-55908663.44444445</v>
+      </c>
     </row>
     <row r="65">
       <c r="B65" s="10" t="inlineStr">
@@ -3749,6 +4290,15 @@
       <c r="W65" s="11" t="n">
         <v>-55908663.44444445</v>
       </c>
+      <c r="X65" s="11" t="n">
+        <v>-10566737391</v>
+      </c>
+      <c r="Y65" s="11" t="n">
+        <v>-621572.7877058823</v>
+      </c>
+      <c r="Z65" s="11" t="n">
+        <v>-55908663.44444445</v>
+      </c>
     </row>
     <row r="66">
       <c r="B66" s="12" t="inlineStr">
@@ -3793,6 +4343,15 @@
         <v>-6786951.495941176</v>
       </c>
       <c r="W66" s="13" t="n">
+        <v>-610466536.6719577</v>
+      </c>
+      <c r="X66" s="13" t="n">
+        <v>-115378175431</v>
+      </c>
+      <c r="Y66" s="13" t="n">
+        <v>-6786951.495941176</v>
+      </c>
+      <c r="Z66" s="13" t="n">
         <v>-610466536.6719577</v>
       </c>
     </row>
@@ -3823,6 +4382,9 @@
       <c r="U67" s="15" t="n"/>
       <c r="V67" s="15" t="n"/>
       <c r="W67" s="15" t="n"/>
+      <c r="X67" s="15" t="n"/>
+      <c r="Y67" s="15" t="n"/>
+      <c r="Z67" s="15" t="n"/>
     </row>
     <row r="68">
       <c r="B68" s="8" t="inlineStr">
@@ -3869,6 +4431,15 @@
       <c r="W68" s="9" t="n">
         <v>-26681372.67724868</v>
       </c>
+      <c r="X68" s="9" t="n">
+        <v>-5042779436</v>
+      </c>
+      <c r="Y68" s="9" t="n">
+        <v>-296634.0844705882</v>
+      </c>
+      <c r="Z68" s="9" t="n">
+        <v>-26681372.67724868</v>
+      </c>
     </row>
     <row r="69">
       <c r="B69" s="12" t="inlineStr">
@@ -3913,6 +4484,15 @@
         <v>-296634.0844705882</v>
       </c>
       <c r="W69" s="13" t="n">
+        <v>-26681372.67724868</v>
+      </c>
+      <c r="X69" s="13" t="n">
+        <v>-5042779436</v>
+      </c>
+      <c r="Y69" s="13" t="n">
+        <v>-296634.0844705882</v>
+      </c>
+      <c r="Z69" s="13" t="n">
         <v>-26681372.67724868</v>
       </c>
     </row>
@@ -3943,6 +4523,9 @@
       <c r="U70" s="15" t="n"/>
       <c r="V70" s="15" t="n"/>
       <c r="W70" s="15" t="n"/>
+      <c r="X70" s="15" t="n"/>
+      <c r="Y70" s="15" t="n"/>
+      <c r="Z70" s="15" t="n"/>
     </row>
     <row r="71">
       <c r="B71" s="8" t="inlineStr">
@@ -3983,6 +4566,15 @@
       <c r="W71" s="9" t="n">
         <v>-92285714.28571428</v>
       </c>
+      <c r="X71" s="9" t="n">
+        <v>-17442000000</v>
+      </c>
+      <c r="Y71" s="9" t="n">
+        <v>-1026000</v>
+      </c>
+      <c r="Z71" s="9" t="n">
+        <v>-92285714.28571428</v>
+      </c>
     </row>
     <row r="72">
       <c r="B72" s="10" t="inlineStr">
@@ -4027,6 +4619,15 @@
         <v>-2588235.294117647</v>
       </c>
       <c r="W72" s="11" t="n">
+        <v>-232804232.8042328</v>
+      </c>
+      <c r="X72" s="11" t="n">
+        <v>-44000000000</v>
+      </c>
+      <c r="Y72" s="11" t="n">
+        <v>-2588235.294117647</v>
+      </c>
+      <c r="Z72" s="11" t="n">
         <v>-232804232.8042328</v>
       </c>
     </row>
@@ -4069,6 +4670,15 @@
       <c r="W73" s="9" t="n">
         <v>-80729414.68253969</v>
       </c>
+      <c r="X73" s="9" t="n">
+        <v>-15257859375</v>
+      </c>
+      <c r="Y73" s="9" t="n">
+        <v>-897521.1397058824</v>
+      </c>
+      <c r="Z73" s="9" t="n">
+        <v>-80729414.68253969</v>
+      </c>
     </row>
     <row r="74">
       <c r="B74" s="12" t="inlineStr">
@@ -4119,6 +4729,15 @@
         <v>-4511756.43382353</v>
       </c>
       <c r="W74" s="13" t="n">
+        <v>-405819361.7724867</v>
+      </c>
+      <c r="X74" s="13" t="n">
+        <v>-76699859375</v>
+      </c>
+      <c r="Y74" s="13" t="n">
+        <v>-4511756.43382353</v>
+      </c>
+      <c r="Z74" s="13" t="n">
         <v>-405819361.7724867</v>
       </c>
     </row>
@@ -4149,6 +4768,9 @@
       <c r="U75" s="15" t="n"/>
       <c r="V75" s="15" t="n"/>
       <c r="W75" s="15" t="n"/>
+      <c r="X75" s="15" t="n"/>
+      <c r="Y75" s="15" t="n"/>
+      <c r="Z75" s="15" t="n"/>
     </row>
     <row r="76">
       <c r="B76" s="8" t="inlineStr">
@@ -4219,6 +4841,15 @@
       <c r="W76" s="9" t="n">
         <v>-29097655.32275132</v>
       </c>
+      <c r="X76" s="9" t="n">
+        <v>-6081007428</v>
+      </c>
+      <c r="Y76" s="9" t="n">
+        <v>-357706.3192941176</v>
+      </c>
+      <c r="Z76" s="9" t="n">
+        <v>-32174642.47619047</v>
+      </c>
     </row>
     <row r="77">
       <c r="B77" s="10" t="inlineStr">
@@ -4289,6 +4920,15 @@
       <c r="W77" s="11" t="n">
         <v>-30154353.86529101</v>
       </c>
+      <c r="X77" s="11" t="n">
+        <v>-7025874357.54</v>
+      </c>
+      <c r="Y77" s="11" t="n">
+        <v>-413286.7269141176</v>
+      </c>
+      <c r="Z77" s="11" t="n">
+        <v>-37173938.39968254</v>
+      </c>
     </row>
     <row r="78">
       <c r="B78" s="8" t="inlineStr">
@@ -4359,6 +4999,15 @@
       <c r="W78" s="9" t="n">
         <v>-28420237.08465608</v>
       </c>
+      <c r="X78" s="9" t="n">
+        <v>-6247229890</v>
+      </c>
+      <c r="Y78" s="9" t="n">
+        <v>-367484.1111764705</v>
+      </c>
+      <c r="Z78" s="9" t="n">
+        <v>-33054126.4021164</v>
+      </c>
     </row>
     <row r="79">
       <c r="B79" s="10" t="inlineStr">
@@ -4429,6 +5078,15 @@
       <c r="W79" s="11" t="n">
         <v>-2004303.851851852</v>
       </c>
+      <c r="X79" s="11" t="n">
+        <v>-386997197</v>
+      </c>
+      <c r="Y79" s="11" t="n">
+        <v>-22764.541</v>
+      </c>
+      <c r="Z79" s="11" t="n">
+        <v>-2047604.216931217</v>
+      </c>
     </row>
     <row r="80">
       <c r="B80" s="12" t="inlineStr">
@@ -4498,6 +5156,15 @@
       </c>
       <c r="W80" s="13" t="n">
         <v>-89676550.12455027</v>
+      </c>
+      <c r="X80" s="13" t="n">
+        <v>-19741108872.54</v>
+      </c>
+      <c r="Y80" s="13" t="n">
+        <v>-1161241.698384706</v>
+      </c>
+      <c r="Z80" s="13" t="n">
+        <v>-104450311.4949206</v>
       </c>
     </row>
     <row r="81">
@@ -4527,6 +5194,9 @@
       <c r="U81" s="15" t="n"/>
       <c r="V81" s="15" t="n"/>
       <c r="W81" s="15" t="n"/>
+      <c r="X81" s="15" t="n"/>
+      <c r="Y81" s="15" t="n"/>
+      <c r="Z81" s="15" t="n"/>
     </row>
     <row r="82">
       <c r="B82" s="14" t="inlineStr">
@@ -4555,6 +5225,9 @@
       <c r="U82" s="15" t="n"/>
       <c r="V82" s="15" t="n"/>
       <c r="W82" s="15" t="n"/>
+      <c r="X82" s="15" t="n"/>
+      <c r="Y82" s="15" t="n"/>
+      <c r="Z82" s="15" t="n"/>
     </row>
     <row r="83">
       <c r="B83" s="8" t="inlineStr">
@@ -4624,6 +5297,15 @@
       </c>
       <c r="W83" s="9" t="n">
         <v>-535741.6243386244</v>
+      </c>
+      <c r="X83" s="9" t="n">
+        <v>-118254829</v>
+      </c>
+      <c r="Y83" s="9" t="n">
+        <v>-6956.166411764707</v>
+      </c>
+      <c r="Z83" s="9" t="n">
+        <v>-625686.925925926</v>
       </c>
     </row>
     <row r="84">
@@ -4653,6 +5335,15 @@
       <c r="U84" s="11" t="n"/>
       <c r="V84" s="11" t="n"/>
       <c r="W84" s="11" t="n"/>
+      <c r="X84" s="11" t="n">
+        <v>-2626600</v>
+      </c>
+      <c r="Y84" s="11" t="n">
+        <v>-154.5058823529412</v>
+      </c>
+      <c r="Z84" s="11" t="n">
+        <v>-13897.3544973545</v>
+      </c>
     </row>
     <row r="85">
       <c r="B85" s="8" t="inlineStr">
@@ -4705,6 +5396,15 @@
       <c r="W85" s="9" t="n">
         <v>-41493.14814814815</v>
       </c>
+      <c r="X85" s="9" t="n">
+        <v>-7842205</v>
+      </c>
+      <c r="Y85" s="9" t="n">
+        <v>-461.3061764705883</v>
+      </c>
+      <c r="Z85" s="9" t="n">
+        <v>-41493.14814814815</v>
+      </c>
     </row>
     <row r="86">
       <c r="B86" s="10" t="inlineStr">
@@ -4757,6 +5457,15 @@
       <c r="W86" s="11" t="n">
         <v>-8627.340952380953</v>
       </c>
+      <c r="X86" s="11" t="n">
+        <v>-1630567.44</v>
+      </c>
+      <c r="Y86" s="11" t="n">
+        <v>-95.91573176470587</v>
+      </c>
+      <c r="Z86" s="11" t="n">
+        <v>-8627.340952380953</v>
+      </c>
     </row>
     <row r="87">
       <c r="B87" s="8" t="inlineStr">
@@ -4826,6 +5535,15 @@
       </c>
       <c r="W87" s="9" t="n">
         <v>-408891.4603174604</v>
+      </c>
+      <c r="X87" s="9" t="n">
+        <v>-97615961</v>
+      </c>
+      <c r="Y87" s="9" t="n">
+        <v>-5742.115352941176</v>
+      </c>
+      <c r="Z87" s="9" t="n">
+        <v>-516486.5661375662</v>
       </c>
     </row>
     <row r="88">
@@ -4885,6 +5603,15 @@
       <c r="W88" s="11" t="n">
         <v>-4466.650793650793</v>
       </c>
+      <c r="X88" s="11" t="n">
+        <v>-1661696</v>
+      </c>
+      <c r="Y88" s="11" t="n">
+        <v>-97.74682352941177</v>
+      </c>
+      <c r="Z88" s="11" t="n">
+        <v>-8792.042328042327</v>
+      </c>
     </row>
     <row r="89">
       <c r="B89" s="12" t="inlineStr">
@@ -4954,6 +5681,15 @@
       </c>
       <c r="W89" s="13" t="n">
         <v>-999220.2245502645</v>
+      </c>
+      <c r="X89" s="13" t="n">
+        <v>-229631858.44</v>
+      </c>
+      <c r="Y89" s="13" t="n">
+        <v>-13507.75637882353</v>
+      </c>
+      <c r="Z89" s="13" t="n">
+        <v>-1214983.377989418</v>
       </c>
     </row>
     <row r="90">
@@ -4983,6 +5719,9 @@
       <c r="U90" s="15" t="n"/>
       <c r="V90" s="15" t="n"/>
       <c r="W90" s="15" t="n"/>
+      <c r="X90" s="15" t="n"/>
+      <c r="Y90" s="15" t="n"/>
+      <c r="Z90" s="15" t="n"/>
     </row>
     <row r="91">
       <c r="B91" s="8" t="inlineStr">
@@ -5035,6 +5774,15 @@
       <c r="W91" s="9" t="n">
         <v>-448105.8201058201</v>
       </c>
+      <c r="X91" s="9" t="n">
+        <v>-85844000</v>
+      </c>
+      <c r="Y91" s="9" t="n">
+        <v>-5049.64705882353</v>
+      </c>
+      <c r="Z91" s="9" t="n">
+        <v>-454201.0582010582</v>
+      </c>
     </row>
     <row r="92">
       <c r="B92" s="10" t="inlineStr">
@@ -5105,6 +5853,15 @@
       <c r="W92" s="11" t="n">
         <v>-928151.4708994708</v>
       </c>
+      <c r="X92" s="11" t="n">
+        <v>-185879421</v>
+      </c>
+      <c r="Y92" s="11" t="n">
+        <v>-10934.08358823529</v>
+      </c>
+      <c r="Z92" s="11" t="n">
+        <v>-983489</v>
+      </c>
     </row>
     <row r="93">
       <c r="B93" s="8" t="inlineStr">
@@ -5175,6 +5932,15 @@
       <c r="W93" s="9" t="n">
         <v>-31322241.6373545</v>
       </c>
+      <c r="X93" s="9" t="n">
+        <v>-6530220650.46</v>
+      </c>
+      <c r="Y93" s="9" t="n">
+        <v>-384130.626497647</v>
+      </c>
+      <c r="Z93" s="9" t="n">
+        <v>-34551432.01301587</v>
+      </c>
     </row>
     <row r="94">
       <c r="B94" s="10" t="inlineStr">
@@ -5245,6 +6011,15 @@
       <c r="W94" s="11" t="n">
         <v>-863608.5714285714</v>
       </c>
+      <c r="X94" s="11" t="n">
+        <v>-193699732</v>
+      </c>
+      <c r="Y94" s="11" t="n">
+        <v>-11394.10188235294</v>
+      </c>
+      <c r="Z94" s="11" t="n">
+        <v>-1024866.306878307</v>
+      </c>
     </row>
     <row r="95">
       <c r="B95" s="8" t="inlineStr">
@@ -5315,6 +6090,15 @@
       <c r="W95" s="9" t="n">
         <v>-1461407.195767196</v>
       </c>
+      <c r="X95" s="9" t="n">
+        <v>-291202982</v>
+      </c>
+      <c r="Y95" s="9" t="n">
+        <v>-17129.58717647059</v>
+      </c>
+      <c r="Z95" s="9" t="n">
+        <v>-1540756.518518518</v>
+      </c>
     </row>
     <row r="96">
       <c r="B96" s="12" t="inlineStr">
@@ -5384,6 +6168,15 @@
       </c>
       <c r="W96" s="13" t="n">
         <v>-35023514.69555555</v>
+      </c>
+      <c r="X96" s="13" t="n">
+        <v>-7286846785.46</v>
+      </c>
+      <c r="Y96" s="13" t="n">
+        <v>-428638.0462035294</v>
+      </c>
+      <c r="Z96" s="13" t="n">
+        <v>-38554744.89661375</v>
       </c>
     </row>
     <row r="97">
@@ -5413,6 +6206,9 @@
       <c r="U97" s="15" t="n"/>
       <c r="V97" s="15" t="n"/>
       <c r="W97" s="15" t="n"/>
+      <c r="X97" s="15" t="n"/>
+      <c r="Y97" s="15" t="n"/>
+      <c r="Z97" s="15" t="n"/>
     </row>
     <row r="98">
       <c r="B98" s="8" t="inlineStr">
@@ -5483,6 +6279,15 @@
       <c r="W98" s="9" t="n">
         <v>-921841.8095238095</v>
       </c>
+      <c r="X98" s="9" t="n">
+        <v>-182969927</v>
+      </c>
+      <c r="Y98" s="9" t="n">
+        <v>-10762.93688235294</v>
+      </c>
+      <c r="Z98" s="9" t="n">
+        <v>-968094.8518518518</v>
+      </c>
     </row>
     <row r="99">
       <c r="B99" s="10" t="inlineStr">
@@ -5553,6 +6358,15 @@
       <c r="W99" s="11" t="n">
         <v>-682307.5502645504</v>
       </c>
+      <c r="X99" s="11" t="n">
+        <v>-160047281</v>
+      </c>
+      <c r="Y99" s="11" t="n">
+        <v>-9414.545941176471</v>
+      </c>
+      <c r="Z99" s="11" t="n">
+        <v>-846811.0105820107</v>
+      </c>
     </row>
     <row r="100">
       <c r="B100" s="8" t="inlineStr">
@@ -5622,6 +6436,15 @@
       </c>
       <c r="W100" s="9" t="n">
         <v>-5278634.232804232</v>
+      </c>
+      <c r="X100" s="9" t="n">
+        <v>-1191659872</v>
+      </c>
+      <c r="Y100" s="9" t="n">
+        <v>-70097.63952941177</v>
+      </c>
+      <c r="Z100" s="9" t="n">
+        <v>-6305078.687830688</v>
       </c>
     </row>
     <row r="101">
@@ -5687,6 +6510,15 @@
       <c r="W101" s="11" t="n">
         <v>-595172.2222222222</v>
       </c>
+      <c r="X101" s="11" t="n">
+        <v>-156363790</v>
+      </c>
+      <c r="Y101" s="11" t="n">
+        <v>-9197.870000000001</v>
+      </c>
+      <c r="Z101" s="11" t="n">
+        <v>-827321.6402116403</v>
+      </c>
     </row>
     <row r="102">
       <c r="B102" s="12" t="inlineStr">
@@ -5756,6 +6588,15 @@
       </c>
       <c r="W102" s="13" t="n">
         <v>-7477955.814814815</v>
+      </c>
+      <c r="X102" s="13" t="n">
+        <v>-1691040870</v>
+      </c>
+      <c r="Y102" s="13" t="n">
+        <v>-99472.99235294119</v>
+      </c>
+      <c r="Z102" s="13" t="n">
+        <v>-8947306.19047619</v>
       </c>
     </row>
     <row r="103">
@@ -5785,6 +6626,9 @@
       <c r="U103" s="15" t="n"/>
       <c r="V103" s="15" t="n"/>
       <c r="W103" s="15" t="n"/>
+      <c r="X103" s="15" t="n"/>
+      <c r="Y103" s="15" t="n"/>
+      <c r="Z103" s="15" t="n"/>
     </row>
     <row r="104">
       <c r="B104" s="8" t="inlineStr">
@@ -5848,6 +6692,15 @@
       </c>
       <c r="W104" s="9" t="n">
         <v>-674262.4338624338</v>
+      </c>
+      <c r="X104" s="9" t="n">
+        <v>-131465600</v>
+      </c>
+      <c r="Y104" s="9" t="n">
+        <v>-7733.270588235294</v>
+      </c>
+      <c r="Z104" s="9" t="n">
+        <v>-695585.1851851851</v>
       </c>
     </row>
     <row r="105">
@@ -5889,6 +6742,15 @@
       <c r="W105" s="11" t="n">
         <v>-12174.60317460317</v>
       </c>
+      <c r="X105" s="11" t="n">
+        <v>-8238500</v>
+      </c>
+      <c r="Y105" s="11" t="n">
+        <v>-484.6176470588235</v>
+      </c>
+      <c r="Z105" s="11" t="n">
+        <v>-43589.94708994709</v>
+      </c>
     </row>
     <row r="106">
       <c r="B106" s="8" t="inlineStr">
@@ -5959,6 +6821,15 @@
       <c r="W106" s="9" t="n">
         <v>-1153318.253968254</v>
       </c>
+      <c r="X106" s="9" t="n">
+        <v>-365550111</v>
+      </c>
+      <c r="Y106" s="9" t="n">
+        <v>-21502.94770588235</v>
+      </c>
+      <c r="Z106" s="9" t="n">
+        <v>-1934127.571428571</v>
+      </c>
     </row>
     <row r="107">
       <c r="B107" s="12" t="inlineStr">
@@ -6028,6 +6899,15 @@
       </c>
       <c r="W107" s="13" t="n">
         <v>-1839755.291005291</v>
+      </c>
+      <c r="X107" s="13" t="n">
+        <v>-505254211</v>
+      </c>
+      <c r="Y107" s="13" t="n">
+        <v>-29720.83594117647</v>
+      </c>
+      <c r="Z107" s="13" t="n">
+        <v>-2673302.703703704</v>
       </c>
     </row>
     <row r="108">
@@ -6057,6 +6937,9 @@
       <c r="U108" s="15" t="n"/>
       <c r="V108" s="15" t="n"/>
       <c r="W108" s="15" t="n"/>
+      <c r="X108" s="15" t="n"/>
+      <c r="Y108" s="15" t="n"/>
+      <c r="Z108" s="15" t="n"/>
     </row>
     <row r="109">
       <c r="B109" s="8" t="inlineStr">
@@ -6120,6 +7003,15 @@
       </c>
       <c r="W109" s="9" t="n">
         <v>-1726759.650793651</v>
+      </c>
+      <c r="X109" s="9" t="n">
+        <v>-352517574</v>
+      </c>
+      <c r="Y109" s="9" t="n">
+        <v>-20736.32788235294</v>
+      </c>
+      <c r="Z109" s="9" t="n">
+        <v>-1865172.349206349</v>
       </c>
     </row>
     <row r="110">
@@ -6149,6 +7041,15 @@
       <c r="U110" s="11" t="n"/>
       <c r="V110" s="11" t="n"/>
       <c r="W110" s="11" t="n"/>
+      <c r="X110" s="11" t="n">
+        <v>-13000000</v>
+      </c>
+      <c r="Y110" s="11" t="n">
+        <v>-764.7058823529412</v>
+      </c>
+      <c r="Z110" s="11" t="n">
+        <v>-68783.06878306878</v>
+      </c>
     </row>
     <row r="111">
       <c r="B111" s="8" t="inlineStr">
@@ -6219,6 +7120,15 @@
       <c r="W111" s="9" t="n">
         <v>-617278.0687830688</v>
       </c>
+      <c r="X111" s="9" t="n">
+        <v>-123269133</v>
+      </c>
+      <c r="Y111" s="9" t="n">
+        <v>-7251.125470588236</v>
+      </c>
+      <c r="Z111" s="9" t="n">
+        <v>-652217.6349206349</v>
+      </c>
     </row>
     <row r="112">
       <c r="B112" s="10" t="inlineStr">
@@ -6289,6 +7199,15 @@
       <c r="W112" s="11" t="n">
         <v>-1315173.513227513</v>
       </c>
+      <c r="X112" s="11" t="n">
+        <v>-413518543</v>
+      </c>
+      <c r="Y112" s="11" t="n">
+        <v>-24324.62017647059</v>
+      </c>
+      <c r="Z112" s="11" t="n">
+        <v>-2187928.798941799</v>
+      </c>
     </row>
     <row r="113">
       <c r="B113" s="12" t="inlineStr">
@@ -6358,6 +7277,15 @@
       </c>
       <c r="W113" s="13" t="n">
         <v>-3659211.232804233</v>
+      </c>
+      <c r="X113" s="13" t="n">
+        <v>-902305250</v>
+      </c>
+      <c r="Y113" s="13" t="n">
+        <v>-53076.77941176471</v>
+      </c>
+      <c r="Z113" s="13" t="n">
+        <v>-4774101.851851852</v>
       </c>
     </row>
     <row r="114">
@@ -6387,6 +7315,9 @@
       <c r="U114" s="15" t="n"/>
       <c r="V114" s="15" t="n"/>
       <c r="W114" s="15" t="n"/>
+      <c r="X114" s="15" t="n"/>
+      <c r="Y114" s="15" t="n"/>
+      <c r="Z114" s="15" t="n"/>
     </row>
     <row r="115">
       <c r="B115" s="8" t="inlineStr">
@@ -6457,6 +7388,15 @@
       <c r="W115" s="9" t="n">
         <v>-21743746.34391534</v>
       </c>
+      <c r="X115" s="9" t="n">
+        <v>-4845172432</v>
+      </c>
+      <c r="Y115" s="9" t="n">
+        <v>-285010.1430588235</v>
+      </c>
+      <c r="Z115" s="9" t="n">
+        <v>-25635832.97354497</v>
+      </c>
     </row>
     <row r="116">
       <c r="B116" s="12" t="inlineStr">
@@ -6526,6 +7466,15 @@
       </c>
       <c r="W116" s="13" t="n">
         <v>-21743746.34391534</v>
+      </c>
+      <c r="X116" s="13" t="n">
+        <v>-4845172432</v>
+      </c>
+      <c r="Y116" s="13" t="n">
+        <v>-285010.1430588235</v>
+      </c>
+      <c r="Z116" s="13" t="n">
+        <v>-25635832.97354497</v>
       </c>
     </row>
     <row r="117">
@@ -6555,6 +7504,9 @@
       <c r="U117" s="15" t="n"/>
       <c r="V117" s="15" t="n"/>
       <c r="W117" s="15" t="n"/>
+      <c r="X117" s="15" t="n"/>
+      <c r="Y117" s="15" t="n"/>
+      <c r="Z117" s="15" t="n"/>
     </row>
     <row r="118">
       <c r="B118" s="8" t="inlineStr">
@@ -6605,6 +7557,15 @@
         <v>-338842.8851764706</v>
       </c>
       <c r="W118" s="9" t="n">
+        <v>-30477931.47089947</v>
+      </c>
+      <c r="X118" s="9" t="n">
+        <v>-5760329048</v>
+      </c>
+      <c r="Y118" s="9" t="n">
+        <v>-338842.8851764706</v>
+      </c>
+      <c r="Z118" s="9" t="n">
         <v>-30477931.47089947</v>
       </c>
     </row>
@@ -6647,6 +7608,15 @@
       <c r="W119" s="11" t="n">
         <v>-9685637.142857144</v>
       </c>
+      <c r="X119" s="11" t="n">
+        <v>-1830585420</v>
+      </c>
+      <c r="Y119" s="11" t="n">
+        <v>-107681.4952941176</v>
+      </c>
+      <c r="Z119" s="11" t="n">
+        <v>-9685637.142857144</v>
+      </c>
     </row>
     <row r="120">
       <c r="B120" s="8" t="inlineStr">
@@ -6717,6 +7687,15 @@
       <c r="W120" s="9" t="n">
         <v>-79822.6507936508</v>
       </c>
+      <c r="X120" s="9" t="n">
+        <v>-16814481</v>
+      </c>
+      <c r="Y120" s="9" t="n">
+        <v>-989.0871176470588</v>
+      </c>
+      <c r="Z120" s="9" t="n">
+        <v>-88965.50793650794</v>
+      </c>
     </row>
     <row r="121">
       <c r="B121" s="10" t="inlineStr">
@@ -6786,6 +7765,15 @@
       </c>
       <c r="W121" s="11" t="n">
         <v>-6957568.632116402</v>
+      </c>
+      <c r="X121" s="11" t="n">
+        <v>-1555850477.47</v>
+      </c>
+      <c r="Y121" s="11" t="n">
+        <v>-91520.6163217647</v>
+      </c>
+      <c r="Z121" s="11" t="n">
+        <v>-8232013.108306877</v>
       </c>
     </row>
     <row r="122">
@@ -6845,6 +7833,15 @@
       <c r="W122" s="9" t="n">
         <v>-952626.9841269843</v>
       </c>
+      <c r="X122" s="9" t="n">
+        <v>-299875500</v>
+      </c>
+      <c r="Y122" s="9" t="n">
+        <v>-17639.73529411765</v>
+      </c>
+      <c r="Z122" s="9" t="n">
+        <v>-1586642.857142857</v>
+      </c>
     </row>
     <row r="123">
       <c r="B123" s="10" t="inlineStr">
@@ -6915,6 +7912,15 @@
       <c r="W123" s="11" t="n">
         <v>-69613980.12698412</v>
       </c>
+      <c r="X123" s="11" t="n">
+        <v>-13932690388</v>
+      </c>
+      <c r="Y123" s="11" t="n">
+        <v>-819570.0228235294</v>
+      </c>
+      <c r="Z123" s="11" t="n">
+        <v>-73717938.56084655</v>
+      </c>
     </row>
     <row r="124">
       <c r="B124" s="12" t="inlineStr">
@@ -6984,6 +7990,15 @@
       </c>
       <c r="W124" s="13" t="n">
         <v>-117767567.0077778</v>
+      </c>
+      <c r="X124" s="13" t="n">
+        <v>-23396145314.47</v>
+      </c>
+      <c r="Y124" s="13" t="n">
+        <v>-1376243.842027647</v>
+      </c>
+      <c r="Z124" s="13" t="n">
+        <v>-123789128.6479894</v>
       </c>
     </row>
     <row r="125">
@@ -7013,6 +8028,9 @@
       <c r="U125" s="15" t="n"/>
       <c r="V125" s="15" t="n"/>
       <c r="W125" s="15" t="n"/>
+      <c r="X125" s="15" t="n"/>
+      <c r="Y125" s="15" t="n"/>
+      <c r="Z125" s="15" t="n"/>
     </row>
     <row r="126">
       <c r="B126" s="8" t="inlineStr">
@@ -7071,6 +8089,15 @@
       <c r="W126" s="9" t="n">
         <v>-121546.9312169312</v>
       </c>
+      <c r="X126" s="9" t="n">
+        <v>-26713320</v>
+      </c>
+      <c r="Y126" s="9" t="n">
+        <v>-1571.371764705882</v>
+      </c>
+      <c r="Z126" s="9" t="n">
+        <v>-141340.3174603175</v>
+      </c>
     </row>
     <row r="127">
       <c r="B127" s="10" t="inlineStr">
@@ -7129,6 +8156,15 @@
       <c r="W127" s="11" t="n">
         <v>-654218.0052910054</v>
       </c>
+      <c r="X127" s="11" t="n">
+        <v>-184037662</v>
+      </c>
+      <c r="Y127" s="11" t="n">
+        <v>-10825.74482352941</v>
+      </c>
+      <c r="Z127" s="11" t="n">
+        <v>-973744.2433862435</v>
+      </c>
     </row>
     <row r="128">
       <c r="B128" s="8" t="inlineStr">
@@ -7199,6 +8235,15 @@
       <c r="W128" s="9" t="n">
         <v>-1093348.444444444</v>
       </c>
+      <c r="X128" s="9" t="n">
+        <v>-206642856</v>
+      </c>
+      <c r="Y128" s="9" t="n">
+        <v>-12155.46211764706</v>
+      </c>
+      <c r="Z128" s="9" t="n">
+        <v>-1093348.444444444</v>
+      </c>
     </row>
     <row r="129">
       <c r="B129" s="10" t="inlineStr">
@@ -7269,6 +8314,15 @@
       <c r="W129" s="11" t="n">
         <v>-424776.1058201058</v>
       </c>
+      <c r="X129" s="11" t="n">
+        <v>-92308428</v>
+      </c>
+      <c r="Y129" s="11" t="n">
+        <v>-5429.907529411764</v>
+      </c>
+      <c r="Z129" s="11" t="n">
+        <v>-488404.3809523809</v>
+      </c>
     </row>
     <row r="130">
       <c r="B130" s="8" t="inlineStr">
@@ -7338,6 +8392,15 @@
       </c>
       <c r="W130" s="9" t="n">
         <v>-933465.5238095238</v>
+      </c>
+      <c r="X130" s="9" t="n">
+        <v>-199819215</v>
+      </c>
+      <c r="Y130" s="9" t="n">
+        <v>-11754.07147058823</v>
+      </c>
+      <c r="Z130" s="9" t="n">
+        <v>-1057244.523809524</v>
       </c>
     </row>
     <row r="131">
@@ -7379,6 +8442,15 @@
       <c r="W131" s="11" t="n">
         <v>-5820.10582010582</v>
       </c>
+      <c r="X131" s="11" t="n">
+        <v>-1100000</v>
+      </c>
+      <c r="Y131" s="11" t="n">
+        <v>-64.70588235294117</v>
+      </c>
+      <c r="Z131" s="11" t="n">
+        <v>-5820.10582010582</v>
+      </c>
     </row>
     <row r="132">
       <c r="B132" s="12" t="inlineStr">
@@ -7449,6 +8521,15 @@
       <c r="W132" s="13" t="n">
         <v>-3233175.116402117</v>
       </c>
+      <c r="X132" s="13" t="n">
+        <v>-710621481</v>
+      </c>
+      <c r="Y132" s="13" t="n">
+        <v>-41801.26358823529</v>
+      </c>
+      <c r="Z132" s="13" t="n">
+        <v>-3759902.015873016</v>
+      </c>
     </row>
     <row r="133">
       <c r="B133" s="12" t="inlineStr">
@@ -7518,6 +8599,15 @@
       </c>
       <c r="W133" s="13" t="n">
         <v>-191744145.7268254</v>
+      </c>
+      <c r="X133" s="13" t="n">
+        <v>-39567018202.37</v>
+      </c>
+      <c r="Y133" s="13" t="n">
+        <v>-2327471.658962942</v>
+      </c>
+      <c r="Z133" s="13" t="n">
+        <v>-209349302.6580423</v>
       </c>
     </row>
     <row r="134">
@@ -7547,6 +8637,9 @@
       <c r="U134" s="15" t="n"/>
       <c r="V134" s="15" t="n"/>
       <c r="W134" s="15" t="n"/>
+      <c r="X134" s="15" t="n"/>
+      <c r="Y134" s="15" t="n"/>
+      <c r="Z134" s="15" t="n"/>
     </row>
     <row r="135">
       <c r="B135" s="8" t="inlineStr">
@@ -7603,6 +8696,15 @@
         <v>-5058.823529411765</v>
       </c>
       <c r="W135" s="9" t="n">
+        <v>-455026.455026455</v>
+      </c>
+      <c r="X135" s="9" t="n">
+        <v>-86000000</v>
+      </c>
+      <c r="Y135" s="9" t="n">
+        <v>-5058.823529411765</v>
+      </c>
+      <c r="Z135" s="9" t="n">
         <v>-455026.455026455</v>
       </c>
     </row>
@@ -7633,6 +8735,15 @@
       <c r="U136" s="11" t="n"/>
       <c r="V136" s="11" t="n"/>
       <c r="W136" s="11" t="n"/>
+      <c r="X136" s="11" t="n">
+        <v>-5000000</v>
+      </c>
+      <c r="Y136" s="11" t="n">
+        <v>-294.1176470588235</v>
+      </c>
+      <c r="Z136" s="11" t="n">
+        <v>-26455.02645502645</v>
+      </c>
     </row>
     <row r="137">
       <c r="B137" s="8" t="inlineStr">
@@ -7702,6 +8813,15 @@
       </c>
       <c r="W137" s="9" t="n">
         <v>-3102749.708994709</v>
+      </c>
+      <c r="X137" s="9" t="n">
+        <v>-678771055</v>
+      </c>
+      <c r="Y137" s="9" t="n">
+        <v>-39927.70911764706</v>
+      </c>
+      <c r="Z137" s="9" t="n">
+        <v>-3591381.243386243</v>
       </c>
     </row>
     <row r="138">
@@ -7743,6 +8863,15 @@
       <c r="W138" s="11" t="n">
         <v>-8289354.497354497</v>
       </c>
+      <c r="X138" s="11" t="n">
+        <v>-1566688000</v>
+      </c>
+      <c r="Y138" s="11" t="n">
+        <v>-92158.11764705883</v>
+      </c>
+      <c r="Z138" s="11" t="n">
+        <v>-8289354.497354497</v>
+      </c>
     </row>
     <row r="139">
       <c r="B139" s="8" t="inlineStr">
@@ -7783,6 +8912,15 @@
       <c r="W139" s="9" t="n">
         <v>-44576.71957671957</v>
       </c>
+      <c r="X139" s="9" t="n">
+        <v>-8425000</v>
+      </c>
+      <c r="Y139" s="9" t="n">
+        <v>-495.5882352941176</v>
+      </c>
+      <c r="Z139" s="9" t="n">
+        <v>-44576.71957671957</v>
+      </c>
     </row>
     <row r="140">
       <c r="B140" s="12" t="inlineStr">
@@ -7852,6 +8990,15 @@
       </c>
       <c r="W140" s="13" t="n">
         <v>-11891707.38095238</v>
+      </c>
+      <c r="X140" s="13" t="n">
+        <v>-2344884055</v>
+      </c>
+      <c r="Y140" s="13" t="n">
+        <v>-137934.3561764706</v>
+      </c>
+      <c r="Z140" s="13" t="n">
+        <v>-12406793.94179894</v>
       </c>
     </row>
     <row r="141">
@@ -7881,6 +9028,9 @@
       <c r="U141" s="15" t="n"/>
       <c r="V141" s="15" t="n"/>
       <c r="W141" s="15" t="n"/>
+      <c r="X141" s="15" t="n"/>
+      <c r="Y141" s="15" t="n"/>
+      <c r="Z141" s="15" t="n"/>
     </row>
     <row r="142">
       <c r="B142" s="8" t="inlineStr">
@@ -7950,6 +9100,15 @@
       </c>
       <c r="W142" s="9" t="n">
         <v>-75097.76550264549</v>
+      </c>
+      <c r="X142" s="9" t="n">
+        <v>-16272731.68</v>
+      </c>
+      <c r="Y142" s="9" t="n">
+        <v>-957.2195105882353</v>
+      </c>
+      <c r="Z142" s="9" t="n">
+        <v>-86099.1094179894</v>
       </c>
     </row>
     <row r="143">
@@ -7997,6 +9156,15 @@
       <c r="W143" s="11" t="n">
         <v>-275204.6190476191</v>
       </c>
+      <c r="X143" s="11" t="n">
+        <v>-52013673</v>
+      </c>
+      <c r="Y143" s="11" t="n">
+        <v>-3059.627823529412</v>
+      </c>
+      <c r="Z143" s="11" t="n">
+        <v>-275204.6190476191</v>
+      </c>
     </row>
     <row r="144">
       <c r="B144" s="8" t="inlineStr">
@@ -8055,6 +9223,15 @@
       <c r="W144" s="9" t="n">
         <v>-49496.48227513227</v>
       </c>
+      <c r="X144" s="9" t="n">
+        <v>-9354835.15</v>
+      </c>
+      <c r="Y144" s="9" t="n">
+        <v>-550.2844205882353</v>
+      </c>
+      <c r="Z144" s="9" t="n">
+        <v>-49496.48227513227</v>
+      </c>
     </row>
     <row r="145">
       <c r="B145" s="10" t="inlineStr">
@@ -8124,6 +9301,15 @@
       </c>
       <c r="W145" s="11" t="n">
         <v>-20527066.32576719</v>
+      </c>
+      <c r="X145" s="11" t="n">
+        <v>-4071177960.57</v>
+      </c>
+      <c r="Y145" s="11" t="n">
+        <v>-239481.0565041177</v>
+      </c>
+      <c r="Z145" s="11" t="n">
+        <v>-21540624.13</v>
       </c>
     </row>
     <row r="146">
@@ -8181,6 +9367,15 @@
         <v>-37801.23429411765</v>
       </c>
       <c r="W146" s="9" t="n">
+        <v>-3400111.021164021</v>
+      </c>
+      <c r="X146" s="9" t="n">
+        <v>-642620983</v>
+      </c>
+      <c r="Y146" s="9" t="n">
+        <v>-37801.23429411765</v>
+      </c>
+      <c r="Z146" s="9" t="n">
         <v>-3400111.021164021</v>
       </c>
     </row>
@@ -8223,6 +9418,15 @@
       <c r="W147" s="11" t="n">
         <v>-4094664.19047619</v>
       </c>
+      <c r="X147" s="11" t="n">
+        <v>-773891532</v>
+      </c>
+      <c r="Y147" s="11" t="n">
+        <v>-45523.03129411765</v>
+      </c>
+      <c r="Z147" s="11" t="n">
+        <v>-4094664.19047619</v>
+      </c>
     </row>
     <row r="148">
       <c r="B148" s="12" t="inlineStr">
@@ -8293,6 +9497,15 @@
       <c r="W148" s="13" t="n">
         <v>-28421640.40423281</v>
       </c>
+      <c r="X148" s="13" t="n">
+        <v>-5565331715.4</v>
+      </c>
+      <c r="Y148" s="13" t="n">
+        <v>-327372.4538470588</v>
+      </c>
+      <c r="Z148" s="13" t="n">
+        <v>-29446199.55238096</v>
+      </c>
     </row>
     <row r="149">
       <c r="B149" s="16" t="inlineStr">
@@ -8363,6 +9576,15 @@
       <c r="W149" s="17" t="n">
         <v>-1435352458.064497</v>
       </c>
+      <c r="X149" s="17" t="n">
+        <v>-278608139779.19</v>
+      </c>
+      <c r="Y149" s="17" t="n">
+        <v>-16388714.10465823</v>
+      </c>
+      <c r="Z149" s="17" t="n">
+        <v>-1474117141.688836</v>
+      </c>
     </row>
     <row r="150">
       <c r="B150" s="16" t="inlineStr">
@@ -8433,6 +9655,15 @@
       <c r="W150" s="17" t="n">
         <v>-347344475.1858202</v>
       </c>
+      <c r="X150" s="17" t="n">
+        <v>-66049022548.12001</v>
+      </c>
+      <c r="Y150" s="17" t="n">
+        <v>-3885236.620477648</v>
+      </c>
+      <c r="Z150" s="17" t="n">
+        <v>-349465727.7678308</v>
+      </c>
     </row>
     <row r="151">
       <c r="B151" s="14" t="inlineStr">
@@ -8503,6 +9734,15 @@
       <c r="W151" s="15" t="n">
         <v>357003496.4357672</v>
       </c>
+      <c r="X151" s="15" t="n">
+        <v>67473660826.36001</v>
+      </c>
+      <c r="Y151" s="15" t="n">
+        <v>3969038.872138824</v>
+      </c>
+      <c r="Z151" s="15" t="n">
+        <v>357003496.4357672</v>
+      </c>
     </row>
     <row r="152">
       <c r="B152" s="16" t="inlineStr">
@@ -8573,15 +9813,25 @@
       <c r="W152" s="17" t="n">
         <v>9659021.255238103</v>
       </c>
+      <c r="X152" s="17" t="n">
+        <v>1424638278.23999</v>
+      </c>
+      <c r="Y152" s="17" t="n">
+        <v>83802.25166117589</v>
+      </c>
+      <c r="Z152" s="17" t="n">
+        <v>7537768.667936456</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
-    <mergeCell ref="B2:W2"/>
+  <mergeCells count="11">
+    <mergeCell ref="B2:Z2"/>
     <mergeCell ref="R3:T3"/>
     <mergeCell ref="U3:W3"/>
     <mergeCell ref="B3:B4"/>
-    <mergeCell ref="B1:W1"/>
+    <mergeCell ref="B1:Z1"/>
     <mergeCell ref="C3:E3"/>
+    <mergeCell ref="X3:Z3"/>
     <mergeCell ref="I3:K3"/>
     <mergeCell ref="F3:H3"/>
     <mergeCell ref="L3:N3"/>
@@ -8599,7 +9849,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:W152"/>
+  <dimension ref="B1:Z152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -8625,6 +9875,9 @@
     <col width="16" customWidth="1" min="21" max="21"/>
     <col width="16" customWidth="1" min="22" max="22"/>
     <col width="16" customWidth="1" min="23" max="23"/>
+    <col width="16" customWidth="1" min="24" max="24"/>
+    <col width="16" customWidth="1" min="25" max="25"/>
+    <col width="16" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -8637,7 +9890,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 28 Jul 2026 16:03 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 28 Jul 2026 16:28 (in IDR Million)</t>
         </is>
       </c>
     </row>
@@ -8696,6 +9949,13 @@
       </c>
       <c r="V3" s="4" t="n"/>
       <c r="W3" s="4" t="n"/>
+      <c r="X3" s="3" t="inlineStr">
+        <is>
+          <t>YTD as of 28 Jul 2026</t>
+        </is>
+      </c>
+      <c r="Y3" s="4" t="n"/>
+      <c r="Z3" s="4" t="n"/>
     </row>
     <row r="4" ht="18" customHeight="1">
       <c r="B4" s="5" t="n"/>
@@ -8800,6 +10060,21 @@
         </is>
       </c>
       <c r="W4" s="3" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="X4" s="3" t="inlineStr">
+        <is>
+          <t>IDR</t>
+        </is>
+      </c>
+      <c r="Y4" s="3" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Z4" s="3" t="inlineStr">
         <is>
           <t>INR</t>
         </is>
@@ -8832,6 +10107,9 @@
       <c r="U5" s="7" t="n"/>
       <c r="V5" s="7" t="n"/>
       <c r="W5" s="7" t="n"/>
+      <c r="X5" s="7" t="n"/>
+      <c r="Y5" s="7" t="n"/>
+      <c r="Z5" s="7" t="n"/>
     </row>
     <row r="6">
       <c r="B6" s="8" t="inlineStr">
@@ -8901,6 +10179,15 @@
       </c>
       <c r="W6" s="9" t="n">
         <v>822.5205241798942</v>
+      </c>
+      <c r="X6" s="9" t="n">
+        <v>162351.695487</v>
+      </c>
+      <c r="Y6" s="9" t="n">
+        <v>9.550099734529411</v>
+      </c>
+      <c r="Z6" s="9" t="n">
+        <v>859.0036798253968</v>
       </c>
     </row>
     <row r="7">
@@ -8954,6 +10241,15 @@
       <c r="W7" s="11" t="n">
         <v>483.8449300899471</v>
       </c>
+      <c r="X7" s="11" t="n">
+        <v>91465.99687899998</v>
+      </c>
+      <c r="Y7" s="11" t="n">
+        <v>5.380352757588236</v>
+      </c>
+      <c r="Z7" s="11" t="n">
+        <v>483.9470734338624</v>
+      </c>
     </row>
     <row r="8">
       <c r="B8" s="8" t="inlineStr">
@@ -9023,6 +10319,15 @@
       </c>
       <c r="W8" s="9" t="n">
         <v>154.6752116666667</v>
+      </c>
+      <c r="X8" s="9" t="n">
+        <v>32823.856519</v>
+      </c>
+      <c r="Y8" s="9" t="n">
+        <v>1.930815089352941</v>
+      </c>
+      <c r="Z8" s="9" t="n">
+        <v>173.6711985132275</v>
       </c>
     </row>
     <row r="9">
@@ -9088,6 +10393,15 @@
       <c r="W9" s="11" t="n">
         <v>142.6768717566137</v>
       </c>
+      <c r="X9" s="11" t="n">
+        <v>29263.769826</v>
+      </c>
+      <c r="Y9" s="11" t="n">
+        <v>1.721398225058824</v>
+      </c>
+      <c r="Z9" s="11" t="n">
+        <v>154.834760984127</v>
+      </c>
     </row>
     <row r="10">
       <c r="B10" s="8" t="inlineStr">
@@ -9152,6 +10466,15 @@
       <c r="W10" s="9" t="n">
         <v>34.98273817989418</v>
       </c>
+      <c r="X10" s="9" t="n">
+        <v>7187.586263000001</v>
+      </c>
+      <c r="Y10" s="9" t="n">
+        <v>0.4227991919411765</v>
+      </c>
+      <c r="Z10" s="9" t="n">
+        <v>38.02955694708995</v>
+      </c>
     </row>
     <row r="11">
       <c r="B11" s="10" t="inlineStr">
@@ -9209,6 +10532,15 @@
       </c>
       <c r="W11" s="11" t="n">
         <v>5.450793650793651</v>
+      </c>
+      <c r="X11" s="11" t="n">
+        <v>1442.28</v>
+      </c>
+      <c r="Y11" s="11" t="n">
+        <v>0.08484</v>
+      </c>
+      <c r="Z11" s="11" t="n">
+        <v>7.631111111111111</v>
       </c>
     </row>
     <row r="12">
@@ -9250,6 +10582,15 @@
       <c r="W12" s="9" t="n">
         <v>0.7408359788359788</v>
       </c>
+      <c r="X12" s="9" t="n">
+        <v>140.018</v>
+      </c>
+      <c r="Y12" s="9" t="n">
+        <v>0.008236352941176471</v>
+      </c>
+      <c r="Z12" s="9" t="n">
+        <v>0.7408359788359788</v>
+      </c>
     </row>
     <row r="13">
       <c r="B13" s="10" t="inlineStr">
@@ -9290,6 +10631,15 @@
       <c r="W13" s="11" t="n">
         <v>0.1491428571428571</v>
       </c>
+      <c r="X13" s="11" t="n">
+        <v>28.188</v>
+      </c>
+      <c r="Y13" s="11" t="n">
+        <v>0.001658117647058823</v>
+      </c>
+      <c r="Z13" s="11" t="n">
+        <v>0.1491428571428571</v>
+      </c>
     </row>
     <row r="14">
       <c r="B14" s="8" t="inlineStr">
@@ -9330,6 +10680,15 @@
       <c r="W14" s="9" t="n">
         <v>262.4126984126984</v>
       </c>
+      <c r="X14" s="9" t="n">
+        <v>49596</v>
+      </c>
+      <c r="Y14" s="9" t="n">
+        <v>2.917411764705882</v>
+      </c>
+      <c r="Z14" s="9" t="n">
+        <v>262.4126984126984</v>
+      </c>
     </row>
     <row r="15">
       <c r="B15" s="10" t="inlineStr">
@@ -9370,6 +10729,15 @@
       <c r="W15" s="11" t="n">
         <v>262.4126984126984</v>
       </c>
+      <c r="X15" s="11" t="n">
+        <v>49596</v>
+      </c>
+      <c r="Y15" s="11" t="n">
+        <v>2.917411764705882</v>
+      </c>
+      <c r="Z15" s="11" t="n">
+        <v>262.4126984126984</v>
+      </c>
     </row>
     <row r="16">
       <c r="B16" s="8" t="inlineStr">
@@ -9440,6 +10808,15 @@
       <c r="W16" s="9" t="n">
         <v>1.910739122063492</v>
       </c>
+      <c r="X16" s="9" t="n">
+        <v>391.4217440699999</v>
+      </c>
+      <c r="Y16" s="9" t="n">
+        <v>0.02302480847470588</v>
+      </c>
+      <c r="Z16" s="9" t="n">
+        <v>2.071014518888889</v>
+      </c>
     </row>
     <row r="17">
       <c r="B17" s="10" t="inlineStr">
@@ -9508,6 +10885,15 @@
         <v>0.00746904232117647</v>
       </c>
       <c r="W17" s="11" t="n">
+        <v>0.6718186214814815</v>
+      </c>
+      <c r="X17" s="11" t="n">
+        <v>126.97371946</v>
+      </c>
+      <c r="Y17" s="11" t="n">
+        <v>0.00746904232117647</v>
+      </c>
+      <c r="Z17" s="11" t="n">
         <v>0.6718186214814815</v>
       </c>
     </row>
@@ -9550,6 +10936,15 @@
       <c r="W18" s="9" t="n">
         <v>0.6579851851851852</v>
       </c>
+      <c r="X18" s="9" t="n">
+        <v>124.3592</v>
+      </c>
+      <c r="Y18" s="9" t="n">
+        <v>0.00731524705882353</v>
+      </c>
+      <c r="Z18" s="9" t="n">
+        <v>0.6579851851851852</v>
+      </c>
     </row>
     <row r="19">
       <c r="B19" s="10" t="inlineStr">
@@ -9590,6 +10985,15 @@
       <c r="W19" s="11" t="n">
         <v>0.1231216931216931</v>
       </c>
+      <c r="X19" s="11" t="n">
+        <v>23.27</v>
+      </c>
+      <c r="Y19" s="11" t="n">
+        <v>0.001368823529411765</v>
+      </c>
+      <c r="Z19" s="11" t="n">
+        <v>0.1231216931216931</v>
+      </c>
     </row>
     <row r="20">
       <c r="B20" s="8" t="inlineStr">
@@ -9647,6 +11051,15 @@
       </c>
       <c r="W20" s="9" t="n">
         <v>0.09770105820105819</v>
+      </c>
+      <c r="X20" s="9" t="n">
+        <v>22.48</v>
+      </c>
+      <c r="Y20" s="9" t="n">
+        <v>0.001322352941176471</v>
+      </c>
+      <c r="Z20" s="9" t="n">
+        <v>0.1189417989417989</v>
       </c>
     </row>
     <row r="21">
@@ -9692,6 +11105,15 @@
         <v>0.001188532352941176</v>
       </c>
       <c r="W21" s="11" t="n">
+        <v>0.1069050264550264</v>
+      </c>
+      <c r="X21" s="11" t="n">
+        <v>20.20505</v>
+      </c>
+      <c r="Y21" s="11" t="n">
+        <v>0.001188532352941176</v>
+      </c>
+      <c r="Z21" s="11" t="n">
         <v>0.1069050264550264</v>
       </c>
     </row>
@@ -9722,6 +11144,15 @@
       <c r="U22" s="9" t="n"/>
       <c r="V22" s="9" t="n"/>
       <c r="W22" s="9" t="n"/>
+      <c r="X22" s="9" t="n">
+        <v>17.865</v>
+      </c>
+      <c r="Y22" s="9" t="n">
+        <v>0.001050882352941176</v>
+      </c>
+      <c r="Z22" s="9" t="n">
+        <v>0.09452380952380951</v>
+      </c>
     </row>
     <row r="23">
       <c r="B23" s="10" t="inlineStr">
@@ -9762,6 +11193,15 @@
       <c r="W23" s="11" t="n">
         <v>0.07447301587301587</v>
       </c>
+      <c r="X23" s="11" t="n">
+        <v>14.0754</v>
+      </c>
+      <c r="Y23" s="11" t="n">
+        <v>0.0008279647058823529</v>
+      </c>
+      <c r="Z23" s="11" t="n">
+        <v>0.07447301587301587</v>
+      </c>
     </row>
     <row r="24">
       <c r="B24" s="8" t="inlineStr">
@@ -9819,6 +11259,15 @@
       </c>
       <c r="W24" s="9" t="n">
         <v>0.04138297354497354</v>
+      </c>
+      <c r="X24" s="9" t="n">
+        <v>11.858382</v>
+      </c>
+      <c r="Y24" s="9" t="n">
+        <v>0.0006975518823529412</v>
+      </c>
+      <c r="Z24" s="9" t="n">
+        <v>0.0627427619047619</v>
       </c>
     </row>
     <row r="25">
@@ -9860,6 +11309,15 @@
       <c r="W25" s="11" t="n">
         <v>0.03976575132275132</v>
       </c>
+      <c r="X25" s="11" t="n">
+        <v>7.515727</v>
+      </c>
+      <c r="Y25" s="11" t="n">
+        <v>0.0004421015882352941</v>
+      </c>
+      <c r="Z25" s="11" t="n">
+        <v>0.03976575132275132</v>
+      </c>
     </row>
     <row r="26">
       <c r="B26" s="8" t="inlineStr">
@@ -9906,6 +11364,15 @@
       <c r="W26" s="9" t="n">
         <v>0.03174603174603174</v>
       </c>
+      <c r="X26" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="Y26" s="9" t="n">
+        <v>0.0003529411764705883</v>
+      </c>
+      <c r="Z26" s="9" t="n">
+        <v>0.03174603174603174</v>
+      </c>
     </row>
     <row r="27">
       <c r="B27" s="10" t="inlineStr">
@@ -9951,6 +11418,15 @@
       </c>
       <c r="W27" s="11" t="n">
         <v>0.0218731746031746</v>
+      </c>
+      <c r="X27" s="11" t="n">
+        <v>4.48403</v>
+      </c>
+      <c r="Y27" s="11" t="n">
+        <v>0.0002637664705882353</v>
+      </c>
+      <c r="Z27" s="11" t="n">
+        <v>0.02372502645502645</v>
       </c>
     </row>
     <row r="28">
@@ -9992,6 +11468,15 @@
       <c r="W28" s="9" t="n">
         <v>0.02022776719576719</v>
       </c>
+      <c r="X28" s="9" t="n">
+        <v>3.823048</v>
+      </c>
+      <c r="Y28" s="9" t="n">
+        <v>0.0002248851764705882</v>
+      </c>
+      <c r="Z28" s="9" t="n">
+        <v>0.02022776719576719</v>
+      </c>
     </row>
     <row r="29">
       <c r="B29" s="10" t="inlineStr">
@@ -10032,6 +11517,15 @@
       <c r="W29" s="11" t="n">
         <v>0.0005566137566137566</v>
       </c>
+      <c r="X29" s="11" t="n">
+        <v>2.70045</v>
+      </c>
+      <c r="Y29" s="11" t="n">
+        <v>0.00015885</v>
+      </c>
+      <c r="Z29" s="11" t="n">
+        <v>0.01428809523809524</v>
+      </c>
     </row>
     <row r="30">
       <c r="B30" s="8" t="inlineStr">
@@ -10082,6 +11576,15 @@
         <v>0.0001031552123529412</v>
       </c>
       <c r="W30" s="9" t="n">
+        <v>0.009278511164021164</v>
+      </c>
+      <c r="X30" s="9" t="n">
+        <v>1.75363861</v>
+      </c>
+      <c r="Y30" s="9" t="n">
+        <v>0.0001031552123529412</v>
+      </c>
+      <c r="Z30" s="9" t="n">
         <v>0.009278511164021164</v>
       </c>
     </row>
@@ -10124,6 +11627,15 @@
       <c r="W31" s="11" t="n">
         <v>0.001502603174603175</v>
       </c>
+      <c r="X31" s="11" t="n">
+        <v>1.644292</v>
+      </c>
+      <c r="Y31" s="11" t="n">
+        <v>9.672305882352941e-05</v>
+      </c>
+      <c r="Z31" s="11" t="n">
+        <v>0.008699957671957671</v>
+      </c>
     </row>
     <row r="32">
       <c r="B32" s="8" t="inlineStr">
@@ -10164,6 +11676,15 @@
       <c r="W32" s="9" t="n">
         <v>0.005291005291005291</v>
       </c>
+      <c r="X32" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y32" s="9" t="n">
+        <v>5.882352941176471e-05</v>
+      </c>
+      <c r="Z32" s="9" t="n">
+        <v>0.005291005291005291</v>
+      </c>
     </row>
     <row r="33">
       <c r="B33" s="10" t="inlineStr">
@@ -10214,6 +11735,15 @@
         <v>4.348235294117647e-05</v>
       </c>
       <c r="W33" s="11" t="n">
+        <v>0.003911111111111111</v>
+      </c>
+      <c r="X33" s="11" t="n">
+        <v>0.7392</v>
+      </c>
+      <c r="Y33" s="11" t="n">
+        <v>4.348235294117647e-05</v>
+      </c>
+      <c r="Z33" s="11" t="n">
         <v>0.003911111111111111</v>
       </c>
     </row>
@@ -10262,6 +11792,15 @@
       <c r="W34" s="9" t="n">
         <v>0.002648703703703704</v>
       </c>
+      <c r="X34" s="9" t="n">
+        <v>0.500605</v>
+      </c>
+      <c r="Y34" s="9" t="n">
+        <v>2.944735294117647e-05</v>
+      </c>
+      <c r="Z34" s="9" t="n">
+        <v>0.002648703703703704</v>
+      </c>
     </row>
     <row r="35">
       <c r="B35" s="10" t="inlineStr">
@@ -10302,6 +11841,15 @@
       <c r="W35" s="11" t="n">
         <v>0.0005291111111111111</v>
       </c>
+      <c r="X35" s="11" t="n">
+        <v>0.170002</v>
+      </c>
+      <c r="Y35" s="11" t="n">
+        <v>1.000011764705882e-05</v>
+      </c>
+      <c r="Z35" s="11" t="n">
+        <v>0.0008994814814814815</v>
+      </c>
     </row>
     <row r="36">
       <c r="B36" s="8" t="inlineStr">
@@ -10342,6 +11890,15 @@
       <c r="W36" s="9" t="n">
         <v>2.116402116402116e-05</v>
       </c>
+      <c r="X36" s="9" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="Y36" s="9" t="n">
+        <v>2.352941176470588e-07</v>
+      </c>
+      <c r="Z36" s="9" t="n">
+        <v>2.116402116402116e-05</v>
+      </c>
     </row>
     <row r="37">
       <c r="B37" s="10" t="inlineStr">
@@ -10382,6 +11939,15 @@
       <c r="W37" s="11" t="n">
         <v>1.164021164021164</v>
       </c>
+      <c r="X37" s="11" t="n">
+        <v>220</v>
+      </c>
+      <c r="Y37" s="11" t="n">
+        <v>0.01294117647058824</v>
+      </c>
+      <c r="Z37" s="11" t="n">
+        <v>1.164021164021164</v>
+      </c>
     </row>
     <row r="38">
       <c r="B38" s="12" t="inlineStr">
@@ -10451,6 +12017,15 @@
       </c>
       <c r="W38" s="13" t="n">
         <v>1088.007982878677</v>
+      </c>
+      <c r="X38" s="13" t="n">
+        <v>212559.11723107</v>
+      </c>
+      <c r="Y38" s="13" t="n">
+        <v>12.50347748418059</v>
+      </c>
+      <c r="Z38" s="13" t="n">
+        <v>1124.651413921005</v>
       </c>
     </row>
     <row r="39">
@@ -10480,6 +12055,9 @@
       <c r="U39" s="7" t="n"/>
       <c r="V39" s="7" t="n"/>
       <c r="W39" s="7" t="n"/>
+      <c r="X39" s="7" t="n"/>
+      <c r="Y39" s="7" t="n"/>
+      <c r="Z39" s="7" t="n"/>
     </row>
     <row r="40">
       <c r="B40" s="14" t="inlineStr">
@@ -10508,6 +12086,9 @@
       <c r="U40" s="15" t="n"/>
       <c r="V40" s="15" t="n"/>
       <c r="W40" s="15" t="n"/>
+      <c r="X40" s="15" t="n"/>
+      <c r="Y40" s="15" t="n"/>
+      <c r="Z40" s="15" t="n"/>
     </row>
     <row r="41">
       <c r="B41" s="8" t="inlineStr">
@@ -10577,6 +12158,15 @@
       </c>
       <c r="W41" s="9" t="n">
         <v>-24.77324962962964</v>
+      </c>
+      <c r="X41" s="9" t="n">
+        <v>-4688.96918</v>
+      </c>
+      <c r="Y41" s="9" t="n">
+        <v>-0.2758217164705882</v>
+      </c>
+      <c r="Z41" s="9" t="n">
+        <v>-24.80936074074075</v>
       </c>
     </row>
     <row r="42">
@@ -10622,6 +12212,15 @@
         <v>-0.009178077352941178</v>
       </c>
       <c r="W42" s="11" t="n">
+        <v>-0.8255413492063493</v>
+      </c>
+      <c r="X42" s="11" t="n">
+        <v>-156.027315</v>
+      </c>
+      <c r="Y42" s="11" t="n">
+        <v>-0.009178077352941178</v>
+      </c>
+      <c r="Z42" s="11" t="n">
         <v>-0.8255413492063493</v>
       </c>
     </row>
@@ -10652,6 +12251,15 @@
       <c r="U43" s="9" t="n"/>
       <c r="V43" s="9" t="n"/>
       <c r="W43" s="9" t="n"/>
+      <c r="X43" s="9" t="n">
+        <v>-172.4435</v>
+      </c>
+      <c r="Y43" s="9" t="n">
+        <v>-0.01014373529411765</v>
+      </c>
+      <c r="Z43" s="9" t="n">
+        <v>-0.9123994708994709</v>
+      </c>
     </row>
     <row r="44">
       <c r="B44" s="10" t="inlineStr">
@@ -10710,6 +12318,15 @@
       <c r="W44" s="11" t="n">
         <v>-5.654963767195767</v>
       </c>
+      <c r="X44" s="11" t="n">
+        <v>-1268.268418</v>
+      </c>
+      <c r="Y44" s="11" t="n">
+        <v>-0.07460402458823531</v>
+      </c>
+      <c r="Z44" s="11" t="n">
+        <v>-6.71041491005291</v>
+      </c>
     </row>
     <row r="45">
       <c r="B45" s="8" t="inlineStr">
@@ -10755,6 +12372,15 @@
       </c>
       <c r="W45" s="9" t="n">
         <v>-0.4427373015873016</v>
+      </c>
+      <c r="X45" s="9" t="n">
+        <v>-134.989875</v>
+      </c>
+      <c r="Y45" s="9" t="n">
+        <v>-0.00794058088235294</v>
+      </c>
+      <c r="Z45" s="9" t="n">
+        <v>-0.7142321428571428</v>
       </c>
     </row>
     <row r="46">
@@ -10784,6 +12410,15 @@
       <c r="U46" s="11" t="n"/>
       <c r="V46" s="11" t="n"/>
       <c r="W46" s="11" t="n"/>
+      <c r="X46" s="11" t="n">
+        <v>-29.4</v>
+      </c>
+      <c r="Y46" s="11" t="n">
+        <v>-0.001729411764705882</v>
+      </c>
+      <c r="Z46" s="11" t="n">
+        <v>-0.1555555555555556</v>
+      </c>
     </row>
     <row r="47">
       <c r="B47" s="8" t="inlineStr">
@@ -10824,6 +12459,15 @@
       <c r="W47" s="9" t="n">
         <v>-0.1844444444444444</v>
       </c>
+      <c r="X47" s="9" t="n">
+        <v>-47.57855</v>
+      </c>
+      <c r="Y47" s="9" t="n">
+        <v>-0.002798738235294117</v>
+      </c>
+      <c r="Z47" s="9" t="n">
+        <v>-0.2517383597883598</v>
+      </c>
     </row>
     <row r="48">
       <c r="B48" s="10" t="inlineStr">
@@ -10882,6 +12526,15 @@
       <c r="W48" s="11" t="n">
         <v>-3.673993804232804</v>
       </c>
+      <c r="X48" s="11" t="n">
+        <v>-1005.168514</v>
+      </c>
+      <c r="Y48" s="11" t="n">
+        <v>-0.05912755964705883</v>
+      </c>
+      <c r="Z48" s="11" t="n">
+        <v>-5.318351925925926</v>
+      </c>
     </row>
     <row r="49">
       <c r="B49" s="8" t="inlineStr">
@@ -10932,6 +12585,15 @@
         <v>-0.005460122647058823</v>
       </c>
       <c r="W49" s="9" t="n">
+        <v>-0.4911221428571428</v>
+      </c>
+      <c r="X49" s="9" t="n">
+        <v>-92.822085</v>
+      </c>
+      <c r="Y49" s="9" t="n">
+        <v>-0.005460122647058823</v>
+      </c>
+      <c r="Z49" s="9" t="n">
         <v>-0.4911221428571428</v>
       </c>
     </row>
@@ -10985,6 +12647,15 @@
       </c>
       <c r="W50" s="11" t="n">
         <v>-6.807835645502645</v>
+      </c>
+      <c r="X50" s="11" t="n">
+        <v>-1328.241875</v>
+      </c>
+      <c r="Y50" s="11" t="n">
+        <v>-0.078131875</v>
+      </c>
+      <c r="Z50" s="11" t="n">
+        <v>-7.027734788359788</v>
       </c>
     </row>
     <row r="51">
@@ -11026,6 +12697,15 @@
       <c r="W51" s="9" t="n">
         <v>-10.04197037037037</v>
       </c>
+      <c r="X51" s="9" t="n">
+        <v>-1897.9324</v>
+      </c>
+      <c r="Y51" s="9" t="n">
+        <v>-0.1116430823529412</v>
+      </c>
+      <c r="Z51" s="9" t="n">
+        <v>-10.04197037037037</v>
+      </c>
     </row>
     <row r="52">
       <c r="B52" s="10" t="inlineStr">
@@ -11095,6 +12775,15 @@
       </c>
       <c r="W52" s="11" t="n">
         <v>-0.7262684444444444</v>
+      </c>
+      <c r="X52" s="11" t="n">
+        <v>-154.499829</v>
+      </c>
+      <c r="Y52" s="11" t="n">
+        <v>-0.009088225235294116</v>
+      </c>
+      <c r="Z52" s="11" t="n">
+        <v>-0.8174594126984126</v>
       </c>
     </row>
     <row r="53">
@@ -11124,6 +12813,15 @@
       <c r="U53" s="9" t="n"/>
       <c r="V53" s="9" t="n"/>
       <c r="W53" s="9" t="n"/>
+      <c r="X53" s="9" t="n">
+        <v>-30.945</v>
+      </c>
+      <c r="Y53" s="9" t="n">
+        <v>-0.001820294117647059</v>
+      </c>
+      <c r="Z53" s="9" t="n">
+        <v>-0.1637301587301587</v>
+      </c>
     </row>
     <row r="54">
       <c r="B54" s="10" t="inlineStr">
@@ -11193,6 +12891,15 @@
       </c>
       <c r="W54" s="11" t="n">
         <v>-7.334781486137566</v>
+      </c>
+      <c r="X54" s="11" t="n">
+        <v>-1408.98575088</v>
+      </c>
+      <c r="Y54" s="11" t="n">
+        <v>-0.08288151475764706</v>
+      </c>
+      <c r="Z54" s="11" t="n">
+        <v>-7.454951062857143</v>
       </c>
     </row>
     <row r="55">
@@ -11232,6 +12939,15 @@
         <v>-0.1012476705882353</v>
       </c>
       <c r="W55" s="9" t="n">
+        <v>-9.106933333333332</v>
+      </c>
+      <c r="X55" s="9" t="n">
+        <v>-1721.2104</v>
+      </c>
+      <c r="Y55" s="9" t="n">
+        <v>-0.1012476705882353</v>
+      </c>
+      <c r="Z55" s="9" t="n">
         <v>-9.106933333333332</v>
       </c>
     </row>
@@ -11262,6 +12978,15 @@
       <c r="U56" s="11" t="n"/>
       <c r="V56" s="11" t="n"/>
       <c r="W56" s="11" t="n"/>
+      <c r="X56" s="11" t="n">
+        <v>-2</v>
+      </c>
+      <c r="Y56" s="11" t="n">
+        <v>-0.0001176470588235294</v>
+      </c>
+      <c r="Z56" s="11" t="n">
+        <v>-0.01058201058201058</v>
+      </c>
     </row>
     <row r="57">
       <c r="B57" s="8" t="inlineStr">
@@ -11326,6 +13051,15 @@
       <c r="W57" s="9" t="n">
         <v>-0.5873015873015872</v>
       </c>
+      <c r="X57" s="9" t="n">
+        <v>-129.5</v>
+      </c>
+      <c r="Y57" s="9" t="n">
+        <v>-0.007617647058823529</v>
+      </c>
+      <c r="Z57" s="9" t="n">
+        <v>-0.6851851851851851</v>
+      </c>
     </row>
     <row r="58">
       <c r="B58" s="12" t="inlineStr">
@@ -11395,6 +13129,15 @@
       </c>
       <c r="W58" s="13" t="n">
         <v>-70.65114330624338</v>
+      </c>
+      <c r="X58" s="13" t="n">
+        <v>-14268.98269188</v>
+      </c>
+      <c r="Y58" s="13" t="n">
+        <v>-0.8393519230517646</v>
+      </c>
+      <c r="Z58" s="13" t="n">
+        <v>-75.49726292</v>
       </c>
     </row>
     <row r="59">
@@ -11424,6 +13167,9 @@
       <c r="U59" s="15" t="n"/>
       <c r="V59" s="15" t="n"/>
       <c r="W59" s="15" t="n"/>
+      <c r="X59" s="15" t="n"/>
+      <c r="Y59" s="15" t="n"/>
+      <c r="Z59" s="15" t="n"/>
     </row>
     <row r="60">
       <c r="B60" s="8" t="inlineStr">
@@ -11464,6 +13210,15 @@
       <c r="W60" s="9" t="n">
         <v>-19.17047917460318</v>
       </c>
+      <c r="X60" s="9" t="n">
+        <v>-3623.220564</v>
+      </c>
+      <c r="Y60" s="9" t="n">
+        <v>-0.2131306214117647</v>
+      </c>
+      <c r="Z60" s="9" t="n">
+        <v>-19.17047917460318</v>
+      </c>
     </row>
     <row r="61">
       <c r="B61" s="10" t="inlineStr">
@@ -11504,6 +13259,15 @@
       <c r="W61" s="11" t="n">
         <v>-19.17047917460318</v>
       </c>
+      <c r="X61" s="11" t="n">
+        <v>-3623.220564</v>
+      </c>
+      <c r="Y61" s="11" t="n">
+        <v>-0.2131306214117647</v>
+      </c>
+      <c r="Z61" s="11" t="n">
+        <v>-19.17047917460318</v>
+      </c>
     </row>
     <row r="62">
       <c r="B62" s="8" t="inlineStr">
@@ -11550,6 +13314,15 @@
       <c r="W62" s="9" t="n">
         <v>-535.3873940529101</v>
       </c>
+      <c r="X62" s="9" t="n">
+        <v>-101188.217476</v>
+      </c>
+      <c r="Y62" s="9" t="n">
+        <v>-5.952248086823529</v>
+      </c>
+      <c r="Z62" s="9" t="n">
+        <v>-535.3873940529101</v>
+      </c>
     </row>
     <row r="63">
       <c r="B63" s="10" t="inlineStr">
@@ -11594,6 +13367,15 @@
         <v>-5.952248086823529</v>
       </c>
       <c r="W63" s="11" t="n">
+        <v>-535.3873940529101</v>
+      </c>
+      <c r="X63" s="11" t="n">
+        <v>-101188.217476</v>
+      </c>
+      <c r="Y63" s="11" t="n">
+        <v>-5.952248086823529</v>
+      </c>
+      <c r="Z63" s="11" t="n">
         <v>-535.3873940529101</v>
       </c>
     </row>
@@ -11636,6 +13418,15 @@
       <c r="W64" s="9" t="n">
         <v>-55.90866344444445</v>
       </c>
+      <c r="X64" s="9" t="n">
+        <v>-10566.737391</v>
+      </c>
+      <c r="Y64" s="9" t="n">
+        <v>-0.6215727877058824</v>
+      </c>
+      <c r="Z64" s="9" t="n">
+        <v>-55.90866344444445</v>
+      </c>
     </row>
     <row r="65">
       <c r="B65" s="10" t="inlineStr">
@@ -11676,6 +13467,15 @@
       <c r="W65" s="11" t="n">
         <v>-55.90866344444445</v>
       </c>
+      <c r="X65" s="11" t="n">
+        <v>-10566.737391</v>
+      </c>
+      <c r="Y65" s="11" t="n">
+        <v>-0.6215727877058824</v>
+      </c>
+      <c r="Z65" s="11" t="n">
+        <v>-55.90866344444445</v>
+      </c>
     </row>
     <row r="66">
       <c r="B66" s="12" t="inlineStr">
@@ -11720,6 +13520,15 @@
         <v>-6.786951495941176</v>
       </c>
       <c r="W66" s="13" t="n">
+        <v>-610.4665366719577</v>
+      </c>
+      <c r="X66" s="13" t="n">
+        <v>-115378.175431</v>
+      </c>
+      <c r="Y66" s="13" t="n">
+        <v>-6.786951495941176</v>
+      </c>
+      <c r="Z66" s="13" t="n">
         <v>-610.4665366719577</v>
       </c>
     </row>
@@ -11750,6 +13559,9 @@
       <c r="U67" s="15" t="n"/>
       <c r="V67" s="15" t="n"/>
       <c r="W67" s="15" t="n"/>
+      <c r="X67" s="15" t="n"/>
+      <c r="Y67" s="15" t="n"/>
+      <c r="Z67" s="15" t="n"/>
     </row>
     <row r="68">
       <c r="B68" s="8" t="inlineStr">
@@ -11796,6 +13608,15 @@
       <c r="W68" s="9" t="n">
         <v>-26.68137267724868</v>
       </c>
+      <c r="X68" s="9" t="n">
+        <v>-5042.779436</v>
+      </c>
+      <c r="Y68" s="9" t="n">
+        <v>-0.2966340844705882</v>
+      </c>
+      <c r="Z68" s="9" t="n">
+        <v>-26.68137267724868</v>
+      </c>
     </row>
     <row r="69">
       <c r="B69" s="12" t="inlineStr">
@@ -11840,6 +13661,15 @@
         <v>-0.2966340844705882</v>
       </c>
       <c r="W69" s="13" t="n">
+        <v>-26.68137267724868</v>
+      </c>
+      <c r="X69" s="13" t="n">
+        <v>-5042.779436</v>
+      </c>
+      <c r="Y69" s="13" t="n">
+        <v>-0.2966340844705882</v>
+      </c>
+      <c r="Z69" s="13" t="n">
         <v>-26.68137267724868</v>
       </c>
     </row>
@@ -11870,6 +13700,9 @@
       <c r="U70" s="15" t="n"/>
       <c r="V70" s="15" t="n"/>
       <c r="W70" s="15" t="n"/>
+      <c r="X70" s="15" t="n"/>
+      <c r="Y70" s="15" t="n"/>
+      <c r="Z70" s="15" t="n"/>
     </row>
     <row r="71">
       <c r="B71" s="8" t="inlineStr">
@@ -11910,6 +13743,15 @@
       <c r="W71" s="9" t="n">
         <v>-92.28571428571429</v>
       </c>
+      <c r="X71" s="9" t="n">
+        <v>-17442</v>
+      </c>
+      <c r="Y71" s="9" t="n">
+        <v>-1.026</v>
+      </c>
+      <c r="Z71" s="9" t="n">
+        <v>-92.28571428571429</v>
+      </c>
     </row>
     <row r="72">
       <c r="B72" s="10" t="inlineStr">
@@ -11954,6 +13796,15 @@
         <v>-2.588235294117647</v>
       </c>
       <c r="W72" s="11" t="n">
+        <v>-232.8042328042328</v>
+      </c>
+      <c r="X72" s="11" t="n">
+        <v>-44000</v>
+      </c>
+      <c r="Y72" s="11" t="n">
+        <v>-2.588235294117647</v>
+      </c>
+      <c r="Z72" s="11" t="n">
         <v>-232.8042328042328</v>
       </c>
     </row>
@@ -11996,6 +13847,15 @@
       <c r="W73" s="9" t="n">
         <v>-80.72941468253968</v>
       </c>
+      <c r="X73" s="9" t="n">
+        <v>-15257.859375</v>
+      </c>
+      <c r="Y73" s="9" t="n">
+        <v>-0.8975211397058823</v>
+      </c>
+      <c r="Z73" s="9" t="n">
+        <v>-80.72941468253968</v>
+      </c>
     </row>
     <row r="74">
       <c r="B74" s="12" t="inlineStr">
@@ -12046,6 +13906,15 @@
         <v>-4.511756433823529</v>
       </c>
       <c r="W74" s="13" t="n">
+        <v>-405.8193617724867</v>
+      </c>
+      <c r="X74" s="13" t="n">
+        <v>-76699.859375</v>
+      </c>
+      <c r="Y74" s="13" t="n">
+        <v>-4.511756433823529</v>
+      </c>
+      <c r="Z74" s="13" t="n">
         <v>-405.8193617724867</v>
       </c>
     </row>
@@ -12076,6 +13945,9 @@
       <c r="U75" s="15" t="n"/>
       <c r="V75" s="15" t="n"/>
       <c r="W75" s="15" t="n"/>
+      <c r="X75" s="15" t="n"/>
+      <c r="Y75" s="15" t="n"/>
+      <c r="Z75" s="15" t="n"/>
     </row>
     <row r="76">
       <c r="B76" s="8" t="inlineStr">
@@ -12146,6 +14018,15 @@
       <c r="W76" s="9" t="n">
         <v>-29.09765532275132</v>
       </c>
+      <c r="X76" s="9" t="n">
+        <v>-6081.007428000001</v>
+      </c>
+      <c r="Y76" s="9" t="n">
+        <v>-0.3577063192941177</v>
+      </c>
+      <c r="Z76" s="9" t="n">
+        <v>-32.17464247619048</v>
+      </c>
     </row>
     <row r="77">
       <c r="B77" s="10" t="inlineStr">
@@ -12216,6 +14097,15 @@
       <c r="W77" s="11" t="n">
         <v>-30.154353865291</v>
       </c>
+      <c r="X77" s="11" t="n">
+        <v>-7025.874357539999</v>
+      </c>
+      <c r="Y77" s="11" t="n">
+        <v>-0.4132867269141176</v>
+      </c>
+      <c r="Z77" s="11" t="n">
+        <v>-37.17393839968254</v>
+      </c>
     </row>
     <row r="78">
       <c r="B78" s="8" t="inlineStr">
@@ -12286,6 +14176,15 @@
       <c r="W78" s="9" t="n">
         <v>-28.42023708465608</v>
       </c>
+      <c r="X78" s="9" t="n">
+        <v>-6247.229889999999</v>
+      </c>
+      <c r="Y78" s="9" t="n">
+        <v>-0.3674841111764706</v>
+      </c>
+      <c r="Z78" s="9" t="n">
+        <v>-33.0541264021164</v>
+      </c>
     </row>
     <row r="79">
       <c r="B79" s="10" t="inlineStr">
@@ -12356,6 +14255,15 @@
       <c r="W79" s="11" t="n">
         <v>-2.004303851851852</v>
       </c>
+      <c r="X79" s="11" t="n">
+        <v>-386.997197</v>
+      </c>
+      <c r="Y79" s="11" t="n">
+        <v>-0.022764541</v>
+      </c>
+      <c r="Z79" s="11" t="n">
+        <v>-2.047604216931217</v>
+      </c>
     </row>
     <row r="80">
       <c r="B80" s="12" t="inlineStr">
@@ -12425,6 +14333,15 @@
       </c>
       <c r="W80" s="13" t="n">
         <v>-89.67655012455025</v>
+      </c>
+      <c r="X80" s="13" t="n">
+        <v>-19741.10887254</v>
+      </c>
+      <c r="Y80" s="13" t="n">
+        <v>-1.161241698384706</v>
+      </c>
+      <c r="Z80" s="13" t="n">
+        <v>-104.4503114949206</v>
       </c>
     </row>
     <row r="81">
@@ -12454,6 +14371,9 @@
       <c r="U81" s="15" t="n"/>
       <c r="V81" s="15" t="n"/>
       <c r="W81" s="15" t="n"/>
+      <c r="X81" s="15" t="n"/>
+      <c r="Y81" s="15" t="n"/>
+      <c r="Z81" s="15" t="n"/>
     </row>
     <row r="82">
       <c r="B82" s="14" t="inlineStr">
@@ -12482,6 +14402,9 @@
       <c r="U82" s="15" t="n"/>
       <c r="V82" s="15" t="n"/>
       <c r="W82" s="15" t="n"/>
+      <c r="X82" s="15" t="n"/>
+      <c r="Y82" s="15" t="n"/>
+      <c r="Z82" s="15" t="n"/>
     </row>
     <row r="83">
       <c r="B83" s="8" t="inlineStr">
@@ -12551,6 +14474,15 @@
       </c>
       <c r="W83" s="9" t="n">
         <v>-0.5357416243386244</v>
+      </c>
+      <c r="X83" s="9" t="n">
+        <v>-118.254829</v>
+      </c>
+      <c r="Y83" s="9" t="n">
+        <v>-0.006956166411764706</v>
+      </c>
+      <c r="Z83" s="9" t="n">
+        <v>-0.625686925925926</v>
       </c>
     </row>
     <row r="84">
@@ -12580,6 +14512,15 @@
       <c r="U84" s="11" t="n"/>
       <c r="V84" s="11" t="n"/>
       <c r="W84" s="11" t="n"/>
+      <c r="X84" s="11" t="n">
+        <v>-2.6266</v>
+      </c>
+      <c r="Y84" s="11" t="n">
+        <v>-0.0001545058823529412</v>
+      </c>
+      <c r="Z84" s="11" t="n">
+        <v>-0.0138973544973545</v>
+      </c>
     </row>
     <row r="85">
       <c r="B85" s="8" t="inlineStr">
@@ -12632,6 +14573,15 @@
       <c r="W85" s="9" t="n">
         <v>-0.04149314814814814</v>
       </c>
+      <c r="X85" s="9" t="n">
+        <v>-7.842205</v>
+      </c>
+      <c r="Y85" s="9" t="n">
+        <v>-0.0004613061764705882</v>
+      </c>
+      <c r="Z85" s="9" t="n">
+        <v>-0.04149314814814814</v>
+      </c>
     </row>
     <row r="86">
       <c r="B86" s="10" t="inlineStr">
@@ -12684,6 +14634,15 @@
       <c r="W86" s="11" t="n">
         <v>-0.008627340952380951</v>
       </c>
+      <c r="X86" s="11" t="n">
+        <v>-1.63056744</v>
+      </c>
+      <c r="Y86" s="11" t="n">
+        <v>-9.591573176470588e-05</v>
+      </c>
+      <c r="Z86" s="11" t="n">
+        <v>-0.008627340952380951</v>
+      </c>
     </row>
     <row r="87">
       <c r="B87" s="8" t="inlineStr">
@@ -12753,6 +14712,15 @@
       </c>
       <c r="W87" s="9" t="n">
         <v>-0.4088914603174603</v>
+      </c>
+      <c r="X87" s="9" t="n">
+        <v>-97.615961</v>
+      </c>
+      <c r="Y87" s="9" t="n">
+        <v>-0.005742115352941176</v>
+      </c>
+      <c r="Z87" s="9" t="n">
+        <v>-0.5164865661375662</v>
       </c>
     </row>
     <row r="88">
@@ -12812,6 +14780,15 @@
       <c r="W88" s="11" t="n">
         <v>-0.004466650793650793</v>
       </c>
+      <c r="X88" s="11" t="n">
+        <v>-1.661696</v>
+      </c>
+      <c r="Y88" s="11" t="n">
+        <v>-9.774682352941177e-05</v>
+      </c>
+      <c r="Z88" s="11" t="n">
+        <v>-0.008792042328042328</v>
+      </c>
     </row>
     <row r="89">
       <c r="B89" s="12" t="inlineStr">
@@ -12881,6 +14858,15 @@
       </c>
       <c r="W89" s="13" t="n">
         <v>-0.9992202245502645</v>
+      </c>
+      <c r="X89" s="13" t="n">
+        <v>-229.63185844</v>
+      </c>
+      <c r="Y89" s="13" t="n">
+        <v>-0.01350775637882353</v>
+      </c>
+      <c r="Z89" s="13" t="n">
+        <v>-1.214983377989418</v>
       </c>
     </row>
     <row r="90">
@@ -12910,6 +14896,9 @@
       <c r="U90" s="15" t="n"/>
       <c r="V90" s="15" t="n"/>
       <c r="W90" s="15" t="n"/>
+      <c r="X90" s="15" t="n"/>
+      <c r="Y90" s="15" t="n"/>
+      <c r="Z90" s="15" t="n"/>
     </row>
     <row r="91">
       <c r="B91" s="8" t="inlineStr">
@@ -12962,6 +14951,15 @@
       <c r="W91" s="9" t="n">
         <v>-0.4481058201058201</v>
       </c>
+      <c r="X91" s="9" t="n">
+        <v>-85.84400000000001</v>
+      </c>
+      <c r="Y91" s="9" t="n">
+        <v>-0.00504964705882353</v>
+      </c>
+      <c r="Z91" s="9" t="n">
+        <v>-0.4542010582010582</v>
+      </c>
     </row>
     <row r="92">
       <c r="B92" s="10" t="inlineStr">
@@ -13032,6 +15030,15 @@
       <c r="W92" s="11" t="n">
         <v>-0.9281514708994709</v>
       </c>
+      <c r="X92" s="11" t="n">
+        <v>-185.879421</v>
+      </c>
+      <c r="Y92" s="11" t="n">
+        <v>-0.01093408358823529</v>
+      </c>
+      <c r="Z92" s="11" t="n">
+        <v>-0.9834890000000001</v>
+      </c>
     </row>
     <row r="93">
       <c r="B93" s="8" t="inlineStr">
@@ -13102,6 +15109,15 @@
       <c r="W93" s="9" t="n">
         <v>-31.3222416373545</v>
       </c>
+      <c r="X93" s="9" t="n">
+        <v>-6530.220650459999</v>
+      </c>
+      <c r="Y93" s="9" t="n">
+        <v>-0.3841306264976471</v>
+      </c>
+      <c r="Z93" s="9" t="n">
+        <v>-34.55143201301588</v>
+      </c>
     </row>
     <row r="94">
       <c r="B94" s="10" t="inlineStr">
@@ -13172,6 +15188,15 @@
       <c r="W94" s="11" t="n">
         <v>-0.8636085714285715</v>
       </c>
+      <c r="X94" s="11" t="n">
+        <v>-193.699732</v>
+      </c>
+      <c r="Y94" s="11" t="n">
+        <v>-0.01139410188235294</v>
+      </c>
+      <c r="Z94" s="11" t="n">
+        <v>-1.024866306878307</v>
+      </c>
     </row>
     <row r="95">
       <c r="B95" s="8" t="inlineStr">
@@ -13242,6 +15267,15 @@
       <c r="W95" s="9" t="n">
         <v>-1.461407195767196</v>
       </c>
+      <c r="X95" s="9" t="n">
+        <v>-291.202982</v>
+      </c>
+      <c r="Y95" s="9" t="n">
+        <v>-0.01712958717647059</v>
+      </c>
+      <c r="Z95" s="9" t="n">
+        <v>-1.540756518518518</v>
+      </c>
     </row>
     <row r="96">
       <c r="B96" s="12" t="inlineStr">
@@ -13311,6 +15345,15 @@
       </c>
       <c r="W96" s="13" t="n">
         <v>-35.02351469555556</v>
+      </c>
+      <c r="X96" s="13" t="n">
+        <v>-7286.846785459999</v>
+      </c>
+      <c r="Y96" s="13" t="n">
+        <v>-0.4286380462035294</v>
+      </c>
+      <c r="Z96" s="13" t="n">
+        <v>-38.55474489661376</v>
       </c>
     </row>
     <row r="97">
@@ -13340,6 +15383,9 @@
       <c r="U97" s="15" t="n"/>
       <c r="V97" s="15" t="n"/>
       <c r="W97" s="15" t="n"/>
+      <c r="X97" s="15" t="n"/>
+      <c r="Y97" s="15" t="n"/>
+      <c r="Z97" s="15" t="n"/>
     </row>
     <row r="98">
       <c r="B98" s="8" t="inlineStr">
@@ -13410,6 +15456,15 @@
       <c r="W98" s="9" t="n">
         <v>-0.9218418095238095</v>
       </c>
+      <c r="X98" s="9" t="n">
+        <v>-182.969927</v>
+      </c>
+      <c r="Y98" s="9" t="n">
+        <v>-0.01076293688235294</v>
+      </c>
+      <c r="Z98" s="9" t="n">
+        <v>-0.9680948518518517</v>
+      </c>
     </row>
     <row r="99">
       <c r="B99" s="10" t="inlineStr">
@@ -13480,6 +15535,15 @@
       <c r="W99" s="11" t="n">
         <v>-0.6823075502645503</v>
       </c>
+      <c r="X99" s="11" t="n">
+        <v>-160.047281</v>
+      </c>
+      <c r="Y99" s="11" t="n">
+        <v>-0.00941454594117647</v>
+      </c>
+      <c r="Z99" s="11" t="n">
+        <v>-0.8468110105820106</v>
+      </c>
     </row>
     <row r="100">
       <c r="B100" s="8" t="inlineStr">
@@ -13549,6 +15613,15 @@
       </c>
       <c r="W100" s="9" t="n">
         <v>-5.278634232804233</v>
+      </c>
+      <c r="X100" s="9" t="n">
+        <v>-1191.659872</v>
+      </c>
+      <c r="Y100" s="9" t="n">
+        <v>-0.07009763952941175</v>
+      </c>
+      <c r="Z100" s="9" t="n">
+        <v>-6.305078687830688</v>
       </c>
     </row>
     <row r="101">
@@ -13614,6 +15687,15 @@
       <c r="W101" s="11" t="n">
         <v>-0.5951722222222222</v>
       </c>
+      <c r="X101" s="11" t="n">
+        <v>-156.36379</v>
+      </c>
+      <c r="Y101" s="11" t="n">
+        <v>-0.00919787</v>
+      </c>
+      <c r="Z101" s="11" t="n">
+        <v>-0.8273216402116402</v>
+      </c>
     </row>
     <row r="102">
       <c r="B102" s="12" t="inlineStr">
@@ -13683,6 +15765,15 @@
       </c>
       <c r="W102" s="13" t="n">
         <v>-7.477955814814814</v>
+      </c>
+      <c r="X102" s="13" t="n">
+        <v>-1691.04087</v>
+      </c>
+      <c r="Y102" s="13" t="n">
+        <v>-0.09947299235294117</v>
+      </c>
+      <c r="Z102" s="13" t="n">
+        <v>-8.947306190476191</v>
       </c>
     </row>
     <row r="103">
@@ -13712,6 +15803,9 @@
       <c r="U103" s="15" t="n"/>
       <c r="V103" s="15" t="n"/>
       <c r="W103" s="15" t="n"/>
+      <c r="X103" s="15" t="n"/>
+      <c r="Y103" s="15" t="n"/>
+      <c r="Z103" s="15" t="n"/>
     </row>
     <row r="104">
       <c r="B104" s="8" t="inlineStr">
@@ -13775,6 +15869,15 @@
       </c>
       <c r="W104" s="9" t="n">
         <v>-0.6742624338624339</v>
+      </c>
+      <c r="X104" s="9" t="n">
+        <v>-131.4656</v>
+      </c>
+      <c r="Y104" s="9" t="n">
+        <v>-0.007733270588235294</v>
+      </c>
+      <c r="Z104" s="9" t="n">
+        <v>-0.6955851851851852</v>
       </c>
     </row>
     <row r="105">
@@ -13816,6 +15919,15 @@
       <c r="W105" s="11" t="n">
         <v>-0.01217460317460317</v>
       </c>
+      <c r="X105" s="11" t="n">
+        <v>-8.2385</v>
+      </c>
+      <c r="Y105" s="11" t="n">
+        <v>-0.0004846176470588235</v>
+      </c>
+      <c r="Z105" s="11" t="n">
+        <v>-0.0435899470899471</v>
+      </c>
     </row>
     <row r="106">
       <c r="B106" s="8" t="inlineStr">
@@ -13886,6 +15998,15 @@
       <c r="W106" s="9" t="n">
         <v>-1.153318253968254</v>
       </c>
+      <c r="X106" s="9" t="n">
+        <v>-365.550111</v>
+      </c>
+      <c r="Y106" s="9" t="n">
+        <v>-0.02150294770588235</v>
+      </c>
+      <c r="Z106" s="9" t="n">
+        <v>-1.934127571428572</v>
+      </c>
     </row>
     <row r="107">
       <c r="B107" s="12" t="inlineStr">
@@ -13955,6 +16076,15 @@
       </c>
       <c r="W107" s="13" t="n">
         <v>-1.839755291005291</v>
+      </c>
+      <c r="X107" s="13" t="n">
+        <v>-505.254211</v>
+      </c>
+      <c r="Y107" s="13" t="n">
+        <v>-0.02972083594117647</v>
+      </c>
+      <c r="Z107" s="13" t="n">
+        <v>-2.673302703703704</v>
       </c>
     </row>
     <row r="108">
@@ -13984,6 +16114,9 @@
       <c r="U108" s="15" t="n"/>
       <c r="V108" s="15" t="n"/>
       <c r="W108" s="15" t="n"/>
+      <c r="X108" s="15" t="n"/>
+      <c r="Y108" s="15" t="n"/>
+      <c r="Z108" s="15" t="n"/>
     </row>
     <row r="109">
       <c r="B109" s="8" t="inlineStr">
@@ -14047,6 +16180,15 @@
       </c>
       <c r="W109" s="9" t="n">
         <v>-1.726759650793651</v>
+      </c>
+      <c r="X109" s="9" t="n">
+        <v>-352.517574</v>
+      </c>
+      <c r="Y109" s="9" t="n">
+        <v>-0.02073632788235294</v>
+      </c>
+      <c r="Z109" s="9" t="n">
+        <v>-1.865172349206349</v>
       </c>
     </row>
     <row r="110">
@@ -14076,6 +16218,15 @@
       <c r="U110" s="11" t="n"/>
       <c r="V110" s="11" t="n"/>
       <c r="W110" s="11" t="n"/>
+      <c r="X110" s="11" t="n">
+        <v>-13</v>
+      </c>
+      <c r="Y110" s="11" t="n">
+        <v>-0.0007647058823529412</v>
+      </c>
+      <c r="Z110" s="11" t="n">
+        <v>-0.06878306878306878</v>
+      </c>
     </row>
     <row r="111">
       <c r="B111" s="8" t="inlineStr">
@@ -14146,6 +16297,15 @@
       <c r="W111" s="9" t="n">
         <v>-0.6172780687830688</v>
       </c>
+      <c r="X111" s="9" t="n">
+        <v>-123.269133</v>
+      </c>
+      <c r="Y111" s="9" t="n">
+        <v>-0.007251125470588235</v>
+      </c>
+      <c r="Z111" s="9" t="n">
+        <v>-0.6522176349206349</v>
+      </c>
     </row>
     <row r="112">
       <c r="B112" s="10" t="inlineStr">
@@ -14216,6 +16376,15 @@
       <c r="W112" s="11" t="n">
         <v>-1.315173513227513</v>
       </c>
+      <c r="X112" s="11" t="n">
+        <v>-413.518543</v>
+      </c>
+      <c r="Y112" s="11" t="n">
+        <v>-0.02432462017647059</v>
+      </c>
+      <c r="Z112" s="11" t="n">
+        <v>-2.187928798941799</v>
+      </c>
     </row>
     <row r="113">
       <c r="B113" s="12" t="inlineStr">
@@ -14285,6 +16454,15 @@
       </c>
       <c r="W113" s="13" t="n">
         <v>-3.659211232804233</v>
+      </c>
+      <c r="X113" s="13" t="n">
+        <v>-902.30525</v>
+      </c>
+      <c r="Y113" s="13" t="n">
+        <v>-0.05307677941176471</v>
+      </c>
+      <c r="Z113" s="13" t="n">
+        <v>-4.774101851851852</v>
       </c>
     </row>
     <row r="114">
@@ -14314,6 +16492,9 @@
       <c r="U114" s="15" t="n"/>
       <c r="V114" s="15" t="n"/>
       <c r="W114" s="15" t="n"/>
+      <c r="X114" s="15" t="n"/>
+      <c r="Y114" s="15" t="n"/>
+      <c r="Z114" s="15" t="n"/>
     </row>
     <row r="115">
       <c r="B115" s="8" t="inlineStr">
@@ -14384,6 +16565,15 @@
       <c r="W115" s="9" t="n">
         <v>-21.74374634391534</v>
       </c>
+      <c r="X115" s="9" t="n">
+        <v>-4845.172432</v>
+      </c>
+      <c r="Y115" s="9" t="n">
+        <v>-0.2850101430588236</v>
+      </c>
+      <c r="Z115" s="9" t="n">
+        <v>-25.63583297354498</v>
+      </c>
     </row>
     <row r="116">
       <c r="B116" s="12" t="inlineStr">
@@ -14453,6 +16643,15 @@
       </c>
       <c r="W116" s="13" t="n">
         <v>-21.74374634391534</v>
+      </c>
+      <c r="X116" s="13" t="n">
+        <v>-4845.172432</v>
+      </c>
+      <c r="Y116" s="13" t="n">
+        <v>-0.2850101430588236</v>
+      </c>
+      <c r="Z116" s="13" t="n">
+        <v>-25.63583297354498</v>
       </c>
     </row>
     <row r="117">
@@ -14482,6 +16681,9 @@
       <c r="U117" s="15" t="n"/>
       <c r="V117" s="15" t="n"/>
       <c r="W117" s="15" t="n"/>
+      <c r="X117" s="15" t="n"/>
+      <c r="Y117" s="15" t="n"/>
+      <c r="Z117" s="15" t="n"/>
     </row>
     <row r="118">
       <c r="B118" s="8" t="inlineStr">
@@ -14532,6 +16734,15 @@
         <v>-0.3388428851764705</v>
       </c>
       <c r="W118" s="9" t="n">
+        <v>-30.47793147089947</v>
+      </c>
+      <c r="X118" s="9" t="n">
+        <v>-5760.329048</v>
+      </c>
+      <c r="Y118" s="9" t="n">
+        <v>-0.3388428851764705</v>
+      </c>
+      <c r="Z118" s="9" t="n">
         <v>-30.47793147089947</v>
       </c>
     </row>
@@ -14574,6 +16785,15 @@
       <c r="W119" s="11" t="n">
         <v>-9.685637142857143</v>
       </c>
+      <c r="X119" s="11" t="n">
+        <v>-1830.58542</v>
+      </c>
+      <c r="Y119" s="11" t="n">
+        <v>-0.1076814952941176</v>
+      </c>
+      <c r="Z119" s="11" t="n">
+        <v>-9.685637142857143</v>
+      </c>
     </row>
     <row r="120">
       <c r="B120" s="8" t="inlineStr">
@@ -14644,6 +16864,15 @@
       <c r="W120" s="9" t="n">
         <v>-0.07982265079365081</v>
       </c>
+      <c r="X120" s="9" t="n">
+        <v>-16.814481</v>
+      </c>
+      <c r="Y120" s="9" t="n">
+        <v>-0.000989087117647059</v>
+      </c>
+      <c r="Z120" s="9" t="n">
+        <v>-0.08896550793650795</v>
+      </c>
     </row>
     <row r="121">
       <c r="B121" s="10" t="inlineStr">
@@ -14713,6 +16942,15 @@
       </c>
       <c r="W121" s="11" t="n">
         <v>-6.957568632116402</v>
+      </c>
+      <c r="X121" s="11" t="n">
+        <v>-1555.85047747</v>
+      </c>
+      <c r="Y121" s="11" t="n">
+        <v>-0.0915206163217647</v>
+      </c>
+      <c r="Z121" s="11" t="n">
+        <v>-8.232013108306878</v>
       </c>
     </row>
     <row r="122">
@@ -14772,6 +17010,15 @@
       <c r="W122" s="9" t="n">
         <v>-0.9526269841269841</v>
       </c>
+      <c r="X122" s="9" t="n">
+        <v>-299.8755</v>
+      </c>
+      <c r="Y122" s="9" t="n">
+        <v>-0.01763973529411765</v>
+      </c>
+      <c r="Z122" s="9" t="n">
+        <v>-1.586642857142857</v>
+      </c>
     </row>
     <row r="123">
       <c r="B123" s="10" t="inlineStr">
@@ -14842,6 +17089,15 @@
       <c r="W123" s="11" t="n">
         <v>-69.61398012698412</v>
       </c>
+      <c r="X123" s="11" t="n">
+        <v>-13932.690388</v>
+      </c>
+      <c r="Y123" s="11" t="n">
+        <v>-0.8195700228235293</v>
+      </c>
+      <c r="Z123" s="11" t="n">
+        <v>-73.71793856084655</v>
+      </c>
     </row>
     <row r="124">
       <c r="B124" s="12" t="inlineStr">
@@ -14911,6 +17167,15 @@
       </c>
       <c r="W124" s="13" t="n">
         <v>-117.7675670077778</v>
+      </c>
+      <c r="X124" s="13" t="n">
+        <v>-23396.14531447</v>
+      </c>
+      <c r="Y124" s="13" t="n">
+        <v>-1.376243842027647</v>
+      </c>
+      <c r="Z124" s="13" t="n">
+        <v>-123.7891286479894</v>
       </c>
     </row>
     <row r="125">
@@ -14940,6 +17205,9 @@
       <c r="U125" s="15" t="n"/>
       <c r="V125" s="15" t="n"/>
       <c r="W125" s="15" t="n"/>
+      <c r="X125" s="15" t="n"/>
+      <c r="Y125" s="15" t="n"/>
+      <c r="Z125" s="15" t="n"/>
     </row>
     <row r="126">
       <c r="B126" s="8" t="inlineStr">
@@ -14998,6 +17266,15 @@
       <c r="W126" s="9" t="n">
         <v>-0.1215469312169312</v>
       </c>
+      <c r="X126" s="9" t="n">
+        <v>-26.71332</v>
+      </c>
+      <c r="Y126" s="9" t="n">
+        <v>-0.001571371764705882</v>
+      </c>
+      <c r="Z126" s="9" t="n">
+        <v>-0.1413403174603174</v>
+      </c>
     </row>
     <row r="127">
       <c r="B127" s="10" t="inlineStr">
@@ -15056,6 +17333,15 @@
       <c r="W127" s="11" t="n">
         <v>-0.6542180052910054</v>
       </c>
+      <c r="X127" s="11" t="n">
+        <v>-184.037662</v>
+      </c>
+      <c r="Y127" s="11" t="n">
+        <v>-0.01082574482352941</v>
+      </c>
+      <c r="Z127" s="11" t="n">
+        <v>-0.9737442433862435</v>
+      </c>
     </row>
     <row r="128">
       <c r="B128" s="8" t="inlineStr">
@@ -15126,6 +17412,15 @@
       <c r="W128" s="9" t="n">
         <v>-1.093348444444444</v>
       </c>
+      <c r="X128" s="9" t="n">
+        <v>-206.642856</v>
+      </c>
+      <c r="Y128" s="9" t="n">
+        <v>-0.01215546211764706</v>
+      </c>
+      <c r="Z128" s="9" t="n">
+        <v>-1.093348444444444</v>
+      </c>
     </row>
     <row r="129">
       <c r="B129" s="10" t="inlineStr">
@@ -15196,6 +17491,15 @@
       <c r="W129" s="11" t="n">
         <v>-0.4247761058201058</v>
       </c>
+      <c r="X129" s="11" t="n">
+        <v>-92.30842800000001</v>
+      </c>
+      <c r="Y129" s="11" t="n">
+        <v>-0.005429907529411766</v>
+      </c>
+      <c r="Z129" s="11" t="n">
+        <v>-0.488404380952381</v>
+      </c>
     </row>
     <row r="130">
       <c r="B130" s="8" t="inlineStr">
@@ -15265,6 +17569,15 @@
       </c>
       <c r="W130" s="9" t="n">
         <v>-0.9334655238095239</v>
+      </c>
+      <c r="X130" s="9" t="n">
+        <v>-199.819215</v>
+      </c>
+      <c r="Y130" s="9" t="n">
+        <v>-0.01175407147058824</v>
+      </c>
+      <c r="Z130" s="9" t="n">
+        <v>-1.057244523809524</v>
       </c>
     </row>
     <row r="131">
@@ -15306,6 +17619,15 @@
       <c r="W131" s="11" t="n">
         <v>-0.005820105820105821</v>
       </c>
+      <c r="X131" s="11" t="n">
+        <v>-1.1</v>
+      </c>
+      <c r="Y131" s="11" t="n">
+        <v>-6.470588235294118e-05</v>
+      </c>
+      <c r="Z131" s="11" t="n">
+        <v>-0.005820105820105821</v>
+      </c>
     </row>
     <row r="132">
       <c r="B132" s="12" t="inlineStr">
@@ -15376,6 +17698,15 @@
       <c r="W132" s="13" t="n">
         <v>-3.233175116402117</v>
       </c>
+      <c r="X132" s="13" t="n">
+        <v>-710.621481</v>
+      </c>
+      <c r="Y132" s="13" t="n">
+        <v>-0.04180126358823529</v>
+      </c>
+      <c r="Z132" s="13" t="n">
+        <v>-3.759902015873016</v>
+      </c>
     </row>
     <row r="133">
       <c r="B133" s="12" t="inlineStr">
@@ -15445,6 +17776,15 @@
       </c>
       <c r="W133" s="13" t="n">
         <v>-191.7441457268254</v>
+      </c>
+      <c r="X133" s="13" t="n">
+        <v>-39567.01820237</v>
+      </c>
+      <c r="Y133" s="13" t="n">
+        <v>-2.327471658962941</v>
+      </c>
+      <c r="Z133" s="13" t="n">
+        <v>-209.3493026580423</v>
       </c>
     </row>
     <row r="134">
@@ -15474,6 +17814,9 @@
       <c r="U134" s="15" t="n"/>
       <c r="V134" s="15" t="n"/>
       <c r="W134" s="15" t="n"/>
+      <c r="X134" s="15" t="n"/>
+      <c r="Y134" s="15" t="n"/>
+      <c r="Z134" s="15" t="n"/>
     </row>
     <row r="135">
       <c r="B135" s="8" t="inlineStr">
@@ -15530,6 +17873,15 @@
         <v>-0.005058823529411765</v>
       </c>
       <c r="W135" s="9" t="n">
+        <v>-0.455026455026455</v>
+      </c>
+      <c r="X135" s="9" t="n">
+        <v>-86</v>
+      </c>
+      <c r="Y135" s="9" t="n">
+        <v>-0.005058823529411765</v>
+      </c>
+      <c r="Z135" s="9" t="n">
         <v>-0.455026455026455</v>
       </c>
     </row>
@@ -15560,6 +17912,15 @@
       <c r="U136" s="11" t="n"/>
       <c r="V136" s="11" t="n"/>
       <c r="W136" s="11" t="n"/>
+      <c r="X136" s="11" t="n">
+        <v>-5</v>
+      </c>
+      <c r="Y136" s="11" t="n">
+        <v>-0.0002941176470588235</v>
+      </c>
+      <c r="Z136" s="11" t="n">
+        <v>-0.02645502645502645</v>
+      </c>
     </row>
     <row r="137">
       <c r="B137" s="8" t="inlineStr">
@@ -15629,6 +17990,15 @@
       </c>
       <c r="W137" s="9" t="n">
         <v>-3.102749708994709</v>
+      </c>
+      <c r="X137" s="9" t="n">
+        <v>-678.771055</v>
+      </c>
+      <c r="Y137" s="9" t="n">
+        <v>-0.03992770911764706</v>
+      </c>
+      <c r="Z137" s="9" t="n">
+        <v>-3.591381243386243</v>
       </c>
     </row>
     <row r="138">
@@ -15670,6 +18040,15 @@
       <c r="W138" s="11" t="n">
         <v>-8.289354497354498</v>
       </c>
+      <c r="X138" s="11" t="n">
+        <v>-1566.688</v>
+      </c>
+      <c r="Y138" s="11" t="n">
+        <v>-0.09215811764705883</v>
+      </c>
+      <c r="Z138" s="11" t="n">
+        <v>-8.289354497354498</v>
+      </c>
     </row>
     <row r="139">
       <c r="B139" s="8" t="inlineStr">
@@ -15710,6 +18089,15 @@
       <c r="W139" s="9" t="n">
         <v>-0.04457671957671958</v>
       </c>
+      <c r="X139" s="9" t="n">
+        <v>-8.425000000000001</v>
+      </c>
+      <c r="Y139" s="9" t="n">
+        <v>-0.0004955882352941177</v>
+      </c>
+      <c r="Z139" s="9" t="n">
+        <v>-0.04457671957671958</v>
+      </c>
     </row>
     <row r="140">
       <c r="B140" s="12" t="inlineStr">
@@ -15779,6 +18167,15 @@
       </c>
       <c r="W140" s="13" t="n">
         <v>-11.89170738095238</v>
+      </c>
+      <c r="X140" s="13" t="n">
+        <v>-2344.884055</v>
+      </c>
+      <c r="Y140" s="13" t="n">
+        <v>-0.1379343561764706</v>
+      </c>
+      <c r="Z140" s="13" t="n">
+        <v>-12.40679394179894</v>
       </c>
     </row>
     <row r="141">
@@ -15808,6 +18205,9 @@
       <c r="U141" s="15" t="n"/>
       <c r="V141" s="15" t="n"/>
       <c r="W141" s="15" t="n"/>
+      <c r="X141" s="15" t="n"/>
+      <c r="Y141" s="15" t="n"/>
+      <c r="Z141" s="15" t="n"/>
     </row>
     <row r="142">
       <c r="B142" s="8" t="inlineStr">
@@ -15877,6 +18277,15 @@
       </c>
       <c r="W142" s="9" t="n">
         <v>-0.07509776550264551</v>
+      </c>
+      <c r="X142" s="9" t="n">
+        <v>-16.27273168</v>
+      </c>
+      <c r="Y142" s="9" t="n">
+        <v>-0.0009572195105882354</v>
+      </c>
+      <c r="Z142" s="9" t="n">
+        <v>-0.08609910941798943</v>
       </c>
     </row>
     <row r="143">
@@ -15924,6 +18333,15 @@
       <c r="W143" s="11" t="n">
         <v>-0.2752046190476191</v>
       </c>
+      <c r="X143" s="11" t="n">
+        <v>-52.013673</v>
+      </c>
+      <c r="Y143" s="11" t="n">
+        <v>-0.003059627823529412</v>
+      </c>
+      <c r="Z143" s="11" t="n">
+        <v>-0.2752046190476191</v>
+      </c>
     </row>
     <row r="144">
       <c r="B144" s="8" t="inlineStr">
@@ -15982,6 +18400,15 @@
       <c r="W144" s="9" t="n">
         <v>-0.04949648227513227</v>
       </c>
+      <c r="X144" s="9" t="n">
+        <v>-9.35483515</v>
+      </c>
+      <c r="Y144" s="9" t="n">
+        <v>-0.0005502844205882353</v>
+      </c>
+      <c r="Z144" s="9" t="n">
+        <v>-0.04949648227513227</v>
+      </c>
     </row>
     <row r="145">
       <c r="B145" s="10" t="inlineStr">
@@ -16051,6 +18478,15 @@
       </c>
       <c r="W145" s="11" t="n">
         <v>-20.5270663257672</v>
+      </c>
+      <c r="X145" s="11" t="n">
+        <v>-4071.17796057</v>
+      </c>
+      <c r="Y145" s="11" t="n">
+        <v>-0.2394810565041176</v>
+      </c>
+      <c r="Z145" s="11" t="n">
+        <v>-21.54062413</v>
       </c>
     </row>
     <row r="146">
@@ -16108,6 +18544,15 @@
         <v>-0.03780123429411764</v>
       </c>
       <c r="W146" s="9" t="n">
+        <v>-3.400111021164021</v>
+      </c>
+      <c r="X146" s="9" t="n">
+        <v>-642.620983</v>
+      </c>
+      <c r="Y146" s="9" t="n">
+        <v>-0.03780123429411764</v>
+      </c>
+      <c r="Z146" s="9" t="n">
         <v>-3.400111021164021</v>
       </c>
     </row>
@@ -16150,6 +18595,15 @@
       <c r="W147" s="11" t="n">
         <v>-4.09466419047619</v>
       </c>
+      <c r="X147" s="11" t="n">
+        <v>-773.891532</v>
+      </c>
+      <c r="Y147" s="11" t="n">
+        <v>-0.04552303129411765</v>
+      </c>
+      <c r="Z147" s="11" t="n">
+        <v>-4.09466419047619</v>
+      </c>
     </row>
     <row r="148">
       <c r="B148" s="12" t="inlineStr">
@@ -16220,6 +18674,15 @@
       <c r="W148" s="13" t="n">
         <v>-28.4216404042328</v>
       </c>
+      <c r="X148" s="13" t="n">
+        <v>-5565.3317154</v>
+      </c>
+      <c r="Y148" s="13" t="n">
+        <v>-0.3273724538470589</v>
+      </c>
+      <c r="Z148" s="13" t="n">
+        <v>-29.44619955238095</v>
+      </c>
     </row>
     <row r="149">
       <c r="B149" s="16" t="inlineStr">
@@ -16290,6 +18753,15 @@
       <c r="W149" s="17" t="n">
         <v>-1435.352458064497</v>
       </c>
+      <c r="X149" s="17" t="n">
+        <v>-278608.13977919</v>
+      </c>
+      <c r="Y149" s="17" t="n">
+        <v>-16.38871410465823</v>
+      </c>
+      <c r="Z149" s="17" t="n">
+        <v>-1474.117141688836</v>
+      </c>
     </row>
     <row r="150">
       <c r="B150" s="16" t="inlineStr">
@@ -16360,6 +18832,15 @@
       <c r="W150" s="17" t="n">
         <v>-347.3444751858202</v>
       </c>
+      <c r="X150" s="17" t="n">
+        <v>-66049.02254812002</v>
+      </c>
+      <c r="Y150" s="17" t="n">
+        <v>-3.885236620477648</v>
+      </c>
+      <c r="Z150" s="17" t="n">
+        <v>-349.4657277678308</v>
+      </c>
     </row>
     <row r="151">
       <c r="B151" s="14" t="inlineStr">
@@ -16430,6 +18911,15 @@
       <c r="W151" s="15" t="n">
         <v>357.0034964357672</v>
       </c>
+      <c r="X151" s="15" t="n">
+        <v>67473.66082636001</v>
+      </c>
+      <c r="Y151" s="15" t="n">
+        <v>3.969038872138824</v>
+      </c>
+      <c r="Z151" s="15" t="n">
+        <v>357.0034964357672</v>
+      </c>
     </row>
     <row r="152">
       <c r="B152" s="16" t="inlineStr">
@@ -16500,15 +18990,25 @@
       <c r="W152" s="17" t="n">
         <v>9.659021255238104</v>
       </c>
+      <c r="X152" s="17" t="n">
+        <v>1424.63827823999</v>
+      </c>
+      <c r="Y152" s="17" t="n">
+        <v>0.0838022516611759</v>
+      </c>
+      <c r="Z152" s="17" t="n">
+        <v>7.537768667936457</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
-    <mergeCell ref="B2:W2"/>
+  <mergeCells count="11">
+    <mergeCell ref="B2:Z2"/>
     <mergeCell ref="R3:T3"/>
     <mergeCell ref="U3:W3"/>
     <mergeCell ref="B3:B4"/>
-    <mergeCell ref="B1:W1"/>
+    <mergeCell ref="B1:Z1"/>
     <mergeCell ref="C3:E3"/>
+    <mergeCell ref="X3:Z3"/>
     <mergeCell ref="I3:K3"/>
     <mergeCell ref="F3:H3"/>
     <mergeCell ref="L3:N3"/>

</xml_diff>

<commit_message>
Refresh dashboard Tue 07/28/2026 16:35
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -672,7 +672,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:Z152"/>
+  <dimension ref="B1:AC152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -701,6 +701,9 @@
     <col width="16" customWidth="1" min="24" max="24"/>
     <col width="16" customWidth="1" min="25" max="25"/>
     <col width="16" customWidth="1" min="26" max="26"/>
+    <col width="16" customWidth="1" min="27" max="27"/>
+    <col width="16" customWidth="1" min="28" max="28"/>
+    <col width="16" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -713,7 +716,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 28 Jul 2026 16:28</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 28 Jul 2026 16:35</t>
         </is>
       </c>
     </row>
@@ -779,6 +782,13 @@
       </c>
       <c r="Y3" s="4" t="n"/>
       <c r="Z3" s="4" t="n"/>
+      <c r="AA3" s="3" t="inlineStr">
+        <is>
+          <t>MTD as of 28 Jul 2026</t>
+        </is>
+      </c>
+      <c r="AB3" s="4" t="n"/>
+      <c r="AC3" s="4" t="n"/>
     </row>
     <row r="4" ht="18" customHeight="1">
       <c r="B4" s="5" t="n"/>
@@ -898,6 +908,21 @@
         </is>
       </c>
       <c r="Z4" s="3" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="AA4" s="3" t="inlineStr">
+        <is>
+          <t>IDR</t>
+        </is>
+      </c>
+      <c r="AB4" s="3" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="AC4" s="3" t="inlineStr">
         <is>
           <t>INR</t>
         </is>
@@ -933,6 +958,9 @@
       <c r="X5" s="7" t="n"/>
       <c r="Y5" s="7" t="n"/>
       <c r="Z5" s="7" t="n"/>
+      <c r="AA5" s="7" t="n"/>
+      <c r="AB5" s="7" t="n"/>
+      <c r="AC5" s="7" t="n"/>
     </row>
     <row r="6">
       <c r="B6" s="8" t="inlineStr">
@@ -1011,6 +1039,15 @@
       </c>
       <c r="Z6" s="9" t="n">
         <v>859003679.8253969</v>
+      </c>
+      <c r="AA6" s="9" t="n">
+        <v>6895316417</v>
+      </c>
+      <c r="AB6" s="9" t="n">
+        <v>405606.8480588236</v>
+      </c>
+      <c r="AC6" s="9" t="n">
+        <v>36483155.64550264</v>
       </c>
     </row>
     <row r="7">
@@ -1073,6 +1110,15 @@
       <c r="Z7" s="11" t="n">
         <v>483947073.4338624</v>
       </c>
+      <c r="AA7" s="11" t="n">
+        <v>19305092</v>
+      </c>
+      <c r="AB7" s="11" t="n">
+        <v>1135.593647058824</v>
+      </c>
+      <c r="AC7" s="11" t="n">
+        <v>102143.3439153439</v>
+      </c>
     </row>
     <row r="8">
       <c r="B8" s="8" t="inlineStr">
@@ -1151,6 +1197,15 @@
       </c>
       <c r="Z8" s="9" t="n">
         <v>173671198.5132275</v>
+      </c>
+      <c r="AA8" s="9" t="n">
+        <v>3590241514</v>
+      </c>
+      <c r="AB8" s="9" t="n">
+        <v>211190.6772941177</v>
+      </c>
+      <c r="AC8" s="9" t="n">
+        <v>18995986.84656085</v>
       </c>
     </row>
     <row r="9">
@@ -1225,6 +1280,15 @@
       <c r="Z9" s="11" t="n">
         <v>154834760.984127</v>
       </c>
+      <c r="AA9" s="11" t="n">
+        <v>2297841064</v>
+      </c>
+      <c r="AB9" s="11" t="n">
+        <v>135167.1214117647</v>
+      </c>
+      <c r="AC9" s="11" t="n">
+        <v>12157889.22751323</v>
+      </c>
     </row>
     <row r="10">
       <c r="B10" s="8" t="inlineStr">
@@ -1298,6 +1362,15 @@
       <c r="Z10" s="9" t="n">
         <v>38029556.94708995</v>
       </c>
+      <c r="AA10" s="9" t="n">
+        <v>575848747</v>
+      </c>
+      <c r="AB10" s="9" t="n">
+        <v>33873.45570588236</v>
+      </c>
+      <c r="AC10" s="9" t="n">
+        <v>3046818.767195767</v>
+      </c>
     </row>
     <row r="11">
       <c r="B11" s="10" t="inlineStr">
@@ -1364,6 +1437,15 @@
       </c>
       <c r="Z11" s="11" t="n">
         <v>7631111.111111112</v>
+      </c>
+      <c r="AA11" s="11" t="n">
+        <v>412080000</v>
+      </c>
+      <c r="AB11" s="11" t="n">
+        <v>24240</v>
+      </c>
+      <c r="AC11" s="11" t="n">
+        <v>2180317.46031746</v>
       </c>
     </row>
     <row r="12">
@@ -1414,6 +1496,9 @@
       <c r="Z12" s="9" t="n">
         <v>740835.9788359788</v>
       </c>
+      <c r="AA12" s="9" t="n"/>
+      <c r="AB12" s="9" t="n"/>
+      <c r="AC12" s="9" t="n"/>
     </row>
     <row r="13">
       <c r="B13" s="10" t="inlineStr">
@@ -1463,6 +1548,9 @@
       <c r="Z13" s="11" t="n">
         <v>149142.8571428571</v>
       </c>
+      <c r="AA13" s="11" t="n"/>
+      <c r="AB13" s="11" t="n"/>
+      <c r="AC13" s="11" t="n"/>
     </row>
     <row r="14">
       <c r="B14" s="8" t="inlineStr">
@@ -1512,6 +1600,9 @@
       <c r="Z14" s="9" t="n">
         <v>262412698.4126984</v>
       </c>
+      <c r="AA14" s="9" t="n"/>
+      <c r="AB14" s="9" t="n"/>
+      <c r="AC14" s="9" t="n"/>
     </row>
     <row r="15">
       <c r="B15" s="10" t="inlineStr">
@@ -1561,6 +1652,9 @@
       <c r="Z15" s="11" t="n">
         <v>262412698.4126984</v>
       </c>
+      <c r="AA15" s="11" t="n"/>
+      <c r="AB15" s="11" t="n"/>
+      <c r="AC15" s="11" t="n"/>
     </row>
     <row r="16">
       <c r="B16" s="8" t="inlineStr">
@@ -1640,6 +1734,15 @@
       <c r="Z16" s="9" t="n">
         <v>2071014.518888889</v>
       </c>
+      <c r="AA16" s="9" t="n">
+        <v>30292050</v>
+      </c>
+      <c r="AB16" s="9" t="n">
+        <v>1781.885294117647</v>
+      </c>
+      <c r="AC16" s="9" t="n">
+        <v>160275.3968253968</v>
+      </c>
     </row>
     <row r="17">
       <c r="B17" s="10" t="inlineStr">
@@ -1719,6 +1822,9 @@
       <c r="Z17" s="11" t="n">
         <v>671818.6214814816</v>
       </c>
+      <c r="AA17" s="11" t="n"/>
+      <c r="AB17" s="11" t="n"/>
+      <c r="AC17" s="11" t="n"/>
     </row>
     <row r="18">
       <c r="B18" s="8" t="inlineStr">
@@ -1768,6 +1874,9 @@
       <c r="Z18" s="9" t="n">
         <v>657985.1851851852</v>
       </c>
+      <c r="AA18" s="9" t="n"/>
+      <c r="AB18" s="9" t="n"/>
+      <c r="AC18" s="9" t="n"/>
     </row>
     <row r="19">
       <c r="B19" s="10" t="inlineStr">
@@ -1817,6 +1926,9 @@
       <c r="Z19" s="11" t="n">
         <v>123121.6931216931</v>
       </c>
+      <c r="AA19" s="11" t="n"/>
+      <c r="AB19" s="11" t="n"/>
+      <c r="AC19" s="11" t="n"/>
     </row>
     <row r="20">
       <c r="B20" s="8" t="inlineStr">
@@ -1883,6 +1995,15 @@
       </c>
       <c r="Z20" s="9" t="n">
         <v>118941.7989417989</v>
+      </c>
+      <c r="AA20" s="9" t="n">
+        <v>4014500</v>
+      </c>
+      <c r="AB20" s="9" t="n">
+        <v>236.1470588235294</v>
+      </c>
+      <c r="AC20" s="9" t="n">
+        <v>21240.74074074074</v>
       </c>
     </row>
     <row r="21">
@@ -1939,6 +2060,9 @@
       <c r="Z21" s="11" t="n">
         <v>106905.0264550265</v>
       </c>
+      <c r="AA21" s="11" t="n"/>
+      <c r="AB21" s="11" t="n"/>
+      <c r="AC21" s="11" t="n"/>
     </row>
     <row r="22">
       <c r="B22" s="8" t="inlineStr">
@@ -1976,6 +2100,15 @@
       <c r="Z22" s="9" t="n">
         <v>94523.80952380953</v>
       </c>
+      <c r="AA22" s="9" t="n">
+        <v>17865000</v>
+      </c>
+      <c r="AB22" s="9" t="n">
+        <v>1050.882352941177</v>
+      </c>
+      <c r="AC22" s="9" t="n">
+        <v>94523.80952380953</v>
+      </c>
     </row>
     <row r="23">
       <c r="B23" s="10" t="inlineStr">
@@ -2025,6 +2158,9 @@
       <c r="Z23" s="11" t="n">
         <v>74473.01587301587</v>
       </c>
+      <c r="AA23" s="11" t="n"/>
+      <c r="AB23" s="11" t="n"/>
+      <c r="AC23" s="11" t="n"/>
     </row>
     <row r="24">
       <c r="B24" s="8" t="inlineStr">
@@ -2091,6 +2227,15 @@
       </c>
       <c r="Z24" s="9" t="n">
         <v>62742.76190476191</v>
+      </c>
+      <c r="AA24" s="9" t="n">
+        <v>4037000</v>
+      </c>
+      <c r="AB24" s="9" t="n">
+        <v>237.4705882352941</v>
+      </c>
+      <c r="AC24" s="9" t="n">
+        <v>21359.78835978836</v>
       </c>
     </row>
     <row r="25">
@@ -2141,6 +2286,9 @@
       <c r="Z25" s="11" t="n">
         <v>39765.75132275133</v>
       </c>
+      <c r="AA25" s="11" t="n"/>
+      <c r="AB25" s="11" t="n"/>
+      <c r="AC25" s="11" t="n"/>
     </row>
     <row r="26">
       <c r="B26" s="8" t="inlineStr">
@@ -2196,6 +2344,9 @@
       <c r="Z26" s="9" t="n">
         <v>31746.03174603175</v>
       </c>
+      <c r="AA26" s="9" t="n"/>
+      <c r="AB26" s="9" t="n"/>
+      <c r="AC26" s="9" t="n"/>
     </row>
     <row r="27">
       <c r="B27" s="10" t="inlineStr">
@@ -2250,6 +2401,15 @@
       </c>
       <c r="Z27" s="11" t="n">
         <v>23725.02645502645</v>
+      </c>
+      <c r="AA27" s="11" t="n">
+        <v>350000</v>
+      </c>
+      <c r="AB27" s="11" t="n">
+        <v>20.58823529411765</v>
+      </c>
+      <c r="AC27" s="11" t="n">
+        <v>1851.851851851852</v>
       </c>
     </row>
     <row r="28">
@@ -2300,6 +2460,9 @@
       <c r="Z28" s="9" t="n">
         <v>20227.7671957672</v>
       </c>
+      <c r="AA28" s="9" t="n"/>
+      <c r="AB28" s="9" t="n"/>
+      <c r="AC28" s="9" t="n"/>
     </row>
     <row r="29">
       <c r="B29" s="10" t="inlineStr">
@@ -2349,6 +2512,15 @@
       <c r="Z29" s="11" t="n">
         <v>14288.09523809524</v>
       </c>
+      <c r="AA29" s="11" t="n">
+        <v>2595250</v>
+      </c>
+      <c r="AB29" s="11" t="n">
+        <v>152.6617647058823</v>
+      </c>
+      <c r="AC29" s="11" t="n">
+        <v>13731.48148148148</v>
+      </c>
     </row>
     <row r="30">
       <c r="B30" s="8" t="inlineStr">
@@ -2410,6 +2582,9 @@
       <c r="Z30" s="9" t="n">
         <v>9278.511164021163</v>
       </c>
+      <c r="AA30" s="9" t="n"/>
+      <c r="AB30" s="9" t="n"/>
+      <c r="AC30" s="9" t="n"/>
     </row>
     <row r="31">
       <c r="B31" s="10" t="inlineStr">
@@ -2459,6 +2634,15 @@
       <c r="Z31" s="11" t="n">
         <v>8699.957671957673</v>
       </c>
+      <c r="AA31" s="11" t="n">
+        <v>1360300</v>
+      </c>
+      <c r="AB31" s="11" t="n">
+        <v>80.01764705882353</v>
+      </c>
+      <c r="AC31" s="11" t="n">
+        <v>7197.354497354498</v>
+      </c>
     </row>
     <row r="32">
       <c r="B32" s="8" t="inlineStr">
@@ -2508,6 +2692,9 @@
       <c r="Z32" s="9" t="n">
         <v>5291.005291005291</v>
       </c>
+      <c r="AA32" s="9" t="n"/>
+      <c r="AB32" s="9" t="n"/>
+      <c r="AC32" s="9" t="n"/>
     </row>
     <row r="33">
       <c r="B33" s="10" t="inlineStr">
@@ -2569,6 +2756,9 @@
       <c r="Z33" s="11" t="n">
         <v>3911.111111111111</v>
       </c>
+      <c r="AA33" s="11" t="n"/>
+      <c r="AB33" s="11" t="n"/>
+      <c r="AC33" s="11" t="n"/>
     </row>
     <row r="34">
       <c r="B34" s="8" t="inlineStr">
@@ -2624,6 +2814,9 @@
       <c r="Z34" s="9" t="n">
         <v>2648.703703703704</v>
       </c>
+      <c r="AA34" s="9" t="n"/>
+      <c r="AB34" s="9" t="n"/>
+      <c r="AC34" s="9" t="n"/>
     </row>
     <row r="35">
       <c r="B35" s="10" t="inlineStr">
@@ -2673,6 +2866,15 @@
       <c r="Z35" s="11" t="n">
         <v>899.4814814814815</v>
       </c>
+      <c r="AA35" s="11" t="n">
+        <v>70000</v>
+      </c>
+      <c r="AB35" s="11" t="n">
+        <v>4.117647058823529</v>
+      </c>
+      <c r="AC35" s="11" t="n">
+        <v>370.3703703703704</v>
+      </c>
     </row>
     <row r="36">
       <c r="B36" s="8" t="inlineStr">
@@ -2722,6 +2924,9 @@
       <c r="Z36" s="9" t="n">
         <v>21.16402116402116</v>
       </c>
+      <c r="AA36" s="9" t="n"/>
+      <c r="AB36" s="9" t="n"/>
+      <c r="AC36" s="9" t="n"/>
     </row>
     <row r="37">
       <c r="B37" s="10" t="inlineStr">
@@ -2771,6 +2976,9 @@
       <c r="Z37" s="11" t="n">
         <v>1164021.164021164</v>
       </c>
+      <c r="AA37" s="11" t="n"/>
+      <c r="AB37" s="11" t="n"/>
+      <c r="AC37" s="11" t="n"/>
     </row>
     <row r="38">
       <c r="B38" s="12" t="inlineStr">
@@ -2849,6 +3057,15 @@
       </c>
       <c r="Z38" s="13" t="n">
         <v>1124651413.921005</v>
+      </c>
+      <c r="AA38" s="13" t="n">
+        <v>6925608467</v>
+      </c>
+      <c r="AB38" s="13" t="n">
+        <v>407388.7333529412</v>
+      </c>
+      <c r="AC38" s="13" t="n">
+        <v>36643431.04232804</v>
       </c>
     </row>
     <row r="39">
@@ -2881,6 +3098,9 @@
       <c r="X39" s="7" t="n"/>
       <c r="Y39" s="7" t="n"/>
       <c r="Z39" s="7" t="n"/>
+      <c r="AA39" s="7" t="n"/>
+      <c r="AB39" s="7" t="n"/>
+      <c r="AC39" s="7" t="n"/>
     </row>
     <row r="40">
       <c r="B40" s="14" t="inlineStr">
@@ -2912,6 +3132,9 @@
       <c r="X40" s="15" t="n"/>
       <c r="Y40" s="15" t="n"/>
       <c r="Z40" s="15" t="n"/>
+      <c r="AA40" s="15" t="n"/>
+      <c r="AB40" s="15" t="n"/>
+      <c r="AC40" s="15" t="n"/>
     </row>
     <row r="41">
       <c r="B41" s="8" t="inlineStr">
@@ -2990,6 +3213,15 @@
       </c>
       <c r="Z41" s="9" t="n">
         <v>-24809360.74074074</v>
+      </c>
+      <c r="AA41" s="9" t="n">
+        <v>-6825000</v>
+      </c>
+      <c r="AB41" s="9" t="n">
+        <v>-401.4705882352941</v>
+      </c>
+      <c r="AC41" s="9" t="n">
+        <v>-36111.11111111111</v>
       </c>
     </row>
     <row r="42">
@@ -3046,6 +3278,9 @@
       <c r="Z42" s="11" t="n">
         <v>-825541.3492063492</v>
       </c>
+      <c r="AA42" s="11" t="n"/>
+      <c r="AB42" s="11" t="n"/>
+      <c r="AC42" s="11" t="n"/>
     </row>
     <row r="43">
       <c r="B43" s="8" t="inlineStr">
@@ -3083,6 +3318,15 @@
       <c r="Z43" s="9" t="n">
         <v>-912399.4708994708</v>
       </c>
+      <c r="AA43" s="9" t="n">
+        <v>-172443500</v>
+      </c>
+      <c r="AB43" s="9" t="n">
+        <v>-10143.73529411765</v>
+      </c>
+      <c r="AC43" s="9" t="n">
+        <v>-912399.4708994708</v>
+      </c>
     </row>
     <row r="44">
       <c r="B44" s="10" t="inlineStr">
@@ -3150,6 +3394,15 @@
       <c r="Z44" s="11" t="n">
         <v>-6710414.91005291</v>
       </c>
+      <c r="AA44" s="11" t="n">
+        <v>-199480266</v>
+      </c>
+      <c r="AB44" s="11" t="n">
+        <v>-11734.13329411765</v>
+      </c>
+      <c r="AC44" s="11" t="n">
+        <v>-1055451.142857143</v>
+      </c>
     </row>
     <row r="45">
       <c r="B45" s="8" t="inlineStr">
@@ -3204,6 +3457,15 @@
       </c>
       <c r="Z45" s="9" t="n">
         <v>-714232.1428571428</v>
+      </c>
+      <c r="AA45" s="9" t="n">
+        <v>-51312525</v>
+      </c>
+      <c r="AB45" s="9" t="n">
+        <v>-3018.383823529412</v>
+      </c>
+      <c r="AC45" s="9" t="n">
+        <v>-271494.8412698412</v>
       </c>
     </row>
     <row r="46">
@@ -3242,6 +3504,15 @@
       <c r="Z46" s="11" t="n">
         <v>-155555.5555555556</v>
       </c>
+      <c r="AA46" s="11" t="n">
+        <v>-29400000</v>
+      </c>
+      <c r="AB46" s="11" t="n">
+        <v>-1729.411764705882</v>
+      </c>
+      <c r="AC46" s="11" t="n">
+        <v>-155555.5555555556</v>
+      </c>
     </row>
     <row r="47">
       <c r="B47" s="8" t="inlineStr">
@@ -3291,6 +3562,15 @@
       <c r="Z47" s="9" t="n">
         <v>-251738.3597883598</v>
       </c>
+      <c r="AA47" s="9" t="n">
+        <v>-12718550</v>
+      </c>
+      <c r="AB47" s="9" t="n">
+        <v>-748.15</v>
+      </c>
+      <c r="AC47" s="9" t="n">
+        <v>-67293.91534391535</v>
+      </c>
     </row>
     <row r="48">
       <c r="B48" s="10" t="inlineStr">
@@ -3358,6 +3638,15 @@
       <c r="Z48" s="11" t="n">
         <v>-5318351.925925925</v>
       </c>
+      <c r="AA48" s="11" t="n">
+        <v>-310783685</v>
+      </c>
+      <c r="AB48" s="11" t="n">
+        <v>-18281.39323529412</v>
+      </c>
+      <c r="AC48" s="11" t="n">
+        <v>-1644358.121693122</v>
+      </c>
     </row>
     <row r="49">
       <c r="B49" s="8" t="inlineStr">
@@ -3419,6 +3708,9 @@
       <c r="Z49" s="9" t="n">
         <v>-491122.1428571428</v>
       </c>
+      <c r="AA49" s="9" t="n"/>
+      <c r="AB49" s="9" t="n"/>
+      <c r="AC49" s="9" t="n"/>
     </row>
     <row r="50">
       <c r="B50" s="10" t="inlineStr">
@@ -3479,6 +3771,15 @@
       </c>
       <c r="Z50" s="11" t="n">
         <v>-7027734.788359787</v>
+      </c>
+      <c r="AA50" s="11" t="n">
+        <v>-41560938</v>
+      </c>
+      <c r="AB50" s="11" t="n">
+        <v>-2444.761058823529</v>
+      </c>
+      <c r="AC50" s="11" t="n">
+        <v>-219899.1428571429</v>
       </c>
     </row>
     <row r="51">
@@ -3529,6 +3830,9 @@
       <c r="Z51" s="9" t="n">
         <v>-10041970.37037037</v>
       </c>
+      <c r="AA51" s="9" t="n"/>
+      <c r="AB51" s="9" t="n"/>
+      <c r="AC51" s="9" t="n"/>
     </row>
     <row r="52">
       <c r="B52" s="10" t="inlineStr">
@@ -3607,6 +3911,15 @@
       </c>
       <c r="Z52" s="11" t="n">
         <v>-817459.4126984128</v>
+      </c>
+      <c r="AA52" s="11" t="n">
+        <v>-17235093</v>
+      </c>
+      <c r="AB52" s="11" t="n">
+        <v>-1013.829</v>
+      </c>
+      <c r="AC52" s="11" t="n">
+        <v>-91190.96825396825</v>
       </c>
     </row>
     <row r="53">
@@ -3645,6 +3958,15 @@
       <c r="Z53" s="9" t="n">
         <v>-163730.1587301587</v>
       </c>
+      <c r="AA53" s="9" t="n">
+        <v>-30945000</v>
+      </c>
+      <c r="AB53" s="9" t="n">
+        <v>-1820.294117647059</v>
+      </c>
+      <c r="AC53" s="9" t="n">
+        <v>-163730.1587301587</v>
+      </c>
     </row>
     <row r="54">
       <c r="B54" s="10" t="inlineStr">
@@ -3723,6 +4045,15 @@
       </c>
       <c r="Z54" s="11" t="n">
         <v>-7454951.062857143</v>
+      </c>
+      <c r="AA54" s="11" t="n">
+        <v>-22712050</v>
+      </c>
+      <c r="AB54" s="11" t="n">
+        <v>-1336.002941176471</v>
+      </c>
+      <c r="AC54" s="11" t="n">
+        <v>-120169.5767195767</v>
       </c>
     </row>
     <row r="55">
@@ -3773,6 +4104,9 @@
       <c r="Z55" s="9" t="n">
         <v>-9106933.333333334</v>
       </c>
+      <c r="AA55" s="9" t="n"/>
+      <c r="AB55" s="9" t="n"/>
+      <c r="AC55" s="9" t="n"/>
     </row>
     <row r="56">
       <c r="B56" s="10" t="inlineStr">
@@ -3810,6 +4144,15 @@
       <c r="Z56" s="11" t="n">
         <v>-10582.01058201058</v>
       </c>
+      <c r="AA56" s="11" t="n">
+        <v>-2000000</v>
+      </c>
+      <c r="AB56" s="11" t="n">
+        <v>-117.6470588235294</v>
+      </c>
+      <c r="AC56" s="11" t="n">
+        <v>-10582.01058201058</v>
+      </c>
     </row>
     <row r="57">
       <c r="B57" s="8" t="inlineStr">
@@ -3883,6 +4226,15 @@
       <c r="Z57" s="9" t="n">
         <v>-685185.1851851852</v>
       </c>
+      <c r="AA57" s="9" t="n">
+        <v>-18500000</v>
+      </c>
+      <c r="AB57" s="9" t="n">
+        <v>-1088.235294117647</v>
+      </c>
+      <c r="AC57" s="9" t="n">
+        <v>-97883.59788359789</v>
+      </c>
     </row>
     <row r="58">
       <c r="B58" s="12" t="inlineStr">
@@ -3961,6 +4313,15 @@
       </c>
       <c r="Z58" s="13" t="n">
         <v>-75497262.92</v>
+      </c>
+      <c r="AA58" s="13" t="n">
+        <v>-915916607</v>
+      </c>
+      <c r="AB58" s="13" t="n">
+        <v>-53877.44747058824</v>
+      </c>
+      <c r="AC58" s="13" t="n">
+        <v>-4846119.613756614</v>
       </c>
     </row>
     <row r="59">
@@ -3993,6 +4354,9 @@
       <c r="X59" s="15" t="n"/>
       <c r="Y59" s="15" t="n"/>
       <c r="Z59" s="15" t="n"/>
+      <c r="AA59" s="15" t="n"/>
+      <c r="AB59" s="15" t="n"/>
+      <c r="AC59" s="15" t="n"/>
     </row>
     <row r="60">
       <c r="B60" s="8" t="inlineStr">
@@ -4042,6 +4406,9 @@
       <c r="Z60" s="9" t="n">
         <v>-19170479.17460318</v>
       </c>
+      <c r="AA60" s="9" t="n"/>
+      <c r="AB60" s="9" t="n"/>
+      <c r="AC60" s="9" t="n"/>
     </row>
     <row r="61">
       <c r="B61" s="10" t="inlineStr">
@@ -4091,6 +4458,9 @@
       <c r="Z61" s="11" t="n">
         <v>-19170479.17460318</v>
       </c>
+      <c r="AA61" s="11" t="n"/>
+      <c r="AB61" s="11" t="n"/>
+      <c r="AC61" s="11" t="n"/>
     </row>
     <row r="62">
       <c r="B62" s="8" t="inlineStr">
@@ -4146,6 +4516,9 @@
       <c r="Z62" s="9" t="n">
         <v>-535387394.05291</v>
       </c>
+      <c r="AA62" s="9" t="n"/>
+      <c r="AB62" s="9" t="n"/>
+      <c r="AC62" s="9" t="n"/>
     </row>
     <row r="63">
       <c r="B63" s="10" t="inlineStr">
@@ -4201,6 +4574,9 @@
       <c r="Z63" s="11" t="n">
         <v>-535387394.05291</v>
       </c>
+      <c r="AA63" s="11" t="n"/>
+      <c r="AB63" s="11" t="n"/>
+      <c r="AC63" s="11" t="n"/>
     </row>
     <row r="64">
       <c r="B64" s="8" t="inlineStr">
@@ -4250,6 +4626,9 @@
       <c r="Z64" s="9" t="n">
         <v>-55908663.44444445</v>
       </c>
+      <c r="AA64" s="9" t="n"/>
+      <c r="AB64" s="9" t="n"/>
+      <c r="AC64" s="9" t="n"/>
     </row>
     <row r="65">
       <c r="B65" s="10" t="inlineStr">
@@ -4299,6 +4678,9 @@
       <c r="Z65" s="11" t="n">
         <v>-55908663.44444445</v>
       </c>
+      <c r="AA65" s="11" t="n"/>
+      <c r="AB65" s="11" t="n"/>
+      <c r="AC65" s="11" t="n"/>
     </row>
     <row r="66">
       <c r="B66" s="12" t="inlineStr">
@@ -4354,6 +4736,9 @@
       <c r="Z66" s="13" t="n">
         <v>-610466536.6719577</v>
       </c>
+      <c r="AA66" s="13" t="n"/>
+      <c r="AB66" s="13" t="n"/>
+      <c r="AC66" s="13" t="n"/>
     </row>
     <row r="67">
       <c r="B67" s="14" t="inlineStr">
@@ -4385,6 +4770,9 @@
       <c r="X67" s="15" t="n"/>
       <c r="Y67" s="15" t="n"/>
       <c r="Z67" s="15" t="n"/>
+      <c r="AA67" s="15" t="n"/>
+      <c r="AB67" s="15" t="n"/>
+      <c r="AC67" s="15" t="n"/>
     </row>
     <row r="68">
       <c r="B68" s="8" t="inlineStr">
@@ -4440,6 +4828,9 @@
       <c r="Z68" s="9" t="n">
         <v>-26681372.67724868</v>
       </c>
+      <c r="AA68" s="9" t="n"/>
+      <c r="AB68" s="9" t="n"/>
+      <c r="AC68" s="9" t="n"/>
     </row>
     <row r="69">
       <c r="B69" s="12" t="inlineStr">
@@ -4495,6 +4886,9 @@
       <c r="Z69" s="13" t="n">
         <v>-26681372.67724868</v>
       </c>
+      <c r="AA69" s="13" t="n"/>
+      <c r="AB69" s="13" t="n"/>
+      <c r="AC69" s="13" t="n"/>
     </row>
     <row r="70">
       <c r="B70" s="14" t="inlineStr">
@@ -4526,6 +4920,9 @@
       <c r="X70" s="15" t="n"/>
       <c r="Y70" s="15" t="n"/>
       <c r="Z70" s="15" t="n"/>
+      <c r="AA70" s="15" t="n"/>
+      <c r="AB70" s="15" t="n"/>
+      <c r="AC70" s="15" t="n"/>
     </row>
     <row r="71">
       <c r="B71" s="8" t="inlineStr">
@@ -4575,6 +4972,9 @@
       <c r="Z71" s="9" t="n">
         <v>-92285714.28571428</v>
       </c>
+      <c r="AA71" s="9" t="n"/>
+      <c r="AB71" s="9" t="n"/>
+      <c r="AC71" s="9" t="n"/>
     </row>
     <row r="72">
       <c r="B72" s="10" t="inlineStr">
@@ -4630,6 +5030,9 @@
       <c r="Z72" s="11" t="n">
         <v>-232804232.8042328</v>
       </c>
+      <c r="AA72" s="11" t="n"/>
+      <c r="AB72" s="11" t="n"/>
+      <c r="AC72" s="11" t="n"/>
     </row>
     <row r="73">
       <c r="B73" s="8" t="inlineStr">
@@ -4679,6 +5082,9 @@
       <c r="Z73" s="9" t="n">
         <v>-80729414.68253969</v>
       </c>
+      <c r="AA73" s="9" t="n"/>
+      <c r="AB73" s="9" t="n"/>
+      <c r="AC73" s="9" t="n"/>
     </row>
     <row r="74">
       <c r="B74" s="12" t="inlineStr">
@@ -4740,6 +5146,9 @@
       <c r="Z74" s="13" t="n">
         <v>-405819361.7724867</v>
       </c>
+      <c r="AA74" s="13" t="n"/>
+      <c r="AB74" s="13" t="n"/>
+      <c r="AC74" s="13" t="n"/>
     </row>
     <row r="75">
       <c r="B75" s="14" t="inlineStr">
@@ -4771,6 +5180,9 @@
       <c r="X75" s="15" t="n"/>
       <c r="Y75" s="15" t="n"/>
       <c r="Z75" s="15" t="n"/>
+      <c r="AA75" s="15" t="n"/>
+      <c r="AB75" s="15" t="n"/>
+      <c r="AC75" s="15" t="n"/>
     </row>
     <row r="76">
       <c r="B76" s="8" t="inlineStr">
@@ -4850,6 +5262,15 @@
       <c r="Z76" s="9" t="n">
         <v>-32174642.47619047</v>
       </c>
+      <c r="AA76" s="9" t="n">
+        <v>-581550572</v>
+      </c>
+      <c r="AB76" s="9" t="n">
+        <v>-34208.85717647058</v>
+      </c>
+      <c r="AC76" s="9" t="n">
+        <v>-3076987.153439153</v>
+      </c>
     </row>
     <row r="77">
       <c r="B77" s="10" t="inlineStr">
@@ -4929,6 +5350,15 @@
       <c r="Z77" s="11" t="n">
         <v>-37173938.39968254</v>
       </c>
+      <c r="AA77" s="11" t="n">
+        <v>-1326701477</v>
+      </c>
+      <c r="AB77" s="11" t="n">
+        <v>-78041.26335294118</v>
+      </c>
+      <c r="AC77" s="11" t="n">
+        <v>-7019584.534391535</v>
+      </c>
     </row>
     <row r="78">
       <c r="B78" s="8" t="inlineStr">
@@ -5008,6 +5438,15 @@
       <c r="Z78" s="9" t="n">
         <v>-33054126.4021164</v>
       </c>
+      <c r="AA78" s="9" t="n">
+        <v>-875805081</v>
+      </c>
+      <c r="AB78" s="9" t="n">
+        <v>-51517.94594117647</v>
+      </c>
+      <c r="AC78" s="9" t="n">
+        <v>-4633889.317460317</v>
+      </c>
     </row>
     <row r="79">
       <c r="B79" s="10" t="inlineStr">
@@ -5087,6 +5526,15 @@
       <c r="Z79" s="11" t="n">
         <v>-2047604.216931217</v>
       </c>
+      <c r="AA79" s="11" t="n">
+        <v>-8183769</v>
+      </c>
+      <c r="AB79" s="11" t="n">
+        <v>-481.3981764705882</v>
+      </c>
+      <c r="AC79" s="11" t="n">
+        <v>-43300.36507936508</v>
+      </c>
     </row>
     <row r="80">
       <c r="B80" s="12" t="inlineStr">
@@ -5165,6 +5613,15 @@
       </c>
       <c r="Z80" s="13" t="n">
         <v>-104450311.4949206</v>
+      </c>
+      <c r="AA80" s="13" t="n">
+        <v>-2792240899</v>
+      </c>
+      <c r="AB80" s="13" t="n">
+        <v>-164249.4646470588</v>
+      </c>
+      <c r="AC80" s="13" t="n">
+        <v>-14773761.37037037</v>
       </c>
     </row>
     <row r="81">
@@ -5197,6 +5654,9 @@
       <c r="X81" s="15" t="n"/>
       <c r="Y81" s="15" t="n"/>
       <c r="Z81" s="15" t="n"/>
+      <c r="AA81" s="15" t="n"/>
+      <c r="AB81" s="15" t="n"/>
+      <c r="AC81" s="15" t="n"/>
     </row>
     <row r="82">
       <c r="B82" s="14" t="inlineStr">
@@ -5228,6 +5688,9 @@
       <c r="X82" s="15" t="n"/>
       <c r="Y82" s="15" t="n"/>
       <c r="Z82" s="15" t="n"/>
+      <c r="AA82" s="15" t="n"/>
+      <c r="AB82" s="15" t="n"/>
+      <c r="AC82" s="15" t="n"/>
     </row>
     <row r="83">
       <c r="B83" s="8" t="inlineStr">
@@ -5306,6 +5769,15 @@
       </c>
       <c r="Z83" s="9" t="n">
         <v>-625686.925925926</v>
+      </c>
+      <c r="AA83" s="9" t="n">
+        <v>-16999662</v>
+      </c>
+      <c r="AB83" s="9" t="n">
+        <v>-999.9801176470588</v>
+      </c>
+      <c r="AC83" s="9" t="n">
+        <v>-89945.30158730158</v>
       </c>
     </row>
     <row r="84">
@@ -5344,6 +5816,15 @@
       <c r="Z84" s="11" t="n">
         <v>-13897.3544973545</v>
       </c>
+      <c r="AA84" s="11" t="n">
+        <v>-2626600</v>
+      </c>
+      <c r="AB84" s="11" t="n">
+        <v>-154.5058823529412</v>
+      </c>
+      <c r="AC84" s="11" t="n">
+        <v>-13897.3544973545</v>
+      </c>
     </row>
     <row r="85">
       <c r="B85" s="8" t="inlineStr">
@@ -5405,6 +5886,9 @@
       <c r="Z85" s="9" t="n">
         <v>-41493.14814814815</v>
       </c>
+      <c r="AA85" s="9" t="n"/>
+      <c r="AB85" s="9" t="n"/>
+      <c r="AC85" s="9" t="n"/>
     </row>
     <row r="86">
       <c r="B86" s="10" t="inlineStr">
@@ -5466,6 +5950,9 @@
       <c r="Z86" s="11" t="n">
         <v>-8627.340952380953</v>
       </c>
+      <c r="AA86" s="11" t="n"/>
+      <c r="AB86" s="11" t="n"/>
+      <c r="AC86" s="11" t="n"/>
     </row>
     <row r="87">
       <c r="B87" s="8" t="inlineStr">
@@ -5544,6 +6031,15 @@
       </c>
       <c r="Z87" s="9" t="n">
         <v>-516486.5661375662</v>
+      </c>
+      <c r="AA87" s="9" t="n">
+        <v>-20335475</v>
+      </c>
+      <c r="AB87" s="9" t="n">
+        <v>-1196.204411764706</v>
+      </c>
+      <c r="AC87" s="9" t="n">
+        <v>-107595.1058201058</v>
       </c>
     </row>
     <row r="88">
@@ -5612,6 +6108,15 @@
       <c r="Z88" s="11" t="n">
         <v>-8792.042328042327</v>
       </c>
+      <c r="AA88" s="11" t="n">
+        <v>-817499</v>
+      </c>
+      <c r="AB88" s="11" t="n">
+        <v>-48.08817647058824</v>
+      </c>
+      <c r="AC88" s="11" t="n">
+        <v>-4325.391534391534</v>
+      </c>
     </row>
     <row r="89">
       <c r="B89" s="12" t="inlineStr">
@@ -5690,6 +6195,15 @@
       </c>
       <c r="Z89" s="13" t="n">
         <v>-1214983.377989418</v>
+      </c>
+      <c r="AA89" s="13" t="n">
+        <v>-40779236</v>
+      </c>
+      <c r="AB89" s="13" t="n">
+        <v>-2398.778588235294</v>
+      </c>
+      <c r="AC89" s="13" t="n">
+        <v>-215763.1534391535</v>
       </c>
     </row>
     <row r="90">
@@ -5722,6 +6236,9 @@
       <c r="X90" s="15" t="n"/>
       <c r="Y90" s="15" t="n"/>
       <c r="Z90" s="15" t="n"/>
+      <c r="AA90" s="15" t="n"/>
+      <c r="AB90" s="15" t="n"/>
+      <c r="AC90" s="15" t="n"/>
     </row>
     <row r="91">
       <c r="B91" s="8" t="inlineStr">
@@ -5783,6 +6300,15 @@
       <c r="Z91" s="9" t="n">
         <v>-454201.0582010582</v>
       </c>
+      <c r="AA91" s="9" t="n">
+        <v>-1152000</v>
+      </c>
+      <c r="AB91" s="9" t="n">
+        <v>-67.76470588235294</v>
+      </c>
+      <c r="AC91" s="9" t="n">
+        <v>-6095.238095238095</v>
+      </c>
     </row>
     <row r="92">
       <c r="B92" s="10" t="inlineStr">
@@ -5862,6 +6388,15 @@
       <c r="Z92" s="11" t="n">
         <v>-983489</v>
       </c>
+      <c r="AA92" s="11" t="n">
+        <v>-10458793</v>
+      </c>
+      <c r="AB92" s="11" t="n">
+        <v>-615.2231176470589</v>
+      </c>
+      <c r="AC92" s="11" t="n">
+        <v>-55337.5291005291</v>
+      </c>
     </row>
     <row r="93">
       <c r="B93" s="8" t="inlineStr">
@@ -5941,6 +6476,15 @@
       <c r="Z93" s="9" t="n">
         <v>-34551432.01301587</v>
       </c>
+      <c r="AA93" s="9" t="n">
+        <v>-610316981</v>
+      </c>
+      <c r="AB93" s="9" t="n">
+        <v>-35900.99888235294</v>
+      </c>
+      <c r="AC93" s="9" t="n">
+        <v>-3229190.375661375</v>
+      </c>
     </row>
     <row r="94">
       <c r="B94" s="10" t="inlineStr">
@@ -6020,6 +6564,15 @@
       <c r="Z94" s="11" t="n">
         <v>-1024866.306878307</v>
       </c>
+      <c r="AA94" s="11" t="n">
+        <v>-30477712</v>
+      </c>
+      <c r="AB94" s="11" t="n">
+        <v>-1792.806588235294</v>
+      </c>
+      <c r="AC94" s="11" t="n">
+        <v>-161257.7354497355</v>
+      </c>
     </row>
     <row r="95">
       <c r="B95" s="8" t="inlineStr">
@@ -6099,6 +6652,15 @@
       <c r="Z95" s="9" t="n">
         <v>-1540756.518518518</v>
       </c>
+      <c r="AA95" s="9" t="n">
+        <v>-14997022</v>
+      </c>
+      <c r="AB95" s="9" t="n">
+        <v>-882.1777647058824</v>
+      </c>
+      <c r="AC95" s="9" t="n">
+        <v>-79349.32275132275</v>
+      </c>
     </row>
     <row r="96">
       <c r="B96" s="12" t="inlineStr">
@@ -6177,6 +6739,15 @@
       </c>
       <c r="Z96" s="13" t="n">
         <v>-38554744.89661375</v>
+      </c>
+      <c r="AA96" s="13" t="n">
+        <v>-667402508</v>
+      </c>
+      <c r="AB96" s="13" t="n">
+        <v>-39258.97105882353</v>
+      </c>
+      <c r="AC96" s="13" t="n">
+        <v>-3531230.201058201</v>
       </c>
     </row>
     <row r="97">
@@ -6209,6 +6780,9 @@
       <c r="X97" s="15" t="n"/>
       <c r="Y97" s="15" t="n"/>
       <c r="Z97" s="15" t="n"/>
+      <c r="AA97" s="15" t="n"/>
+      <c r="AB97" s="15" t="n"/>
+      <c r="AC97" s="15" t="n"/>
     </row>
     <row r="98">
       <c r="B98" s="8" t="inlineStr">
@@ -6288,6 +6862,15 @@
       <c r="Z98" s="9" t="n">
         <v>-968094.8518518518</v>
       </c>
+      <c r="AA98" s="9" t="n">
+        <v>-8741825</v>
+      </c>
+      <c r="AB98" s="9" t="n">
+        <v>-514.225</v>
+      </c>
+      <c r="AC98" s="9" t="n">
+        <v>-46253.04232804233</v>
+      </c>
     </row>
     <row r="99">
       <c r="B99" s="10" t="inlineStr">
@@ -6367,6 +6950,15 @@
       <c r="Z99" s="11" t="n">
         <v>-846811.0105820107</v>
       </c>
+      <c r="AA99" s="11" t="n">
+        <v>-31091154</v>
+      </c>
+      <c r="AB99" s="11" t="n">
+        <v>-1828.891411764706</v>
+      </c>
+      <c r="AC99" s="11" t="n">
+        <v>-164503.4603174603</v>
+      </c>
     </row>
     <row r="100">
       <c r="B100" s="8" t="inlineStr">
@@ -6445,6 +7037,15 @@
       </c>
       <c r="Z100" s="9" t="n">
         <v>-6305078.687830688</v>
+      </c>
+      <c r="AA100" s="9" t="n">
+        <v>-193998002</v>
+      </c>
+      <c r="AB100" s="9" t="n">
+        <v>-11411.64717647059</v>
+      </c>
+      <c r="AC100" s="9" t="n">
+        <v>-1026444.455026455</v>
       </c>
     </row>
     <row r="101">
@@ -6519,6 +7120,15 @@
       <c r="Z101" s="11" t="n">
         <v>-827321.6402116403</v>
       </c>
+      <c r="AA101" s="11" t="n">
+        <v>-43876240</v>
+      </c>
+      <c r="AB101" s="11" t="n">
+        <v>-2580.955294117647</v>
+      </c>
+      <c r="AC101" s="11" t="n">
+        <v>-232149.417989418</v>
+      </c>
     </row>
     <row r="102">
       <c r="B102" s="12" t="inlineStr">
@@ -6597,6 +7207,15 @@
       </c>
       <c r="Z102" s="13" t="n">
         <v>-8947306.19047619</v>
+      </c>
+      <c r="AA102" s="13" t="n">
+        <v>-277707221</v>
+      </c>
+      <c r="AB102" s="13" t="n">
+        <v>-16335.71888235294</v>
+      </c>
+      <c r="AC102" s="13" t="n">
+        <v>-1469350.375661376</v>
       </c>
     </row>
     <row r="103">
@@ -6629,6 +7248,9 @@
       <c r="X103" s="15" t="n"/>
       <c r="Y103" s="15" t="n"/>
       <c r="Z103" s="15" t="n"/>
+      <c r="AA103" s="15" t="n"/>
+      <c r="AB103" s="15" t="n"/>
+      <c r="AC103" s="15" t="n"/>
     </row>
     <row r="104">
       <c r="B104" s="8" t="inlineStr">
@@ -6701,6 +7323,15 @@
       </c>
       <c r="Z104" s="9" t="n">
         <v>-695585.1851851851</v>
+      </c>
+      <c r="AA104" s="9" t="n">
+        <v>-4030000</v>
+      </c>
+      <c r="AB104" s="9" t="n">
+        <v>-237.0588235294118</v>
+      </c>
+      <c r="AC104" s="9" t="n">
+        <v>-21322.75132275132</v>
       </c>
     </row>
     <row r="105">
@@ -6751,6 +7382,15 @@
       <c r="Z105" s="11" t="n">
         <v>-43589.94708994709</v>
       </c>
+      <c r="AA105" s="11" t="n">
+        <v>-5937500</v>
+      </c>
+      <c r="AB105" s="11" t="n">
+        <v>-349.2647058823529</v>
+      </c>
+      <c r="AC105" s="11" t="n">
+        <v>-31415.34391534391</v>
+      </c>
     </row>
     <row r="106">
       <c r="B106" s="8" t="inlineStr">
@@ -6830,6 +7470,15 @@
       <c r="Z106" s="9" t="n">
         <v>-1934127.571428571</v>
       </c>
+      <c r="AA106" s="9" t="n">
+        <v>-147572961</v>
+      </c>
+      <c r="AB106" s="9" t="n">
+        <v>-8680.762411764706</v>
+      </c>
+      <c r="AC106" s="9" t="n">
+        <v>-780809.3174603175</v>
+      </c>
     </row>
     <row r="107">
       <c r="B107" s="12" t="inlineStr">
@@ -6908,6 +7557,15 @@
       </c>
       <c r="Z107" s="13" t="n">
         <v>-2673302.703703704</v>
+      </c>
+      <c r="AA107" s="13" t="n">
+        <v>-157540461</v>
+      </c>
+      <c r="AB107" s="13" t="n">
+        <v>-9267.08594117647</v>
+      </c>
+      <c r="AC107" s="13" t="n">
+        <v>-833547.4126984127</v>
       </c>
     </row>
     <row r="108">
@@ -6940,6 +7598,9 @@
       <c r="X108" s="15" t="n"/>
       <c r="Y108" s="15" t="n"/>
       <c r="Z108" s="15" t="n"/>
+      <c r="AA108" s="15" t="n"/>
+      <c r="AB108" s="15" t="n"/>
+      <c r="AC108" s="15" t="n"/>
     </row>
     <row r="109">
       <c r="B109" s="8" t="inlineStr">
@@ -7012,6 +7673,15 @@
       </c>
       <c r="Z109" s="9" t="n">
         <v>-1865172.349206349</v>
+      </c>
+      <c r="AA109" s="9" t="n">
+        <v>-26160000</v>
+      </c>
+      <c r="AB109" s="9" t="n">
+        <v>-1538.823529411765</v>
+      </c>
+      <c r="AC109" s="9" t="n">
+        <v>-138412.6984126984</v>
       </c>
     </row>
     <row r="110">
@@ -7050,6 +7720,15 @@
       <c r="Z110" s="11" t="n">
         <v>-68783.06878306878</v>
       </c>
+      <c r="AA110" s="11" t="n">
+        <v>-13000000</v>
+      </c>
+      <c r="AB110" s="11" t="n">
+        <v>-764.7058823529412</v>
+      </c>
+      <c r="AC110" s="11" t="n">
+        <v>-68783.06878306878</v>
+      </c>
     </row>
     <row r="111">
       <c r="B111" s="8" t="inlineStr">
@@ -7129,6 +7808,15 @@
       <c r="Z111" s="9" t="n">
         <v>-652217.6349206349</v>
       </c>
+      <c r="AA111" s="9" t="n">
+        <v>-6603578</v>
+      </c>
+      <c r="AB111" s="9" t="n">
+        <v>-388.4457647058824</v>
+      </c>
+      <c r="AC111" s="9" t="n">
+        <v>-34939.56613756614</v>
+      </c>
     </row>
     <row r="112">
       <c r="B112" s="10" t="inlineStr">
@@ -7208,6 +7896,15 @@
       <c r="Z112" s="11" t="n">
         <v>-2187928.798941799</v>
       </c>
+      <c r="AA112" s="11" t="n">
+        <v>-164950749</v>
+      </c>
+      <c r="AB112" s="11" t="n">
+        <v>-9702.985235294118</v>
+      </c>
+      <c r="AC112" s="11" t="n">
+        <v>-872755.2857142857</v>
+      </c>
     </row>
     <row r="113">
       <c r="B113" s="12" t="inlineStr">
@@ -7286,6 +7983,15 @@
       </c>
       <c r="Z113" s="13" t="n">
         <v>-4774101.851851852</v>
+      </c>
+      <c r="AA113" s="13" t="n">
+        <v>-210714327</v>
+      </c>
+      <c r="AB113" s="13" t="n">
+        <v>-12394.9604117647</v>
+      </c>
+      <c r="AC113" s="13" t="n">
+        <v>-1114890.619047619</v>
       </c>
     </row>
     <row r="114">
@@ -7318,6 +8024,9 @@
       <c r="X114" s="15" t="n"/>
       <c r="Y114" s="15" t="n"/>
       <c r="Z114" s="15" t="n"/>
+      <c r="AA114" s="15" t="n"/>
+      <c r="AB114" s="15" t="n"/>
+      <c r="AC114" s="15" t="n"/>
     </row>
     <row r="115">
       <c r="B115" s="8" t="inlineStr">
@@ -7397,6 +8106,15 @@
       <c r="Z115" s="9" t="n">
         <v>-25635832.97354497</v>
       </c>
+      <c r="AA115" s="9" t="n">
+        <v>-735604373</v>
+      </c>
+      <c r="AB115" s="9" t="n">
+        <v>-43270.84547058823</v>
+      </c>
+      <c r="AC115" s="9" t="n">
+        <v>-3892086.62962963</v>
+      </c>
     </row>
     <row r="116">
       <c r="B116" s="12" t="inlineStr">
@@ -7475,6 +8193,15 @@
       </c>
       <c r="Z116" s="13" t="n">
         <v>-25635832.97354497</v>
+      </c>
+      <c r="AA116" s="13" t="n">
+        <v>-735604373</v>
+      </c>
+      <c r="AB116" s="13" t="n">
+        <v>-43270.84547058823</v>
+      </c>
+      <c r="AC116" s="13" t="n">
+        <v>-3892086.62962963</v>
       </c>
     </row>
     <row r="117">
@@ -7507,6 +8234,9 @@
       <c r="X117" s="15" t="n"/>
       <c r="Y117" s="15" t="n"/>
       <c r="Z117" s="15" t="n"/>
+      <c r="AA117" s="15" t="n"/>
+      <c r="AB117" s="15" t="n"/>
+      <c r="AC117" s="15" t="n"/>
     </row>
     <row r="118">
       <c r="B118" s="8" t="inlineStr">
@@ -7568,6 +8298,9 @@
       <c r="Z118" s="9" t="n">
         <v>-30477931.47089947</v>
       </c>
+      <c r="AA118" s="9" t="n"/>
+      <c r="AB118" s="9" t="n"/>
+      <c r="AC118" s="9" t="n"/>
     </row>
     <row r="119">
       <c r="B119" s="10" t="inlineStr">
@@ -7617,6 +8350,9 @@
       <c r="Z119" s="11" t="n">
         <v>-9685637.142857144</v>
       </c>
+      <c r="AA119" s="11" t="n"/>
+      <c r="AB119" s="11" t="n"/>
+      <c r="AC119" s="11" t="n"/>
     </row>
     <row r="120">
       <c r="B120" s="8" t="inlineStr">
@@ -7696,6 +8432,15 @@
       <c r="Z120" s="9" t="n">
         <v>-88965.50793650794</v>
       </c>
+      <c r="AA120" s="9" t="n">
+        <v>-1728000</v>
+      </c>
+      <c r="AB120" s="9" t="n">
+        <v>-101.6470588235294</v>
+      </c>
+      <c r="AC120" s="9" t="n">
+        <v>-9142.857142857143</v>
+      </c>
     </row>
     <row r="121">
       <c r="B121" s="10" t="inlineStr">
@@ -7774,6 +8519,15 @@
       </c>
       <c r="Z121" s="11" t="n">
         <v>-8232013.108306877</v>
+      </c>
+      <c r="AA121" s="11" t="n">
+        <v>-240870006</v>
+      </c>
+      <c r="AB121" s="11" t="n">
+        <v>-14168.82388235294</v>
+      </c>
+      <c r="AC121" s="11" t="n">
+        <v>-1274444.476190476</v>
       </c>
     </row>
     <row r="122">
@@ -7842,6 +8596,15 @@
       <c r="Z122" s="9" t="n">
         <v>-1586642.857142857</v>
       </c>
+      <c r="AA122" s="9" t="n">
+        <v>-119829000</v>
+      </c>
+      <c r="AB122" s="9" t="n">
+        <v>-7048.764705882353</v>
+      </c>
+      <c r="AC122" s="9" t="n">
+        <v>-634015.873015873</v>
+      </c>
     </row>
     <row r="123">
       <c r="B123" s="10" t="inlineStr">
@@ -7921,6 +8684,15 @@
       <c r="Z123" s="11" t="n">
         <v>-73717938.56084655</v>
       </c>
+      <c r="AA123" s="11" t="n">
+        <v>-775648144</v>
+      </c>
+      <c r="AB123" s="11" t="n">
+        <v>-45626.36141176471</v>
+      </c>
+      <c r="AC123" s="11" t="n">
+        <v>-4103958.433862434</v>
+      </c>
     </row>
     <row r="124">
       <c r="B124" s="12" t="inlineStr">
@@ -7999,6 +8771,15 @@
       </c>
       <c r="Z124" s="13" t="n">
         <v>-123789128.6479894</v>
+      </c>
+      <c r="AA124" s="13" t="n">
+        <v>-1138075150</v>
+      </c>
+      <c r="AB124" s="13" t="n">
+        <v>-66945.59705882354</v>
+      </c>
+      <c r="AC124" s="13" t="n">
+        <v>-6021561.64021164</v>
       </c>
     </row>
     <row r="125">
@@ -8031,6 +8812,9 @@
       <c r="X125" s="15" t="n"/>
       <c r="Y125" s="15" t="n"/>
       <c r="Z125" s="15" t="n"/>
+      <c r="AA125" s="15" t="n"/>
+      <c r="AB125" s="15" t="n"/>
+      <c r="AC125" s="15" t="n"/>
     </row>
     <row r="126">
       <c r="B126" s="8" t="inlineStr">
@@ -8098,6 +8882,15 @@
       <c r="Z126" s="9" t="n">
         <v>-141340.3174603175</v>
       </c>
+      <c r="AA126" s="9" t="n">
+        <v>-3740950</v>
+      </c>
+      <c r="AB126" s="9" t="n">
+        <v>-220.0558823529412</v>
+      </c>
+      <c r="AC126" s="9" t="n">
+        <v>-19793.38624338625</v>
+      </c>
     </row>
     <row r="127">
       <c r="B127" s="10" t="inlineStr">
@@ -8165,6 +8958,15 @@
       <c r="Z127" s="11" t="n">
         <v>-973744.2433862435</v>
       </c>
+      <c r="AA127" s="11" t="n">
+        <v>-60390459</v>
+      </c>
+      <c r="AB127" s="11" t="n">
+        <v>-3552.379941176471</v>
+      </c>
+      <c r="AC127" s="11" t="n">
+        <v>-319526.2380952381</v>
+      </c>
     </row>
     <row r="128">
       <c r="B128" s="8" t="inlineStr">
@@ -8244,6 +9046,9 @@
       <c r="Z128" s="9" t="n">
         <v>-1093348.444444444</v>
       </c>
+      <c r="AA128" s="9" t="n"/>
+      <c r="AB128" s="9" t="n"/>
+      <c r="AC128" s="9" t="n"/>
     </row>
     <row r="129">
       <c r="B129" s="10" t="inlineStr">
@@ -8323,6 +9128,15 @@
       <c r="Z129" s="11" t="n">
         <v>-488404.3809523809</v>
       </c>
+      <c r="AA129" s="11" t="n">
+        <v>-12025744</v>
+      </c>
+      <c r="AB129" s="11" t="n">
+        <v>-707.396705882353</v>
+      </c>
+      <c r="AC129" s="11" t="n">
+        <v>-63628.27513227514</v>
+      </c>
     </row>
     <row r="130">
       <c r="B130" s="8" t="inlineStr">
@@ -8401,6 +9215,15 @@
       </c>
       <c r="Z130" s="9" t="n">
         <v>-1057244.523809524</v>
+      </c>
+      <c r="AA130" s="9" t="n">
+        <v>-23394231</v>
+      </c>
+      <c r="AB130" s="9" t="n">
+        <v>-1376.131235294118</v>
+      </c>
+      <c r="AC130" s="9" t="n">
+        <v>-123779</v>
       </c>
     </row>
     <row r="131">
@@ -8451,6 +9274,9 @@
       <c r="Z131" s="11" t="n">
         <v>-5820.10582010582</v>
       </c>
+      <c r="AA131" s="11" t="n"/>
+      <c r="AB131" s="11" t="n"/>
+      <c r="AC131" s="11" t="n"/>
     </row>
     <row r="132">
       <c r="B132" s="12" t="inlineStr">
@@ -8530,6 +9356,15 @@
       <c r="Z132" s="13" t="n">
         <v>-3759902.015873016</v>
       </c>
+      <c r="AA132" s="13" t="n">
+        <v>-99551384</v>
+      </c>
+      <c r="AB132" s="13" t="n">
+        <v>-5855.963764705883</v>
+      </c>
+      <c r="AC132" s="13" t="n">
+        <v>-526726.8994708995</v>
+      </c>
     </row>
     <row r="133">
       <c r="B133" s="12" t="inlineStr">
@@ -8608,6 +9443,15 @@
       </c>
       <c r="Z133" s="13" t="n">
         <v>-209349302.6580423</v>
+      </c>
+      <c r="AA133" s="13" t="n">
+        <v>-3327374660</v>
+      </c>
+      <c r="AB133" s="13" t="n">
+        <v>-195727.9211764706</v>
+      </c>
+      <c r="AC133" s="13" t="n">
+        <v>-17605156.93121693</v>
       </c>
     </row>
     <row r="134">
@@ -8640,6 +9484,9 @@
       <c r="X134" s="15" t="n"/>
       <c r="Y134" s="15" t="n"/>
       <c r="Z134" s="15" t="n"/>
+      <c r="AA134" s="15" t="n"/>
+      <c r="AB134" s="15" t="n"/>
+      <c r="AC134" s="15" t="n"/>
     </row>
     <row r="135">
       <c r="B135" s="8" t="inlineStr">
@@ -8707,6 +9554,9 @@
       <c r="Z135" s="9" t="n">
         <v>-455026.455026455</v>
       </c>
+      <c r="AA135" s="9" t="n"/>
+      <c r="AB135" s="9" t="n"/>
+      <c r="AC135" s="9" t="n"/>
     </row>
     <row r="136">
       <c r="B136" s="10" t="inlineStr">
@@ -8744,6 +9594,15 @@
       <c r="Z136" s="11" t="n">
         <v>-26455.02645502645</v>
       </c>
+      <c r="AA136" s="11" t="n">
+        <v>-5000000</v>
+      </c>
+      <c r="AB136" s="11" t="n">
+        <v>-294.1176470588235</v>
+      </c>
+      <c r="AC136" s="11" t="n">
+        <v>-26455.02645502645</v>
+      </c>
     </row>
     <row r="137">
       <c r="B137" s="8" t="inlineStr">
@@ -8822,6 +9681,15 @@
       </c>
       <c r="Z137" s="9" t="n">
         <v>-3591381.243386243</v>
+      </c>
+      <c r="AA137" s="9" t="n">
+        <v>-92351360</v>
+      </c>
+      <c r="AB137" s="9" t="n">
+        <v>-5432.43294117647</v>
+      </c>
+      <c r="AC137" s="9" t="n">
+        <v>-488631.5343915344</v>
       </c>
     </row>
     <row r="138">
@@ -8872,6 +9740,9 @@
       <c r="Z138" s="11" t="n">
         <v>-8289354.497354497</v>
       </c>
+      <c r="AA138" s="11" t="n"/>
+      <c r="AB138" s="11" t="n"/>
+      <c r="AC138" s="11" t="n"/>
     </row>
     <row r="139">
       <c r="B139" s="8" t="inlineStr">
@@ -8921,6 +9792,9 @@
       <c r="Z139" s="9" t="n">
         <v>-44576.71957671957</v>
       </c>
+      <c r="AA139" s="9" t="n"/>
+      <c r="AB139" s="9" t="n"/>
+      <c r="AC139" s="9" t="n"/>
     </row>
     <row r="140">
       <c r="B140" s="12" t="inlineStr">
@@ -8999,6 +9873,15 @@
       </c>
       <c r="Z140" s="13" t="n">
         <v>-12406793.94179894</v>
+      </c>
+      <c r="AA140" s="13" t="n">
+        <v>-97351360</v>
+      </c>
+      <c r="AB140" s="13" t="n">
+        <v>-5726.550588235295</v>
+      </c>
+      <c r="AC140" s="13" t="n">
+        <v>-515086.5608465609</v>
       </c>
     </row>
     <row r="141">
@@ -9031,6 +9914,9 @@
       <c r="X141" s="15" t="n"/>
       <c r="Y141" s="15" t="n"/>
       <c r="Z141" s="15" t="n"/>
+      <c r="AA141" s="15" t="n"/>
+      <c r="AB141" s="15" t="n"/>
+      <c r="AC141" s="15" t="n"/>
     </row>
     <row r="142">
       <c r="B142" s="8" t="inlineStr">
@@ -9109,6 +9995,15 @@
       </c>
       <c r="Z142" s="9" t="n">
         <v>-86099.1094179894</v>
+      </c>
+      <c r="AA142" s="9" t="n">
+        <v>-2079254</v>
+      </c>
+      <c r="AB142" s="9" t="n">
+        <v>-122.3090588235294</v>
+      </c>
+      <c r="AC142" s="9" t="n">
+        <v>-11001.34391534392</v>
       </c>
     </row>
     <row r="143">
@@ -9165,6 +10060,9 @@
       <c r="Z143" s="11" t="n">
         <v>-275204.6190476191</v>
       </c>
+      <c r="AA143" s="11" t="n"/>
+      <c r="AB143" s="11" t="n"/>
+      <c r="AC143" s="11" t="n"/>
     </row>
     <row r="144">
       <c r="B144" s="8" t="inlineStr">
@@ -9232,6 +10130,9 @@
       <c r="Z144" s="9" t="n">
         <v>-49496.48227513227</v>
       </c>
+      <c r="AA144" s="9" t="n"/>
+      <c r="AB144" s="9" t="n"/>
+      <c r="AC144" s="9" t="n"/>
     </row>
     <row r="145">
       <c r="B145" s="10" t="inlineStr">
@@ -9310,6 +10211,15 @@
       </c>
       <c r="Z145" s="11" t="n">
         <v>-21540624.13</v>
+      </c>
+      <c r="AA145" s="11" t="n">
+        <v>-191562425</v>
+      </c>
+      <c r="AB145" s="11" t="n">
+        <v>-11268.37794117647</v>
+      </c>
+      <c r="AC145" s="11" t="n">
+        <v>-1013557.804232804</v>
       </c>
     </row>
     <row r="146">
@@ -9378,6 +10288,9 @@
       <c r="Z146" s="9" t="n">
         <v>-3400111.021164021</v>
       </c>
+      <c r="AA146" s="9" t="n"/>
+      <c r="AB146" s="9" t="n"/>
+      <c r="AC146" s="9" t="n"/>
     </row>
     <row r="147">
       <c r="B147" s="10" t="inlineStr">
@@ -9427,6 +10340,9 @@
       <c r="Z147" s="11" t="n">
         <v>-4094664.19047619</v>
       </c>
+      <c r="AA147" s="11" t="n"/>
+      <c r="AB147" s="11" t="n"/>
+      <c r="AC147" s="11" t="n"/>
     </row>
     <row r="148">
       <c r="B148" s="12" t="inlineStr">
@@ -9506,6 +10422,15 @@
       <c r="Z148" s="13" t="n">
         <v>-29446199.55238096</v>
       </c>
+      <c r="AA148" s="13" t="n">
+        <v>-193641679</v>
+      </c>
+      <c r="AB148" s="13" t="n">
+        <v>-11390.687</v>
+      </c>
+      <c r="AC148" s="13" t="n">
+        <v>-1024559.148148148</v>
+      </c>
     </row>
     <row r="149">
       <c r="B149" s="16" t="inlineStr">
@@ -9585,6 +10510,15 @@
       <c r="Z149" s="17" t="n">
         <v>-1474117141.688836</v>
       </c>
+      <c r="AA149" s="17" t="n">
+        <v>-7326525205</v>
+      </c>
+      <c r="AB149" s="17" t="n">
+        <v>-430972.0708823529</v>
+      </c>
+      <c r="AC149" s="17" t="n">
+        <v>-38764683.62433863</v>
+      </c>
     </row>
     <row r="150">
       <c r="B150" s="16" t="inlineStr">
@@ -9664,6 +10598,15 @@
       <c r="Z150" s="17" t="n">
         <v>-349465727.7678308</v>
       </c>
+      <c r="AA150" s="17" t="n">
+        <v>-400916738</v>
+      </c>
+      <c r="AB150" s="17" t="n">
+        <v>-23583.33752941176</v>
+      </c>
+      <c r="AC150" s="17" t="n">
+        <v>-2121252.582010582</v>
+      </c>
     </row>
     <row r="151">
       <c r="B151" s="14" t="inlineStr">
@@ -9743,6 +10686,15 @@
       <c r="Z151" s="15" t="n">
         <v>357003496.4357672</v>
       </c>
+      <c r="AA151" s="15" t="n">
+        <v>1825555016.239998</v>
+      </c>
+      <c r="AB151" s="15" t="n">
+        <v>107385.5891905881</v>
+      </c>
+      <c r="AC151" s="15" t="n">
+        <v>9659021.249947079</v>
+      </c>
     </row>
     <row r="152">
       <c r="B152" s="16" t="inlineStr">
@@ -9822,19 +10774,29 @@
       <c r="Z152" s="17" t="n">
         <v>7537768.667936456</v>
       </c>
+      <c r="AA152" s="17" t="n">
+        <v>1424638278.239998</v>
+      </c>
+      <c r="AB152" s="17" t="n">
+        <v>83802.25166117634</v>
+      </c>
+      <c r="AC152" s="17" t="n">
+        <v>7537768.667936496</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="11">
-    <mergeCell ref="B2:Z2"/>
+  <mergeCells count="12">
+    <mergeCell ref="B2:AC2"/>
     <mergeCell ref="R3:T3"/>
     <mergeCell ref="U3:W3"/>
     <mergeCell ref="B3:B4"/>
-    <mergeCell ref="B1:Z1"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="X3:Z3"/>
+    <mergeCell ref="B1:AC1"/>
     <mergeCell ref="I3:K3"/>
     <mergeCell ref="F3:H3"/>
     <mergeCell ref="L3:N3"/>
+    <mergeCell ref="AA3:AC3"/>
     <mergeCell ref="O3:Q3"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
@@ -9849,7 +10811,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:Z152"/>
+  <dimension ref="B1:AC152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -9878,6 +10840,9 @@
     <col width="16" customWidth="1" min="24" max="24"/>
     <col width="16" customWidth="1" min="25" max="25"/>
     <col width="16" customWidth="1" min="26" max="26"/>
+    <col width="16" customWidth="1" min="27" max="27"/>
+    <col width="16" customWidth="1" min="28" max="28"/>
+    <col width="16" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -9890,7 +10855,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 28 Jul 2026 16:28 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 28 Jul 2026 16:35 (in IDR Million)</t>
         </is>
       </c>
     </row>
@@ -9956,6 +10921,13 @@
       </c>
       <c r="Y3" s="4" t="n"/>
       <c r="Z3" s="4" t="n"/>
+      <c r="AA3" s="3" t="inlineStr">
+        <is>
+          <t>MTD as of 28 Jul 2026</t>
+        </is>
+      </c>
+      <c r="AB3" s="4" t="n"/>
+      <c r="AC3" s="4" t="n"/>
     </row>
     <row r="4" ht="18" customHeight="1">
       <c r="B4" s="5" t="n"/>
@@ -10075,6 +11047,21 @@
         </is>
       </c>
       <c r="Z4" s="3" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="AA4" s="3" t="inlineStr">
+        <is>
+          <t>IDR</t>
+        </is>
+      </c>
+      <c r="AB4" s="3" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="AC4" s="3" t="inlineStr">
         <is>
           <t>INR</t>
         </is>
@@ -10110,6 +11097,9 @@
       <c r="X5" s="7" t="n"/>
       <c r="Y5" s="7" t="n"/>
       <c r="Z5" s="7" t="n"/>
+      <c r="AA5" s="7" t="n"/>
+      <c r="AB5" s="7" t="n"/>
+      <c r="AC5" s="7" t="n"/>
     </row>
     <row r="6">
       <c r="B6" s="8" t="inlineStr">
@@ -10188,6 +11178,15 @@
       </c>
       <c r="Z6" s="9" t="n">
         <v>859.0036798253968</v>
+      </c>
+      <c r="AA6" s="9" t="n">
+        <v>6895.316417</v>
+      </c>
+      <c r="AB6" s="9" t="n">
+        <v>0.4056068480588235</v>
+      </c>
+      <c r="AC6" s="9" t="n">
+        <v>36.48315564550265</v>
       </c>
     </row>
     <row r="7">
@@ -10250,6 +11249,15 @@
       <c r="Z7" s="11" t="n">
         <v>483.9470734338624</v>
       </c>
+      <c r="AA7" s="11" t="n">
+        <v>19.305092</v>
+      </c>
+      <c r="AB7" s="11" t="n">
+        <v>0.001135593647058823</v>
+      </c>
+      <c r="AC7" s="11" t="n">
+        <v>0.1021433439153439</v>
+      </c>
     </row>
     <row r="8">
       <c r="B8" s="8" t="inlineStr">
@@ -10328,6 +11336,15 @@
       </c>
       <c r="Z8" s="9" t="n">
         <v>173.6711985132275</v>
+      </c>
+      <c r="AA8" s="9" t="n">
+        <v>3590.241514</v>
+      </c>
+      <c r="AB8" s="9" t="n">
+        <v>0.2111906772941176</v>
+      </c>
+      <c r="AC8" s="9" t="n">
+        <v>18.99598684656085</v>
       </c>
     </row>
     <row r="9">
@@ -10402,6 +11419,15 @@
       <c r="Z9" s="11" t="n">
         <v>154.834760984127</v>
       </c>
+      <c r="AA9" s="11" t="n">
+        <v>2297.841064</v>
+      </c>
+      <c r="AB9" s="11" t="n">
+        <v>0.1351671214117647</v>
+      </c>
+      <c r="AC9" s="11" t="n">
+        <v>12.15788922751323</v>
+      </c>
     </row>
     <row r="10">
       <c r="B10" s="8" t="inlineStr">
@@ -10475,6 +11501,15 @@
       <c r="Z10" s="9" t="n">
         <v>38.02955694708995</v>
       </c>
+      <c r="AA10" s="9" t="n">
+        <v>575.848747</v>
+      </c>
+      <c r="AB10" s="9" t="n">
+        <v>0.03387345570588236</v>
+      </c>
+      <c r="AC10" s="9" t="n">
+        <v>3.046818767195767</v>
+      </c>
     </row>
     <row r="11">
       <c r="B11" s="10" t="inlineStr">
@@ -10541,6 +11576,15 @@
       </c>
       <c r="Z11" s="11" t="n">
         <v>7.631111111111111</v>
+      </c>
+      <c r="AA11" s="11" t="n">
+        <v>412.08</v>
+      </c>
+      <c r="AB11" s="11" t="n">
+        <v>0.02424</v>
+      </c>
+      <c r="AC11" s="11" t="n">
+        <v>2.18031746031746</v>
       </c>
     </row>
     <row r="12">
@@ -10591,6 +11635,9 @@
       <c r="Z12" s="9" t="n">
         <v>0.7408359788359788</v>
       </c>
+      <c r="AA12" s="9" t="n"/>
+      <c r="AB12" s="9" t="n"/>
+      <c r="AC12" s="9" t="n"/>
     </row>
     <row r="13">
       <c r="B13" s="10" t="inlineStr">
@@ -10640,6 +11687,9 @@
       <c r="Z13" s="11" t="n">
         <v>0.1491428571428571</v>
       </c>
+      <c r="AA13" s="11" t="n"/>
+      <c r="AB13" s="11" t="n"/>
+      <c r="AC13" s="11" t="n"/>
     </row>
     <row r="14">
       <c r="B14" s="8" t="inlineStr">
@@ -10689,6 +11739,9 @@
       <c r="Z14" s="9" t="n">
         <v>262.4126984126984</v>
       </c>
+      <c r="AA14" s="9" t="n"/>
+      <c r="AB14" s="9" t="n"/>
+      <c r="AC14" s="9" t="n"/>
     </row>
     <row r="15">
       <c r="B15" s="10" t="inlineStr">
@@ -10738,6 +11791,9 @@
       <c r="Z15" s="11" t="n">
         <v>262.4126984126984</v>
       </c>
+      <c r="AA15" s="11" t="n"/>
+      <c r="AB15" s="11" t="n"/>
+      <c r="AC15" s="11" t="n"/>
     </row>
     <row r="16">
       <c r="B16" s="8" t="inlineStr">
@@ -10817,6 +11873,15 @@
       <c r="Z16" s="9" t="n">
         <v>2.071014518888889</v>
       </c>
+      <c r="AA16" s="9" t="n">
+        <v>30.29205</v>
+      </c>
+      <c r="AB16" s="9" t="n">
+        <v>0.001781885294117647</v>
+      </c>
+      <c r="AC16" s="9" t="n">
+        <v>0.1602753968253968</v>
+      </c>
     </row>
     <row r="17">
       <c r="B17" s="10" t="inlineStr">
@@ -10896,6 +11961,9 @@
       <c r="Z17" s="11" t="n">
         <v>0.6718186214814815</v>
       </c>
+      <c r="AA17" s="11" t="n"/>
+      <c r="AB17" s="11" t="n"/>
+      <c r="AC17" s="11" t="n"/>
     </row>
     <row r="18">
       <c r="B18" s="8" t="inlineStr">
@@ -10945,6 +12013,9 @@
       <c r="Z18" s="9" t="n">
         <v>0.6579851851851852</v>
       </c>
+      <c r="AA18" s="9" t="n"/>
+      <c r="AB18" s="9" t="n"/>
+      <c r="AC18" s="9" t="n"/>
     </row>
     <row r="19">
       <c r="B19" s="10" t="inlineStr">
@@ -10994,6 +12065,9 @@
       <c r="Z19" s="11" t="n">
         <v>0.1231216931216931</v>
       </c>
+      <c r="AA19" s="11" t="n"/>
+      <c r="AB19" s="11" t="n"/>
+      <c r="AC19" s="11" t="n"/>
     </row>
     <row r="20">
       <c r="B20" s="8" t="inlineStr">
@@ -11060,6 +12134,15 @@
       </c>
       <c r="Z20" s="9" t="n">
         <v>0.1189417989417989</v>
+      </c>
+      <c r="AA20" s="9" t="n">
+        <v>4.0145</v>
+      </c>
+      <c r="AB20" s="9" t="n">
+        <v>0.0002361470588235294</v>
+      </c>
+      <c r="AC20" s="9" t="n">
+        <v>0.02124074074074074</v>
       </c>
     </row>
     <row r="21">
@@ -11116,6 +12199,9 @@
       <c r="Z21" s="11" t="n">
         <v>0.1069050264550264</v>
       </c>
+      <c r="AA21" s="11" t="n"/>
+      <c r="AB21" s="11" t="n"/>
+      <c r="AC21" s="11" t="n"/>
     </row>
     <row r="22">
       <c r="B22" s="8" t="inlineStr">
@@ -11153,6 +12239,15 @@
       <c r="Z22" s="9" t="n">
         <v>0.09452380952380951</v>
       </c>
+      <c r="AA22" s="9" t="n">
+        <v>17.865</v>
+      </c>
+      <c r="AB22" s="9" t="n">
+        <v>0.001050882352941176</v>
+      </c>
+      <c r="AC22" s="9" t="n">
+        <v>0.09452380952380951</v>
+      </c>
     </row>
     <row r="23">
       <c r="B23" s="10" t="inlineStr">
@@ -11202,6 +12297,9 @@
       <c r="Z23" s="11" t="n">
         <v>0.07447301587301587</v>
       </c>
+      <c r="AA23" s="11" t="n"/>
+      <c r="AB23" s="11" t="n"/>
+      <c r="AC23" s="11" t="n"/>
     </row>
     <row r="24">
       <c r="B24" s="8" t="inlineStr">
@@ -11268,6 +12366,15 @@
       </c>
       <c r="Z24" s="9" t="n">
         <v>0.0627427619047619</v>
+      </c>
+      <c r="AA24" s="9" t="n">
+        <v>4.037</v>
+      </c>
+      <c r="AB24" s="9" t="n">
+        <v>0.0002374705882352941</v>
+      </c>
+      <c r="AC24" s="9" t="n">
+        <v>0.02135978835978836</v>
       </c>
     </row>
     <row r="25">
@@ -11318,6 +12425,9 @@
       <c r="Z25" s="11" t="n">
         <v>0.03976575132275132</v>
       </c>
+      <c r="AA25" s="11" t="n"/>
+      <c r="AB25" s="11" t="n"/>
+      <c r="AC25" s="11" t="n"/>
     </row>
     <row r="26">
       <c r="B26" s="8" t="inlineStr">
@@ -11373,6 +12483,9 @@
       <c r="Z26" s="9" t="n">
         <v>0.03174603174603174</v>
       </c>
+      <c r="AA26" s="9" t="n"/>
+      <c r="AB26" s="9" t="n"/>
+      <c r="AC26" s="9" t="n"/>
     </row>
     <row r="27">
       <c r="B27" s="10" t="inlineStr">
@@ -11427,6 +12540,15 @@
       </c>
       <c r="Z27" s="11" t="n">
         <v>0.02372502645502645</v>
+      </c>
+      <c r="AA27" s="11" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="AB27" s="11" t="n">
+        <v>2.058823529411765e-05</v>
+      </c>
+      <c r="AC27" s="11" t="n">
+        <v>0.001851851851851852</v>
       </c>
     </row>
     <row r="28">
@@ -11477,6 +12599,9 @@
       <c r="Z28" s="9" t="n">
         <v>0.02022776719576719</v>
       </c>
+      <c r="AA28" s="9" t="n"/>
+      <c r="AB28" s="9" t="n"/>
+      <c r="AC28" s="9" t="n"/>
     </row>
     <row r="29">
       <c r="B29" s="10" t="inlineStr">
@@ -11526,6 +12651,15 @@
       <c r="Z29" s="11" t="n">
         <v>0.01428809523809524</v>
       </c>
+      <c r="AA29" s="11" t="n">
+        <v>2.59525</v>
+      </c>
+      <c r="AB29" s="11" t="n">
+        <v>0.0001526617647058824</v>
+      </c>
+      <c r="AC29" s="11" t="n">
+        <v>0.01373148148148148</v>
+      </c>
     </row>
     <row r="30">
       <c r="B30" s="8" t="inlineStr">
@@ -11587,6 +12721,9 @@
       <c r="Z30" s="9" t="n">
         <v>0.009278511164021164</v>
       </c>
+      <c r="AA30" s="9" t="n"/>
+      <c r="AB30" s="9" t="n"/>
+      <c r="AC30" s="9" t="n"/>
     </row>
     <row r="31">
       <c r="B31" s="10" t="inlineStr">
@@ -11636,6 +12773,15 @@
       <c r="Z31" s="11" t="n">
         <v>0.008699957671957671</v>
       </c>
+      <c r="AA31" s="11" t="n">
+        <v>1.3603</v>
+      </c>
+      <c r="AB31" s="11" t="n">
+        <v>8.001764705882353e-05</v>
+      </c>
+      <c r="AC31" s="11" t="n">
+        <v>0.007197354497354497</v>
+      </c>
     </row>
     <row r="32">
       <c r="B32" s="8" t="inlineStr">
@@ -11685,6 +12831,9 @@
       <c r="Z32" s="9" t="n">
         <v>0.005291005291005291</v>
       </c>
+      <c r="AA32" s="9" t="n"/>
+      <c r="AB32" s="9" t="n"/>
+      <c r="AC32" s="9" t="n"/>
     </row>
     <row r="33">
       <c r="B33" s="10" t="inlineStr">
@@ -11746,6 +12895,9 @@
       <c r="Z33" s="11" t="n">
         <v>0.003911111111111111</v>
       </c>
+      <c r="AA33" s="11" t="n"/>
+      <c r="AB33" s="11" t="n"/>
+      <c r="AC33" s="11" t="n"/>
     </row>
     <row r="34">
       <c r="B34" s="8" t="inlineStr">
@@ -11801,6 +12953,9 @@
       <c r="Z34" s="9" t="n">
         <v>0.002648703703703704</v>
       </c>
+      <c r="AA34" s="9" t="n"/>
+      <c r="AB34" s="9" t="n"/>
+      <c r="AC34" s="9" t="n"/>
     </row>
     <row r="35">
       <c r="B35" s="10" t="inlineStr">
@@ -11850,6 +13005,15 @@
       <c r="Z35" s="11" t="n">
         <v>0.0008994814814814815</v>
       </c>
+      <c r="AA35" s="11" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="AB35" s="11" t="n">
+        <v>4.11764705882353e-06</v>
+      </c>
+      <c r="AC35" s="11" t="n">
+        <v>0.0003703703703703704</v>
+      </c>
     </row>
     <row r="36">
       <c r="B36" s="8" t="inlineStr">
@@ -11899,6 +13063,9 @@
       <c r="Z36" s="9" t="n">
         <v>2.116402116402116e-05</v>
       </c>
+      <c r="AA36" s="9" t="n"/>
+      <c r="AB36" s="9" t="n"/>
+      <c r="AC36" s="9" t="n"/>
     </row>
     <row r="37">
       <c r="B37" s="10" t="inlineStr">
@@ -11948,6 +13115,9 @@
       <c r="Z37" s="11" t="n">
         <v>1.164021164021164</v>
       </c>
+      <c r="AA37" s="11" t="n"/>
+      <c r="AB37" s="11" t="n"/>
+      <c r="AC37" s="11" t="n"/>
     </row>
     <row r="38">
       <c r="B38" s="12" t="inlineStr">
@@ -12026,6 +13196,15 @@
       </c>
       <c r="Z38" s="13" t="n">
         <v>1124.651413921005</v>
+      </c>
+      <c r="AA38" s="13" t="n">
+        <v>6925.608467</v>
+      </c>
+      <c r="AB38" s="13" t="n">
+        <v>0.4073887333529412</v>
+      </c>
+      <c r="AC38" s="13" t="n">
+        <v>36.64343104232804</v>
       </c>
     </row>
     <row r="39">
@@ -12058,6 +13237,9 @@
       <c r="X39" s="7" t="n"/>
       <c r="Y39" s="7" t="n"/>
       <c r="Z39" s="7" t="n"/>
+      <c r="AA39" s="7" t="n"/>
+      <c r="AB39" s="7" t="n"/>
+      <c r="AC39" s="7" t="n"/>
     </row>
     <row r="40">
       <c r="B40" s="14" t="inlineStr">
@@ -12089,6 +13271,9 @@
       <c r="X40" s="15" t="n"/>
       <c r="Y40" s="15" t="n"/>
       <c r="Z40" s="15" t="n"/>
+      <c r="AA40" s="15" t="n"/>
+      <c r="AB40" s="15" t="n"/>
+      <c r="AC40" s="15" t="n"/>
     </row>
     <row r="41">
       <c r="B41" s="8" t="inlineStr">
@@ -12167,6 +13352,15 @@
       </c>
       <c r="Z41" s="9" t="n">
         <v>-24.80936074074075</v>
+      </c>
+      <c r="AA41" s="9" t="n">
+        <v>-6.825</v>
+      </c>
+      <c r="AB41" s="9" t="n">
+        <v>-0.0004014705882352942</v>
+      </c>
+      <c r="AC41" s="9" t="n">
+        <v>-0.03611111111111111</v>
       </c>
     </row>
     <row r="42">
@@ -12223,6 +13417,9 @@
       <c r="Z42" s="11" t="n">
         <v>-0.8255413492063493</v>
       </c>
+      <c r="AA42" s="11" t="n"/>
+      <c r="AB42" s="11" t="n"/>
+      <c r="AC42" s="11" t="n"/>
     </row>
     <row r="43">
       <c r="B43" s="8" t="inlineStr">
@@ -12260,6 +13457,15 @@
       <c r="Z43" s="9" t="n">
         <v>-0.9123994708994709</v>
       </c>
+      <c r="AA43" s="9" t="n">
+        <v>-172.4435</v>
+      </c>
+      <c r="AB43" s="9" t="n">
+        <v>-0.01014373529411765</v>
+      </c>
+      <c r="AC43" s="9" t="n">
+        <v>-0.9123994708994709</v>
+      </c>
     </row>
     <row r="44">
       <c r="B44" s="10" t="inlineStr">
@@ -12327,6 +13533,15 @@
       <c r="Z44" s="11" t="n">
         <v>-6.71041491005291</v>
       </c>
+      <c r="AA44" s="11" t="n">
+        <v>-199.480266</v>
+      </c>
+      <c r="AB44" s="11" t="n">
+        <v>-0.01173413329411765</v>
+      </c>
+      <c r="AC44" s="11" t="n">
+        <v>-1.055451142857143</v>
+      </c>
     </row>
     <row r="45">
       <c r="B45" s="8" t="inlineStr">
@@ -12381,6 +13596,15 @@
       </c>
       <c r="Z45" s="9" t="n">
         <v>-0.7142321428571428</v>
+      </c>
+      <c r="AA45" s="9" t="n">
+        <v>-51.312525</v>
+      </c>
+      <c r="AB45" s="9" t="n">
+        <v>-0.003018383823529412</v>
+      </c>
+      <c r="AC45" s="9" t="n">
+        <v>-0.2714948412698412</v>
       </c>
     </row>
     <row r="46">
@@ -12419,6 +13643,15 @@
       <c r="Z46" s="11" t="n">
         <v>-0.1555555555555556</v>
       </c>
+      <c r="AA46" s="11" t="n">
+        <v>-29.4</v>
+      </c>
+      <c r="AB46" s="11" t="n">
+        <v>-0.001729411764705882</v>
+      </c>
+      <c r="AC46" s="11" t="n">
+        <v>-0.1555555555555556</v>
+      </c>
     </row>
     <row r="47">
       <c r="B47" s="8" t="inlineStr">
@@ -12468,6 +13701,15 @@
       <c r="Z47" s="9" t="n">
         <v>-0.2517383597883598</v>
       </c>
+      <c r="AA47" s="9" t="n">
+        <v>-12.71855</v>
+      </c>
+      <c r="AB47" s="9" t="n">
+        <v>-0.0007481500000000001</v>
+      </c>
+      <c r="AC47" s="9" t="n">
+        <v>-0.06729391534391535</v>
+      </c>
     </row>
     <row r="48">
       <c r="B48" s="10" t="inlineStr">
@@ -12535,6 +13777,15 @@
       <c r="Z48" s="11" t="n">
         <v>-5.318351925925926</v>
       </c>
+      <c r="AA48" s="11" t="n">
+        <v>-310.783685</v>
+      </c>
+      <c r="AB48" s="11" t="n">
+        <v>-0.01828139323529412</v>
+      </c>
+      <c r="AC48" s="11" t="n">
+        <v>-1.644358121693122</v>
+      </c>
     </row>
     <row r="49">
       <c r="B49" s="8" t="inlineStr">
@@ -12596,6 +13847,9 @@
       <c r="Z49" s="9" t="n">
         <v>-0.4911221428571428</v>
       </c>
+      <c r="AA49" s="9" t="n"/>
+      <c r="AB49" s="9" t="n"/>
+      <c r="AC49" s="9" t="n"/>
     </row>
     <row r="50">
       <c r="B50" s="10" t="inlineStr">
@@ -12656,6 +13910,15 @@
       </c>
       <c r="Z50" s="11" t="n">
         <v>-7.027734788359788</v>
+      </c>
+      <c r="AA50" s="11" t="n">
+        <v>-41.560938</v>
+      </c>
+      <c r="AB50" s="11" t="n">
+        <v>-0.00244476105882353</v>
+      </c>
+      <c r="AC50" s="11" t="n">
+        <v>-0.2198991428571428</v>
       </c>
     </row>
     <row r="51">
@@ -12706,6 +13969,9 @@
       <c r="Z51" s="9" t="n">
         <v>-10.04197037037037</v>
       </c>
+      <c r="AA51" s="9" t="n"/>
+      <c r="AB51" s="9" t="n"/>
+      <c r="AC51" s="9" t="n"/>
     </row>
     <row r="52">
       <c r="B52" s="10" t="inlineStr">
@@ -12784,6 +14050,15 @@
       </c>
       <c r="Z52" s="11" t="n">
         <v>-0.8174594126984126</v>
+      </c>
+      <c r="AA52" s="11" t="n">
+        <v>-17.235093</v>
+      </c>
+      <c r="AB52" s="11" t="n">
+        <v>-0.001013829</v>
+      </c>
+      <c r="AC52" s="11" t="n">
+        <v>-0.09119096825396825</v>
       </c>
     </row>
     <row r="53">
@@ -12822,6 +14097,15 @@
       <c r="Z53" s="9" t="n">
         <v>-0.1637301587301587</v>
       </c>
+      <c r="AA53" s="9" t="n">
+        <v>-30.945</v>
+      </c>
+      <c r="AB53" s="9" t="n">
+        <v>-0.001820294117647059</v>
+      </c>
+      <c r="AC53" s="9" t="n">
+        <v>-0.1637301587301587</v>
+      </c>
     </row>
     <row r="54">
       <c r="B54" s="10" t="inlineStr">
@@ -12900,6 +14184,15 @@
       </c>
       <c r="Z54" s="11" t="n">
         <v>-7.454951062857143</v>
+      </c>
+      <c r="AA54" s="11" t="n">
+        <v>-22.71205</v>
+      </c>
+      <c r="AB54" s="11" t="n">
+        <v>-0.001336002941176471</v>
+      </c>
+      <c r="AC54" s="11" t="n">
+        <v>-0.1201695767195767</v>
       </c>
     </row>
     <row r="55">
@@ -12950,6 +14243,9 @@
       <c r="Z55" s="9" t="n">
         <v>-9.106933333333332</v>
       </c>
+      <c r="AA55" s="9" t="n"/>
+      <c r="AB55" s="9" t="n"/>
+      <c r="AC55" s="9" t="n"/>
     </row>
     <row r="56">
       <c r="B56" s="10" t="inlineStr">
@@ -12987,6 +14283,15 @@
       <c r="Z56" s="11" t="n">
         <v>-0.01058201058201058</v>
       </c>
+      <c r="AA56" s="11" t="n">
+        <v>-2</v>
+      </c>
+      <c r="AB56" s="11" t="n">
+        <v>-0.0001176470588235294</v>
+      </c>
+      <c r="AC56" s="11" t="n">
+        <v>-0.01058201058201058</v>
+      </c>
     </row>
     <row r="57">
       <c r="B57" s="8" t="inlineStr">
@@ -13060,6 +14365,15 @@
       <c r="Z57" s="9" t="n">
         <v>-0.6851851851851851</v>
       </c>
+      <c r="AA57" s="9" t="n">
+        <v>-18.5</v>
+      </c>
+      <c r="AB57" s="9" t="n">
+        <v>-0.001088235294117647</v>
+      </c>
+      <c r="AC57" s="9" t="n">
+        <v>-0.09788359788359788</v>
+      </c>
     </row>
     <row r="58">
       <c r="B58" s="12" t="inlineStr">
@@ -13138,6 +14452,15 @@
       </c>
       <c r="Z58" s="13" t="n">
         <v>-75.49726292</v>
+      </c>
+      <c r="AA58" s="13" t="n">
+        <v>-915.916607</v>
+      </c>
+      <c r="AB58" s="13" t="n">
+        <v>-0.05387744747058824</v>
+      </c>
+      <c r="AC58" s="13" t="n">
+        <v>-4.846119613756613</v>
       </c>
     </row>
     <row r="59">
@@ -13170,6 +14493,9 @@
       <c r="X59" s="15" t="n"/>
       <c r="Y59" s="15" t="n"/>
       <c r="Z59" s="15" t="n"/>
+      <c r="AA59" s="15" t="n"/>
+      <c r="AB59" s="15" t="n"/>
+      <c r="AC59" s="15" t="n"/>
     </row>
     <row r="60">
       <c r="B60" s="8" t="inlineStr">
@@ -13219,6 +14545,9 @@
       <c r="Z60" s="9" t="n">
         <v>-19.17047917460318</v>
       </c>
+      <c r="AA60" s="9" t="n"/>
+      <c r="AB60" s="9" t="n"/>
+      <c r="AC60" s="9" t="n"/>
     </row>
     <row r="61">
       <c r="B61" s="10" t="inlineStr">
@@ -13268,6 +14597,9 @@
       <c r="Z61" s="11" t="n">
         <v>-19.17047917460318</v>
       </c>
+      <c r="AA61" s="11" t="n"/>
+      <c r="AB61" s="11" t="n"/>
+      <c r="AC61" s="11" t="n"/>
     </row>
     <row r="62">
       <c r="B62" s="8" t="inlineStr">
@@ -13323,6 +14655,9 @@
       <c r="Z62" s="9" t="n">
         <v>-535.3873940529101</v>
       </c>
+      <c r="AA62" s="9" t="n"/>
+      <c r="AB62" s="9" t="n"/>
+      <c r="AC62" s="9" t="n"/>
     </row>
     <row r="63">
       <c r="B63" s="10" t="inlineStr">
@@ -13378,6 +14713,9 @@
       <c r="Z63" s="11" t="n">
         <v>-535.3873940529101</v>
       </c>
+      <c r="AA63" s="11" t="n"/>
+      <c r="AB63" s="11" t="n"/>
+      <c r="AC63" s="11" t="n"/>
     </row>
     <row r="64">
       <c r="B64" s="8" t="inlineStr">
@@ -13427,6 +14765,9 @@
       <c r="Z64" s="9" t="n">
         <v>-55.90866344444445</v>
       </c>
+      <c r="AA64" s="9" t="n"/>
+      <c r="AB64" s="9" t="n"/>
+      <c r="AC64" s="9" t="n"/>
     </row>
     <row r="65">
       <c r="B65" s="10" t="inlineStr">
@@ -13476,6 +14817,9 @@
       <c r="Z65" s="11" t="n">
         <v>-55.90866344444445</v>
       </c>
+      <c r="AA65" s="11" t="n"/>
+      <c r="AB65" s="11" t="n"/>
+      <c r="AC65" s="11" t="n"/>
     </row>
     <row r="66">
       <c r="B66" s="12" t="inlineStr">
@@ -13531,6 +14875,9 @@
       <c r="Z66" s="13" t="n">
         <v>-610.4665366719577</v>
       </c>
+      <c r="AA66" s="13" t="n"/>
+      <c r="AB66" s="13" t="n"/>
+      <c r="AC66" s="13" t="n"/>
     </row>
     <row r="67">
       <c r="B67" s="14" t="inlineStr">
@@ -13562,6 +14909,9 @@
       <c r="X67" s="15" t="n"/>
       <c r="Y67" s="15" t="n"/>
       <c r="Z67" s="15" t="n"/>
+      <c r="AA67" s="15" t="n"/>
+      <c r="AB67" s="15" t="n"/>
+      <c r="AC67" s="15" t="n"/>
     </row>
     <row r="68">
       <c r="B68" s="8" t="inlineStr">
@@ -13617,6 +14967,9 @@
       <c r="Z68" s="9" t="n">
         <v>-26.68137267724868</v>
       </c>
+      <c r="AA68" s="9" t="n"/>
+      <c r="AB68" s="9" t="n"/>
+      <c r="AC68" s="9" t="n"/>
     </row>
     <row r="69">
       <c r="B69" s="12" t="inlineStr">
@@ -13672,6 +15025,9 @@
       <c r="Z69" s="13" t="n">
         <v>-26.68137267724868</v>
       </c>
+      <c r="AA69" s="13" t="n"/>
+      <c r="AB69" s="13" t="n"/>
+      <c r="AC69" s="13" t="n"/>
     </row>
     <row r="70">
       <c r="B70" s="14" t="inlineStr">
@@ -13703,6 +15059,9 @@
       <c r="X70" s="15" t="n"/>
       <c r="Y70" s="15" t="n"/>
       <c r="Z70" s="15" t="n"/>
+      <c r="AA70" s="15" t="n"/>
+      <c r="AB70" s="15" t="n"/>
+      <c r="AC70" s="15" t="n"/>
     </row>
     <row r="71">
       <c r="B71" s="8" t="inlineStr">
@@ -13752,6 +15111,9 @@
       <c r="Z71" s="9" t="n">
         <v>-92.28571428571429</v>
       </c>
+      <c r="AA71" s="9" t="n"/>
+      <c r="AB71" s="9" t="n"/>
+      <c r="AC71" s="9" t="n"/>
     </row>
     <row r="72">
       <c r="B72" s="10" t="inlineStr">
@@ -13807,6 +15169,9 @@
       <c r="Z72" s="11" t="n">
         <v>-232.8042328042328</v>
       </c>
+      <c r="AA72" s="11" t="n"/>
+      <c r="AB72" s="11" t="n"/>
+      <c r="AC72" s="11" t="n"/>
     </row>
     <row r="73">
       <c r="B73" s="8" t="inlineStr">
@@ -13856,6 +15221,9 @@
       <c r="Z73" s="9" t="n">
         <v>-80.72941468253968</v>
       </c>
+      <c r="AA73" s="9" t="n"/>
+      <c r="AB73" s="9" t="n"/>
+      <c r="AC73" s="9" t="n"/>
     </row>
     <row r="74">
       <c r="B74" s="12" t="inlineStr">
@@ -13917,6 +15285,9 @@
       <c r="Z74" s="13" t="n">
         <v>-405.8193617724867</v>
       </c>
+      <c r="AA74" s="13" t="n"/>
+      <c r="AB74" s="13" t="n"/>
+      <c r="AC74" s="13" t="n"/>
     </row>
     <row r="75">
       <c r="B75" s="14" t="inlineStr">
@@ -13948,6 +15319,9 @@
       <c r="X75" s="15" t="n"/>
       <c r="Y75" s="15" t="n"/>
       <c r="Z75" s="15" t="n"/>
+      <c r="AA75" s="15" t="n"/>
+      <c r="AB75" s="15" t="n"/>
+      <c r="AC75" s="15" t="n"/>
     </row>
     <row r="76">
       <c r="B76" s="8" t="inlineStr">
@@ -14027,6 +15401,15 @@
       <c r="Z76" s="9" t="n">
         <v>-32.17464247619048</v>
       </c>
+      <c r="AA76" s="9" t="n">
+        <v>-581.550572</v>
+      </c>
+      <c r="AB76" s="9" t="n">
+        <v>-0.03420885717647059</v>
+      </c>
+      <c r="AC76" s="9" t="n">
+        <v>-3.076987153439153</v>
+      </c>
     </row>
     <row r="77">
       <c r="B77" s="10" t="inlineStr">
@@ -14106,6 +15489,15 @@
       <c r="Z77" s="11" t="n">
         <v>-37.17393839968254</v>
       </c>
+      <c r="AA77" s="11" t="n">
+        <v>-1326.701477</v>
+      </c>
+      <c r="AB77" s="11" t="n">
+        <v>-0.07804126335294118</v>
+      </c>
+      <c r="AC77" s="11" t="n">
+        <v>-7.019584534391535</v>
+      </c>
     </row>
     <row r="78">
       <c r="B78" s="8" t="inlineStr">
@@ -14185,6 +15577,15 @@
       <c r="Z78" s="9" t="n">
         <v>-33.0541264021164</v>
       </c>
+      <c r="AA78" s="9" t="n">
+        <v>-875.805081</v>
+      </c>
+      <c r="AB78" s="9" t="n">
+        <v>-0.05151794594117647</v>
+      </c>
+      <c r="AC78" s="9" t="n">
+        <v>-4.633889317460318</v>
+      </c>
     </row>
     <row r="79">
       <c r="B79" s="10" t="inlineStr">
@@ -14264,6 +15665,15 @@
       <c r="Z79" s="11" t="n">
         <v>-2.047604216931217</v>
       </c>
+      <c r="AA79" s="11" t="n">
+        <v>-8.183769</v>
+      </c>
+      <c r="AB79" s="11" t="n">
+        <v>-0.0004813981764705882</v>
+      </c>
+      <c r="AC79" s="11" t="n">
+        <v>-0.04330036507936508</v>
+      </c>
     </row>
     <row r="80">
       <c r="B80" s="12" t="inlineStr">
@@ -14342,6 +15752,15 @@
       </c>
       <c r="Z80" s="13" t="n">
         <v>-104.4503114949206</v>
+      </c>
+      <c r="AA80" s="13" t="n">
+        <v>-2792.240899</v>
+      </c>
+      <c r="AB80" s="13" t="n">
+        <v>-0.1642494646470588</v>
+      </c>
+      <c r="AC80" s="13" t="n">
+        <v>-14.77376137037037</v>
       </c>
     </row>
     <row r="81">
@@ -14374,6 +15793,9 @@
       <c r="X81" s="15" t="n"/>
       <c r="Y81" s="15" t="n"/>
       <c r="Z81" s="15" t="n"/>
+      <c r="AA81" s="15" t="n"/>
+      <c r="AB81" s="15" t="n"/>
+      <c r="AC81" s="15" t="n"/>
     </row>
     <row r="82">
       <c r="B82" s="14" t="inlineStr">
@@ -14405,6 +15827,9 @@
       <c r="X82" s="15" t="n"/>
       <c r="Y82" s="15" t="n"/>
       <c r="Z82" s="15" t="n"/>
+      <c r="AA82" s="15" t="n"/>
+      <c r="AB82" s="15" t="n"/>
+      <c r="AC82" s="15" t="n"/>
     </row>
     <row r="83">
       <c r="B83" s="8" t="inlineStr">
@@ -14483,6 +15908,15 @@
       </c>
       <c r="Z83" s="9" t="n">
         <v>-0.625686925925926</v>
+      </c>
+      <c r="AA83" s="9" t="n">
+        <v>-16.999662</v>
+      </c>
+      <c r="AB83" s="9" t="n">
+        <v>-0.0009999801176470589</v>
+      </c>
+      <c r="AC83" s="9" t="n">
+        <v>-0.08994530158730159</v>
       </c>
     </row>
     <row r="84">
@@ -14521,6 +15955,15 @@
       <c r="Z84" s="11" t="n">
         <v>-0.0138973544973545</v>
       </c>
+      <c r="AA84" s="11" t="n">
+        <v>-2.6266</v>
+      </c>
+      <c r="AB84" s="11" t="n">
+        <v>-0.0001545058823529412</v>
+      </c>
+      <c r="AC84" s="11" t="n">
+        <v>-0.0138973544973545</v>
+      </c>
     </row>
     <row r="85">
       <c r="B85" s="8" t="inlineStr">
@@ -14582,6 +16025,9 @@
       <c r="Z85" s="9" t="n">
         <v>-0.04149314814814814</v>
       </c>
+      <c r="AA85" s="9" t="n"/>
+      <c r="AB85" s="9" t="n"/>
+      <c r="AC85" s="9" t="n"/>
     </row>
     <row r="86">
       <c r="B86" s="10" t="inlineStr">
@@ -14643,6 +16089,9 @@
       <c r="Z86" s="11" t="n">
         <v>-0.008627340952380951</v>
       </c>
+      <c r="AA86" s="11" t="n"/>
+      <c r="AB86" s="11" t="n"/>
+      <c r="AC86" s="11" t="n"/>
     </row>
     <row r="87">
       <c r="B87" s="8" t="inlineStr">
@@ -14721,6 +16170,15 @@
       </c>
       <c r="Z87" s="9" t="n">
         <v>-0.5164865661375662</v>
+      </c>
+      <c r="AA87" s="9" t="n">
+        <v>-20.335475</v>
+      </c>
+      <c r="AB87" s="9" t="n">
+        <v>-0.001196204411764706</v>
+      </c>
+      <c r="AC87" s="9" t="n">
+        <v>-0.1075951058201058</v>
       </c>
     </row>
     <row r="88">
@@ -14789,6 +16247,15 @@
       <c r="Z88" s="11" t="n">
         <v>-0.008792042328042328</v>
       </c>
+      <c r="AA88" s="11" t="n">
+        <v>-0.817499</v>
+      </c>
+      <c r="AB88" s="11" t="n">
+        <v>-4.808817647058823e-05</v>
+      </c>
+      <c r="AC88" s="11" t="n">
+        <v>-0.004325391534391534</v>
+      </c>
     </row>
     <row r="89">
       <c r="B89" s="12" t="inlineStr">
@@ -14867,6 +16334,15 @@
       </c>
       <c r="Z89" s="13" t="n">
         <v>-1.214983377989418</v>
+      </c>
+      <c r="AA89" s="13" t="n">
+        <v>-40.779236</v>
+      </c>
+      <c r="AB89" s="13" t="n">
+        <v>-0.002398778588235294</v>
+      </c>
+      <c r="AC89" s="13" t="n">
+        <v>-0.2157631534391534</v>
       </c>
     </row>
     <row r="90">
@@ -14899,6 +16375,9 @@
       <c r="X90" s="15" t="n"/>
       <c r="Y90" s="15" t="n"/>
       <c r="Z90" s="15" t="n"/>
+      <c r="AA90" s="15" t="n"/>
+      <c r="AB90" s="15" t="n"/>
+      <c r="AC90" s="15" t="n"/>
     </row>
     <row r="91">
       <c r="B91" s="8" t="inlineStr">
@@ -14960,6 +16439,15 @@
       <c r="Z91" s="9" t="n">
         <v>-0.4542010582010582</v>
       </c>
+      <c r="AA91" s="9" t="n">
+        <v>-1.152</v>
+      </c>
+      <c r="AB91" s="9" t="n">
+        <v>-6.776470588235293e-05</v>
+      </c>
+      <c r="AC91" s="9" t="n">
+        <v>-0.006095238095238095</v>
+      </c>
     </row>
     <row r="92">
       <c r="B92" s="10" t="inlineStr">
@@ -15039,6 +16527,15 @@
       <c r="Z92" s="11" t="n">
         <v>-0.9834890000000001</v>
       </c>
+      <c r="AA92" s="11" t="n">
+        <v>-10.458793</v>
+      </c>
+      <c r="AB92" s="11" t="n">
+        <v>-0.0006152231176470588</v>
+      </c>
+      <c r="AC92" s="11" t="n">
+        <v>-0.0553375291005291</v>
+      </c>
     </row>
     <row r="93">
       <c r="B93" s="8" t="inlineStr">
@@ -15118,6 +16615,15 @@
       <c r="Z93" s="9" t="n">
         <v>-34.55143201301588</v>
       </c>
+      <c r="AA93" s="9" t="n">
+        <v>-610.3169810000001</v>
+      </c>
+      <c r="AB93" s="9" t="n">
+        <v>-0.03590099888235294</v>
+      </c>
+      <c r="AC93" s="9" t="n">
+        <v>-3.229190375661376</v>
+      </c>
     </row>
     <row r="94">
       <c r="B94" s="10" t="inlineStr">
@@ -15197,6 +16703,15 @@
       <c r="Z94" s="11" t="n">
         <v>-1.024866306878307</v>
       </c>
+      <c r="AA94" s="11" t="n">
+        <v>-30.477712</v>
+      </c>
+      <c r="AB94" s="11" t="n">
+        <v>-0.001792806588235294</v>
+      </c>
+      <c r="AC94" s="11" t="n">
+        <v>-0.1612577354497355</v>
+      </c>
     </row>
     <row r="95">
       <c r="B95" s="8" t="inlineStr">
@@ -15276,6 +16791,15 @@
       <c r="Z95" s="9" t="n">
         <v>-1.540756518518518</v>
       </c>
+      <c r="AA95" s="9" t="n">
+        <v>-14.997022</v>
+      </c>
+      <c r="AB95" s="9" t="n">
+        <v>-0.0008821777647058823</v>
+      </c>
+      <c r="AC95" s="9" t="n">
+        <v>-0.07934932275132275</v>
+      </c>
     </row>
     <row r="96">
       <c r="B96" s="12" t="inlineStr">
@@ -15354,6 +16878,15 @@
       </c>
       <c r="Z96" s="13" t="n">
         <v>-38.55474489661376</v>
+      </c>
+      <c r="AA96" s="13" t="n">
+        <v>-667.402508</v>
+      </c>
+      <c r="AB96" s="13" t="n">
+        <v>-0.03925897105882353</v>
+      </c>
+      <c r="AC96" s="13" t="n">
+        <v>-3.531230201058201</v>
       </c>
     </row>
     <row r="97">
@@ -15386,6 +16919,9 @@
       <c r="X97" s="15" t="n"/>
       <c r="Y97" s="15" t="n"/>
       <c r="Z97" s="15" t="n"/>
+      <c r="AA97" s="15" t="n"/>
+      <c r="AB97" s="15" t="n"/>
+      <c r="AC97" s="15" t="n"/>
     </row>
     <row r="98">
       <c r="B98" s="8" t="inlineStr">
@@ -15465,6 +17001,15 @@
       <c r="Z98" s="9" t="n">
         <v>-0.9680948518518517</v>
       </c>
+      <c r="AA98" s="9" t="n">
+        <v>-8.741825</v>
+      </c>
+      <c r="AB98" s="9" t="n">
+        <v>-0.000514225</v>
+      </c>
+      <c r="AC98" s="9" t="n">
+        <v>-0.04625304232804233</v>
+      </c>
     </row>
     <row r="99">
       <c r="B99" s="10" t="inlineStr">
@@ -15544,6 +17089,15 @@
       <c r="Z99" s="11" t="n">
         <v>-0.8468110105820106</v>
       </c>
+      <c r="AA99" s="11" t="n">
+        <v>-31.091154</v>
+      </c>
+      <c r="AB99" s="11" t="n">
+        <v>-0.001828891411764706</v>
+      </c>
+      <c r="AC99" s="11" t="n">
+        <v>-0.1645034603174603</v>
+      </c>
     </row>
     <row r="100">
       <c r="B100" s="8" t="inlineStr">
@@ -15622,6 +17176,15 @@
       </c>
       <c r="Z100" s="9" t="n">
         <v>-6.305078687830688</v>
+      </c>
+      <c r="AA100" s="9" t="n">
+        <v>-193.998002</v>
+      </c>
+      <c r="AB100" s="9" t="n">
+        <v>-0.01141164717647059</v>
+      </c>
+      <c r="AC100" s="9" t="n">
+        <v>-1.026444455026455</v>
       </c>
     </row>
     <row r="101">
@@ -15696,6 +17259,15 @@
       <c r="Z101" s="11" t="n">
         <v>-0.8273216402116402</v>
       </c>
+      <c r="AA101" s="11" t="n">
+        <v>-43.87624</v>
+      </c>
+      <c r="AB101" s="11" t="n">
+        <v>-0.002580955294117647</v>
+      </c>
+      <c r="AC101" s="11" t="n">
+        <v>-0.232149417989418</v>
+      </c>
     </row>
     <row r="102">
       <c r="B102" s="12" t="inlineStr">
@@ -15774,6 +17346,15 @@
       </c>
       <c r="Z102" s="13" t="n">
         <v>-8.947306190476191</v>
+      </c>
+      <c r="AA102" s="13" t="n">
+        <v>-277.707221</v>
+      </c>
+      <c r="AB102" s="13" t="n">
+        <v>-0.01633571888235294</v>
+      </c>
+      <c r="AC102" s="13" t="n">
+        <v>-1.469350375661376</v>
       </c>
     </row>
     <row r="103">
@@ -15806,6 +17387,9 @@
       <c r="X103" s="15" t="n"/>
       <c r="Y103" s="15" t="n"/>
       <c r="Z103" s="15" t="n"/>
+      <c r="AA103" s="15" t="n"/>
+      <c r="AB103" s="15" t="n"/>
+      <c r="AC103" s="15" t="n"/>
     </row>
     <row r="104">
       <c r="B104" s="8" t="inlineStr">
@@ -15878,6 +17462,15 @@
       </c>
       <c r="Z104" s="9" t="n">
         <v>-0.6955851851851852</v>
+      </c>
+      <c r="AA104" s="9" t="n">
+        <v>-4.03</v>
+      </c>
+      <c r="AB104" s="9" t="n">
+        <v>-0.0002370588235294118</v>
+      </c>
+      <c r="AC104" s="9" t="n">
+        <v>-0.02132275132275132</v>
       </c>
     </row>
     <row r="105">
@@ -15928,6 +17521,15 @@
       <c r="Z105" s="11" t="n">
         <v>-0.0435899470899471</v>
       </c>
+      <c r="AA105" s="11" t="n">
+        <v>-5.9375</v>
+      </c>
+      <c r="AB105" s="11" t="n">
+        <v>-0.000349264705882353</v>
+      </c>
+      <c r="AC105" s="11" t="n">
+        <v>-0.03141534391534392</v>
+      </c>
     </row>
     <row r="106">
       <c r="B106" s="8" t="inlineStr">
@@ -16007,6 +17609,15 @@
       <c r="Z106" s="9" t="n">
         <v>-1.934127571428572</v>
       </c>
+      <c r="AA106" s="9" t="n">
+        <v>-147.572961</v>
+      </c>
+      <c r="AB106" s="9" t="n">
+        <v>-0.008680762411764706</v>
+      </c>
+      <c r="AC106" s="9" t="n">
+        <v>-0.7808093174603175</v>
+      </c>
     </row>
     <row r="107">
       <c r="B107" s="12" t="inlineStr">
@@ -16085,6 +17696,15 @@
       </c>
       <c r="Z107" s="13" t="n">
         <v>-2.673302703703704</v>
+      </c>
+      <c r="AA107" s="13" t="n">
+        <v>-157.540461</v>
+      </c>
+      <c r="AB107" s="13" t="n">
+        <v>-0.00926708594117647</v>
+      </c>
+      <c r="AC107" s="13" t="n">
+        <v>-0.8335474126984127</v>
       </c>
     </row>
     <row r="108">
@@ -16117,6 +17737,9 @@
       <c r="X108" s="15" t="n"/>
       <c r="Y108" s="15" t="n"/>
       <c r="Z108" s="15" t="n"/>
+      <c r="AA108" s="15" t="n"/>
+      <c r="AB108" s="15" t="n"/>
+      <c r="AC108" s="15" t="n"/>
     </row>
     <row r="109">
       <c r="B109" s="8" t="inlineStr">
@@ -16189,6 +17812,15 @@
       </c>
       <c r="Z109" s="9" t="n">
         <v>-1.865172349206349</v>
+      </c>
+      <c r="AA109" s="9" t="n">
+        <v>-26.16</v>
+      </c>
+      <c r="AB109" s="9" t="n">
+        <v>-0.001538823529411765</v>
+      </c>
+      <c r="AC109" s="9" t="n">
+        <v>-0.1384126984126984</v>
       </c>
     </row>
     <row r="110">
@@ -16227,6 +17859,15 @@
       <c r="Z110" s="11" t="n">
         <v>-0.06878306878306878</v>
       </c>
+      <c r="AA110" s="11" t="n">
+        <v>-13</v>
+      </c>
+      <c r="AB110" s="11" t="n">
+        <v>-0.0007647058823529412</v>
+      </c>
+      <c r="AC110" s="11" t="n">
+        <v>-0.06878306878306878</v>
+      </c>
     </row>
     <row r="111">
       <c r="B111" s="8" t="inlineStr">
@@ -16306,6 +17947,15 @@
       <c r="Z111" s="9" t="n">
         <v>-0.6522176349206349</v>
       </c>
+      <c r="AA111" s="9" t="n">
+        <v>-6.603578</v>
+      </c>
+      <c r="AB111" s="9" t="n">
+        <v>-0.0003884457647058823</v>
+      </c>
+      <c r="AC111" s="9" t="n">
+        <v>-0.03493956613756614</v>
+      </c>
     </row>
     <row r="112">
       <c r="B112" s="10" t="inlineStr">
@@ -16385,6 +18035,15 @@
       <c r="Z112" s="11" t="n">
         <v>-2.187928798941799</v>
       </c>
+      <c r="AA112" s="11" t="n">
+        <v>-164.950749</v>
+      </c>
+      <c r="AB112" s="11" t="n">
+        <v>-0.009702985235294118</v>
+      </c>
+      <c r="AC112" s="11" t="n">
+        <v>-0.8727552857142857</v>
+      </c>
     </row>
     <row r="113">
       <c r="B113" s="12" t="inlineStr">
@@ -16463,6 +18122,15 @@
       </c>
       <c r="Z113" s="13" t="n">
         <v>-4.774101851851852</v>
+      </c>
+      <c r="AA113" s="13" t="n">
+        <v>-210.714327</v>
+      </c>
+      <c r="AB113" s="13" t="n">
+        <v>-0.01239496041176471</v>
+      </c>
+      <c r="AC113" s="13" t="n">
+        <v>-1.114890619047619</v>
       </c>
     </row>
     <row r="114">
@@ -16495,6 +18163,9 @@
       <c r="X114" s="15" t="n"/>
       <c r="Y114" s="15" t="n"/>
       <c r="Z114" s="15" t="n"/>
+      <c r="AA114" s="15" t="n"/>
+      <c r="AB114" s="15" t="n"/>
+      <c r="AC114" s="15" t="n"/>
     </row>
     <row r="115">
       <c r="B115" s="8" t="inlineStr">
@@ -16574,6 +18245,15 @@
       <c r="Z115" s="9" t="n">
         <v>-25.63583297354498</v>
       </c>
+      <c r="AA115" s="9" t="n">
+        <v>-735.604373</v>
+      </c>
+      <c r="AB115" s="9" t="n">
+        <v>-0.04327084547058824</v>
+      </c>
+      <c r="AC115" s="9" t="n">
+        <v>-3.89208662962963</v>
+      </c>
     </row>
     <row r="116">
       <c r="B116" s="12" t="inlineStr">
@@ -16652,6 +18332,15 @@
       </c>
       <c r="Z116" s="13" t="n">
         <v>-25.63583297354498</v>
+      </c>
+      <c r="AA116" s="13" t="n">
+        <v>-735.604373</v>
+      </c>
+      <c r="AB116" s="13" t="n">
+        <v>-0.04327084547058824</v>
+      </c>
+      <c r="AC116" s="13" t="n">
+        <v>-3.89208662962963</v>
       </c>
     </row>
     <row r="117">
@@ -16684,6 +18373,9 @@
       <c r="X117" s="15" t="n"/>
       <c r="Y117" s="15" t="n"/>
       <c r="Z117" s="15" t="n"/>
+      <c r="AA117" s="15" t="n"/>
+      <c r="AB117" s="15" t="n"/>
+      <c r="AC117" s="15" t="n"/>
     </row>
     <row r="118">
       <c r="B118" s="8" t="inlineStr">
@@ -16745,6 +18437,9 @@
       <c r="Z118" s="9" t="n">
         <v>-30.47793147089947</v>
       </c>
+      <c r="AA118" s="9" t="n"/>
+      <c r="AB118" s="9" t="n"/>
+      <c r="AC118" s="9" t="n"/>
     </row>
     <row r="119">
       <c r="B119" s="10" t="inlineStr">
@@ -16794,6 +18489,9 @@
       <c r="Z119" s="11" t="n">
         <v>-9.685637142857143</v>
       </c>
+      <c r="AA119" s="11" t="n"/>
+      <c r="AB119" s="11" t="n"/>
+      <c r="AC119" s="11" t="n"/>
     </row>
     <row r="120">
       <c r="B120" s="8" t="inlineStr">
@@ -16873,6 +18571,15 @@
       <c r="Z120" s="9" t="n">
         <v>-0.08896550793650795</v>
       </c>
+      <c r="AA120" s="9" t="n">
+        <v>-1.728</v>
+      </c>
+      <c r="AB120" s="9" t="n">
+        <v>-0.0001016470588235294</v>
+      </c>
+      <c r="AC120" s="9" t="n">
+        <v>-0.009142857142857144</v>
+      </c>
     </row>
     <row r="121">
       <c r="B121" s="10" t="inlineStr">
@@ -16951,6 +18658,15 @@
       </c>
       <c r="Z121" s="11" t="n">
         <v>-8.232013108306878</v>
+      </c>
+      <c r="AA121" s="11" t="n">
+        <v>-240.870006</v>
+      </c>
+      <c r="AB121" s="11" t="n">
+        <v>-0.01416882388235294</v>
+      </c>
+      <c r="AC121" s="11" t="n">
+        <v>-1.274444476190476</v>
       </c>
     </row>
     <row r="122">
@@ -17019,6 +18735,15 @@
       <c r="Z122" s="9" t="n">
         <v>-1.586642857142857</v>
       </c>
+      <c r="AA122" s="9" t="n">
+        <v>-119.829</v>
+      </c>
+      <c r="AB122" s="9" t="n">
+        <v>-0.007048764705882352</v>
+      </c>
+      <c r="AC122" s="9" t="n">
+        <v>-0.634015873015873</v>
+      </c>
     </row>
     <row r="123">
       <c r="B123" s="10" t="inlineStr">
@@ -17098,6 +18823,15 @@
       <c r="Z123" s="11" t="n">
         <v>-73.71793856084655</v>
       </c>
+      <c r="AA123" s="11" t="n">
+        <v>-775.648144</v>
+      </c>
+      <c r="AB123" s="11" t="n">
+        <v>-0.0456263614117647</v>
+      </c>
+      <c r="AC123" s="11" t="n">
+        <v>-4.103958433862434</v>
+      </c>
     </row>
     <row r="124">
       <c r="B124" s="12" t="inlineStr">
@@ -17176,6 +18910,15 @@
       </c>
       <c r="Z124" s="13" t="n">
         <v>-123.7891286479894</v>
+      </c>
+      <c r="AA124" s="13" t="n">
+        <v>-1138.07515</v>
+      </c>
+      <c r="AB124" s="13" t="n">
+        <v>-0.06694559705882352</v>
+      </c>
+      <c r="AC124" s="13" t="n">
+        <v>-6.021561640211639</v>
       </c>
     </row>
     <row r="125">
@@ -17208,6 +18951,9 @@
       <c r="X125" s="15" t="n"/>
       <c r="Y125" s="15" t="n"/>
       <c r="Z125" s="15" t="n"/>
+      <c r="AA125" s="15" t="n"/>
+      <c r="AB125" s="15" t="n"/>
+      <c r="AC125" s="15" t="n"/>
     </row>
     <row r="126">
       <c r="B126" s="8" t="inlineStr">
@@ -17275,6 +19021,15 @@
       <c r="Z126" s="9" t="n">
         <v>-0.1413403174603174</v>
       </c>
+      <c r="AA126" s="9" t="n">
+        <v>-3.74095</v>
+      </c>
+      <c r="AB126" s="9" t="n">
+        <v>-0.0002200558823529412</v>
+      </c>
+      <c r="AC126" s="9" t="n">
+        <v>-0.01979338624338624</v>
+      </c>
     </row>
     <row r="127">
       <c r="B127" s="10" t="inlineStr">
@@ -17342,6 +19097,15 @@
       <c r="Z127" s="11" t="n">
         <v>-0.9737442433862435</v>
       </c>
+      <c r="AA127" s="11" t="n">
+        <v>-60.390459</v>
+      </c>
+      <c r="AB127" s="11" t="n">
+        <v>-0.003552379941176471</v>
+      </c>
+      <c r="AC127" s="11" t="n">
+        <v>-0.3195262380952381</v>
+      </c>
     </row>
     <row r="128">
       <c r="B128" s="8" t="inlineStr">
@@ -17421,6 +19185,9 @@
       <c r="Z128" s="9" t="n">
         <v>-1.093348444444444</v>
       </c>
+      <c r="AA128" s="9" t="n"/>
+      <c r="AB128" s="9" t="n"/>
+      <c r="AC128" s="9" t="n"/>
     </row>
     <row r="129">
       <c r="B129" s="10" t="inlineStr">
@@ -17500,6 +19267,15 @@
       <c r="Z129" s="11" t="n">
         <v>-0.488404380952381</v>
       </c>
+      <c r="AA129" s="11" t="n">
+        <v>-12.025744</v>
+      </c>
+      <c r="AB129" s="11" t="n">
+        <v>-0.0007073967058823529</v>
+      </c>
+      <c r="AC129" s="11" t="n">
+        <v>-0.06362827513227513</v>
+      </c>
     </row>
     <row r="130">
       <c r="B130" s="8" t="inlineStr">
@@ -17578,6 +19354,15 @@
       </c>
       <c r="Z130" s="9" t="n">
         <v>-1.057244523809524</v>
+      </c>
+      <c r="AA130" s="9" t="n">
+        <v>-23.394231</v>
+      </c>
+      <c r="AB130" s="9" t="n">
+        <v>-0.001376131235294118</v>
+      </c>
+      <c r="AC130" s="9" t="n">
+        <v>-0.123779</v>
       </c>
     </row>
     <row r="131">
@@ -17628,6 +19413,9 @@
       <c r="Z131" s="11" t="n">
         <v>-0.005820105820105821</v>
       </c>
+      <c r="AA131" s="11" t="n"/>
+      <c r="AB131" s="11" t="n"/>
+      <c r="AC131" s="11" t="n"/>
     </row>
     <row r="132">
       <c r="B132" s="12" t="inlineStr">
@@ -17707,6 +19495,15 @@
       <c r="Z132" s="13" t="n">
         <v>-3.759902015873016</v>
       </c>
+      <c r="AA132" s="13" t="n">
+        <v>-99.551384</v>
+      </c>
+      <c r="AB132" s="13" t="n">
+        <v>-0.005855963764705882</v>
+      </c>
+      <c r="AC132" s="13" t="n">
+        <v>-0.5267268994708995</v>
+      </c>
     </row>
     <row r="133">
       <c r="B133" s="12" t="inlineStr">
@@ -17785,6 +19582,15 @@
       </c>
       <c r="Z133" s="13" t="n">
         <v>-209.3493026580423</v>
+      </c>
+      <c r="AA133" s="13" t="n">
+        <v>-3327.37466</v>
+      </c>
+      <c r="AB133" s="13" t="n">
+        <v>-0.1957279211764706</v>
+      </c>
+      <c r="AC133" s="13" t="n">
+        <v>-17.60515693121693</v>
       </c>
     </row>
     <row r="134">
@@ -17817,6 +19623,9 @@
       <c r="X134" s="15" t="n"/>
       <c r="Y134" s="15" t="n"/>
       <c r="Z134" s="15" t="n"/>
+      <c r="AA134" s="15" t="n"/>
+      <c r="AB134" s="15" t="n"/>
+      <c r="AC134" s="15" t="n"/>
     </row>
     <row r="135">
       <c r="B135" s="8" t="inlineStr">
@@ -17884,6 +19693,9 @@
       <c r="Z135" s="9" t="n">
         <v>-0.455026455026455</v>
       </c>
+      <c r="AA135" s="9" t="n"/>
+      <c r="AB135" s="9" t="n"/>
+      <c r="AC135" s="9" t="n"/>
     </row>
     <row r="136">
       <c r="B136" s="10" t="inlineStr">
@@ -17921,6 +19733,15 @@
       <c r="Z136" s="11" t="n">
         <v>-0.02645502645502645</v>
       </c>
+      <c r="AA136" s="11" t="n">
+        <v>-5</v>
+      </c>
+      <c r="AB136" s="11" t="n">
+        <v>-0.0002941176470588235</v>
+      </c>
+      <c r="AC136" s="11" t="n">
+        <v>-0.02645502645502645</v>
+      </c>
     </row>
     <row r="137">
       <c r="B137" s="8" t="inlineStr">
@@ -17999,6 +19820,15 @@
       </c>
       <c r="Z137" s="9" t="n">
         <v>-3.591381243386243</v>
+      </c>
+      <c r="AA137" s="9" t="n">
+        <v>-92.35136</v>
+      </c>
+      <c r="AB137" s="9" t="n">
+        <v>-0.00543243294117647</v>
+      </c>
+      <c r="AC137" s="9" t="n">
+        <v>-0.4886315343915344</v>
       </c>
     </row>
     <row r="138">
@@ -18049,6 +19879,9 @@
       <c r="Z138" s="11" t="n">
         <v>-8.289354497354498</v>
       </c>
+      <c r="AA138" s="11" t="n"/>
+      <c r="AB138" s="11" t="n"/>
+      <c r="AC138" s="11" t="n"/>
     </row>
     <row r="139">
       <c r="B139" s="8" t="inlineStr">
@@ -18098,6 +19931,9 @@
       <c r="Z139" s="9" t="n">
         <v>-0.04457671957671958</v>
       </c>
+      <c r="AA139" s="9" t="n"/>
+      <c r="AB139" s="9" t="n"/>
+      <c r="AC139" s="9" t="n"/>
     </row>
     <row r="140">
       <c r="B140" s="12" t="inlineStr">
@@ -18176,6 +20012,15 @@
       </c>
       <c r="Z140" s="13" t="n">
         <v>-12.40679394179894</v>
+      </c>
+      <c r="AA140" s="13" t="n">
+        <v>-97.35136</v>
+      </c>
+      <c r="AB140" s="13" t="n">
+        <v>-0.005726550588235294</v>
+      </c>
+      <c r="AC140" s="13" t="n">
+        <v>-0.5150865608465608</v>
       </c>
     </row>
     <row r="141">
@@ -18208,6 +20053,9 @@
       <c r="X141" s="15" t="n"/>
       <c r="Y141" s="15" t="n"/>
       <c r="Z141" s="15" t="n"/>
+      <c r="AA141" s="15" t="n"/>
+      <c r="AB141" s="15" t="n"/>
+      <c r="AC141" s="15" t="n"/>
     </row>
     <row r="142">
       <c r="B142" s="8" t="inlineStr">
@@ -18286,6 +20134,15 @@
       </c>
       <c r="Z142" s="9" t="n">
         <v>-0.08609910941798943</v>
+      </c>
+      <c r="AA142" s="9" t="n">
+        <v>-2.079254</v>
+      </c>
+      <c r="AB142" s="9" t="n">
+        <v>-0.0001223090588235294</v>
+      </c>
+      <c r="AC142" s="9" t="n">
+        <v>-0.01100134391534392</v>
       </c>
     </row>
     <row r="143">
@@ -18342,6 +20199,9 @@
       <c r="Z143" s="11" t="n">
         <v>-0.2752046190476191</v>
       </c>
+      <c r="AA143" s="11" t="n"/>
+      <c r="AB143" s="11" t="n"/>
+      <c r="AC143" s="11" t="n"/>
     </row>
     <row r="144">
       <c r="B144" s="8" t="inlineStr">
@@ -18409,6 +20269,9 @@
       <c r="Z144" s="9" t="n">
         <v>-0.04949648227513227</v>
       </c>
+      <c r="AA144" s="9" t="n"/>
+      <c r="AB144" s="9" t="n"/>
+      <c r="AC144" s="9" t="n"/>
     </row>
     <row r="145">
       <c r="B145" s="10" t="inlineStr">
@@ -18487,6 +20350,15 @@
       </c>
       <c r="Z145" s="11" t="n">
         <v>-21.54062413</v>
+      </c>
+      <c r="AA145" s="11" t="n">
+        <v>-191.562425</v>
+      </c>
+      <c r="AB145" s="11" t="n">
+        <v>-0.01126837794117647</v>
+      </c>
+      <c r="AC145" s="11" t="n">
+        <v>-1.013557804232804</v>
       </c>
     </row>
     <row r="146">
@@ -18555,6 +20427,9 @@
       <c r="Z146" s="9" t="n">
         <v>-3.400111021164021</v>
       </c>
+      <c r="AA146" s="9" t="n"/>
+      <c r="AB146" s="9" t="n"/>
+      <c r="AC146" s="9" t="n"/>
     </row>
     <row r="147">
       <c r="B147" s="10" t="inlineStr">
@@ -18604,6 +20479,9 @@
       <c r="Z147" s="11" t="n">
         <v>-4.09466419047619</v>
       </c>
+      <c r="AA147" s="11" t="n"/>
+      <c r="AB147" s="11" t="n"/>
+      <c r="AC147" s="11" t="n"/>
     </row>
     <row r="148">
       <c r="B148" s="12" t="inlineStr">
@@ -18683,6 +20561,15 @@
       <c r="Z148" s="13" t="n">
         <v>-29.44619955238095</v>
       </c>
+      <c r="AA148" s="13" t="n">
+        <v>-193.641679</v>
+      </c>
+      <c r="AB148" s="13" t="n">
+        <v>-0.011390687</v>
+      </c>
+      <c r="AC148" s="13" t="n">
+        <v>-1.024559148148148</v>
+      </c>
     </row>
     <row r="149">
       <c r="B149" s="16" t="inlineStr">
@@ -18762,6 +20649,15 @@
       <c r="Z149" s="17" t="n">
         <v>-1474.117141688836</v>
       </c>
+      <c r="AA149" s="17" t="n">
+        <v>-7326.525205</v>
+      </c>
+      <c r="AB149" s="17" t="n">
+        <v>-0.430972070882353</v>
+      </c>
+      <c r="AC149" s="17" t="n">
+        <v>-38.76468362433862</v>
+      </c>
     </row>
     <row r="150">
       <c r="B150" s="16" t="inlineStr">
@@ -18841,6 +20737,15 @@
       <c r="Z150" s="17" t="n">
         <v>-349.4657277678308</v>
       </c>
+      <c r="AA150" s="17" t="n">
+        <v>-400.916738</v>
+      </c>
+      <c r="AB150" s="17" t="n">
+        <v>-0.02358333752941176</v>
+      </c>
+      <c r="AC150" s="17" t="n">
+        <v>-2.121252582010582</v>
+      </c>
     </row>
     <row r="151">
       <c r="B151" s="14" t="inlineStr">
@@ -18920,6 +20825,15 @@
       <c r="Z151" s="15" t="n">
         <v>357.0034964357672</v>
       </c>
+      <c r="AA151" s="15" t="n">
+        <v>1825.555016239998</v>
+      </c>
+      <c r="AB151" s="15" t="n">
+        <v>0.1073855891905881</v>
+      </c>
+      <c r="AC151" s="15" t="n">
+        <v>9.659021249947079</v>
+      </c>
     </row>
     <row r="152">
       <c r="B152" s="16" t="inlineStr">
@@ -18999,19 +20913,29 @@
       <c r="Z152" s="17" t="n">
         <v>7.537768667936457</v>
       </c>
+      <c r="AA152" s="17" t="n">
+        <v>1424.638278239998</v>
+      </c>
+      <c r="AB152" s="17" t="n">
+        <v>0.08380225166117634</v>
+      </c>
+      <c r="AC152" s="17" t="n">
+        <v>7.537768667936496</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="11">
-    <mergeCell ref="B2:Z2"/>
+  <mergeCells count="12">
+    <mergeCell ref="B2:AC2"/>
     <mergeCell ref="R3:T3"/>
     <mergeCell ref="U3:W3"/>
     <mergeCell ref="B3:B4"/>
-    <mergeCell ref="B1:Z1"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="X3:Z3"/>
+    <mergeCell ref="B1:AC1"/>
     <mergeCell ref="I3:K3"/>
     <mergeCell ref="F3:H3"/>
     <mergeCell ref="L3:N3"/>
+    <mergeCell ref="AA3:AC3"/>
     <mergeCell ref="O3:Q3"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>

</xml_diff>

<commit_message>
Refresh dashboard Tue 07/28/2026 16:40
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -716,7 +716,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 28 Jul 2026 16:35</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 28 Jul 2026 16:40</t>
         </is>
       </c>
     </row>
@@ -10855,7 +10855,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 28 Jul 2026 16:35 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 28 Jul 2026 16:40 (in IDR Million)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh dashboard Wed 07/29/2026  9:06
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -722,7 +722,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 28 Jul 2026 16:56</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 29 Jul 2026 09:06</t>
         </is>
       </c>
     </row>
@@ -783,14 +783,14 @@
       <c r="W3" s="4" t="n"/>
       <c r="X3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 28 Jul 2026</t>
+          <t>MTD as of 29 Jul 2026</t>
         </is>
       </c>
       <c r="Y3" s="4" t="n"/>
       <c r="Z3" s="4" t="n"/>
       <c r="AA3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 28 Jul 2026</t>
+          <t>YTD as of 29 Jul 2026</t>
         </is>
       </c>
       <c r="AB3" s="4" t="n"/>
@@ -10861,7 +10861,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 28 Jul 2026 16:56 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 29 Jul 2026 09:06 (in IDR Million)</t>
         </is>
       </c>
     </row>
@@ -10922,14 +10922,14 @@
       <c r="W3" s="4" t="n"/>
       <c r="X3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 28 Jul 2026</t>
+          <t>MTD as of 29 Jul 2026</t>
         </is>
       </c>
       <c r="Y3" s="4" t="n"/>
       <c r="Z3" s="4" t="n"/>
       <c r="AA3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 28 Jul 2026</t>
+          <t>YTD as of 29 Jul 2026</t>
         </is>
       </c>
       <c r="AB3" s="4" t="n"/>

</xml_diff>

<commit_message>
Refresh dashboard Wed 07/29/2026 16:15
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -722,7 +722,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 29 Jul 2026 09:06</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 29 Jul 2026 16:15</t>
         </is>
       </c>
     </row>
@@ -1126,22 +1126,22 @@
         <v>822520524.1798942</v>
       </c>
       <c r="X7" s="11" t="n">
-        <v>6895316417</v>
+        <v>6908036417</v>
       </c>
       <c r="Y7" s="11" t="n">
-        <v>405606.8480588236</v>
+        <v>406355.0833529412</v>
       </c>
       <c r="Z7" s="11" t="n">
-        <v>36483155.64550264</v>
+        <v>36550457.23280423</v>
       </c>
       <c r="AA7" s="11" t="n">
-        <v>162351695487</v>
+        <v>162364415487</v>
       </c>
       <c r="AB7" s="11" t="n">
-        <v>9550099.734529411</v>
+        <v>9550847.96982353</v>
       </c>
       <c r="AC7" s="11" t="n">
-        <v>859003679.8253969</v>
+        <v>859070981.4126984</v>
       </c>
     </row>
     <row r="8">
@@ -1633,17 +1633,23 @@
       <c r="W14" s="13" t="n">
         <v>149142.8571428571</v>
       </c>
-      <c r="X14" s="13" t="n"/>
-      <c r="Y14" s="13" t="n"/>
-      <c r="Z14" s="13" t="n"/>
+      <c r="X14" s="13" t="n">
+        <v>12720000</v>
+      </c>
+      <c r="Y14" s="13" t="n">
+        <v>748.2352941176471</v>
+      </c>
+      <c r="Z14" s="13" t="n">
+        <v>67301.58730158731</v>
+      </c>
       <c r="AA14" s="13" t="n">
-        <v>28188000</v>
+        <v>40908000</v>
       </c>
       <c r="AB14" s="13" t="n">
-        <v>1658.117647058823</v>
+        <v>2406.35294117647</v>
       </c>
       <c r="AC14" s="13" t="n">
-        <v>149142.8571428571</v>
+        <v>216444.4444444444</v>
       </c>
     </row>
     <row r="15">
@@ -1820,22 +1826,22 @@
         <v>1910739.122063492</v>
       </c>
       <c r="X17" s="11" t="n">
-        <v>30292050</v>
+        <v>31538050</v>
       </c>
       <c r="Y17" s="11" t="n">
-        <v>1781.885294117647</v>
+        <v>1855.179411764706</v>
       </c>
       <c r="Z17" s="11" t="n">
-        <v>160275.3968253968</v>
+        <v>166867.9894179894</v>
       </c>
       <c r="AA17" s="11" t="n">
-        <v>391421744.07</v>
+        <v>392667744.07</v>
       </c>
       <c r="AB17" s="11" t="n">
-        <v>23024.80847470588</v>
+        <v>23098.10259235294</v>
       </c>
       <c r="AC17" s="11" t="n">
-        <v>2071014.518888889</v>
+        <v>2077607.111481482</v>
       </c>
     </row>
     <row r="18">
@@ -1975,7 +1981,7 @@
     <row r="20">
       <c r="B20" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">        CV Adni Diffa Swandana</t>
+          <t xml:space="preserve">        Scrap Sales</t>
         </is>
       </c>
       <c r="C20" s="13" t="n"/>
@@ -1984,50 +1990,74 @@
       <c r="F20" s="13" t="n"/>
       <c r="G20" s="13" t="n"/>
       <c r="H20" s="13" t="n"/>
-      <c r="I20" s="13" t="n"/>
-      <c r="J20" s="13" t="n"/>
-      <c r="K20" s="13" t="n"/>
-      <c r="L20" s="13" t="n"/>
-      <c r="M20" s="13" t="n"/>
-      <c r="N20" s="13" t="n"/>
+      <c r="I20" s="13" t="n">
+        <v>1673000</v>
+      </c>
+      <c r="J20" s="13" t="n">
+        <v>98.41176470588235</v>
+      </c>
+      <c r="K20" s="13" t="n">
+        <v>8851.851851851852</v>
+      </c>
+      <c r="L20" s="13" t="n">
+        <v>12959000</v>
+      </c>
+      <c r="M20" s="13" t="n">
+        <v>762.2941176470588</v>
+      </c>
+      <c r="N20" s="13" t="n">
+        <v>68566.13756613756</v>
+      </c>
       <c r="O20" s="13" t="n">
-        <v>23270000</v>
+        <v>682500</v>
       </c>
       <c r="P20" s="13" t="n">
-        <v>1368.823529411765</v>
+        <v>40.14705882352941</v>
       </c>
       <c r="Q20" s="13" t="n">
-        <v>123121.6931216931</v>
-      </c>
-      <c r="R20" s="13" t="n"/>
-      <c r="S20" s="13" t="n"/>
-      <c r="T20" s="13" t="n"/>
+        <v>3611.111111111111</v>
+      </c>
+      <c r="R20" s="13" t="n">
+        <v>3151000</v>
+      </c>
+      <c r="S20" s="13" t="n">
+        <v>185.3529411764706</v>
+      </c>
+      <c r="T20" s="13" t="n">
+        <v>16671.95767195767</v>
+      </c>
       <c r="U20" s="13" t="n">
-        <v>23270000</v>
+        <v>18465500</v>
       </c>
       <c r="V20" s="13" t="n">
-        <v>1368.823529411765</v>
+        <v>1086.205882352941</v>
       </c>
       <c r="W20" s="13" t="n">
-        <v>123121.6931216931</v>
-      </c>
-      <c r="X20" s="13" t="n"/>
-      <c r="Y20" s="13" t="n"/>
-      <c r="Z20" s="13" t="n"/>
+        <v>97701.0582010582</v>
+      </c>
+      <c r="X20" s="13" t="n">
+        <v>5260500</v>
+      </c>
+      <c r="Y20" s="13" t="n">
+        <v>309.4411764705882</v>
+      </c>
+      <c r="Z20" s="13" t="n">
+        <v>27833.33333333333</v>
+      </c>
       <c r="AA20" s="13" t="n">
-        <v>23270000</v>
+        <v>23726000</v>
       </c>
       <c r="AB20" s="13" t="n">
-        <v>1368.823529411765</v>
+        <v>1395.647058823529</v>
       </c>
       <c r="AC20" s="13" t="n">
-        <v>123121.6931216931</v>
+        <v>125534.3915343915</v>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">        Scrap Sales</t>
+          <t xml:space="preserve">        CV Adni Diffa Swandana</t>
         </is>
       </c>
       <c r="C21" s="11" t="n"/>
@@ -2036,68 +2066,44 @@
       <c r="F21" s="11" t="n"/>
       <c r="G21" s="11" t="n"/>
       <c r="H21" s="11" t="n"/>
-      <c r="I21" s="11" t="n">
-        <v>1673000</v>
-      </c>
-      <c r="J21" s="11" t="n">
-        <v>98.41176470588235</v>
-      </c>
-      <c r="K21" s="11" t="n">
-        <v>8851.851851851852</v>
-      </c>
-      <c r="L21" s="11" t="n">
-        <v>12959000</v>
-      </c>
-      <c r="M21" s="11" t="n">
-        <v>762.2941176470588</v>
-      </c>
-      <c r="N21" s="11" t="n">
-        <v>68566.13756613756</v>
-      </c>
+      <c r="I21" s="11" t="n"/>
+      <c r="J21" s="11" t="n"/>
+      <c r="K21" s="11" t="n"/>
+      <c r="L21" s="11" t="n"/>
+      <c r="M21" s="11" t="n"/>
+      <c r="N21" s="11" t="n"/>
       <c r="O21" s="11" t="n">
-        <v>682500</v>
+        <v>23270000</v>
       </c>
       <c r="P21" s="11" t="n">
-        <v>40.14705882352941</v>
+        <v>1368.823529411765</v>
       </c>
       <c r="Q21" s="11" t="n">
-        <v>3611.111111111111</v>
-      </c>
-      <c r="R21" s="11" t="n">
-        <v>3151000</v>
-      </c>
-      <c r="S21" s="11" t="n">
-        <v>185.3529411764706</v>
-      </c>
-      <c r="T21" s="11" t="n">
-        <v>16671.95767195767</v>
-      </c>
+        <v>123121.6931216931</v>
+      </c>
+      <c r="R21" s="11" t="n"/>
+      <c r="S21" s="11" t="n"/>
+      <c r="T21" s="11" t="n"/>
       <c r="U21" s="11" t="n">
-        <v>18465500</v>
+        <v>23270000</v>
       </c>
       <c r="V21" s="11" t="n">
-        <v>1086.205882352941</v>
+        <v>1368.823529411765</v>
       </c>
       <c r="W21" s="11" t="n">
-        <v>97701.0582010582</v>
-      </c>
-      <c r="X21" s="11" t="n">
-        <v>4014500</v>
-      </c>
-      <c r="Y21" s="11" t="n">
-        <v>236.1470588235294</v>
-      </c>
-      <c r="Z21" s="11" t="n">
-        <v>21240.74074074074</v>
-      </c>
+        <v>123121.6931216931</v>
+      </c>
+      <c r="X21" s="11" t="n"/>
+      <c r="Y21" s="11" t="n"/>
+      <c r="Z21" s="11" t="n"/>
       <c r="AA21" s="11" t="n">
-        <v>22480000</v>
+        <v>23270000</v>
       </c>
       <c r="AB21" s="11" t="n">
-        <v>1322.35294117647</v>
+        <v>1368.823529411765</v>
       </c>
       <c r="AC21" s="11" t="n">
-        <v>118941.7989417989</v>
+        <v>123121.6931216931</v>
       </c>
     </row>
     <row r="22">
@@ -3144,22 +3150,22 @@
         <v>1088007982.878677</v>
       </c>
       <c r="X39" s="15" t="n">
-        <v>6925608467</v>
+        <v>6939574467</v>
       </c>
       <c r="Y39" s="15" t="n">
-        <v>407388.7333529412</v>
+        <v>408210.2627647059</v>
       </c>
       <c r="Z39" s="15" t="n">
-        <v>36643431.04232804</v>
+        <v>36717325.22222222</v>
       </c>
       <c r="AA39" s="15" t="n">
-        <v>212559117231.07</v>
+        <v>212573083231.07</v>
       </c>
       <c r="AB39" s="15" t="n">
-        <v>12503477.48418059</v>
+        <v>12504299.01359235</v>
       </c>
       <c r="AC39" s="15" t="n">
-        <v>1124651413.921005</v>
+        <v>1124725308.100899</v>
       </c>
     </row>
     <row r="40">
@@ -3321,7 +3327,7 @@
     <row r="43">
       <c r="B43" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">        Building Facility &amp; Infrastructure</t>
+          <t xml:space="preserve">        Building Facilities and Infrastructure</t>
         </is>
       </c>
       <c r="C43" s="13" t="n"/>
@@ -3379,7 +3385,7 @@
     <row r="44">
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">        CWIP - Building Facility &amp; Infrastructure</t>
+          <t xml:space="preserve">        CWIP - Building Facilities and Infrastructure</t>
         </is>
       </c>
       <c r="C44" s="11" t="n"/>
@@ -3404,22 +3410,22 @@
       <c r="V44" s="11" t="n"/>
       <c r="W44" s="11" t="n"/>
       <c r="X44" s="11" t="n">
-        <v>-172443500</v>
+        <v>-196234940</v>
       </c>
       <c r="Y44" s="11" t="n">
-        <v>-10143.73529411765</v>
+        <v>-11543.23176470588</v>
       </c>
       <c r="Z44" s="11" t="n">
-        <v>-912399.4708994708</v>
+        <v>-1038280.105820106</v>
       </c>
       <c r="AA44" s="11" t="n">
-        <v>-172443500</v>
+        <v>-196234940</v>
       </c>
       <c r="AB44" s="11" t="n">
-        <v>-10143.73529411765</v>
+        <v>-11543.23176470588</v>
       </c>
       <c r="AC44" s="11" t="n">
-        <v>-912399.4708994708</v>
+        <v>-1038280.105820106</v>
       </c>
     </row>
     <row r="45">
@@ -4400,22 +4406,22 @@
         <v>-70651143.30624339</v>
       </c>
       <c r="X59" s="15" t="n">
-        <v>-915916607</v>
+        <v>-939708047</v>
       </c>
       <c r="Y59" s="15" t="n">
-        <v>-53877.44747058824</v>
+        <v>-55276.94394117647</v>
       </c>
       <c r="Z59" s="15" t="n">
-        <v>-4846119.613756614</v>
+        <v>-4972000.248677249</v>
       </c>
       <c r="AA59" s="15" t="n">
-        <v>-14268982691.88</v>
+        <v>-14292774131.88</v>
       </c>
       <c r="AB59" s="15" t="n">
-        <v>-839351.9230517646</v>
+        <v>-840751.4195223529</v>
       </c>
       <c r="AC59" s="15" t="n">
-        <v>-75497262.92</v>
+        <v>-75623143.55492064</v>
       </c>
     </row>
     <row r="60">
@@ -5856,22 +5862,22 @@
         <v>-535741.6243386244</v>
       </c>
       <c r="X84" s="11" t="n">
-        <v>-16999662</v>
+        <v>-17294034</v>
       </c>
       <c r="Y84" s="11" t="n">
-        <v>-999.9801176470588</v>
+        <v>-1017.296117647059</v>
       </c>
       <c r="Z84" s="11" t="n">
-        <v>-89945.30158730158</v>
+        <v>-91502.8253968254</v>
       </c>
       <c r="AA84" s="11" t="n">
-        <v>-118254829</v>
+        <v>-118549201</v>
       </c>
       <c r="AB84" s="11" t="n">
-        <v>-6956.166411764707</v>
+        <v>-6973.482411764707</v>
       </c>
       <c r="AC84" s="11" t="n">
-        <v>-625686.925925926</v>
+        <v>-627244.4497354499</v>
       </c>
     </row>
     <row r="85">
@@ -6282,22 +6288,22 @@
         <v>-999220.2245502645</v>
       </c>
       <c r="X90" s="15" t="n">
-        <v>-40779236</v>
+        <v>-41073608</v>
       </c>
       <c r="Y90" s="15" t="n">
-        <v>-2398.778588235294</v>
+        <v>-2416.094588235294</v>
       </c>
       <c r="Z90" s="15" t="n">
-        <v>-215763.1534391535</v>
+        <v>-217320.6772486772</v>
       </c>
       <c r="AA90" s="15" t="n">
-        <v>-229631858.44</v>
+        <v>-229926230.44</v>
       </c>
       <c r="AB90" s="15" t="n">
-        <v>-13507.75637882353</v>
+        <v>-13525.07237882353</v>
       </c>
       <c r="AC90" s="15" t="n">
-        <v>-1214983.377989418</v>
+        <v>-1216540.901798942</v>
       </c>
     </row>
     <row r="91">
@@ -6474,22 +6480,22 @@
         <v>-928151.4708994708</v>
       </c>
       <c r="X93" s="13" t="n">
-        <v>-10458793</v>
+        <v>-11413271</v>
       </c>
       <c r="Y93" s="13" t="n">
-        <v>-615.2231176470589</v>
+        <v>-671.3688823529412</v>
       </c>
       <c r="Z93" s="13" t="n">
-        <v>-55337.5291005291</v>
+        <v>-60387.67724867725</v>
       </c>
       <c r="AA93" s="13" t="n">
-        <v>-185879421</v>
+        <v>-186833899</v>
       </c>
       <c r="AB93" s="13" t="n">
-        <v>-10934.08358823529</v>
+        <v>-10990.22935294118</v>
       </c>
       <c r="AC93" s="13" t="n">
-        <v>-983489</v>
+        <v>-988539.1481481481</v>
       </c>
     </row>
     <row r="94">
@@ -6738,22 +6744,22 @@
         <v>-1461407.195767196</v>
       </c>
       <c r="X96" s="11" t="n">
-        <v>-14997022</v>
+        <v>-16927322</v>
       </c>
       <c r="Y96" s="11" t="n">
-        <v>-882.1777647058824</v>
+        <v>-995.7248235294118</v>
       </c>
       <c r="Z96" s="11" t="n">
-        <v>-79349.32275132275</v>
+        <v>-89562.55026455027</v>
       </c>
       <c r="AA96" s="11" t="n">
-        <v>-291202982</v>
+        <v>-293133282</v>
       </c>
       <c r="AB96" s="11" t="n">
-        <v>-17129.58717647059</v>
+        <v>-17243.13423529412</v>
       </c>
       <c r="AC96" s="11" t="n">
-        <v>-1540756.518518518</v>
+        <v>-1550969.746031746</v>
       </c>
     </row>
     <row r="97">
@@ -6826,22 +6832,22 @@
         <v>-35023514.69555555</v>
       </c>
       <c r="X97" s="15" t="n">
-        <v>-667402508</v>
+        <v>-670287286</v>
       </c>
       <c r="Y97" s="15" t="n">
-        <v>-39258.97105882353</v>
+        <v>-39428.66388235294</v>
       </c>
       <c r="Z97" s="15" t="n">
-        <v>-3531230.201058201</v>
+        <v>-3546493.576719576</v>
       </c>
       <c r="AA97" s="15" t="n">
-        <v>-7286846785.46</v>
+        <v>-7289731563.46</v>
       </c>
       <c r="AB97" s="15" t="n">
-        <v>-428638.0462035294</v>
+        <v>-428807.7390270588</v>
       </c>
       <c r="AC97" s="15" t="n">
-        <v>-38554744.89661375</v>
+        <v>-38570008.27227513</v>
       </c>
     </row>
     <row r="98">
@@ -6948,22 +6954,22 @@
         <v>-921841.8095238095</v>
       </c>
       <c r="X99" s="11" t="n">
-        <v>-8741825</v>
+        <v>-9003325</v>
       </c>
       <c r="Y99" s="11" t="n">
-        <v>-514.225</v>
+        <v>-529.6073529411765</v>
       </c>
       <c r="Z99" s="11" t="n">
-        <v>-46253.04232804233</v>
+        <v>-47636.64021164021</v>
       </c>
       <c r="AA99" s="11" t="n">
-        <v>-182969927</v>
+        <v>-183231427</v>
       </c>
       <c r="AB99" s="11" t="n">
-        <v>-10762.93688235294</v>
+        <v>-10778.31923529412</v>
       </c>
       <c r="AC99" s="11" t="n">
-        <v>-968094.8518518518</v>
+        <v>-969478.4497354496</v>
       </c>
     </row>
     <row r="100">
@@ -7036,22 +7042,22 @@
         <v>-682307.5502645504</v>
       </c>
       <c r="X100" s="13" t="n">
-        <v>-31091154</v>
+        <v>-31371654</v>
       </c>
       <c r="Y100" s="13" t="n">
-        <v>-1828.891411764706</v>
+        <v>-1845.391411764706</v>
       </c>
       <c r="Z100" s="13" t="n">
-        <v>-164503.4603174603</v>
+        <v>-165987.5873015873</v>
       </c>
       <c r="AA100" s="13" t="n">
-        <v>-160047281</v>
+        <v>-160327781</v>
       </c>
       <c r="AB100" s="13" t="n">
-        <v>-9414.545941176471</v>
+        <v>-9431.045941176471</v>
       </c>
       <c r="AC100" s="13" t="n">
-        <v>-846811.0105820107</v>
+        <v>-848295.1375661377</v>
       </c>
     </row>
     <row r="101">
@@ -7294,22 +7300,22 @@
         <v>-7477955.814814815</v>
       </c>
       <c r="X103" s="15" t="n">
-        <v>-277707221</v>
+        <v>-278249221</v>
       </c>
       <c r="Y103" s="15" t="n">
-        <v>-16335.71888235294</v>
+        <v>-16367.60123529412</v>
       </c>
       <c r="Z103" s="15" t="n">
-        <v>-1469350.375661376</v>
+        <v>-1472218.100529101</v>
       </c>
       <c r="AA103" s="15" t="n">
-        <v>-1691040870</v>
+        <v>-1691582870</v>
       </c>
       <c r="AB103" s="15" t="n">
-        <v>-99472.99235294119</v>
+        <v>-99504.87470588236</v>
       </c>
       <c r="AC103" s="15" t="n">
-        <v>-8947306.19047619</v>
+        <v>-8950173.915343916</v>
       </c>
     </row>
     <row r="104">
@@ -7556,22 +7562,22 @@
         <v>-1153318.253968254</v>
       </c>
       <c r="X107" s="11" t="n">
-        <v>-147572961</v>
+        <v>-147792961</v>
       </c>
       <c r="Y107" s="11" t="n">
-        <v>-8680.762411764706</v>
+        <v>-8693.703588235294</v>
       </c>
       <c r="Z107" s="11" t="n">
-        <v>-780809.3174603175</v>
+        <v>-781973.3386243386</v>
       </c>
       <c r="AA107" s="11" t="n">
-        <v>-365550111</v>
+        <v>-365770111</v>
       </c>
       <c r="AB107" s="11" t="n">
-        <v>-21502.94770588235</v>
+        <v>-21515.88888235294</v>
       </c>
       <c r="AC107" s="11" t="n">
-        <v>-1934127.571428571</v>
+        <v>-1935291.592592593</v>
       </c>
     </row>
     <row r="108">
@@ -7644,22 +7650,22 @@
         <v>-1839755.291005291</v>
       </c>
       <c r="X108" s="15" t="n">
-        <v>-157540461</v>
+        <v>-157760461</v>
       </c>
       <c r="Y108" s="15" t="n">
-        <v>-9267.08594117647</v>
+        <v>-9280.02711764706</v>
       </c>
       <c r="Z108" s="15" t="n">
-        <v>-833547.4126984127</v>
+        <v>-834711.4338624339</v>
       </c>
       <c r="AA108" s="15" t="n">
-        <v>-505254211</v>
+        <v>-505474211</v>
       </c>
       <c r="AB108" s="15" t="n">
-        <v>-29720.83594117647</v>
+        <v>-29733.77711764706</v>
       </c>
       <c r="AC108" s="15" t="n">
-        <v>-2673302.703703704</v>
+        <v>-2674466.724867725</v>
       </c>
     </row>
     <row r="109">
@@ -8192,22 +8198,22 @@
         <v>-21743746.34391534</v>
       </c>
       <c r="X116" s="11" t="n">
-        <v>-735604373</v>
+        <v>-714165559</v>
       </c>
       <c r="Y116" s="11" t="n">
-        <v>-43270.84547058823</v>
+        <v>-42009.73876470589</v>
       </c>
       <c r="Z116" s="11" t="n">
-        <v>-3892086.62962963</v>
+        <v>-3778653.751322751</v>
       </c>
       <c r="AA116" s="11" t="n">
-        <v>-4845172432</v>
+        <v>-4823733618</v>
       </c>
       <c r="AB116" s="11" t="n">
-        <v>-285010.1430588235</v>
+        <v>-283749.0363529412</v>
       </c>
       <c r="AC116" s="11" t="n">
-        <v>-25635832.97354497</v>
+        <v>-25522400.09523809</v>
       </c>
     </row>
     <row r="117">
@@ -8280,22 +8286,22 @@
         <v>-21743746.34391534</v>
       </c>
       <c r="X117" s="15" t="n">
-        <v>-735604373</v>
+        <v>-714165559</v>
       </c>
       <c r="Y117" s="15" t="n">
-        <v>-43270.84547058823</v>
+        <v>-42009.73876470589</v>
       </c>
       <c r="Z117" s="15" t="n">
-        <v>-3892086.62962963</v>
+        <v>-3778653.751322751</v>
       </c>
       <c r="AA117" s="15" t="n">
-        <v>-4845172432</v>
+        <v>-4823733618</v>
       </c>
       <c r="AB117" s="15" t="n">
-        <v>-285010.1430588235</v>
+        <v>-283749.0363529412</v>
       </c>
       <c r="AC117" s="15" t="n">
-        <v>-25635832.97354497</v>
+        <v>-25522400.09523809</v>
       </c>
     </row>
     <row r="118">
@@ -8606,22 +8612,22 @@
         <v>-6957568.632116402</v>
       </c>
       <c r="X122" s="13" t="n">
-        <v>-240870006</v>
+        <v>-243375606</v>
       </c>
       <c r="Y122" s="13" t="n">
-        <v>-14168.82388235294</v>
+        <v>-14316.21211764706</v>
       </c>
       <c r="Z122" s="13" t="n">
-        <v>-1274444.476190476</v>
+        <v>-1287701.619047619</v>
       </c>
       <c r="AA122" s="13" t="n">
-        <v>-1555850477.47</v>
+        <v>-1558356077.47</v>
       </c>
       <c r="AB122" s="13" t="n">
-        <v>-91520.6163217647</v>
+        <v>-91668.00455705881</v>
       </c>
       <c r="AC122" s="13" t="n">
-        <v>-8232013.108306877</v>
+        <v>-8245270.251164021</v>
       </c>
     </row>
     <row r="123">
@@ -8858,22 +8864,22 @@
         <v>-117767567.0077778</v>
       </c>
       <c r="X125" s="15" t="n">
-        <v>-1138075150</v>
+        <v>-1140580750</v>
       </c>
       <c r="Y125" s="15" t="n">
-        <v>-66945.59705882354</v>
+        <v>-67092.98529411765</v>
       </c>
       <c r="Z125" s="15" t="n">
-        <v>-6021561.64021164</v>
+        <v>-6034818.783068783</v>
       </c>
       <c r="AA125" s="15" t="n">
-        <v>-23396145314.47</v>
+        <v>-23398650914.47</v>
       </c>
       <c r="AB125" s="15" t="n">
-        <v>-1376243.842027647</v>
+        <v>-1376391.230262941</v>
       </c>
       <c r="AC125" s="15" t="n">
-        <v>-123789128.6479894</v>
+        <v>-123802385.7908466</v>
       </c>
     </row>
     <row r="126">
@@ -8968,22 +8974,22 @@
         <v>-121546.9312169312</v>
       </c>
       <c r="X127" s="11" t="n">
-        <v>-3740950</v>
+        <v>-5518450</v>
       </c>
       <c r="Y127" s="11" t="n">
-        <v>-220.0558823529412</v>
+        <v>-324.614705882353</v>
       </c>
       <c r="Z127" s="11" t="n">
-        <v>-19793.38624338625</v>
+        <v>-29198.14814814815</v>
       </c>
       <c r="AA127" s="11" t="n">
-        <v>-26713320</v>
+        <v>-28490820</v>
       </c>
       <c r="AB127" s="11" t="n">
-        <v>-1571.371764705882</v>
+        <v>-1675.930588235294</v>
       </c>
       <c r="AC127" s="11" t="n">
-        <v>-141340.3174603175</v>
+        <v>-150745.0793650794</v>
       </c>
     </row>
     <row r="128">
@@ -9214,22 +9220,22 @@
         <v>-424776.1058201058</v>
       </c>
       <c r="X130" s="13" t="n">
-        <v>-12025744</v>
+        <v>-12327744</v>
       </c>
       <c r="Y130" s="13" t="n">
-        <v>-707.396705882353</v>
+        <v>-725.1614117647059</v>
       </c>
       <c r="Z130" s="13" t="n">
-        <v>-63628.27513227514</v>
+        <v>-65226.15873015873</v>
       </c>
       <c r="AA130" s="13" t="n">
-        <v>-92308428</v>
+        <v>-92610428</v>
       </c>
       <c r="AB130" s="13" t="n">
-        <v>-5429.907529411764</v>
+        <v>-5447.672235294117</v>
       </c>
       <c r="AC130" s="13" t="n">
-        <v>-488404.3809523809</v>
+        <v>-490002.2645502645</v>
       </c>
     </row>
     <row r="131">
@@ -9442,22 +9448,22 @@
         <v>-3233175.116402117</v>
       </c>
       <c r="X133" s="15" t="n">
-        <v>-99551384</v>
+        <v>-101630884</v>
       </c>
       <c r="Y133" s="15" t="n">
-        <v>-5855.963764705883</v>
+        <v>-5978.287294117647</v>
       </c>
       <c r="Z133" s="15" t="n">
-        <v>-526726.8994708995</v>
+        <v>-537729.544973545</v>
       </c>
       <c r="AA133" s="15" t="n">
-        <v>-710621481</v>
+        <v>-712700981</v>
       </c>
       <c r="AB133" s="15" t="n">
-        <v>-41801.26358823529</v>
+        <v>-41923.58711764705</v>
       </c>
       <c r="AC133" s="15" t="n">
-        <v>-3759902.015873016</v>
+        <v>-3770904.661375661</v>
       </c>
     </row>
     <row r="134">
@@ -9530,22 +9536,22 @@
         <v>-191744145.7268254</v>
       </c>
       <c r="X134" s="15" t="n">
-        <v>-3327374660</v>
+        <v>-3314462096</v>
       </c>
       <c r="Y134" s="15" t="n">
-        <v>-195727.9211764706</v>
+        <v>-194968.3585882353</v>
       </c>
       <c r="Z134" s="15" t="n">
-        <v>-17605156.93121693</v>
+        <v>-17536836.48677249</v>
       </c>
       <c r="AA134" s="15" t="n">
-        <v>-39567018202.37</v>
+        <v>-39554105638.37</v>
       </c>
       <c r="AB134" s="15" t="n">
-        <v>-2327471.658962942</v>
+        <v>-2326712.096374706</v>
       </c>
       <c r="AC134" s="15" t="n">
-        <v>-209349302.6580423</v>
+        <v>-209280982.2135978</v>
       </c>
     </row>
     <row r="135">
@@ -9680,22 +9686,22 @@
       <c r="V137" s="13" t="n"/>
       <c r="W137" s="13" t="n"/>
       <c r="X137" s="13" t="n">
-        <v>-5000000</v>
+        <v>-10000000</v>
       </c>
       <c r="Y137" s="13" t="n">
-        <v>-294.1176470588235</v>
+        <v>-588.2352941176471</v>
       </c>
       <c r="Z137" s="13" t="n">
-        <v>-26455.02645502645</v>
+        <v>-52910.05291005291</v>
       </c>
       <c r="AA137" s="13" t="n">
-        <v>-5000000</v>
+        <v>-10000000</v>
       </c>
       <c r="AB137" s="13" t="n">
-        <v>-294.1176470588235</v>
+        <v>-588.2352941176471</v>
       </c>
       <c r="AC137" s="13" t="n">
-        <v>-26455.02645502645</v>
+        <v>-52910.05291005291</v>
       </c>
     </row>
     <row r="138">
@@ -9768,22 +9774,22 @@
         <v>-3102749.708994709</v>
       </c>
       <c r="X138" s="11" t="n">
-        <v>-92351360</v>
+        <v>-142351360</v>
       </c>
       <c r="Y138" s="11" t="n">
-        <v>-5432.43294117647</v>
+        <v>-8373.609411764706</v>
       </c>
       <c r="Z138" s="11" t="n">
-        <v>-488631.5343915344</v>
+        <v>-753181.798941799</v>
       </c>
       <c r="AA138" s="11" t="n">
-        <v>-678771055</v>
+        <v>-728771055</v>
       </c>
       <c r="AB138" s="11" t="n">
-        <v>-39927.70911764706</v>
+        <v>-42868.88558823529</v>
       </c>
       <c r="AC138" s="11" t="n">
-        <v>-3591381.243386243</v>
+        <v>-3855931.507936508</v>
       </c>
     </row>
     <row r="139">
@@ -9960,22 +9966,22 @@
         <v>-11891707.38095238</v>
       </c>
       <c r="X141" s="15" t="n">
-        <v>-97351360</v>
+        <v>-152351360</v>
       </c>
       <c r="Y141" s="15" t="n">
-        <v>-5726.550588235295</v>
+        <v>-8961.844705882353</v>
       </c>
       <c r="Z141" s="15" t="n">
-        <v>-515086.5608465609</v>
+        <v>-806091.8518518518</v>
       </c>
       <c r="AA141" s="15" t="n">
-        <v>-2344884055</v>
+        <v>-2399884055</v>
       </c>
       <c r="AB141" s="15" t="n">
-        <v>-137934.3561764706</v>
+        <v>-141169.6502941177</v>
       </c>
       <c r="AC141" s="15" t="n">
-        <v>-12406793.94179894</v>
+        <v>-12697799.23280423</v>
       </c>
     </row>
     <row r="142">
@@ -10082,22 +10088,22 @@
         <v>-75097.76550264549</v>
       </c>
       <c r="X143" s="11" t="n">
-        <v>-2079254</v>
+        <v>-2107754</v>
       </c>
       <c r="Y143" s="11" t="n">
-        <v>-122.3090588235294</v>
+        <v>-123.9855294117647</v>
       </c>
       <c r="Z143" s="11" t="n">
-        <v>-11001.34391534392</v>
+        <v>-11152.13756613757</v>
       </c>
       <c r="AA143" s="11" t="n">
-        <v>-16272731.68</v>
+        <v>-16301231.68</v>
       </c>
       <c r="AB143" s="11" t="n">
-        <v>-957.2195105882353</v>
+        <v>-958.8959811764705</v>
       </c>
       <c r="AC143" s="11" t="n">
-        <v>-86099.1094179894</v>
+        <v>-86249.90306878305</v>
       </c>
     </row>
     <row r="144">
@@ -10508,22 +10514,22 @@
         <v>-28421640.40423281</v>
       </c>
       <c r="X149" s="15" t="n">
-        <v>-193641679</v>
+        <v>-193670179</v>
       </c>
       <c r="Y149" s="15" t="n">
-        <v>-11390.687</v>
+        <v>-11392.36347058824</v>
       </c>
       <c r="Z149" s="15" t="n">
-        <v>-1024559.148148148</v>
+        <v>-1024709.941798942</v>
       </c>
       <c r="AA149" s="15" t="n">
-        <v>-5565331715.4</v>
+        <v>-5565360215.4</v>
       </c>
       <c r="AB149" s="15" t="n">
-        <v>-327372.4538470588</v>
+        <v>-327374.130317647</v>
       </c>
       <c r="AC149" s="15" t="n">
-        <v>-29446199.55238096</v>
+        <v>-29446350.34603175</v>
       </c>
     </row>
     <row r="150">
@@ -10596,22 +10602,22 @@
         <v>-1435352458.064497</v>
       </c>
       <c r="X150" s="19" t="n">
-        <v>-7326525205</v>
+        <v>-7392432581</v>
       </c>
       <c r="Y150" s="19" t="n">
-        <v>-430972.0708823529</v>
+        <v>-434848.9753529412</v>
       </c>
       <c r="Z150" s="19" t="n">
-        <v>-38764683.62433863</v>
+        <v>-39113399.8994709</v>
       </c>
       <c r="AA150" s="19" t="n">
-        <v>-278608139779.19</v>
+        <v>-278674047155.19</v>
       </c>
       <c r="AB150" s="19" t="n">
-        <v>-16388714.10465823</v>
+        <v>-16392591.00912882</v>
       </c>
       <c r="AC150" s="19" t="n">
-        <v>-1474117141.688836</v>
+        <v>-1474465857.963968</v>
       </c>
     </row>
     <row r="151">
@@ -10684,22 +10690,22 @@
         <v>-347344475.1858202</v>
       </c>
       <c r="X151" s="19" t="n">
-        <v>-400916738</v>
+        <v>-452858114</v>
       </c>
       <c r="Y151" s="19" t="n">
-        <v>-23583.33752941176</v>
+        <v>-26638.7125882353</v>
       </c>
       <c r="Z151" s="19" t="n">
-        <v>-2121252.582010582</v>
+        <v>-2396074.677248677</v>
       </c>
       <c r="AA151" s="19" t="n">
-        <v>-66049022548.12001</v>
+        <v>-66100963924.12001</v>
       </c>
       <c r="AB151" s="19" t="n">
-        <v>-3885236.620477648</v>
+        <v>-3888291.995536471</v>
       </c>
       <c r="AC151" s="19" t="n">
-        <v>-349465727.7678308</v>
+        <v>-349740549.8630689</v>
       </c>
     </row>
     <row r="152">
@@ -10772,22 +10778,22 @@
         <v>9659021.249947079</v>
       </c>
       <c r="X152" s="7" t="n">
-        <v>1424638278.239998</v>
+        <v>1372696902.239998</v>
       </c>
       <c r="Y152" s="7" t="n">
-        <v>83802.25166117634</v>
+        <v>80746.87660235282</v>
       </c>
       <c r="Z152" s="7" t="n">
-        <v>7537768.667936496</v>
+        <v>7262946.572698401</v>
       </c>
       <c r="AA152" s="7" t="n">
-        <v>1424638278.239998</v>
+        <v>1372696902.239998</v>
       </c>
       <c r="AB152" s="7" t="n">
-        <v>83802.25166117634</v>
+        <v>80746.87660235282</v>
       </c>
       <c r="AC152" s="7" t="n">
-        <v>7537768.667936496</v>
+        <v>7262946.572698401</v>
       </c>
     </row>
   </sheetData>
@@ -10861,7 +10867,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 29 Jul 2026 09:06 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 29 Jul 2026 16:15 (in IDR Million)</t>
         </is>
       </c>
     </row>
@@ -11265,22 +11271,22 @@
         <v>822.5205241798942</v>
       </c>
       <c r="X7" s="11" t="n">
-        <v>6895.316417</v>
+        <v>6908.036417</v>
       </c>
       <c r="Y7" s="11" t="n">
-        <v>0.4056068480588235</v>
+        <v>0.4063550833529412</v>
       </c>
       <c r="Z7" s="11" t="n">
-        <v>36.48315564550265</v>
+        <v>36.55045723280423</v>
       </c>
       <c r="AA7" s="11" t="n">
-        <v>162351.695487</v>
+        <v>162364.415487</v>
       </c>
       <c r="AB7" s="11" t="n">
-        <v>9.550099734529411</v>
+        <v>9.550847969823529</v>
       </c>
       <c r="AC7" s="11" t="n">
-        <v>859.0036798253968</v>
+        <v>859.0709814126984</v>
       </c>
     </row>
     <row r="8">
@@ -11772,17 +11778,23 @@
       <c r="W14" s="13" t="n">
         <v>0.1491428571428571</v>
       </c>
-      <c r="X14" s="13" t="n"/>
-      <c r="Y14" s="13" t="n"/>
-      <c r="Z14" s="13" t="n"/>
+      <c r="X14" s="13" t="n">
+        <v>12.72</v>
+      </c>
+      <c r="Y14" s="13" t="n">
+        <v>0.0007482352941176471</v>
+      </c>
+      <c r="Z14" s="13" t="n">
+        <v>0.06730158730158731</v>
+      </c>
       <c r="AA14" s="13" t="n">
-        <v>28.188</v>
+        <v>40.908</v>
       </c>
       <c r="AB14" s="13" t="n">
-        <v>0.001658117647058823</v>
+        <v>0.002406352941176471</v>
       </c>
       <c r="AC14" s="13" t="n">
-        <v>0.1491428571428571</v>
+        <v>0.2164444444444444</v>
       </c>
     </row>
     <row r="15">
@@ -11959,22 +11971,22 @@
         <v>1.910739122063492</v>
       </c>
       <c r="X17" s="11" t="n">
-        <v>30.29205</v>
+        <v>31.53805</v>
       </c>
       <c r="Y17" s="11" t="n">
-        <v>0.001781885294117647</v>
+        <v>0.001855179411764706</v>
       </c>
       <c r="Z17" s="11" t="n">
-        <v>0.1602753968253968</v>
+        <v>0.1668679894179894</v>
       </c>
       <c r="AA17" s="11" t="n">
-        <v>391.4217440699999</v>
+        <v>392.6677440699999</v>
       </c>
       <c r="AB17" s="11" t="n">
-        <v>0.02302480847470588</v>
+        <v>0.02309810259235294</v>
       </c>
       <c r="AC17" s="11" t="n">
-        <v>2.071014518888889</v>
+        <v>2.077607111481481</v>
       </c>
     </row>
     <row r="18">
@@ -12114,7 +12126,7 @@
     <row r="20">
       <c r="B20" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">        CV Adni Diffa Swandana</t>
+          <t xml:space="preserve">        Scrap Sales</t>
         </is>
       </c>
       <c r="C20" s="13" t="n"/>
@@ -12123,50 +12135,74 @@
       <c r="F20" s="13" t="n"/>
       <c r="G20" s="13" t="n"/>
       <c r="H20" s="13" t="n"/>
-      <c r="I20" s="13" t="n"/>
-      <c r="J20" s="13" t="n"/>
-      <c r="K20" s="13" t="n"/>
-      <c r="L20" s="13" t="n"/>
-      <c r="M20" s="13" t="n"/>
-      <c r="N20" s="13" t="n"/>
+      <c r="I20" s="13" t="n">
+        <v>1.673</v>
+      </c>
+      <c r="J20" s="13" t="n">
+        <v>9.841176470588236e-05</v>
+      </c>
+      <c r="K20" s="13" t="n">
+        <v>0.008851851851851852</v>
+      </c>
+      <c r="L20" s="13" t="n">
+        <v>12.959</v>
+      </c>
+      <c r="M20" s="13" t="n">
+        <v>0.0007622941176470588</v>
+      </c>
+      <c r="N20" s="13" t="n">
+        <v>0.06856613756613757</v>
+      </c>
       <c r="O20" s="13" t="n">
-        <v>23.27</v>
+        <v>0.6825</v>
       </c>
       <c r="P20" s="13" t="n">
-        <v>0.001368823529411765</v>
+        <v>4.014705882352941e-05</v>
       </c>
       <c r="Q20" s="13" t="n">
-        <v>0.1231216931216931</v>
-      </c>
-      <c r="R20" s="13" t="n"/>
-      <c r="S20" s="13" t="n"/>
-      <c r="T20" s="13" t="n"/>
+        <v>0.003611111111111111</v>
+      </c>
+      <c r="R20" s="13" t="n">
+        <v>3.151</v>
+      </c>
+      <c r="S20" s="13" t="n">
+        <v>0.0001853529411764706</v>
+      </c>
+      <c r="T20" s="13" t="n">
+        <v>0.01667195767195767</v>
+      </c>
       <c r="U20" s="13" t="n">
-        <v>23.27</v>
+        <v>18.4655</v>
       </c>
       <c r="V20" s="13" t="n">
-        <v>0.001368823529411765</v>
+        <v>0.001086205882352941</v>
       </c>
       <c r="W20" s="13" t="n">
-        <v>0.1231216931216931</v>
-      </c>
-      <c r="X20" s="13" t="n"/>
-      <c r="Y20" s="13" t="n"/>
-      <c r="Z20" s="13" t="n"/>
+        <v>0.09770105820105819</v>
+      </c>
+      <c r="X20" s="13" t="n">
+        <v>5.2605</v>
+      </c>
+      <c r="Y20" s="13" t="n">
+        <v>0.0003094411764705883</v>
+      </c>
+      <c r="Z20" s="13" t="n">
+        <v>0.02783333333333333</v>
+      </c>
       <c r="AA20" s="13" t="n">
-        <v>23.27</v>
+        <v>23.726</v>
       </c>
       <c r="AB20" s="13" t="n">
-        <v>0.001368823529411765</v>
+        <v>0.001395647058823529</v>
       </c>
       <c r="AC20" s="13" t="n">
-        <v>0.1231216931216931</v>
+        <v>0.1255343915343915</v>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">        Scrap Sales</t>
+          <t xml:space="preserve">        CV Adni Diffa Swandana</t>
         </is>
       </c>
       <c r="C21" s="11" t="n"/>
@@ -12175,68 +12211,44 @@
       <c r="F21" s="11" t="n"/>
       <c r="G21" s="11" t="n"/>
       <c r="H21" s="11" t="n"/>
-      <c r="I21" s="11" t="n">
-        <v>1.673</v>
-      </c>
-      <c r="J21" s="11" t="n">
-        <v>9.841176470588236e-05</v>
-      </c>
-      <c r="K21" s="11" t="n">
-        <v>0.008851851851851852</v>
-      </c>
-      <c r="L21" s="11" t="n">
-        <v>12.959</v>
-      </c>
-      <c r="M21" s="11" t="n">
-        <v>0.0007622941176470588</v>
-      </c>
-      <c r="N21" s="11" t="n">
-        <v>0.06856613756613757</v>
-      </c>
+      <c r="I21" s="11" t="n"/>
+      <c r="J21" s="11" t="n"/>
+      <c r="K21" s="11" t="n"/>
+      <c r="L21" s="11" t="n"/>
+      <c r="M21" s="11" t="n"/>
+      <c r="N21" s="11" t="n"/>
       <c r="O21" s="11" t="n">
-        <v>0.6825</v>
+        <v>23.27</v>
       </c>
       <c r="P21" s="11" t="n">
-        <v>4.014705882352941e-05</v>
+        <v>0.001368823529411765</v>
       </c>
       <c r="Q21" s="11" t="n">
-        <v>0.003611111111111111</v>
-      </c>
-      <c r="R21" s="11" t="n">
-        <v>3.151</v>
-      </c>
-      <c r="S21" s="11" t="n">
-        <v>0.0001853529411764706</v>
-      </c>
-      <c r="T21" s="11" t="n">
-        <v>0.01667195767195767</v>
-      </c>
+        <v>0.1231216931216931</v>
+      </c>
+      <c r="R21" s="11" t="n"/>
+      <c r="S21" s="11" t="n"/>
+      <c r="T21" s="11" t="n"/>
       <c r="U21" s="11" t="n">
-        <v>18.4655</v>
+        <v>23.27</v>
       </c>
       <c r="V21" s="11" t="n">
-        <v>0.001086205882352941</v>
+        <v>0.001368823529411765</v>
       </c>
       <c r="W21" s="11" t="n">
-        <v>0.09770105820105819</v>
-      </c>
-      <c r="X21" s="11" t="n">
-        <v>4.0145</v>
-      </c>
-      <c r="Y21" s="11" t="n">
-        <v>0.0002361470588235294</v>
-      </c>
-      <c r="Z21" s="11" t="n">
-        <v>0.02124074074074074</v>
-      </c>
+        <v>0.1231216931216931</v>
+      </c>
+      <c r="X21" s="11" t="n"/>
+      <c r="Y21" s="11" t="n"/>
+      <c r="Z21" s="11" t="n"/>
       <c r="AA21" s="11" t="n">
-        <v>22.48</v>
+        <v>23.27</v>
       </c>
       <c r="AB21" s="11" t="n">
-        <v>0.001322352941176471</v>
+        <v>0.001368823529411765</v>
       </c>
       <c r="AC21" s="11" t="n">
-        <v>0.1189417989417989</v>
+        <v>0.1231216931216931</v>
       </c>
     </row>
     <row r="22">
@@ -13283,22 +13295,22 @@
         <v>1088.007982878677</v>
       </c>
       <c r="X39" s="15" t="n">
-        <v>6925.608467</v>
+        <v>6939.574467</v>
       </c>
       <c r="Y39" s="15" t="n">
-        <v>0.4073887333529412</v>
+        <v>0.4082102627647059</v>
       </c>
       <c r="Z39" s="15" t="n">
-        <v>36.64343104232804</v>
+        <v>36.71732522222222</v>
       </c>
       <c r="AA39" s="15" t="n">
-        <v>212559.11723107</v>
+        <v>212573.08323107</v>
       </c>
       <c r="AB39" s="15" t="n">
-        <v>12.50347748418059</v>
+        <v>12.50429901359235</v>
       </c>
       <c r="AC39" s="15" t="n">
-        <v>1124.651413921005</v>
+        <v>1124.725308100899</v>
       </c>
     </row>
     <row r="40">
@@ -13460,7 +13472,7 @@
     <row r="43">
       <c r="B43" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">        Building Facility &amp; Infrastructure</t>
+          <t xml:space="preserve">        Building Facilities and Infrastructure</t>
         </is>
       </c>
       <c r="C43" s="13" t="n"/>
@@ -13518,7 +13530,7 @@
     <row r="44">
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">        CWIP - Building Facility &amp; Infrastructure</t>
+          <t xml:space="preserve">        CWIP - Building Facilities and Infrastructure</t>
         </is>
       </c>
       <c r="C44" s="11" t="n"/>
@@ -13543,22 +13555,22 @@
       <c r="V44" s="11" t="n"/>
       <c r="W44" s="11" t="n"/>
       <c r="X44" s="11" t="n">
-        <v>-172.4435</v>
+        <v>-196.23494</v>
       </c>
       <c r="Y44" s="11" t="n">
-        <v>-0.01014373529411765</v>
+        <v>-0.01154323176470588</v>
       </c>
       <c r="Z44" s="11" t="n">
-        <v>-0.9123994708994709</v>
+        <v>-1.038280105820106</v>
       </c>
       <c r="AA44" s="11" t="n">
-        <v>-172.4435</v>
+        <v>-196.23494</v>
       </c>
       <c r="AB44" s="11" t="n">
-        <v>-0.01014373529411765</v>
+        <v>-0.01154323176470588</v>
       </c>
       <c r="AC44" s="11" t="n">
-        <v>-0.9123994708994709</v>
+        <v>-1.038280105820106</v>
       </c>
     </row>
     <row r="45">
@@ -14539,22 +14551,22 @@
         <v>-70.65114330624338</v>
       </c>
       <c r="X59" s="15" t="n">
-        <v>-915.916607</v>
+        <v>-939.708047</v>
       </c>
       <c r="Y59" s="15" t="n">
-        <v>-0.05387744747058824</v>
+        <v>-0.05527694394117647</v>
       </c>
       <c r="Z59" s="15" t="n">
-        <v>-4.846119613756613</v>
+        <v>-4.972000248677248</v>
       </c>
       <c r="AA59" s="15" t="n">
-        <v>-14268.98269188</v>
+        <v>-14292.77413188</v>
       </c>
       <c r="AB59" s="15" t="n">
-        <v>-0.8393519230517646</v>
+        <v>-0.8407514195223529</v>
       </c>
       <c r="AC59" s="15" t="n">
-        <v>-75.49726292</v>
+        <v>-75.62314355492063</v>
       </c>
     </row>
     <row r="60">
@@ -15995,22 +16007,22 @@
         <v>-0.5357416243386244</v>
       </c>
       <c r="X84" s="11" t="n">
-        <v>-16.999662</v>
+        <v>-17.294034</v>
       </c>
       <c r="Y84" s="11" t="n">
-        <v>-0.0009999801176470589</v>
+        <v>-0.001017296117647059</v>
       </c>
       <c r="Z84" s="11" t="n">
-        <v>-0.08994530158730159</v>
+        <v>-0.0915028253968254</v>
       </c>
       <c r="AA84" s="11" t="n">
-        <v>-118.254829</v>
+        <v>-118.549201</v>
       </c>
       <c r="AB84" s="11" t="n">
-        <v>-0.006956166411764706</v>
+        <v>-0.006973482411764706</v>
       </c>
       <c r="AC84" s="11" t="n">
-        <v>-0.625686925925926</v>
+        <v>-0.6272444497354498</v>
       </c>
     </row>
     <row r="85">
@@ -16421,22 +16433,22 @@
         <v>-0.9992202245502645</v>
       </c>
       <c r="X90" s="15" t="n">
-        <v>-40.779236</v>
+        <v>-41.073608</v>
       </c>
       <c r="Y90" s="15" t="n">
-        <v>-0.002398778588235294</v>
+        <v>-0.002416094588235294</v>
       </c>
       <c r="Z90" s="15" t="n">
-        <v>-0.2157631534391534</v>
+        <v>-0.2173206772486773</v>
       </c>
       <c r="AA90" s="15" t="n">
-        <v>-229.63185844</v>
+        <v>-229.92623044</v>
       </c>
       <c r="AB90" s="15" t="n">
-        <v>-0.01350775637882353</v>
+        <v>-0.01352507237882353</v>
       </c>
       <c r="AC90" s="15" t="n">
-        <v>-1.214983377989418</v>
+        <v>-1.216540901798942</v>
       </c>
     </row>
     <row r="91">
@@ -16613,22 +16625,22 @@
         <v>-0.9281514708994709</v>
       </c>
       <c r="X93" s="13" t="n">
-        <v>-10.458793</v>
+        <v>-11.413271</v>
       </c>
       <c r="Y93" s="13" t="n">
-        <v>-0.0006152231176470588</v>
+        <v>-0.0006713688823529411</v>
       </c>
       <c r="Z93" s="13" t="n">
-        <v>-0.0553375291005291</v>
+        <v>-0.06038767724867725</v>
       </c>
       <c r="AA93" s="13" t="n">
-        <v>-185.879421</v>
+        <v>-186.833899</v>
       </c>
       <c r="AB93" s="13" t="n">
-        <v>-0.01093408358823529</v>
+        <v>-0.01099022935294118</v>
       </c>
       <c r="AC93" s="13" t="n">
-        <v>-0.9834890000000001</v>
+        <v>-0.9885391481481481</v>
       </c>
     </row>
     <row r="94">
@@ -16877,22 +16889,22 @@
         <v>-1.461407195767196</v>
       </c>
       <c r="X96" s="11" t="n">
-        <v>-14.997022</v>
+        <v>-16.927322</v>
       </c>
       <c r="Y96" s="11" t="n">
-        <v>-0.0008821777647058823</v>
+        <v>-0.0009957248235294117</v>
       </c>
       <c r="Z96" s="11" t="n">
-        <v>-0.07934932275132275</v>
+        <v>-0.08956255026455026</v>
       </c>
       <c r="AA96" s="11" t="n">
-        <v>-291.202982</v>
+        <v>-293.133282</v>
       </c>
       <c r="AB96" s="11" t="n">
-        <v>-0.01712958717647059</v>
+        <v>-0.01724313423529412</v>
       </c>
       <c r="AC96" s="11" t="n">
-        <v>-1.540756518518518</v>
+        <v>-1.550969746031746</v>
       </c>
     </row>
     <row r="97">
@@ -16965,22 +16977,22 @@
         <v>-35.02351469555556</v>
       </c>
       <c r="X97" s="15" t="n">
-        <v>-667.402508</v>
+        <v>-670.287286</v>
       </c>
       <c r="Y97" s="15" t="n">
-        <v>-0.03925897105882353</v>
+        <v>-0.03942866388235294</v>
       </c>
       <c r="Z97" s="15" t="n">
-        <v>-3.531230201058201</v>
+        <v>-3.546493576719577</v>
       </c>
       <c r="AA97" s="15" t="n">
-        <v>-7286.846785459999</v>
+        <v>-7289.731563459999</v>
       </c>
       <c r="AB97" s="15" t="n">
-        <v>-0.4286380462035294</v>
+        <v>-0.4288077390270588</v>
       </c>
       <c r="AC97" s="15" t="n">
-        <v>-38.55474489661376</v>
+        <v>-38.57000827227514</v>
       </c>
     </row>
     <row r="98">
@@ -17087,22 +17099,22 @@
         <v>-0.9218418095238095</v>
       </c>
       <c r="X99" s="11" t="n">
-        <v>-8.741825</v>
+        <v>-9.003325</v>
       </c>
       <c r="Y99" s="11" t="n">
-        <v>-0.000514225</v>
+        <v>-0.0005296073529411765</v>
       </c>
       <c r="Z99" s="11" t="n">
-        <v>-0.04625304232804233</v>
+        <v>-0.04763664021164021</v>
       </c>
       <c r="AA99" s="11" t="n">
-        <v>-182.969927</v>
+        <v>-183.231427</v>
       </c>
       <c r="AB99" s="11" t="n">
-        <v>-0.01076293688235294</v>
+        <v>-0.01077831923529412</v>
       </c>
       <c r="AC99" s="11" t="n">
-        <v>-0.9680948518518517</v>
+        <v>-0.9694784497354496</v>
       </c>
     </row>
     <row r="100">
@@ -17175,22 +17187,22 @@
         <v>-0.6823075502645503</v>
       </c>
       <c r="X100" s="13" t="n">
-        <v>-31.091154</v>
+        <v>-31.371654</v>
       </c>
       <c r="Y100" s="13" t="n">
-        <v>-0.001828891411764706</v>
+        <v>-0.001845391411764706</v>
       </c>
       <c r="Z100" s="13" t="n">
-        <v>-0.1645034603174603</v>
+        <v>-0.1659875873015873</v>
       </c>
       <c r="AA100" s="13" t="n">
-        <v>-160.047281</v>
+        <v>-160.327781</v>
       </c>
       <c r="AB100" s="13" t="n">
-        <v>-0.00941454594117647</v>
+        <v>-0.009431045941176471</v>
       </c>
       <c r="AC100" s="13" t="n">
-        <v>-0.8468110105820106</v>
+        <v>-0.8482951375661376</v>
       </c>
     </row>
     <row r="101">
@@ -17433,22 +17445,22 @@
         <v>-7.477955814814814</v>
       </c>
       <c r="X103" s="15" t="n">
-        <v>-277.707221</v>
+        <v>-278.249221</v>
       </c>
       <c r="Y103" s="15" t="n">
-        <v>-0.01633571888235294</v>
+        <v>-0.01636760123529412</v>
       </c>
       <c r="Z103" s="15" t="n">
-        <v>-1.469350375661376</v>
+        <v>-1.4722181005291</v>
       </c>
       <c r="AA103" s="15" t="n">
-        <v>-1691.04087</v>
+        <v>-1691.58287</v>
       </c>
       <c r="AB103" s="15" t="n">
-        <v>-0.09947299235294117</v>
+        <v>-0.09950487470588235</v>
       </c>
       <c r="AC103" s="15" t="n">
-        <v>-8.947306190476191</v>
+        <v>-8.950173915343914</v>
       </c>
     </row>
     <row r="104">
@@ -17695,22 +17707,22 @@
         <v>-1.153318253968254</v>
       </c>
       <c r="X107" s="11" t="n">
-        <v>-147.572961</v>
+        <v>-147.792961</v>
       </c>
       <c r="Y107" s="11" t="n">
-        <v>-0.008680762411764706</v>
+        <v>-0.008693703588235294</v>
       </c>
       <c r="Z107" s="11" t="n">
-        <v>-0.7808093174603175</v>
+        <v>-0.7819733386243386</v>
       </c>
       <c r="AA107" s="11" t="n">
-        <v>-365.550111</v>
+        <v>-365.770111</v>
       </c>
       <c r="AB107" s="11" t="n">
-        <v>-0.02150294770588235</v>
+        <v>-0.02151588888235294</v>
       </c>
       <c r="AC107" s="11" t="n">
-        <v>-1.934127571428572</v>
+        <v>-1.935291592592593</v>
       </c>
     </row>
     <row r="108">
@@ -17783,22 +17795,22 @@
         <v>-1.839755291005291</v>
       </c>
       <c r="X108" s="15" t="n">
-        <v>-157.540461</v>
+        <v>-157.760461</v>
       </c>
       <c r="Y108" s="15" t="n">
-        <v>-0.00926708594117647</v>
+        <v>-0.009280027117647058</v>
       </c>
       <c r="Z108" s="15" t="n">
-        <v>-0.8335474126984127</v>
+        <v>-0.8347114338624338</v>
       </c>
       <c r="AA108" s="15" t="n">
-        <v>-505.254211</v>
+        <v>-505.474211</v>
       </c>
       <c r="AB108" s="15" t="n">
-        <v>-0.02972083594117647</v>
+        <v>-0.02973377711764706</v>
       </c>
       <c r="AC108" s="15" t="n">
-        <v>-2.673302703703704</v>
+        <v>-2.674466724867725</v>
       </c>
     </row>
     <row r="109">
@@ -18331,22 +18343,22 @@
         <v>-21.74374634391534</v>
       </c>
       <c r="X116" s="11" t="n">
-        <v>-735.604373</v>
+        <v>-714.165559</v>
       </c>
       <c r="Y116" s="11" t="n">
-        <v>-0.04327084547058824</v>
+        <v>-0.04200973876470589</v>
       </c>
       <c r="Z116" s="11" t="n">
-        <v>-3.89208662962963</v>
+        <v>-3.778653751322751</v>
       </c>
       <c r="AA116" s="11" t="n">
-        <v>-4845.172432</v>
+        <v>-4823.733618</v>
       </c>
       <c r="AB116" s="11" t="n">
-        <v>-0.2850101430588236</v>
+        <v>-0.2837490363529412</v>
       </c>
       <c r="AC116" s="11" t="n">
-        <v>-25.63583297354498</v>
+        <v>-25.52240009523809</v>
       </c>
     </row>
     <row r="117">
@@ -18419,22 +18431,22 @@
         <v>-21.74374634391534</v>
       </c>
       <c r="X117" s="15" t="n">
-        <v>-735.604373</v>
+        <v>-714.165559</v>
       </c>
       <c r="Y117" s="15" t="n">
-        <v>-0.04327084547058824</v>
+        <v>-0.04200973876470589</v>
       </c>
       <c r="Z117" s="15" t="n">
-        <v>-3.89208662962963</v>
+        <v>-3.778653751322751</v>
       </c>
       <c r="AA117" s="15" t="n">
-        <v>-4845.172432</v>
+        <v>-4823.733618</v>
       </c>
       <c r="AB117" s="15" t="n">
-        <v>-0.2850101430588236</v>
+        <v>-0.2837490363529412</v>
       </c>
       <c r="AC117" s="15" t="n">
-        <v>-25.63583297354498</v>
+        <v>-25.52240009523809</v>
       </c>
     </row>
     <row r="118">
@@ -18745,22 +18757,22 @@
         <v>-6.957568632116402</v>
       </c>
       <c r="X122" s="13" t="n">
-        <v>-240.870006</v>
+        <v>-243.375606</v>
       </c>
       <c r="Y122" s="13" t="n">
-        <v>-0.01416882388235294</v>
+        <v>-0.01431621211764706</v>
       </c>
       <c r="Z122" s="13" t="n">
-        <v>-1.274444476190476</v>
+        <v>-1.287701619047619</v>
       </c>
       <c r="AA122" s="13" t="n">
-        <v>-1555.85047747</v>
+        <v>-1558.35607747</v>
       </c>
       <c r="AB122" s="13" t="n">
-        <v>-0.0915206163217647</v>
+        <v>-0.09166800455705881</v>
       </c>
       <c r="AC122" s="13" t="n">
-        <v>-8.232013108306878</v>
+        <v>-8.245270251164021</v>
       </c>
     </row>
     <row r="123">
@@ -18997,22 +19009,22 @@
         <v>-117.7675670077778</v>
       </c>
       <c r="X125" s="15" t="n">
-        <v>-1138.07515</v>
+        <v>-1140.58075</v>
       </c>
       <c r="Y125" s="15" t="n">
-        <v>-0.06694559705882352</v>
+        <v>-0.06709298529411765</v>
       </c>
       <c r="Z125" s="15" t="n">
-        <v>-6.021561640211639</v>
+        <v>-6.034818783068784</v>
       </c>
       <c r="AA125" s="15" t="n">
-        <v>-23396.14531447</v>
+        <v>-23398.65091447</v>
       </c>
       <c r="AB125" s="15" t="n">
-        <v>-1.376243842027647</v>
+        <v>-1.376391230262941</v>
       </c>
       <c r="AC125" s="15" t="n">
-        <v>-123.7891286479894</v>
+        <v>-123.8023857908466</v>
       </c>
     </row>
     <row r="126">
@@ -19107,22 +19119,22 @@
         <v>-0.1215469312169312</v>
       </c>
       <c r="X127" s="11" t="n">
-        <v>-3.74095</v>
+        <v>-5.51845</v>
       </c>
       <c r="Y127" s="11" t="n">
-        <v>-0.0002200558823529412</v>
+        <v>-0.0003246147058823529</v>
       </c>
       <c r="Z127" s="11" t="n">
-        <v>-0.01979338624338624</v>
+        <v>-0.02919814814814815</v>
       </c>
       <c r="AA127" s="11" t="n">
-        <v>-26.71332</v>
+        <v>-28.49082</v>
       </c>
       <c r="AB127" s="11" t="n">
-        <v>-0.001571371764705882</v>
+        <v>-0.001675930588235294</v>
       </c>
       <c r="AC127" s="11" t="n">
-        <v>-0.1413403174603174</v>
+        <v>-0.1507450793650794</v>
       </c>
     </row>
     <row r="128">
@@ -19353,22 +19365,22 @@
         <v>-0.4247761058201058</v>
       </c>
       <c r="X130" s="13" t="n">
-        <v>-12.025744</v>
+        <v>-12.327744</v>
       </c>
       <c r="Y130" s="13" t="n">
-        <v>-0.0007073967058823529</v>
+        <v>-0.0007251614117647059</v>
       </c>
       <c r="Z130" s="13" t="n">
-        <v>-0.06362827513227513</v>
+        <v>-0.06522615873015873</v>
       </c>
       <c r="AA130" s="13" t="n">
-        <v>-92.30842800000001</v>
+        <v>-92.610428</v>
       </c>
       <c r="AB130" s="13" t="n">
-        <v>-0.005429907529411766</v>
+        <v>-0.005447672235294118</v>
       </c>
       <c r="AC130" s="13" t="n">
-        <v>-0.488404380952381</v>
+        <v>-0.4900022645502646</v>
       </c>
     </row>
     <row r="131">
@@ -19581,22 +19593,22 @@
         <v>-3.233175116402117</v>
       </c>
       <c r="X133" s="15" t="n">
-        <v>-99.551384</v>
+        <v>-101.630884</v>
       </c>
       <c r="Y133" s="15" t="n">
-        <v>-0.005855963764705882</v>
+        <v>-0.005978287294117647</v>
       </c>
       <c r="Z133" s="15" t="n">
-        <v>-0.5267268994708995</v>
+        <v>-0.537729544973545</v>
       </c>
       <c r="AA133" s="15" t="n">
-        <v>-710.621481</v>
+        <v>-712.7009810000001</v>
       </c>
       <c r="AB133" s="15" t="n">
-        <v>-0.04180126358823529</v>
+        <v>-0.04192358711764706</v>
       </c>
       <c r="AC133" s="15" t="n">
-        <v>-3.759902015873016</v>
+        <v>-3.770904661375662</v>
       </c>
     </row>
     <row r="134">
@@ -19669,22 +19681,22 @@
         <v>-191.7441457268254</v>
       </c>
       <c r="X134" s="15" t="n">
-        <v>-3327.37466</v>
+        <v>-3314.462096</v>
       </c>
       <c r="Y134" s="15" t="n">
-        <v>-0.1957279211764706</v>
+        <v>-0.1949683585882353</v>
       </c>
       <c r="Z134" s="15" t="n">
-        <v>-17.60515693121693</v>
+        <v>-17.53683648677249</v>
       </c>
       <c r="AA134" s="15" t="n">
-        <v>-39567.01820237</v>
+        <v>-39554.10563837001</v>
       </c>
       <c r="AB134" s="15" t="n">
-        <v>-2.327471658962941</v>
+        <v>-2.326712096374706</v>
       </c>
       <c r="AC134" s="15" t="n">
-        <v>-209.3493026580423</v>
+        <v>-209.2809822135978</v>
       </c>
     </row>
     <row r="135">
@@ -19819,22 +19831,22 @@
       <c r="V137" s="13" t="n"/>
       <c r="W137" s="13" t="n"/>
       <c r="X137" s="13" t="n">
-        <v>-5</v>
+        <v>-10</v>
       </c>
       <c r="Y137" s="13" t="n">
-        <v>-0.0002941176470588235</v>
+        <v>-0.000588235294117647</v>
       </c>
       <c r="Z137" s="13" t="n">
-        <v>-0.02645502645502645</v>
+        <v>-0.05291005291005291</v>
       </c>
       <c r="AA137" s="13" t="n">
-        <v>-5</v>
+        <v>-10</v>
       </c>
       <c r="AB137" s="13" t="n">
-        <v>-0.0002941176470588235</v>
+        <v>-0.000588235294117647</v>
       </c>
       <c r="AC137" s="13" t="n">
-        <v>-0.02645502645502645</v>
+        <v>-0.05291005291005291</v>
       </c>
     </row>
     <row r="138">
@@ -19907,22 +19919,22 @@
         <v>-3.102749708994709</v>
       </c>
       <c r="X138" s="11" t="n">
-        <v>-92.35136</v>
+        <v>-142.35136</v>
       </c>
       <c r="Y138" s="11" t="n">
-        <v>-0.00543243294117647</v>
+        <v>-0.008373609411764706</v>
       </c>
       <c r="Z138" s="11" t="n">
-        <v>-0.4886315343915344</v>
+        <v>-0.7531817989417989</v>
       </c>
       <c r="AA138" s="11" t="n">
-        <v>-678.771055</v>
+        <v>-728.771055</v>
       </c>
       <c r="AB138" s="11" t="n">
-        <v>-0.03992770911764706</v>
+        <v>-0.0428688855882353</v>
       </c>
       <c r="AC138" s="11" t="n">
-        <v>-3.591381243386243</v>
+        <v>-3.855931507936508</v>
       </c>
     </row>
     <row r="139">
@@ -20099,22 +20111,22 @@
         <v>-11.89170738095238</v>
       </c>
       <c r="X141" s="15" t="n">
-        <v>-97.35136</v>
+        <v>-152.35136</v>
       </c>
       <c r="Y141" s="15" t="n">
-        <v>-0.005726550588235294</v>
+        <v>-0.008961844705882353</v>
       </c>
       <c r="Z141" s="15" t="n">
-        <v>-0.5150865608465608</v>
+        <v>-0.8060918518518518</v>
       </c>
       <c r="AA141" s="15" t="n">
-        <v>-2344.884055</v>
+        <v>-2399.884055</v>
       </c>
       <c r="AB141" s="15" t="n">
-        <v>-0.1379343561764706</v>
+        <v>-0.1411696502941177</v>
       </c>
       <c r="AC141" s="15" t="n">
-        <v>-12.40679394179894</v>
+        <v>-12.69779923280423</v>
       </c>
     </row>
     <row r="142">
@@ -20221,22 +20233,22 @@
         <v>-0.07509776550264551</v>
       </c>
       <c r="X143" s="11" t="n">
-        <v>-2.079254</v>
+        <v>-2.107754</v>
       </c>
       <c r="Y143" s="11" t="n">
-        <v>-0.0001223090588235294</v>
+        <v>-0.0001239855294117647</v>
       </c>
       <c r="Z143" s="11" t="n">
-        <v>-0.01100134391534392</v>
+        <v>-0.01115213756613757</v>
       </c>
       <c r="AA143" s="11" t="n">
-        <v>-16.27273168</v>
+        <v>-16.30123168</v>
       </c>
       <c r="AB143" s="11" t="n">
-        <v>-0.0009572195105882354</v>
+        <v>-0.0009588959811764707</v>
       </c>
       <c r="AC143" s="11" t="n">
-        <v>-0.08609910941798943</v>
+        <v>-0.08624990306878307</v>
       </c>
     </row>
     <row r="144">
@@ -20647,22 +20659,22 @@
         <v>-28.4216404042328</v>
       </c>
       <c r="X149" s="15" t="n">
-        <v>-193.641679</v>
+        <v>-193.670179</v>
       </c>
       <c r="Y149" s="15" t="n">
-        <v>-0.011390687</v>
+        <v>-0.01139236347058823</v>
       </c>
       <c r="Z149" s="15" t="n">
-        <v>-1.024559148148148</v>
+        <v>-1.024709941798942</v>
       </c>
       <c r="AA149" s="15" t="n">
-        <v>-5565.3317154</v>
+        <v>-5565.360215399999</v>
       </c>
       <c r="AB149" s="15" t="n">
-        <v>-0.3273724538470589</v>
+        <v>-0.3273741303176471</v>
       </c>
       <c r="AC149" s="15" t="n">
-        <v>-29.44619955238095</v>
+        <v>-29.44635034603175</v>
       </c>
     </row>
     <row r="150">
@@ -20735,22 +20747,22 @@
         <v>-1435.352458064497</v>
       </c>
       <c r="X150" s="19" t="n">
-        <v>-7326.525205</v>
+        <v>-7392.432581</v>
       </c>
       <c r="Y150" s="19" t="n">
-        <v>-0.430972070882353</v>
+        <v>-0.4348489753529412</v>
       </c>
       <c r="Z150" s="19" t="n">
-        <v>-38.76468362433862</v>
+        <v>-39.1133998994709</v>
       </c>
       <c r="AA150" s="19" t="n">
-        <v>-278608.13977919</v>
+        <v>-278674.0471551899</v>
       </c>
       <c r="AB150" s="19" t="n">
-        <v>-16.38871410465823</v>
+        <v>-16.39259100912883</v>
       </c>
       <c r="AC150" s="19" t="n">
-        <v>-1474.117141688836</v>
+        <v>-1474.465857963968</v>
       </c>
     </row>
     <row r="151">
@@ -20823,22 +20835,22 @@
         <v>-347.3444751858202</v>
       </c>
       <c r="X151" s="19" t="n">
-        <v>-400.916738</v>
+        <v>-452.858114</v>
       </c>
       <c r="Y151" s="19" t="n">
-        <v>-0.02358333752941176</v>
+        <v>-0.0266387125882353</v>
       </c>
       <c r="Z151" s="19" t="n">
-        <v>-2.121252582010582</v>
+        <v>-2.396074677248677</v>
       </c>
       <c r="AA151" s="19" t="n">
-        <v>-66049.02254812002</v>
+        <v>-66100.96392412002</v>
       </c>
       <c r="AB151" s="19" t="n">
-        <v>-3.885236620477648</v>
+        <v>-3.888291995536472</v>
       </c>
       <c r="AC151" s="19" t="n">
-        <v>-349.4657277678308</v>
+        <v>-349.7405498630689</v>
       </c>
     </row>
     <row r="152">
@@ -20911,22 +20923,22 @@
         <v>9.659021249947079</v>
       </c>
       <c r="X152" s="7" t="n">
-        <v>1424.638278239998</v>
+        <v>1372.696902239998</v>
       </c>
       <c r="Y152" s="7" t="n">
-        <v>0.08380225166117634</v>
+        <v>0.08074687660235282</v>
       </c>
       <c r="Z152" s="7" t="n">
-        <v>7.537768667936496</v>
+        <v>7.262946572698401</v>
       </c>
       <c r="AA152" s="7" t="n">
-        <v>1424.638278239998</v>
+        <v>1372.696902239998</v>
       </c>
       <c r="AB152" s="7" t="n">
-        <v>0.08380225166117634</v>
+        <v>0.08074687660235282</v>
       </c>
       <c r="AC152" s="7" t="n">
-        <v>7.537768667936496</v>
+        <v>7.262946572698401</v>
       </c>
     </row>
   </sheetData>
@@ -23010,16 +23022,16 @@
         <v>631754694</v>
       </c>
       <c r="E6" s="11" t="n">
-        <v>366812219</v>
+        <v>-471576557</v>
       </c>
       <c r="F6" s="11" t="n">
-        <v>998566913</v>
+        <v>160178137</v>
       </c>
       <c r="G6" s="23" t="n">
-        <v>58739.23017647059</v>
+        <v>9422.243352941177</v>
       </c>
       <c r="H6" s="23" t="n">
-        <v>5283422.82010582</v>
+        <v>847503.3703703703</v>
       </c>
     </row>
     <row r="7">
@@ -23106,16 +23118,16 @@
         <v>310487173.9</v>
       </c>
       <c r="E9" s="13" t="n">
-        <v>-302049275</v>
+        <v>459398125</v>
       </c>
       <c r="F9" s="13" t="n">
-        <v>8437898.899999976</v>
+        <v>769885298.9</v>
       </c>
       <c r="G9" s="24" t="n">
-        <v>496.3469941176456</v>
+        <v>45287.37052352941</v>
       </c>
       <c r="H9" s="24" t="n">
-        <v>44644.9677248676</v>
+        <v>4073467.18994709</v>
       </c>
     </row>
     <row r="10">
@@ -23170,16 +23182,16 @@
         <v>534977305.5</v>
       </c>
       <c r="E11" s="13" t="n">
-        <v>-489146568</v>
+        <v>-464146568</v>
       </c>
       <c r="F11" s="13" t="n">
-        <v>45830737.5</v>
+        <v>70830737.5</v>
       </c>
       <c r="G11" s="24" t="n">
-        <v>2695.925735294118</v>
+        <v>4166.513970588236</v>
       </c>
       <c r="H11" s="24" t="n">
-        <v>242490.6746031746</v>
+        <v>374765.8068783069</v>
       </c>
     </row>
     <row r="12">
@@ -23225,13 +23237,13 @@
       <c r="D13" s="26" t="n"/>
       <c r="E13" s="26" t="n"/>
       <c r="F13" s="27" t="n">
-        <v>1424638280.24</v>
+        <v>1372696904.24</v>
       </c>
       <c r="G13" s="28" t="n">
-        <v>83802.25177882353</v>
+        <v>80746.87672</v>
       </c>
       <c r="H13" s="28" t="n">
-        <v>7537768.678518519</v>
+        <v>7262946.583280424</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh dashboard Fri 07/31/2026 13:59
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -722,7 +722,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 29 Jul 2026 16:15</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 31 Jul 2026 13:59</t>
         </is>
       </c>
     </row>
@@ -783,14 +783,14 @@
       <c r="W3" s="4" t="n"/>
       <c r="X3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 29 Jul 2026</t>
+          <t>MTD as of 31 Jul 2026</t>
         </is>
       </c>
       <c r="Y3" s="4" t="n"/>
       <c r="Z3" s="4" t="n"/>
       <c r="AA3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 29 Jul 2026</t>
+          <t>YTD as of 31 Jul 2026</t>
         </is>
       </c>
       <c r="AB3" s="4" t="n"/>
@@ -1826,22 +1826,22 @@
         <v>1910739.122063492</v>
       </c>
       <c r="X17" s="11" t="n">
-        <v>31538050</v>
+        <v>33995050</v>
       </c>
       <c r="Y17" s="11" t="n">
-        <v>1855.179411764706</v>
+        <v>1999.708823529412</v>
       </c>
       <c r="Z17" s="11" t="n">
-        <v>166867.9894179894</v>
+        <v>179867.9894179894</v>
       </c>
       <c r="AA17" s="11" t="n">
-        <v>392667744.07</v>
+        <v>395124744.07</v>
       </c>
       <c r="AB17" s="11" t="n">
-        <v>23098.10259235294</v>
+        <v>23242.63200411764</v>
       </c>
       <c r="AC17" s="11" t="n">
-        <v>2077607.111481482</v>
+        <v>2090607.111481482</v>
       </c>
     </row>
     <row r="18">
@@ -2036,22 +2036,22 @@
         <v>97701.0582010582</v>
       </c>
       <c r="X20" s="13" t="n">
-        <v>5260500</v>
+        <v>7717500</v>
       </c>
       <c r="Y20" s="13" t="n">
-        <v>309.4411764705882</v>
+        <v>453.9705882352941</v>
       </c>
       <c r="Z20" s="13" t="n">
-        <v>27833.33333333333</v>
+        <v>40833.33333333334</v>
       </c>
       <c r="AA20" s="13" t="n">
-        <v>23726000</v>
+        <v>26183000</v>
       </c>
       <c r="AB20" s="13" t="n">
-        <v>1395.647058823529</v>
+        <v>1540.176470588235</v>
       </c>
       <c r="AC20" s="13" t="n">
-        <v>125534.3915343915</v>
+        <v>138534.3915343915</v>
       </c>
     </row>
     <row r="21">
@@ -3150,22 +3150,22 @@
         <v>1088007982.878677</v>
       </c>
       <c r="X39" s="15" t="n">
-        <v>6939574467</v>
+        <v>6942031467</v>
       </c>
       <c r="Y39" s="15" t="n">
-        <v>408210.2627647059</v>
+        <v>408354.7921764706</v>
       </c>
       <c r="Z39" s="15" t="n">
-        <v>36717325.22222222</v>
+        <v>36730325.22222222</v>
       </c>
       <c r="AA39" s="15" t="n">
-        <v>212573083231.07</v>
+        <v>212575540231.07</v>
       </c>
       <c r="AB39" s="15" t="n">
-        <v>12504299.01359235</v>
+        <v>12504443.54300412</v>
       </c>
       <c r="AC39" s="15" t="n">
-        <v>1124725308.100899</v>
+        <v>1124738308.100899</v>
       </c>
     </row>
     <row r="40">
@@ -10379,17 +10379,23 @@
       <c r="W147" s="11" t="n">
         <v>-3400111.021164021</v>
       </c>
-      <c r="X147" s="11" t="n"/>
-      <c r="Y147" s="11" t="n"/>
-      <c r="Z147" s="11" t="n"/>
+      <c r="X147" s="11" t="n">
+        <v>-103034108</v>
+      </c>
+      <c r="Y147" s="11" t="n">
+        <v>-6060.829882352941</v>
+      </c>
+      <c r="Z147" s="11" t="n">
+        <v>-545154.0105820106</v>
+      </c>
       <c r="AA147" s="11" t="n">
-        <v>-642620983</v>
+        <v>-745655091</v>
       </c>
       <c r="AB147" s="11" t="n">
-        <v>-37801.23429411765</v>
+        <v>-43862.06417647059</v>
       </c>
       <c r="AC147" s="11" t="n">
-        <v>-3400111.021164021</v>
+        <v>-3945265.031746032</v>
       </c>
     </row>
     <row r="148">
@@ -10514,22 +10520,22 @@
         <v>-28421640.40423281</v>
       </c>
       <c r="X149" s="15" t="n">
-        <v>-193670179</v>
+        <v>-296704287</v>
       </c>
       <c r="Y149" s="15" t="n">
-        <v>-11392.36347058824</v>
+        <v>-17453.19335294118</v>
       </c>
       <c r="Z149" s="15" t="n">
-        <v>-1024709.941798942</v>
+        <v>-1569863.952380952</v>
       </c>
       <c r="AA149" s="15" t="n">
-        <v>-5565360215.4</v>
+        <v>-5668394323.4</v>
       </c>
       <c r="AB149" s="15" t="n">
-        <v>-327374.130317647</v>
+        <v>-333434.9602</v>
       </c>
       <c r="AC149" s="15" t="n">
-        <v>-29446350.34603175</v>
+        <v>-29991504.35661376</v>
       </c>
     </row>
     <row r="150">
@@ -10602,22 +10608,22 @@
         <v>-1435352458.064497</v>
       </c>
       <c r="X150" s="19" t="n">
-        <v>-7392432581</v>
+        <v>-7495466689</v>
       </c>
       <c r="Y150" s="19" t="n">
-        <v>-434848.9753529412</v>
+        <v>-440909.8052352941</v>
       </c>
       <c r="Z150" s="19" t="n">
-        <v>-39113399.8994709</v>
+        <v>-39658553.91005291</v>
       </c>
       <c r="AA150" s="19" t="n">
-        <v>-278674047155.19</v>
+        <v>-278777081263.19</v>
       </c>
       <c r="AB150" s="19" t="n">
-        <v>-16392591.00912882</v>
+        <v>-16398651.83901118</v>
       </c>
       <c r="AC150" s="19" t="n">
-        <v>-1474465857.963968</v>
+        <v>-1475011011.97455</v>
       </c>
     </row>
     <row r="151">
@@ -10690,22 +10696,22 @@
         <v>-347344475.1858202</v>
       </c>
       <c r="X151" s="19" t="n">
-        <v>-452858114</v>
+        <v>-553435222</v>
       </c>
       <c r="Y151" s="19" t="n">
-        <v>-26638.7125882353</v>
+        <v>-32555.01305882353</v>
       </c>
       <c r="Z151" s="19" t="n">
-        <v>-2396074.677248677</v>
+        <v>-2928228.687830688</v>
       </c>
       <c r="AA151" s="19" t="n">
-        <v>-66100963924.12001</v>
+        <v>-66201541032.12001</v>
       </c>
       <c r="AB151" s="19" t="n">
-        <v>-3888291.995536471</v>
+        <v>-3894208.29600706</v>
       </c>
       <c r="AC151" s="19" t="n">
-        <v>-349740549.8630689</v>
+        <v>-350272703.8736509</v>
       </c>
     </row>
     <row r="152">
@@ -10778,22 +10784,22 @@
         <v>9659021.249947079</v>
       </c>
       <c r="X152" s="7" t="n">
-        <v>1372696902.239998</v>
+        <v>1272119794.239998</v>
       </c>
       <c r="Y152" s="7" t="n">
-        <v>80746.87660235282</v>
+        <v>74830.57613176458</v>
       </c>
       <c r="Z152" s="7" t="n">
-        <v>7262946.572698401</v>
+        <v>6730792.562116391</v>
       </c>
       <c r="AA152" s="7" t="n">
-        <v>1372696902.239998</v>
+        <v>1272119794.239998</v>
       </c>
       <c r="AB152" s="7" t="n">
-        <v>80746.87660235282</v>
+        <v>74830.57613176458</v>
       </c>
       <c r="AC152" s="7" t="n">
-        <v>7262946.572698401</v>
+        <v>6730792.562116391</v>
       </c>
     </row>
   </sheetData>
@@ -10867,7 +10873,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 29 Jul 2026 16:15 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 31 Jul 2026 13:59 (in IDR Million)</t>
         </is>
       </c>
     </row>
@@ -10928,14 +10934,14 @@
       <c r="W3" s="4" t="n"/>
       <c r="X3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 29 Jul 2026</t>
+          <t>MTD as of 31 Jul 2026</t>
         </is>
       </c>
       <c r="Y3" s="4" t="n"/>
       <c r="Z3" s="4" t="n"/>
       <c r="AA3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 29 Jul 2026</t>
+          <t>YTD as of 31 Jul 2026</t>
         </is>
       </c>
       <c r="AB3" s="4" t="n"/>
@@ -11971,22 +11977,22 @@
         <v>1.910739122063492</v>
       </c>
       <c r="X17" s="11" t="n">
-        <v>31.53805</v>
+        <v>33.99505</v>
       </c>
       <c r="Y17" s="11" t="n">
-        <v>0.001855179411764706</v>
+        <v>0.001999708823529412</v>
       </c>
       <c r="Z17" s="11" t="n">
-        <v>0.1668679894179894</v>
+        <v>0.1798679894179894</v>
       </c>
       <c r="AA17" s="11" t="n">
-        <v>392.6677440699999</v>
+        <v>395.1247440699999</v>
       </c>
       <c r="AB17" s="11" t="n">
-        <v>0.02309810259235294</v>
+        <v>0.02324263200411765</v>
       </c>
       <c r="AC17" s="11" t="n">
-        <v>2.077607111481481</v>
+        <v>2.090607111481482</v>
       </c>
     </row>
     <row r="18">
@@ -12181,22 +12187,22 @@
         <v>0.09770105820105819</v>
       </c>
       <c r="X20" s="13" t="n">
-        <v>5.2605</v>
+        <v>7.7175</v>
       </c>
       <c r="Y20" s="13" t="n">
-        <v>0.0003094411764705883</v>
+        <v>0.0004539705882352941</v>
       </c>
       <c r="Z20" s="13" t="n">
-        <v>0.02783333333333333</v>
+        <v>0.04083333333333333</v>
       </c>
       <c r="AA20" s="13" t="n">
-        <v>23.726</v>
+        <v>26.183</v>
       </c>
       <c r="AB20" s="13" t="n">
-        <v>0.001395647058823529</v>
+        <v>0.001540176470588235</v>
       </c>
       <c r="AC20" s="13" t="n">
-        <v>0.1255343915343915</v>
+        <v>0.1385343915343915</v>
       </c>
     </row>
     <row r="21">
@@ -13295,22 +13301,22 @@
         <v>1088.007982878677</v>
       </c>
       <c r="X39" s="15" t="n">
-        <v>6939.574467</v>
+        <v>6942.031467</v>
       </c>
       <c r="Y39" s="15" t="n">
-        <v>0.4082102627647059</v>
+        <v>0.4083547921764706</v>
       </c>
       <c r="Z39" s="15" t="n">
-        <v>36.71732522222222</v>
+        <v>36.73032522222222</v>
       </c>
       <c r="AA39" s="15" t="n">
-        <v>212573.08323107</v>
+        <v>212575.54023107</v>
       </c>
       <c r="AB39" s="15" t="n">
-        <v>12.50429901359235</v>
+        <v>12.50444354300412</v>
       </c>
       <c r="AC39" s="15" t="n">
-        <v>1124.725308100899</v>
+        <v>1124.7383081009</v>
       </c>
     </row>
     <row r="40">
@@ -20524,17 +20530,23 @@
       <c r="W147" s="11" t="n">
         <v>-3.400111021164021</v>
       </c>
-      <c r="X147" s="11" t="n"/>
-      <c r="Y147" s="11" t="n"/>
-      <c r="Z147" s="11" t="n"/>
+      <c r="X147" s="11" t="n">
+        <v>-103.034108</v>
+      </c>
+      <c r="Y147" s="11" t="n">
+        <v>-0.006060829882352942</v>
+      </c>
+      <c r="Z147" s="11" t="n">
+        <v>-0.5451540105820106</v>
+      </c>
       <c r="AA147" s="11" t="n">
-        <v>-642.620983</v>
+        <v>-745.6550910000001</v>
       </c>
       <c r="AB147" s="11" t="n">
-        <v>-0.03780123429411764</v>
+        <v>-0.04386206417647059</v>
       </c>
       <c r="AC147" s="11" t="n">
-        <v>-3.400111021164021</v>
+        <v>-3.945265031746032</v>
       </c>
     </row>
     <row r="148">
@@ -20659,22 +20671,22 @@
         <v>-28.4216404042328</v>
       </c>
       <c r="X149" s="15" t="n">
-        <v>-193.670179</v>
+        <v>-296.704287</v>
       </c>
       <c r="Y149" s="15" t="n">
-        <v>-0.01139236347058823</v>
+        <v>-0.01745319335294118</v>
       </c>
       <c r="Z149" s="15" t="n">
-        <v>-1.024709941798942</v>
+        <v>-1.569863952380953</v>
       </c>
       <c r="AA149" s="15" t="n">
-        <v>-5565.360215399999</v>
+        <v>-5668.3943234</v>
       </c>
       <c r="AB149" s="15" t="n">
-        <v>-0.3273741303176471</v>
+        <v>-0.3334349602</v>
       </c>
       <c r="AC149" s="15" t="n">
-        <v>-29.44635034603175</v>
+        <v>-29.99150435661376</v>
       </c>
     </row>
     <row r="150">
@@ -20747,22 +20759,22 @@
         <v>-1435.352458064497</v>
       </c>
       <c r="X150" s="19" t="n">
-        <v>-7392.432581</v>
+        <v>-7495.466689</v>
       </c>
       <c r="Y150" s="19" t="n">
-        <v>-0.4348489753529412</v>
+        <v>-0.4409098052352941</v>
       </c>
       <c r="Z150" s="19" t="n">
-        <v>-39.1133998994709</v>
+        <v>-39.65855391005291</v>
       </c>
       <c r="AA150" s="19" t="n">
-        <v>-278674.0471551899</v>
+        <v>-278777.08126319</v>
       </c>
       <c r="AB150" s="19" t="n">
-        <v>-16.39259100912883</v>
+        <v>-16.39865183901118</v>
       </c>
       <c r="AC150" s="19" t="n">
-        <v>-1474.465857963968</v>
+        <v>-1475.01101197455</v>
       </c>
     </row>
     <row r="151">
@@ -20835,22 +20847,22 @@
         <v>-347.3444751858202</v>
       </c>
       <c r="X151" s="19" t="n">
-        <v>-452.858114</v>
+        <v>-553.435222</v>
       </c>
       <c r="Y151" s="19" t="n">
-        <v>-0.0266387125882353</v>
+        <v>-0.03255501305882353</v>
       </c>
       <c r="Z151" s="19" t="n">
-        <v>-2.396074677248677</v>
+        <v>-2.928228687830688</v>
       </c>
       <c r="AA151" s="19" t="n">
-        <v>-66100.96392412002</v>
+        <v>-66201.54103212002</v>
       </c>
       <c r="AB151" s="19" t="n">
-        <v>-3.888291995536472</v>
+        <v>-3.89420829600706</v>
       </c>
       <c r="AC151" s="19" t="n">
-        <v>-349.7405498630689</v>
+        <v>-350.2727038736509</v>
       </c>
     </row>
     <row r="152">
@@ -20923,22 +20935,22 @@
         <v>9.659021249947079</v>
       </c>
       <c r="X152" s="7" t="n">
-        <v>1372.696902239998</v>
+        <v>1272.119794239998</v>
       </c>
       <c r="Y152" s="7" t="n">
-        <v>0.08074687660235282</v>
+        <v>0.07483057613176458</v>
       </c>
       <c r="Z152" s="7" t="n">
-        <v>7.262946572698401</v>
+        <v>6.730792562116391</v>
       </c>
       <c r="AA152" s="7" t="n">
-        <v>1372.696902239998</v>
+        <v>1272.119794239998</v>
       </c>
       <c r="AB152" s="7" t="n">
-        <v>0.08074687660235282</v>
+        <v>0.07483057613176458</v>
       </c>
       <c r="AC152" s="7" t="n">
-        <v>7.262946572698401</v>
+        <v>6.730792562116391</v>
       </c>
     </row>
   </sheetData>
@@ -23022,16 +23034,16 @@
         <v>631754694</v>
       </c>
       <c r="E6" s="11" t="n">
-        <v>-471576557</v>
+        <v>-574610665</v>
       </c>
       <c r="F6" s="11" t="n">
-        <v>160178137</v>
+        <v>57144029</v>
       </c>
       <c r="G6" s="23" t="n">
-        <v>9422.243352941177</v>
+        <v>3361.413470588235</v>
       </c>
       <c r="H6" s="23" t="n">
-        <v>847503.3703703703</v>
+        <v>302349.3597883598</v>
       </c>
     </row>
     <row r="7">
@@ -23118,16 +23130,16 @@
         <v>310487173.9</v>
       </c>
       <c r="E9" s="13" t="n">
-        <v>459398125</v>
+        <v>461855125</v>
       </c>
       <c r="F9" s="13" t="n">
-        <v>769885298.9</v>
+        <v>772342298.9</v>
       </c>
       <c r="G9" s="24" t="n">
-        <v>45287.37052352941</v>
+        <v>45431.89993529412</v>
       </c>
       <c r="H9" s="24" t="n">
-        <v>4073467.18994709</v>
+        <v>4086467.18994709</v>
       </c>
     </row>
     <row r="10">
@@ -23237,13 +23249,13 @@
       <c r="D13" s="26" t="n"/>
       <c r="E13" s="26" t="n"/>
       <c r="F13" s="27" t="n">
-        <v>1372696904.24</v>
+        <v>1272119796.24</v>
       </c>
       <c r="G13" s="28" t="n">
-        <v>80746.87672</v>
+        <v>74830.57624941177</v>
       </c>
       <c r="H13" s="28" t="n">
-        <v>7262946.583280424</v>
+        <v>6730792.572698412</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh dashboard Fri 07/31/2026 14:02
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -722,7 +722,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 31 Jul 2026 13:59</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 31 Jul 2026 14:02</t>
         </is>
       </c>
     </row>
@@ -10873,7 +10873,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 31 Jul 2026 13:59 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 31 Jul 2026 14:02 (in IDR Million)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh dashboard Fri 08/07/2026 16:43
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -726,7 +726,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 06 Aug 2026 19:30</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 07 Aug 2026 16:43</t>
         </is>
       </c>
     </row>
@@ -794,14 +794,14 @@
       <c r="Z3" s="4" t="n"/>
       <c r="AA3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 06 Aug 2026</t>
+          <t>MTD as of 07 Aug 2026</t>
         </is>
       </c>
       <c r="AB3" s="4" t="n"/>
       <c r="AC3" s="4" t="n"/>
       <c r="AD3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 06 Aug 2026</t>
+          <t>YTD as of 07 Aug 2026</t>
         </is>
       </c>
       <c r="AE3" s="4" t="n"/>
@@ -1173,22 +1173,22 @@
         <v>873088236.8412699</v>
       </c>
       <c r="AA7" s="11" t="n">
-        <v>1634218723</v>
+        <v>3196868712</v>
       </c>
       <c r="AB7" s="11" t="n">
-        <v>96130.51311764706</v>
+        <v>188051.1007058824</v>
       </c>
       <c r="AC7" s="11" t="n">
-        <v>8646659.91005291</v>
+        <v>16914649.26984127</v>
       </c>
       <c r="AD7" s="11" t="n">
-        <v>166647895486</v>
+        <v>168210545475</v>
       </c>
       <c r="AE7" s="11" t="n">
-        <v>9802817.381529411</v>
+        <v>9894737.969117647</v>
       </c>
       <c r="AF7" s="11" t="n">
-        <v>881734896.7513227</v>
+        <v>890002886.1111112</v>
       </c>
     </row>
     <row r="8">
@@ -1267,177 +1267,183 @@
     <row r="9">
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">        PT Syngenta Seed Indonesia</t>
+          <t xml:space="preserve">        PT Corteva Agriscience Seeds Indonesia</t>
         </is>
       </c>
       <c r="C9" s="11" t="n">
-        <v>4917371048</v>
+        <v>14774062032</v>
       </c>
       <c r="D9" s="11" t="n">
-        <v>289257.1204705882</v>
+        <v>869062.4724705883</v>
       </c>
       <c r="E9" s="11" t="n">
-        <v>26017836.23280423</v>
-      </c>
-      <c r="F9" s="11" t="n">
-        <v>377499498</v>
-      </c>
-      <c r="G9" s="11" t="n">
-        <v>22205.85282352941</v>
-      </c>
-      <c r="H9" s="11" t="n">
-        <v>1997351.841269841</v>
-      </c>
+        <v>78169640.38095239</v>
+      </c>
+      <c r="F9" s="11" t="n"/>
+      <c r="G9" s="11" t="n"/>
+      <c r="H9" s="11" t="n"/>
       <c r="I9" s="11" t="n">
-        <v>5249034721</v>
+        <v>3060445998</v>
       </c>
       <c r="J9" s="11" t="n">
-        <v>308766.7482941176</v>
+        <v>180026.2351764706</v>
       </c>
       <c r="K9" s="11" t="n">
-        <v>27772670.48148148</v>
+        <v>16192835.96825397</v>
       </c>
       <c r="L9" s="11" t="n">
-        <v>5409395616</v>
+        <v>2647239849</v>
       </c>
       <c r="M9" s="11" t="n">
-        <v>318199.7421176471</v>
+        <v>155719.9911176471</v>
       </c>
       <c r="N9" s="11" t="n">
-        <v>28621140.82539682</v>
+        <v>14006560.04761905</v>
       </c>
       <c r="O9" s="11" t="n">
-        <v>7986730445</v>
+        <v>4342041733</v>
       </c>
       <c r="P9" s="11" t="n">
-        <v>469807.6732352941</v>
+        <v>255414.2195882353</v>
       </c>
       <c r="Q9" s="11" t="n">
-        <v>42257833.04232804</v>
+        <v>22973765.78306878</v>
       </c>
       <c r="R9" s="11" t="n">
-        <v>5293583677</v>
+        <v>2142139150</v>
       </c>
       <c r="S9" s="11" t="n">
-        <v>311387.2751176471</v>
+        <v>126008.1852941176</v>
       </c>
       <c r="T9" s="11" t="n">
-        <v>28008379.24338624</v>
+        <v>11334069.57671958</v>
       </c>
       <c r="U9" s="11" t="n">
-        <v>3590241514</v>
+        <v>4939206340</v>
       </c>
       <c r="V9" s="11" t="n">
-        <v>211190.6772941177</v>
+        <v>290541.5494117647</v>
       </c>
       <c r="W9" s="11" t="n">
-        <v>18995986.84656085</v>
+        <v>26133366.87830688</v>
       </c>
       <c r="X9" s="11" t="n">
-        <v>32823856519</v>
+        <v>31905135102</v>
       </c>
       <c r="Y9" s="11" t="n">
-        <v>1930815.089352941</v>
+        <v>1876772.653058824</v>
       </c>
       <c r="Z9" s="11" t="n">
-        <v>173671198.5132275</v>
-      </c>
-      <c r="AA9" s="11" t="n"/>
-      <c r="AB9" s="11" t="n"/>
-      <c r="AC9" s="11" t="n"/>
+        <v>168810238.6349206</v>
+      </c>
+      <c r="AA9" s="11" t="n">
+        <v>1562649989</v>
+      </c>
+      <c r="AB9" s="11" t="n">
+        <v>91920.5875882353</v>
+      </c>
+      <c r="AC9" s="11" t="n">
+        <v>8267989.35978836</v>
+      </c>
       <c r="AD9" s="11" t="n">
-        <v>32823856519</v>
+        <v>33467785091</v>
       </c>
       <c r="AE9" s="11" t="n">
-        <v>1930815.089352941</v>
+        <v>1968693.240647059</v>
       </c>
       <c r="AF9" s="11" t="n">
-        <v>173671198.5132275</v>
+        <v>177078227.994709</v>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">        PT Corteva Agriscience Seeds Indonesia</t>
+          <t xml:space="preserve">        PT Syngenta Seed Indonesia</t>
         </is>
       </c>
       <c r="C10" s="13" t="n">
-        <v>14774062032</v>
+        <v>4917371048</v>
       </c>
       <c r="D10" s="13" t="n">
-        <v>869062.4724705883</v>
+        <v>289257.1204705882</v>
       </c>
       <c r="E10" s="13" t="n">
-        <v>78169640.38095239</v>
-      </c>
-      <c r="F10" s="13" t="n"/>
-      <c r="G10" s="13" t="n"/>
-      <c r="H10" s="13" t="n"/>
+        <v>26017836.23280423</v>
+      </c>
+      <c r="F10" s="13" t="n">
+        <v>377499498</v>
+      </c>
+      <c r="G10" s="13" t="n">
+        <v>22205.85282352941</v>
+      </c>
+      <c r="H10" s="13" t="n">
+        <v>1997351.841269841</v>
+      </c>
       <c r="I10" s="13" t="n">
-        <v>3060445998</v>
+        <v>5249034721</v>
       </c>
       <c r="J10" s="13" t="n">
-        <v>180026.2351764706</v>
+        <v>308766.7482941176</v>
       </c>
       <c r="K10" s="13" t="n">
-        <v>16192835.96825397</v>
+        <v>27772670.48148148</v>
       </c>
       <c r="L10" s="13" t="n">
-        <v>2647239849</v>
+        <v>5409395616</v>
       </c>
       <c r="M10" s="13" t="n">
-        <v>155719.9911176471</v>
+        <v>318199.7421176471</v>
       </c>
       <c r="N10" s="13" t="n">
-        <v>14006560.04761905</v>
+        <v>28621140.82539682</v>
       </c>
       <c r="O10" s="13" t="n">
-        <v>4342041733</v>
+        <v>7986730445</v>
       </c>
       <c r="P10" s="13" t="n">
-        <v>255414.2195882353</v>
+        <v>469807.6732352941</v>
       </c>
       <c r="Q10" s="13" t="n">
-        <v>22973765.78306878</v>
+        <v>42257833.04232804</v>
       </c>
       <c r="R10" s="13" t="n">
-        <v>2142139150</v>
+        <v>5293583677</v>
       </c>
       <c r="S10" s="13" t="n">
-        <v>126008.1852941176</v>
+        <v>311387.2751176471</v>
       </c>
       <c r="T10" s="13" t="n">
-        <v>11334069.57671958</v>
+        <v>28008379.24338624</v>
       </c>
       <c r="U10" s="13" t="n">
-        <v>4939206340</v>
+        <v>3590241514</v>
       </c>
       <c r="V10" s="13" t="n">
-        <v>290541.5494117647</v>
+        <v>211190.6772941177</v>
       </c>
       <c r="W10" s="13" t="n">
-        <v>26133366.87830688</v>
+        <v>18995986.84656085</v>
       </c>
       <c r="X10" s="13" t="n">
-        <v>31905135102</v>
+        <v>32823856519</v>
       </c>
       <c r="Y10" s="13" t="n">
-        <v>1876772.653058824</v>
+        <v>1930815.089352941</v>
       </c>
       <c r="Z10" s="13" t="n">
-        <v>168810238.6349206</v>
+        <v>173671198.5132275</v>
       </c>
       <c r="AA10" s="13" t="n"/>
       <c r="AB10" s="13" t="n"/>
       <c r="AC10" s="13" t="n"/>
       <c r="AD10" s="13" t="n">
-        <v>31905135102</v>
+        <v>32823856519</v>
       </c>
       <c r="AE10" s="13" t="n">
-        <v>1876772.653058824</v>
+        <v>1930815.089352941</v>
       </c>
       <c r="AF10" s="13" t="n">
-        <v>168810238.6349206</v>
+        <v>173671198.5132275</v>
       </c>
     </row>
     <row r="11">
@@ -2013,22 +2019,22 @@
         <v>2099643.822698413</v>
       </c>
       <c r="AA19" s="11" t="n">
-        <v>2174720</v>
+        <v>3732220</v>
       </c>
       <c r="AB19" s="11" t="n">
-        <v>127.9247058823529</v>
+        <v>219.5423529411765</v>
       </c>
       <c r="AC19" s="11" t="n">
-        <v>11506.45502645503</v>
+        <v>19747.19576719577</v>
       </c>
       <c r="AD19" s="11" t="n">
-        <v>399007402.49</v>
+        <v>400564902.49</v>
       </c>
       <c r="AE19" s="11" t="n">
-        <v>23471.02367588235</v>
+        <v>23562.64132294118</v>
       </c>
       <c r="AF19" s="11" t="n">
-        <v>2111150.277724868</v>
+        <v>2119391.018465609</v>
       </c>
     </row>
     <row r="20">
@@ -2244,22 +2250,22 @@
         <v>140849.2063492063</v>
       </c>
       <c r="AA22" s="13" t="n">
-        <v>1883000</v>
+        <v>3440500</v>
       </c>
       <c r="AB22" s="13" t="n">
-        <v>110.7647058823529</v>
+        <v>202.3823529411765</v>
       </c>
       <c r="AC22" s="13" t="n">
-        <v>9962.962962962964</v>
+        <v>18203.7037037037</v>
       </c>
       <c r="AD22" s="13" t="n">
-        <v>28503500</v>
+        <v>30061000</v>
       </c>
       <c r="AE22" s="13" t="n">
-        <v>1676.676470588235</v>
+        <v>1768.294117647059</v>
       </c>
       <c r="AF22" s="13" t="n">
-        <v>150812.1693121693</v>
+        <v>159052.91005291</v>
       </c>
     </row>
     <row r="23">
@@ -3451,22 +3457,22 @@
         <v>1138764600.240688</v>
       </c>
       <c r="AA41" s="15" t="n">
-        <v>1636393443</v>
+        <v>3200600932</v>
       </c>
       <c r="AB41" s="15" t="n">
-        <v>96258.43782352941</v>
+        <v>188270.6430588235</v>
       </c>
       <c r="AC41" s="15" t="n">
-        <v>8658166.365079366</v>
+        <v>16934396.46560847</v>
       </c>
       <c r="AD41" s="15" t="n">
-        <v>216862902888.49</v>
+        <v>218427110377.49</v>
       </c>
       <c r="AE41" s="15" t="n">
-        <v>12756641.34638176</v>
+        <v>12848653.55161706</v>
       </c>
       <c r="AF41" s="15" t="n">
-        <v>1147422766.605767</v>
+        <v>1155698996.706296</v>
       </c>
     </row>
     <row r="42">
@@ -3817,22 +3823,22 @@
         <v>-6710414.91005291</v>
       </c>
       <c r="AA47" s="13" t="n">
-        <v>-168087391</v>
+        <v>-175119091</v>
       </c>
       <c r="AB47" s="13" t="n">
-        <v>-9887.493588235295</v>
+        <v>-10301.123</v>
       </c>
       <c r="AC47" s="13" t="n">
-        <v>-889351.2751322752</v>
+        <v>-926556.0370370371</v>
       </c>
       <c r="AD47" s="13" t="n">
-        <v>-1436355809</v>
+        <v>-1443387509</v>
       </c>
       <c r="AE47" s="13" t="n">
-        <v>-84491.51817647059</v>
+        <v>-84905.1475882353</v>
       </c>
       <c r="AF47" s="13" t="n">
-        <v>-7599766.185185185</v>
+        <v>-7636970.947089947</v>
       </c>
     </row>
     <row r="48">
@@ -4693,22 +4699,22 @@
         <v>-75623143.55492064</v>
       </c>
       <c r="AA59" s="15" t="n">
-        <v>-273730041</v>
+        <v>-280761741</v>
       </c>
       <c r="AB59" s="15" t="n">
-        <v>-16101.76711764706</v>
+        <v>-16515.39652941177</v>
       </c>
       <c r="AC59" s="15" t="n">
-        <v>-1448307.095238095</v>
+        <v>-1485511.857142857</v>
       </c>
       <c r="AD59" s="15" t="n">
-        <v>-14566504172.88</v>
+        <v>-14573535872.88</v>
       </c>
       <c r="AE59" s="15" t="n">
-        <v>-856853.18664</v>
+        <v>-857266.8160517646</v>
       </c>
       <c r="AF59" s="15" t="n">
-        <v>-77071450.65015873</v>
+        <v>-77108655.41206349</v>
       </c>
     </row>
     <row r="60">
@@ -5935,13 +5941,13 @@
         <v>-44761.71957671957</v>
       </c>
       <c r="L80" s="13" t="n">
-        <v>-16481670</v>
+        <v>-9454108</v>
       </c>
       <c r="M80" s="13" t="n">
-        <v>-969.51</v>
+        <v>-556.124</v>
       </c>
       <c r="N80" s="13" t="n">
-        <v>-87204.60317460318</v>
+        <v>-50021.73544973545</v>
       </c>
       <c r="O80" s="13" t="n">
         <v>-11129454</v>
@@ -5971,13 +5977,13 @@
         <v>-43300.36507936508</v>
       </c>
       <c r="X80" s="13" t="n">
-        <v>-386997197</v>
+        <v>-379969635</v>
       </c>
       <c r="Y80" s="13" t="n">
-        <v>-22764.541</v>
+        <v>-22351.155</v>
       </c>
       <c r="Z80" s="13" t="n">
-        <v>-2047604.216931217</v>
+        <v>-2010421.349206349</v>
       </c>
       <c r="AA80" s="13" t="n">
         <v>-4350012</v>
@@ -5989,13 +5995,13 @@
         <v>-23015.93650793651</v>
       </c>
       <c r="AD80" s="13" t="n">
-        <v>-391347209</v>
+        <v>-384319647</v>
       </c>
       <c r="AE80" s="13" t="n">
-        <v>-23020.42405882353</v>
+        <v>-22607.03805882353</v>
       </c>
       <c r="AF80" s="13" t="n">
-        <v>-2070620.153439153</v>
+        <v>-2033437.285714286</v>
       </c>
     </row>
     <row r="81">
@@ -6032,13 +6038,13 @@
         <v>-8149575.227513228</v>
       </c>
       <c r="L81" s="15" t="n">
-        <v>-2947191108</v>
+        <v>-2940163546</v>
       </c>
       <c r="M81" s="15" t="n">
-        <v>-173364.1828235294</v>
+        <v>-172950.7968235294</v>
       </c>
       <c r="N81" s="15" t="n">
-        <v>-15593603.74603175</v>
+        <v>-15556420.87830688</v>
       </c>
       <c r="O81" s="15" t="n">
         <v>-2557069174.54</v>
@@ -6068,13 +6074,13 @@
         <v>-14773761.37037037</v>
       </c>
       <c r="X81" s="15" t="n">
-        <v>-19741108872.54</v>
+        <v>-19734081310.54</v>
       </c>
       <c r="Y81" s="15" t="n">
-        <v>-1161241.698384706</v>
+        <v>-1160828.312384706</v>
       </c>
       <c r="Z81" s="15" t="n">
-        <v>-104450311.4949206</v>
+        <v>-104413128.6271958</v>
       </c>
       <c r="AA81" s="15" t="n">
         <v>-1030020506</v>
@@ -6086,13 +6092,13 @@
         <v>-5449843.947089947</v>
       </c>
       <c r="AD81" s="15" t="n">
-        <v>-20771129378.54</v>
+        <v>-20764101816.54</v>
       </c>
       <c r="AE81" s="15" t="n">
-        <v>-1221831.139914118</v>
+        <v>-1221417.753914118</v>
       </c>
       <c r="AF81" s="15" t="n">
-        <v>-109900155.4420106</v>
+        <v>-109862972.5742857</v>
       </c>
     </row>
     <row r="82">
@@ -7226,22 +7232,22 @@
         <v>-1550969.746031746</v>
       </c>
       <c r="AA96" s="11" t="n">
-        <v>-8996525</v>
+        <v>-2281700</v>
       </c>
       <c r="AB96" s="11" t="n">
-        <v>-529.2073529411765</v>
+        <v>-134.2176470588235</v>
       </c>
       <c r="AC96" s="11" t="n">
-        <v>-47600.66137566137</v>
+        <v>-12072.48677248677</v>
       </c>
       <c r="AD96" s="11" t="n">
-        <v>-302129807</v>
+        <v>-295414982</v>
       </c>
       <c r="AE96" s="11" t="n">
-        <v>-17772.34158823529</v>
+        <v>-17377.35188235294</v>
       </c>
       <c r="AF96" s="11" t="n">
-        <v>-1598570.407407407</v>
+        <v>-1563042.232804233</v>
       </c>
     </row>
     <row r="97">
@@ -7323,22 +7329,22 @@
         <v>-37700914.92835979</v>
       </c>
       <c r="AA97" s="15" t="n">
-        <v>-51016672</v>
+        <v>-44301847</v>
       </c>
       <c r="AB97" s="15" t="n">
-        <v>-3000.980705882353</v>
+        <v>-2605.991</v>
       </c>
       <c r="AC97" s="15" t="n">
-        <v>-269929.4814814815</v>
+        <v>-234401.3068783069</v>
       </c>
       <c r="AD97" s="15" t="n">
-        <v>-7176489593.46</v>
+        <v>-7169774768.46</v>
       </c>
       <c r="AE97" s="15" t="n">
-        <v>-422146.4466741176</v>
+        <v>-421751.4569682353</v>
       </c>
       <c r="AF97" s="15" t="n">
-        <v>-37970844.40984128</v>
+        <v>-37935316.2352381</v>
       </c>
     </row>
     <row r="98">
@@ -8824,22 +8830,22 @@
         <v>-24120218.13227513</v>
       </c>
       <c r="AA116" s="11" t="n">
-        <v>-232028585</v>
+        <v>-231711710</v>
       </c>
       <c r="AB116" s="11" t="n">
-        <v>-13648.74029411765</v>
+        <v>-13630.10058823529</v>
       </c>
       <c r="AC116" s="11" t="n">
-        <v>-1227664.470899471</v>
+        <v>-1225987.883597884</v>
       </c>
       <c r="AD116" s="11" t="n">
-        <v>-4790749812</v>
+        <v>-4790432937</v>
       </c>
       <c r="AE116" s="11" t="n">
-        <v>-281808.8124705883</v>
+        <v>-281790.1727647059</v>
       </c>
       <c r="AF116" s="11" t="n">
-        <v>-25347882.6031746</v>
+        <v>-25346206.01587302</v>
       </c>
     </row>
     <row r="117">
@@ -8921,22 +8927,22 @@
         <v>-24120218.13227513</v>
       </c>
       <c r="AA117" s="15" t="n">
-        <v>-232028585</v>
+        <v>-231711710</v>
       </c>
       <c r="AB117" s="15" t="n">
-        <v>-13648.74029411765</v>
+        <v>-13630.10058823529</v>
       </c>
       <c r="AC117" s="15" t="n">
-        <v>-1227664.470899471</v>
+        <v>-1225987.883597884</v>
       </c>
       <c r="AD117" s="15" t="n">
-        <v>-4790749812</v>
+        <v>-4790432937</v>
       </c>
       <c r="AE117" s="15" t="n">
-        <v>-281808.8124705883</v>
+        <v>-281790.1727647059</v>
       </c>
       <c r="AF117" s="15" t="n">
-        <v>-25347882.6031746</v>
+        <v>-25346206.01587302</v>
       </c>
     </row>
     <row r="118">
@@ -9496,13 +9502,13 @@
         <v>-455974.7513227513</v>
       </c>
       <c r="L125" s="11" t="n">
-        <v>-43468282</v>
+        <v>-50495844</v>
       </c>
       <c r="M125" s="11" t="n">
-        <v>-2556.957764705882</v>
+        <v>-2970.343764705882</v>
       </c>
       <c r="N125" s="11" t="n">
-        <v>-229990.91005291</v>
+        <v>-267173.7777777778</v>
       </c>
       <c r="O125" s="11" t="n">
         <v>-50240918</v>
@@ -9532,25 +9538,25 @@
         <v>-315554.3968253968</v>
       </c>
       <c r="X125" s="11" t="n">
-        <v>-1040425127</v>
+        <v>-1047452689</v>
       </c>
       <c r="Y125" s="11" t="n">
-        <v>-61201.47805882354</v>
+        <v>-61614.86405882354</v>
       </c>
       <c r="Z125" s="11" t="n">
-        <v>-5504894.851851851</v>
+        <v>-5542077.719576718</v>
       </c>
       <c r="AA125" s="11" t="n"/>
       <c r="AB125" s="11" t="n"/>
       <c r="AC125" s="11" t="n"/>
       <c r="AD125" s="11" t="n">
-        <v>-1040425127</v>
+        <v>-1047452689</v>
       </c>
       <c r="AE125" s="11" t="n">
-        <v>-61201.47805882354</v>
+        <v>-61614.86405882354</v>
       </c>
       <c r="AF125" s="11" t="n">
-        <v>-5504894.851851851</v>
+        <v>-5542077.719576718</v>
       </c>
     </row>
     <row r="126">
@@ -9587,13 +9593,13 @@
         <v>-5085715.19047619</v>
       </c>
       <c r="L126" s="15" t="n">
-        <v>-6458994316.059999</v>
+        <v>-6466021878.059999</v>
       </c>
       <c r="M126" s="15" t="n">
-        <v>-379940.8421211764</v>
+        <v>-380354.2281211764</v>
       </c>
       <c r="N126" s="15" t="n">
-        <v>-34174573.10084656</v>
+        <v>-34211755.96857142</v>
       </c>
       <c r="O126" s="15" t="n">
         <v>-1318812959.4</v>
@@ -9623,13 +9629,13 @@
         <v>-10206510.8621164</v>
       </c>
       <c r="X126" s="15" t="n">
-        <v>-24556731969.41</v>
+        <v>-24563759531.41</v>
       </c>
       <c r="Y126" s="15" t="n">
-        <v>-1444513.645259412</v>
+        <v>-1444927.031259412</v>
       </c>
       <c r="Z126" s="15" t="n">
-        <v>-129929798.7799471</v>
+        <v>-129966981.6476719</v>
       </c>
       <c r="AA126" s="15" t="n">
         <v>-28138500</v>
@@ -9641,13 +9647,13 @@
         <v>-148880.9523809524</v>
       </c>
       <c r="AD126" s="15" t="n">
-        <v>-24584870469.41</v>
+        <v>-24591898031.41</v>
       </c>
       <c r="AE126" s="15" t="n">
-        <v>-1446168.851141765</v>
+        <v>-1446582.237141765</v>
       </c>
       <c r="AF126" s="15" t="n">
-        <v>-130078679.732328</v>
+        <v>-130115862.6000529</v>
       </c>
     </row>
     <row r="127">
@@ -10310,13 +10316,13 @@
         <v>-14621315.66666667</v>
       </c>
       <c r="L135" s="15" t="n">
-        <v>-8651599269.059999</v>
+        <v>-8658626831.059999</v>
       </c>
       <c r="M135" s="15" t="n">
-        <v>-508917.6040623529</v>
+        <v>-509330.9900623529</v>
       </c>
       <c r="N135" s="15" t="n">
-        <v>-45775657.50825396</v>
+        <v>-45812840.37597883</v>
       </c>
       <c r="O135" s="15" t="n">
         <v>-2654292760.86</v>
@@ -10346,31 +10352,31 @@
         <v>-21392974.16899471</v>
       </c>
       <c r="X135" s="15" t="n">
-        <v>-40282915660.31001</v>
+        <v>-40289943222.31001</v>
       </c>
       <c r="Y135" s="15" t="n">
-        <v>-2369583.274135883</v>
+        <v>-2369996.660135882</v>
       </c>
       <c r="Z135" s="15" t="n">
-        <v>-213137119.8958201</v>
+        <v>-213174302.763545</v>
       </c>
       <c r="AA135" s="15" t="n">
-        <v>-482046975</v>
+        <v>-475015275</v>
       </c>
       <c r="AB135" s="15" t="n">
-        <v>-28355.70441176471</v>
+        <v>-27942.075</v>
       </c>
       <c r="AC135" s="15" t="n">
-        <v>-2550513.095238095</v>
+        <v>-2513308.333333333</v>
       </c>
       <c r="AD135" s="15" t="n">
-        <v>-40764962635.31001</v>
+        <v>-40764958497.31001</v>
       </c>
       <c r="AE135" s="15" t="n">
-        <v>-2397938.978547647</v>
+        <v>-2397938.735135883</v>
       </c>
       <c r="AF135" s="15" t="n">
-        <v>-215687632.9910582</v>
+        <v>-215687611.0968783</v>
       </c>
     </row>
     <row r="136">
@@ -11596,22 +11602,22 @@
         <v>-340104393.7373017</v>
       </c>
       <c r="AA152" s="19" t="n">
-        <v>-149999402</v>
+        <v>1414208087</v>
       </c>
       <c r="AB152" s="19" t="n">
-        <v>-8823.494235294118</v>
+        <v>83188.711</v>
       </c>
       <c r="AC152" s="19" t="n">
-        <v>-793647.6296296297</v>
+        <v>7482582.470899471</v>
       </c>
       <c r="AD152" s="19" t="n">
-        <v>-64429729818.35001</v>
+        <v>-62865522329.35001</v>
       </c>
       <c r="AE152" s="19" t="n">
-        <v>-3789984.106961765</v>
+        <v>-3697971.901726471</v>
       </c>
       <c r="AF152" s="19" t="n">
-        <v>-340898041.3669313</v>
+        <v>-332621811.2664022</v>
       </c>
     </row>
     <row r="153">
@@ -11693,22 +11699,22 @@
         <v>16899102.6984656</v>
       </c>
       <c r="AA153" s="7" t="n">
-        <v>3043931008.009999</v>
+        <v>4608138497.009999</v>
       </c>
       <c r="AB153" s="7" t="n">
-        <v>179054.7651770588</v>
+        <v>271066.9704123529</v>
       </c>
       <c r="AC153" s="7" t="n">
-        <v>16105455.06883598</v>
+        <v>24381685.16936507</v>
       </c>
       <c r="AD153" s="7" t="n">
-        <v>3043931008.009999</v>
+        <v>4608138497.009999</v>
       </c>
       <c r="AE153" s="7" t="n">
-        <v>179054.7651770588</v>
+        <v>271066.9704123529</v>
       </c>
       <c r="AF153" s="7" t="n">
-        <v>16105455.06883598</v>
+        <v>24381685.16936507</v>
       </c>
     </row>
   </sheetData>
@@ -11835,16 +11841,16 @@
         <v>2698509305</v>
       </c>
       <c r="E6" s="11" t="n">
-        <v>226785940</v>
+        <v>1789435929</v>
       </c>
       <c r="F6" s="11" t="n">
-        <v>2925295245</v>
+        <v>4487945234</v>
       </c>
       <c r="G6" s="23" t="n">
-        <v>172076.1908823529</v>
+        <v>263996.7784705882</v>
       </c>
       <c r="H6" s="23" t="n">
-        <v>15477752.61904762</v>
+        <v>23745741.97883598</v>
       </c>
     </row>
     <row r="7">
@@ -11931,16 +11937,16 @@
         <v>44055921.71</v>
       </c>
       <c r="E9" s="13" t="n">
-        <v>-16561019</v>
+        <v>-15003519</v>
       </c>
       <c r="F9" s="13" t="n">
-        <v>27494902.71</v>
+        <v>29052402.71</v>
       </c>
       <c r="G9" s="24" t="n">
-        <v>1617.347218235294</v>
+        <v>1708.964865294118</v>
       </c>
       <c r="H9" s="24" t="n">
-        <v>145475.6757142857</v>
+        <v>153716.4164550265</v>
       </c>
     </row>
     <row r="10">
@@ -12050,13 +12056,13 @@
       <c r="D13" s="26" t="n"/>
       <c r="E13" s="26" t="n"/>
       <c r="F13" s="27" t="n">
-        <v>3043931010.01</v>
+        <v>4608138499.01</v>
       </c>
       <c r="G13" s="28" t="n">
-        <v>179054.7652947059</v>
+        <v>271066.97053</v>
       </c>
       <c r="H13" s="28" t="n">
-        <v>16105455.07941799</v>
+        <v>24381685.17994709</v>
       </c>
     </row>
   </sheetData>
@@ -12123,7 +12129,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 06 Aug 2026 19:30 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 07 Aug 2026 16:43 (in IDR Million)</t>
         </is>
       </c>
     </row>
@@ -12191,14 +12197,14 @@
       <c r="Z3" s="4" t="n"/>
       <c r="AA3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 06 Aug 2026</t>
+          <t>MTD as of 07 Aug 2026</t>
         </is>
       </c>
       <c r="AB3" s="4" t="n"/>
       <c r="AC3" s="4" t="n"/>
       <c r="AD3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 06 Aug 2026</t>
+          <t>YTD as of 07 Aug 2026</t>
         </is>
       </c>
       <c r="AE3" s="4" t="n"/>
@@ -12570,22 +12576,22 @@
         <v>873.0882368412699</v>
       </c>
       <c r="AA7" s="11" t="n">
-        <v>1634.218723</v>
+        <v>3196.868712</v>
       </c>
       <c r="AB7" s="11" t="n">
-        <v>0.09613051311764706</v>
+        <v>0.1880511007058824</v>
       </c>
       <c r="AC7" s="11" t="n">
-        <v>8.646659910052909</v>
+        <v>16.91464926984127</v>
       </c>
       <c r="AD7" s="11" t="n">
-        <v>166647.895486</v>
+        <v>168210.545475</v>
       </c>
       <c r="AE7" s="11" t="n">
-        <v>9.80281738152941</v>
+        <v>9.894737969117646</v>
       </c>
       <c r="AF7" s="11" t="n">
-        <v>881.7348967513228</v>
+        <v>890.0028861111111</v>
       </c>
     </row>
     <row r="8">
@@ -12664,177 +12670,183 @@
     <row r="9">
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">        PT Syngenta Seed Indonesia</t>
+          <t xml:space="preserve">        PT Corteva Agriscience Seeds Indonesia</t>
         </is>
       </c>
       <c r="C9" s="11" t="n">
-        <v>4917.371048</v>
+        <v>14774.062032</v>
       </c>
       <c r="D9" s="11" t="n">
-        <v>0.2892571204705882</v>
+        <v>0.8690624724705882</v>
       </c>
       <c r="E9" s="11" t="n">
-        <v>26.01783623280423</v>
-      </c>
-      <c r="F9" s="11" t="n">
-        <v>377.499498</v>
-      </c>
-      <c r="G9" s="11" t="n">
-        <v>0.02220585282352941</v>
-      </c>
-      <c r="H9" s="11" t="n">
-        <v>1.997351841269841</v>
-      </c>
+        <v>78.16964038095237</v>
+      </c>
+      <c r="F9" s="11" t="n"/>
+      <c r="G9" s="11" t="n"/>
+      <c r="H9" s="11" t="n"/>
       <c r="I9" s="11" t="n">
-        <v>5249.034721</v>
+        <v>3060.445998</v>
       </c>
       <c r="J9" s="11" t="n">
-        <v>0.3087667482941177</v>
+        <v>0.1800262351764706</v>
       </c>
       <c r="K9" s="11" t="n">
-        <v>27.77267048148148</v>
+        <v>16.19283596825397</v>
       </c>
       <c r="L9" s="11" t="n">
-        <v>5409.395616</v>
+        <v>2647.239849</v>
       </c>
       <c r="M9" s="11" t="n">
-        <v>0.3181997421176471</v>
+        <v>0.1557199911176471</v>
       </c>
       <c r="N9" s="11" t="n">
-        <v>28.62114082539683</v>
+        <v>14.00656004761905</v>
       </c>
       <c r="O9" s="11" t="n">
-        <v>7986.730445</v>
+        <v>4342.041733</v>
       </c>
       <c r="P9" s="11" t="n">
-        <v>0.4698076732352941</v>
+        <v>0.2554142195882353</v>
       </c>
       <c r="Q9" s="11" t="n">
-        <v>42.25783304232804</v>
+        <v>22.97376578306878</v>
       </c>
       <c r="R9" s="11" t="n">
-        <v>5293.583677</v>
+        <v>2142.13915</v>
       </c>
       <c r="S9" s="11" t="n">
-        <v>0.311387275117647</v>
+        <v>0.1260081852941176</v>
       </c>
       <c r="T9" s="11" t="n">
-        <v>28.00837924338624</v>
+        <v>11.33406957671958</v>
       </c>
       <c r="U9" s="11" t="n">
-        <v>3590.241514</v>
+        <v>4939.20634</v>
       </c>
       <c r="V9" s="11" t="n">
-        <v>0.2111906772941176</v>
+        <v>0.2905415494117647</v>
       </c>
       <c r="W9" s="11" t="n">
-        <v>18.99598684656085</v>
+        <v>26.13336687830688</v>
       </c>
       <c r="X9" s="11" t="n">
-        <v>32823.856519</v>
+        <v>31905.135102</v>
       </c>
       <c r="Y9" s="11" t="n">
-        <v>1.930815089352941</v>
+        <v>1.876772653058824</v>
       </c>
       <c r="Z9" s="11" t="n">
-        <v>173.6711985132275</v>
-      </c>
-      <c r="AA9" s="11" t="n"/>
-      <c r="AB9" s="11" t="n"/>
-      <c r="AC9" s="11" t="n"/>
+        <v>168.8102386349206</v>
+      </c>
+      <c r="AA9" s="11" t="n">
+        <v>1562.649989</v>
+      </c>
+      <c r="AB9" s="11" t="n">
+        <v>0.09192058758823529</v>
+      </c>
+      <c r="AC9" s="11" t="n">
+        <v>8.267989359788359</v>
+      </c>
       <c r="AD9" s="11" t="n">
-        <v>32823.856519</v>
+        <v>33467.785091</v>
       </c>
       <c r="AE9" s="11" t="n">
-        <v>1.930815089352941</v>
+        <v>1.968693240647059</v>
       </c>
       <c r="AF9" s="11" t="n">
-        <v>173.6711985132275</v>
+        <v>177.078227994709</v>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">        PT Corteva Agriscience Seeds Indonesia</t>
+          <t xml:space="preserve">        PT Syngenta Seed Indonesia</t>
         </is>
       </c>
       <c r="C10" s="13" t="n">
-        <v>14774.062032</v>
+        <v>4917.371048</v>
       </c>
       <c r="D10" s="13" t="n">
-        <v>0.8690624724705882</v>
+        <v>0.2892571204705882</v>
       </c>
       <c r="E10" s="13" t="n">
-        <v>78.16964038095237</v>
-      </c>
-      <c r="F10" s="13" t="n"/>
-      <c r="G10" s="13" t="n"/>
-      <c r="H10" s="13" t="n"/>
+        <v>26.01783623280423</v>
+      </c>
+      <c r="F10" s="13" t="n">
+        <v>377.499498</v>
+      </c>
+      <c r="G10" s="13" t="n">
+        <v>0.02220585282352941</v>
+      </c>
+      <c r="H10" s="13" t="n">
+        <v>1.997351841269841</v>
+      </c>
       <c r="I10" s="13" t="n">
-        <v>3060.445998</v>
+        <v>5249.034721</v>
       </c>
       <c r="J10" s="13" t="n">
-        <v>0.1800262351764706</v>
+        <v>0.3087667482941177</v>
       </c>
       <c r="K10" s="13" t="n">
-        <v>16.19283596825397</v>
+        <v>27.77267048148148</v>
       </c>
       <c r="L10" s="13" t="n">
-        <v>2647.239849</v>
+        <v>5409.395616</v>
       </c>
       <c r="M10" s="13" t="n">
-        <v>0.1557199911176471</v>
+        <v>0.3181997421176471</v>
       </c>
       <c r="N10" s="13" t="n">
-        <v>14.00656004761905</v>
+        <v>28.62114082539683</v>
       </c>
       <c r="O10" s="13" t="n">
-        <v>4342.041733</v>
+        <v>7986.730445</v>
       </c>
       <c r="P10" s="13" t="n">
-        <v>0.2554142195882353</v>
+        <v>0.4698076732352941</v>
       </c>
       <c r="Q10" s="13" t="n">
-        <v>22.97376578306878</v>
+        <v>42.25783304232804</v>
       </c>
       <c r="R10" s="13" t="n">
-        <v>2142.13915</v>
+        <v>5293.583677</v>
       </c>
       <c r="S10" s="13" t="n">
-        <v>0.1260081852941176</v>
+        <v>0.311387275117647</v>
       </c>
       <c r="T10" s="13" t="n">
-        <v>11.33406957671958</v>
+        <v>28.00837924338624</v>
       </c>
       <c r="U10" s="13" t="n">
-        <v>4939.20634</v>
+        <v>3590.241514</v>
       </c>
       <c r="V10" s="13" t="n">
-        <v>0.2905415494117647</v>
+        <v>0.2111906772941176</v>
       </c>
       <c r="W10" s="13" t="n">
-        <v>26.13336687830688</v>
+        <v>18.99598684656085</v>
       </c>
       <c r="X10" s="13" t="n">
-        <v>31905.135102</v>
+        <v>32823.856519</v>
       </c>
       <c r="Y10" s="13" t="n">
-        <v>1.876772653058824</v>
+        <v>1.930815089352941</v>
       </c>
       <c r="Z10" s="13" t="n">
-        <v>168.8102386349206</v>
+        <v>173.6711985132275</v>
       </c>
       <c r="AA10" s="13" t="n"/>
       <c r="AB10" s="13" t="n"/>
       <c r="AC10" s="13" t="n"/>
       <c r="AD10" s="13" t="n">
-        <v>31905.135102</v>
+        <v>32823.856519</v>
       </c>
       <c r="AE10" s="13" t="n">
-        <v>1.876772653058824</v>
+        <v>1.930815089352941</v>
       </c>
       <c r="AF10" s="13" t="n">
-        <v>168.8102386349206</v>
+        <v>173.6711985132275</v>
       </c>
     </row>
     <row r="11">
@@ -13410,22 +13422,22 @@
         <v>2.099643822698413</v>
       </c>
       <c r="AA19" s="11" t="n">
-        <v>2.17472</v>
+        <v>3.73222</v>
       </c>
       <c r="AB19" s="11" t="n">
-        <v>0.000127924705882353</v>
+        <v>0.0002195423529411765</v>
       </c>
       <c r="AC19" s="11" t="n">
-        <v>0.01150645502645503</v>
+        <v>0.01974719576719577</v>
       </c>
       <c r="AD19" s="11" t="n">
-        <v>399.0074024899999</v>
+        <v>400.56490249</v>
       </c>
       <c r="AE19" s="11" t="n">
-        <v>0.02347102367588235</v>
+        <v>0.02356264132294118</v>
       </c>
       <c r="AF19" s="11" t="n">
-        <v>2.111150277724868</v>
+        <v>2.119391018465609</v>
       </c>
     </row>
     <row r="20">
@@ -13641,22 +13653,22 @@
         <v>0.1408492063492063</v>
       </c>
       <c r="AA22" s="13" t="n">
-        <v>1.883</v>
+        <v>3.4405</v>
       </c>
       <c r="AB22" s="13" t="n">
-        <v>0.0001107647058823529</v>
+        <v>0.0002023823529411765</v>
       </c>
       <c r="AC22" s="13" t="n">
-        <v>0.009962962962962963</v>
+        <v>0.0182037037037037</v>
       </c>
       <c r="AD22" s="13" t="n">
-        <v>28.5035</v>
+        <v>30.061</v>
       </c>
       <c r="AE22" s="13" t="n">
-        <v>0.001676676470588235</v>
+        <v>0.001768294117647059</v>
       </c>
       <c r="AF22" s="13" t="n">
-        <v>0.1508121693121693</v>
+        <v>0.15905291005291</v>
       </c>
     </row>
     <row r="23">
@@ -14848,22 +14860,22 @@
         <v>1138.764600240688</v>
       </c>
       <c r="AA41" s="15" t="n">
-        <v>1636.393443</v>
+        <v>3200.600932</v>
       </c>
       <c r="AB41" s="15" t="n">
-        <v>0.09625843782352941</v>
+        <v>0.1882706430588235</v>
       </c>
       <c r="AC41" s="15" t="n">
-        <v>8.658166365079365</v>
+        <v>16.93439646560847</v>
       </c>
       <c r="AD41" s="15" t="n">
-        <v>216862.90288849</v>
+        <v>218427.11037749</v>
       </c>
       <c r="AE41" s="15" t="n">
-        <v>12.75664134638176</v>
+        <v>12.84865355161706</v>
       </c>
       <c r="AF41" s="15" t="n">
-        <v>1147.422766605767</v>
+        <v>1155.698996706296</v>
       </c>
     </row>
     <row r="42">
@@ -15214,22 +15226,22 @@
         <v>-6.71041491005291</v>
       </c>
       <c r="AA47" s="13" t="n">
-        <v>-168.087391</v>
+        <v>-175.119091</v>
       </c>
       <c r="AB47" s="13" t="n">
-        <v>-0.009887493588235294</v>
+        <v>-0.010301123</v>
       </c>
       <c r="AC47" s="13" t="n">
-        <v>-0.8893512751322751</v>
+        <v>-0.926556037037037</v>
       </c>
       <c r="AD47" s="13" t="n">
-        <v>-1436.355809</v>
+        <v>-1443.387509</v>
       </c>
       <c r="AE47" s="13" t="n">
-        <v>-0.0844915181764706</v>
+        <v>-0.08490514758823531</v>
       </c>
       <c r="AF47" s="13" t="n">
-        <v>-7.599766185185184</v>
+        <v>-7.636970947089947</v>
       </c>
     </row>
     <row r="48">
@@ -16090,22 +16102,22 @@
         <v>-75.62314355492063</v>
       </c>
       <c r="AA59" s="15" t="n">
-        <v>-273.730041</v>
+        <v>-280.761741</v>
       </c>
       <c r="AB59" s="15" t="n">
-        <v>-0.01610176711764706</v>
+        <v>-0.01651539652941176</v>
       </c>
       <c r="AC59" s="15" t="n">
-        <v>-1.448307095238095</v>
+        <v>-1.485511857142857</v>
       </c>
       <c r="AD59" s="15" t="n">
-        <v>-14566.50417288</v>
+        <v>-14573.53587288</v>
       </c>
       <c r="AE59" s="15" t="n">
-        <v>-0.85685318664</v>
+        <v>-0.8572668160517647</v>
       </c>
       <c r="AF59" s="15" t="n">
-        <v>-77.07145065015872</v>
+        <v>-77.10865541206348</v>
       </c>
     </row>
     <row r="60">
@@ -17332,13 +17344,13 @@
         <v>-0.04476171957671958</v>
       </c>
       <c r="L80" s="13" t="n">
-        <v>-16.48167</v>
+        <v>-9.454108</v>
       </c>
       <c r="M80" s="13" t="n">
-        <v>-0.00096951</v>
+        <v>-0.000556124</v>
       </c>
       <c r="N80" s="13" t="n">
-        <v>-0.08720460317460318</v>
+        <v>-0.05002173544973545</v>
       </c>
       <c r="O80" s="13" t="n">
         <v>-11.129454</v>
@@ -17368,13 +17380,13 @@
         <v>-0.04330036507936508</v>
       </c>
       <c r="X80" s="13" t="n">
-        <v>-386.997197</v>
+        <v>-379.969635</v>
       </c>
       <c r="Y80" s="13" t="n">
-        <v>-0.022764541</v>
+        <v>-0.022351155</v>
       </c>
       <c r="Z80" s="13" t="n">
-        <v>-2.047604216931217</v>
+        <v>-2.010421349206349</v>
       </c>
       <c r="AA80" s="13" t="n">
         <v>-4.350012</v>
@@ -17386,13 +17398,13 @@
         <v>-0.02301593650793651</v>
       </c>
       <c r="AD80" s="13" t="n">
-        <v>-391.347209</v>
+        <v>-384.319647</v>
       </c>
       <c r="AE80" s="13" t="n">
-        <v>-0.02302042405882353</v>
+        <v>-0.02260703805882353</v>
       </c>
       <c r="AF80" s="13" t="n">
-        <v>-2.070620153439153</v>
+        <v>-2.033437285714286</v>
       </c>
     </row>
     <row r="81">
@@ -17429,13 +17441,13 @@
         <v>-8.149575227513228</v>
       </c>
       <c r="L81" s="15" t="n">
-        <v>-2947.191108</v>
+        <v>-2940.163546</v>
       </c>
       <c r="M81" s="15" t="n">
-        <v>-0.1733641828235294</v>
+        <v>-0.1729507968235294</v>
       </c>
       <c r="N81" s="15" t="n">
-        <v>-15.59360374603175</v>
+        <v>-15.55642087830688</v>
       </c>
       <c r="O81" s="15" t="n">
         <v>-2557.06917454</v>
@@ -17465,13 +17477,13 @@
         <v>-14.77376137037037</v>
       </c>
       <c r="X81" s="15" t="n">
-        <v>-19741.10887254</v>
+        <v>-19734.08131054</v>
       </c>
       <c r="Y81" s="15" t="n">
-        <v>-1.161241698384706</v>
+        <v>-1.160828312384706</v>
       </c>
       <c r="Z81" s="15" t="n">
-        <v>-104.4503114949206</v>
+        <v>-104.4131286271957</v>
       </c>
       <c r="AA81" s="15" t="n">
         <v>-1030.020506</v>
@@ -17483,13 +17495,13 @@
         <v>-5.449843947089947</v>
       </c>
       <c r="AD81" s="15" t="n">
-        <v>-20771.12937854</v>
+        <v>-20764.10181654</v>
       </c>
       <c r="AE81" s="15" t="n">
-        <v>-1.221831139914118</v>
+        <v>-1.221417753914118</v>
       </c>
       <c r="AF81" s="15" t="n">
-        <v>-109.9001554420106</v>
+        <v>-109.8629725742857</v>
       </c>
     </row>
     <row r="82">
@@ -18623,22 +18635,22 @@
         <v>-1.550969746031746</v>
       </c>
       <c r="AA96" s="11" t="n">
-        <v>-8.996525</v>
+        <v>-2.2817</v>
       </c>
       <c r="AB96" s="11" t="n">
-        <v>-0.0005292073529411765</v>
+        <v>-0.0001342176470588235</v>
       </c>
       <c r="AC96" s="11" t="n">
-        <v>-0.04760066137566138</v>
+        <v>-0.01207248677248677</v>
       </c>
       <c r="AD96" s="11" t="n">
-        <v>-302.129807</v>
+        <v>-295.414982</v>
       </c>
       <c r="AE96" s="11" t="n">
-        <v>-0.01777234158823529</v>
+        <v>-0.01737735188235294</v>
       </c>
       <c r="AF96" s="11" t="n">
-        <v>-1.598570407407407</v>
+        <v>-1.563042232804233</v>
       </c>
     </row>
     <row r="97">
@@ -18720,22 +18732,22 @@
         <v>-37.70091492835979</v>
       </c>
       <c r="AA97" s="15" t="n">
-        <v>-51.016672</v>
+        <v>-44.301847</v>
       </c>
       <c r="AB97" s="15" t="n">
-        <v>-0.003000980705882353</v>
+        <v>-0.002605991</v>
       </c>
       <c r="AC97" s="15" t="n">
-        <v>-0.2699294814814815</v>
+        <v>-0.2344013068783069</v>
       </c>
       <c r="AD97" s="15" t="n">
-        <v>-7176.48959346</v>
+        <v>-7169.77476846</v>
       </c>
       <c r="AE97" s="15" t="n">
-        <v>-0.4221464466741177</v>
+        <v>-0.4217514569682353</v>
       </c>
       <c r="AF97" s="15" t="n">
-        <v>-37.97084440984127</v>
+        <v>-37.93531623523809</v>
       </c>
     </row>
     <row r="98">
@@ -20221,22 +20233,22 @@
         <v>-24.12021813227513</v>
       </c>
       <c r="AA116" s="11" t="n">
-        <v>-232.028585</v>
+        <v>-231.71171</v>
       </c>
       <c r="AB116" s="11" t="n">
-        <v>-0.01364874029411765</v>
+        <v>-0.01363010058823529</v>
       </c>
       <c r="AC116" s="11" t="n">
-        <v>-1.227664470899471</v>
+        <v>-1.225987883597884</v>
       </c>
       <c r="AD116" s="11" t="n">
-        <v>-4790.749812</v>
+        <v>-4790.432937</v>
       </c>
       <c r="AE116" s="11" t="n">
-        <v>-0.2818088124705883</v>
+        <v>-0.2817901727647059</v>
       </c>
       <c r="AF116" s="11" t="n">
-        <v>-25.3478826031746</v>
+        <v>-25.34620601587302</v>
       </c>
     </row>
     <row r="117">
@@ -20318,22 +20330,22 @@
         <v>-24.12021813227513</v>
       </c>
       <c r="AA117" s="15" t="n">
-        <v>-232.028585</v>
+        <v>-231.71171</v>
       </c>
       <c r="AB117" s="15" t="n">
-        <v>-0.01364874029411765</v>
+        <v>-0.01363010058823529</v>
       </c>
       <c r="AC117" s="15" t="n">
-        <v>-1.227664470899471</v>
+        <v>-1.225987883597884</v>
       </c>
       <c r="AD117" s="15" t="n">
-        <v>-4790.749812</v>
+        <v>-4790.432937</v>
       </c>
       <c r="AE117" s="15" t="n">
-        <v>-0.2818088124705883</v>
+        <v>-0.2817901727647059</v>
       </c>
       <c r="AF117" s="15" t="n">
-        <v>-25.3478826031746</v>
+        <v>-25.34620601587302</v>
       </c>
     </row>
     <row r="118">
@@ -20893,13 +20905,13 @@
         <v>-0.4559747513227513</v>
       </c>
       <c r="L125" s="11" t="n">
-        <v>-43.468282</v>
+        <v>-50.495844</v>
       </c>
       <c r="M125" s="11" t="n">
-        <v>-0.002556957764705882</v>
+        <v>-0.002970343764705882</v>
       </c>
       <c r="N125" s="11" t="n">
-        <v>-0.2299909100529101</v>
+        <v>-0.2671737777777778</v>
       </c>
       <c r="O125" s="11" t="n">
         <v>-50.240918</v>
@@ -20929,25 +20941,25 @@
         <v>-0.3155543968253968</v>
       </c>
       <c r="X125" s="11" t="n">
-        <v>-1040.425127</v>
+        <v>-1047.452689</v>
       </c>
       <c r="Y125" s="11" t="n">
-        <v>-0.06120147805882353</v>
+        <v>-0.06161486405882353</v>
       </c>
       <c r="Z125" s="11" t="n">
-        <v>-5.504894851851852</v>
+        <v>-5.54207771957672</v>
       </c>
       <c r="AA125" s="11" t="n"/>
       <c r="AB125" s="11" t="n"/>
       <c r="AC125" s="11" t="n"/>
       <c r="AD125" s="11" t="n">
-        <v>-1040.425127</v>
+        <v>-1047.452689</v>
       </c>
       <c r="AE125" s="11" t="n">
-        <v>-0.06120147805882353</v>
+        <v>-0.06161486405882353</v>
       </c>
       <c r="AF125" s="11" t="n">
-        <v>-5.504894851851852</v>
+        <v>-5.54207771957672</v>
       </c>
     </row>
     <row r="126">
@@ -20984,13 +20996,13 @@
         <v>-5.08571519047619</v>
       </c>
       <c r="L126" s="15" t="n">
-        <v>-6458.99431606</v>
+        <v>-6466.02187806</v>
       </c>
       <c r="M126" s="15" t="n">
-        <v>-0.3799408421211765</v>
+        <v>-0.3803542281211765</v>
       </c>
       <c r="N126" s="15" t="n">
-        <v>-34.17457310084656</v>
+        <v>-34.21175596857143</v>
       </c>
       <c r="O126" s="15" t="n">
         <v>-1318.8129594</v>
@@ -21020,13 +21032,13 @@
         <v>-10.2065108621164</v>
       </c>
       <c r="X126" s="15" t="n">
-        <v>-24556.73196941</v>
+        <v>-24563.75953141</v>
       </c>
       <c r="Y126" s="15" t="n">
-        <v>-1.444513645259412</v>
+        <v>-1.444927031259412</v>
       </c>
       <c r="Z126" s="15" t="n">
-        <v>-129.9297987799471</v>
+        <v>-129.966981647672</v>
       </c>
       <c r="AA126" s="15" t="n">
         <v>-28.1385</v>
@@ -21038,13 +21050,13 @@
         <v>-0.1488809523809524</v>
       </c>
       <c r="AD126" s="15" t="n">
-        <v>-24584.87046941</v>
+        <v>-24591.89803141</v>
       </c>
       <c r="AE126" s="15" t="n">
-        <v>-1.446168851141765</v>
+        <v>-1.446582237141765</v>
       </c>
       <c r="AF126" s="15" t="n">
-        <v>-130.078679732328</v>
+        <v>-130.1158626000529</v>
       </c>
     </row>
     <row r="127">
@@ -21707,13 +21719,13 @@
         <v>-14.62131566666667</v>
       </c>
       <c r="L135" s="15" t="n">
-        <v>-8651.59926906</v>
+        <v>-8658.626831059999</v>
       </c>
       <c r="M135" s="15" t="n">
-        <v>-0.5089176040623529</v>
+        <v>-0.5093309900623528</v>
       </c>
       <c r="N135" s="15" t="n">
-        <v>-45.77565750825396</v>
+        <v>-45.81284037597883</v>
       </c>
       <c r="O135" s="15" t="n">
         <v>-2654.29276086</v>
@@ -21743,31 +21755,31 @@
         <v>-21.39297416899471</v>
       </c>
       <c r="X135" s="15" t="n">
-        <v>-40282.91566031001</v>
+        <v>-40289.94322231</v>
       </c>
       <c r="Y135" s="15" t="n">
-        <v>-2.369583274135882</v>
+        <v>-2.369996660135882</v>
       </c>
       <c r="Z135" s="15" t="n">
-        <v>-213.1371198958201</v>
+        <v>-213.1743027635449</v>
       </c>
       <c r="AA135" s="15" t="n">
-        <v>-482.046975</v>
+        <v>-475.015275</v>
       </c>
       <c r="AB135" s="15" t="n">
-        <v>-0.0283557044117647</v>
+        <v>-0.027942075</v>
       </c>
       <c r="AC135" s="15" t="n">
-        <v>-2.550513095238095</v>
+        <v>-2.513308333333333</v>
       </c>
       <c r="AD135" s="15" t="n">
-        <v>-40764.96263531</v>
+        <v>-40764.95849731</v>
       </c>
       <c r="AE135" s="15" t="n">
-        <v>-2.397938978547647</v>
+        <v>-2.397938735135882</v>
       </c>
       <c r="AF135" s="15" t="n">
-        <v>-215.6876329910582</v>
+        <v>-215.6876110968783</v>
       </c>
     </row>
     <row r="136">
@@ -22993,22 +23005,22 @@
         <v>-340.1043937373017</v>
       </c>
       <c r="AA152" s="19" t="n">
-        <v>-149.999402</v>
+        <v>1414.208087</v>
       </c>
       <c r="AB152" s="19" t="n">
-        <v>-0.008823494235294119</v>
+        <v>0.083188711</v>
       </c>
       <c r="AC152" s="19" t="n">
-        <v>-0.7936476296296296</v>
+        <v>7.48258247089947</v>
       </c>
       <c r="AD152" s="19" t="n">
-        <v>-64429.72981835002</v>
+        <v>-62865.52232935002</v>
       </c>
       <c r="AE152" s="19" t="n">
-        <v>-3.789984106961766</v>
+        <v>-3.697971901726472</v>
       </c>
       <c r="AF152" s="19" t="n">
-        <v>-340.8980413669313</v>
+        <v>-332.6218112664022</v>
       </c>
     </row>
     <row r="153">
@@ -23090,22 +23102,22 @@
         <v>16.8991026984656</v>
       </c>
       <c r="AA153" s="7" t="n">
-        <v>3043.931008009999</v>
+        <v>4608.138497009999</v>
       </c>
       <c r="AB153" s="7" t="n">
-        <v>0.1790547651770588</v>
+        <v>0.2710669704123529</v>
       </c>
       <c r="AC153" s="7" t="n">
-        <v>16.10545506883598</v>
+        <v>24.38168516936507</v>
       </c>
       <c r="AD153" s="7" t="n">
-        <v>3043.931008009999</v>
+        <v>4608.138497009999</v>
       </c>
       <c r="AE153" s="7" t="n">
-        <v>0.1790547651770588</v>
+        <v>0.2710669704123529</v>
       </c>
       <c r="AF153" s="7" t="n">
-        <v>16.10545506883598</v>
+        <v>24.38168516936507</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh dashboard Tue 08/11/2026 17:18
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -726,7 +726,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 10 Aug 2026 16:54</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 11 Aug 2026 17:18</t>
         </is>
       </c>
     </row>
@@ -794,14 +794,14 @@
       <c r="Z3" s="4" t="n"/>
       <c r="AA3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 10 Aug 2026</t>
+          <t>MTD as of 11 Aug 2026</t>
         </is>
       </c>
       <c r="AB3" s="4" t="n"/>
       <c r="AC3" s="4" t="n"/>
       <c r="AD3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 10 Aug 2026</t>
+          <t>YTD as of 11 Aug 2026</t>
         </is>
       </c>
       <c r="AE3" s="4" t="n"/>
@@ -2025,22 +2025,22 @@
         <v>2099643.822698413</v>
       </c>
       <c r="AA19" s="11" t="n">
-        <v>8297720</v>
+        <v>9708220</v>
       </c>
       <c r="AB19" s="11" t="n">
-        <v>488.1011764705883</v>
+        <v>571.0717647058824</v>
       </c>
       <c r="AC19" s="11" t="n">
-        <v>43903.28042328043</v>
+        <v>51366.24338624338</v>
       </c>
       <c r="AD19" s="11" t="n">
-        <v>405130402.49</v>
+        <v>406540902.49</v>
       </c>
       <c r="AE19" s="11" t="n">
-        <v>23831.20014647059</v>
+        <v>23914.17073470588</v>
       </c>
       <c r="AF19" s="11" t="n">
-        <v>2143547.103121693</v>
+        <v>2151010.066084656</v>
       </c>
     </row>
     <row r="20">
@@ -2256,22 +2256,22 @@
         <v>140849.2063492063</v>
       </c>
       <c r="AA22" s="13" t="n">
-        <v>3906000</v>
+        <v>5316500</v>
       </c>
       <c r="AB22" s="13" t="n">
-        <v>229.7647058823529</v>
+        <v>312.7352941176471</v>
       </c>
       <c r="AC22" s="13" t="n">
-        <v>20666.66666666667</v>
+        <v>28129.62962962963</v>
       </c>
       <c r="AD22" s="13" t="n">
-        <v>30526500</v>
+        <v>31937000</v>
       </c>
       <c r="AE22" s="13" t="n">
-        <v>1795.676470588235</v>
+        <v>1878.647058823529</v>
       </c>
       <c r="AF22" s="13" t="n">
-        <v>161515.873015873</v>
+        <v>168978.835978836</v>
       </c>
     </row>
     <row r="23">
@@ -3512,22 +3512,22 @@
         <v>1138764600.240688</v>
       </c>
       <c r="AA42" s="15" t="n">
-        <v>3425597528</v>
+        <v>3427008028</v>
       </c>
       <c r="AB42" s="15" t="n">
-        <v>201505.7369411765</v>
+        <v>201588.7075294118</v>
       </c>
       <c r="AC42" s="15" t="n">
-        <v>18124854.64550265</v>
+        <v>18132317.60846561</v>
       </c>
       <c r="AD42" s="15" t="n">
-        <v>218652106973.49</v>
+        <v>218653517473.49</v>
       </c>
       <c r="AE42" s="15" t="n">
-        <v>12861888.64549941</v>
+        <v>12861971.61608765</v>
       </c>
       <c r="AF42" s="15" t="n">
-        <v>1156889454.88619</v>
+        <v>1156896917.849154</v>
       </c>
     </row>
     <row r="43">
@@ -10678,22 +10678,22 @@
         <v>-3855931.507936508</v>
       </c>
       <c r="AA140" s="11" t="n">
-        <v>-20000000</v>
+        <v>-26550000</v>
       </c>
       <c r="AB140" s="11" t="n">
-        <v>-1176.470588235294</v>
+        <v>-1561.764705882353</v>
       </c>
       <c r="AC140" s="11" t="n">
-        <v>-105820.1058201058</v>
+        <v>-140476.1904761905</v>
       </c>
       <c r="AD140" s="11" t="n">
-        <v>-748771055</v>
+        <v>-755321055</v>
       </c>
       <c r="AE140" s="11" t="n">
-        <v>-44045.35617647059</v>
+        <v>-44430.65029411764</v>
       </c>
       <c r="AF140" s="11" t="n">
-        <v>-3961751.613756614</v>
+        <v>-3996407.698412698</v>
       </c>
     </row>
     <row r="141">
@@ -10885,22 +10885,22 @@
         <v>-12697799.23280423</v>
       </c>
       <c r="AA143" s="15" t="n">
-        <v>-20000000</v>
+        <v>-26550000</v>
       </c>
       <c r="AB143" s="15" t="n">
-        <v>-1176.470588235294</v>
+        <v>-1561.764705882353</v>
       </c>
       <c r="AC143" s="15" t="n">
-        <v>-105820.1058201058</v>
+        <v>-140476.1904761905</v>
       </c>
       <c r="AD143" s="15" t="n">
-        <v>-2419884055</v>
+        <v>-2426434055</v>
       </c>
       <c r="AE143" s="15" t="n">
-        <v>-142346.120882353</v>
+        <v>-142731.415</v>
       </c>
       <c r="AF143" s="15" t="n">
-        <v>-12803619.33862434</v>
+        <v>-12838275.42328042</v>
       </c>
     </row>
     <row r="144">
@@ -11019,22 +11019,22 @@
         <v>-87167.31047619047</v>
       </c>
       <c r="AA145" s="11" t="n">
-        <v>-604723</v>
+        <v>-607223</v>
       </c>
       <c r="AB145" s="11" t="n">
-        <v>-35.57194117647059</v>
+        <v>-35.719</v>
       </c>
       <c r="AC145" s="11" t="n">
-        <v>-3199.592592592593</v>
+        <v>-3212.820105820106</v>
       </c>
       <c r="AD145" s="11" t="n">
-        <v>-17079344.68</v>
+        <v>-17081844.68</v>
       </c>
       <c r="AE145" s="11" t="n">
-        <v>-1004.667334117647</v>
+        <v>-1004.814392941176</v>
       </c>
       <c r="AF145" s="11" t="n">
-        <v>-90366.90306878307</v>
+        <v>-90380.13058201058</v>
       </c>
     </row>
     <row r="146">
@@ -11475,22 +11475,22 @@
         <v>-29993348.67783069</v>
       </c>
       <c r="AA151" s="15" t="n">
-        <v>-604723</v>
+        <v>-607223</v>
       </c>
       <c r="AB151" s="15" t="n">
-        <v>-35.57194117647059</v>
+        <v>-35.719</v>
       </c>
       <c r="AC151" s="15" t="n">
-        <v>-3199.592592592593</v>
+        <v>-3212.820105820106</v>
       </c>
       <c r="AD151" s="15" t="n">
-        <v>-5669347623.110001</v>
+        <v>-5669350123.110001</v>
       </c>
       <c r="AE151" s="15" t="n">
-        <v>-333491.0366535294</v>
+        <v>-333491.1837123529</v>
       </c>
       <c r="AF151" s="15" t="n">
-        <v>-29996548.27042328</v>
+        <v>-29996561.49793651</v>
       </c>
     </row>
     <row r="152">
@@ -11572,22 +11572,22 @@
         <v>-1478868993.977989</v>
       </c>
       <c r="AA152" s="19" t="n">
-        <v>-1808087363</v>
+        <v>-1814639863</v>
       </c>
       <c r="AB152" s="19" t="n">
-        <v>-106358.0801764706</v>
+        <v>-106743.5213529412</v>
       </c>
       <c r="AC152" s="19" t="n">
-        <v>-9566599.804232804</v>
+        <v>-9601269.116402116</v>
       </c>
       <c r="AD152" s="19" t="n">
-        <v>-281314327224.84</v>
+        <v>-281320879724.84</v>
       </c>
       <c r="AE152" s="19" t="n">
-        <v>-16547901.60146117</v>
+        <v>-16548287.04263764</v>
       </c>
       <c r="AF152" s="19" t="n">
-        <v>-1488435593.782222</v>
+        <v>-1488470263.094392</v>
       </c>
     </row>
     <row r="153">
@@ -11669,22 +11669,22 @@
         <v>-340104393.7373017</v>
       </c>
       <c r="AA153" s="19" t="n">
-        <v>1617510165</v>
+        <v>1612368165</v>
       </c>
       <c r="AB153" s="19" t="n">
-        <v>95147.65676470588</v>
+        <v>94845.18617647058</v>
       </c>
       <c r="AC153" s="19" t="n">
-        <v>8558254.841269841</v>
+        <v>8531048.492063493</v>
       </c>
       <c r="AD153" s="19" t="n">
-        <v>-62662220251.35001</v>
+        <v>-62667362251.35001</v>
       </c>
       <c r="AE153" s="19" t="n">
-        <v>-3686012.955961766</v>
+        <v>-3686315.426550001</v>
       </c>
       <c r="AF153" s="19" t="n">
-        <v>-331546138.8960319</v>
+        <v>-331573345.2452382</v>
       </c>
     </row>
     <row r="154">
@@ -11766,22 +11766,22 @@
         <v>16899102.6984656</v>
       </c>
       <c r="AA154" s="7" t="n">
-        <v>4811440575.009999</v>
+        <v>4806298575.009999</v>
       </c>
       <c r="AB154" s="7" t="n">
-        <v>283025.9161770588</v>
+        <v>282723.4455888235</v>
       </c>
       <c r="AC154" s="7" t="n">
-        <v>25457357.53973545</v>
+        <v>25430151.1905291</v>
       </c>
       <c r="AD154" s="7" t="n">
-        <v>4811440575.009999</v>
+        <v>4806298575.009999</v>
       </c>
       <c r="AE154" s="7" t="n">
-        <v>283025.9161770588</v>
+        <v>282723.4455888235</v>
       </c>
       <c r="AF154" s="7" t="n">
-        <v>25457357.53973545</v>
+        <v>25430151.1905291</v>
       </c>
     </row>
   </sheetData>
@@ -12004,16 +12004,16 @@
         <v>44055921.71</v>
       </c>
       <c r="E9" s="13" t="n">
-        <v>-32129637</v>
+        <v>-37271637</v>
       </c>
       <c r="F9" s="13" t="n">
-        <v>11926284.71</v>
+        <v>6784284.710000001</v>
       </c>
       <c r="G9" s="24" t="n">
-        <v>701.5461594117647</v>
+        <v>399.0755711764706</v>
       </c>
       <c r="H9" s="24" t="n">
-        <v>63102.03550264551</v>
+        <v>35895.6862962963</v>
       </c>
     </row>
     <row r="10">
@@ -12123,13 +12123,13 @@
       <c r="D13" s="26" t="n"/>
       <c r="E13" s="26" t="n"/>
       <c r="F13" s="27" t="n">
-        <v>4811440577.01</v>
+        <v>4806298577.01</v>
       </c>
       <c r="G13" s="28" t="n">
-        <v>283025.9162947059</v>
+        <v>282723.4457064706</v>
       </c>
       <c r="H13" s="28" t="n">
-        <v>25457357.55031746</v>
+        <v>25430151.20111111</v>
       </c>
     </row>
   </sheetData>
@@ -12196,7 +12196,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 10 Aug 2026 16:54 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 11 Aug 2026 17:18 (in IDR Million)</t>
         </is>
       </c>
     </row>
@@ -12264,14 +12264,14 @@
       <c r="Z3" s="4" t="n"/>
       <c r="AA3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 10 Aug 2026</t>
+          <t>MTD as of 11 Aug 2026</t>
         </is>
       </c>
       <c r="AB3" s="4" t="n"/>
       <c r="AC3" s="4" t="n"/>
       <c r="AD3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 10 Aug 2026</t>
+          <t>YTD as of 11 Aug 2026</t>
         </is>
       </c>
       <c r="AE3" s="4" t="n"/>
@@ -13495,22 +13495,22 @@
         <v>2.099643822698413</v>
       </c>
       <c r="AA19" s="11" t="n">
-        <v>8.29772</v>
+        <v>9.708220000000001</v>
       </c>
       <c r="AB19" s="11" t="n">
-        <v>0.0004881011764705883</v>
+        <v>0.0005710717647058824</v>
       </c>
       <c r="AC19" s="11" t="n">
-        <v>0.04390328042328042</v>
+        <v>0.05136624338624339</v>
       </c>
       <c r="AD19" s="11" t="n">
-        <v>405.13040249</v>
+        <v>406.54090249</v>
       </c>
       <c r="AE19" s="11" t="n">
-        <v>0.02383120014647059</v>
+        <v>0.02391417073470588</v>
       </c>
       <c r="AF19" s="11" t="n">
-        <v>2.143547103121693</v>
+        <v>2.151010066084656</v>
       </c>
     </row>
     <row r="20">
@@ -13726,22 +13726,22 @@
         <v>0.1408492063492063</v>
       </c>
       <c r="AA22" s="13" t="n">
-        <v>3.906</v>
+        <v>5.3165</v>
       </c>
       <c r="AB22" s="13" t="n">
-        <v>0.000229764705882353</v>
+        <v>0.000312735294117647</v>
       </c>
       <c r="AC22" s="13" t="n">
-        <v>0.02066666666666667</v>
+        <v>0.02812962962962963</v>
       </c>
       <c r="AD22" s="13" t="n">
-        <v>30.5265</v>
+        <v>31.937</v>
       </c>
       <c r="AE22" s="13" t="n">
-        <v>0.001795676470588235</v>
+        <v>0.001878647058823529</v>
       </c>
       <c r="AF22" s="13" t="n">
-        <v>0.161515873015873</v>
+        <v>0.168978835978836</v>
       </c>
     </row>
     <row r="23">
@@ -14982,22 +14982,22 @@
         <v>1138.764600240688</v>
       </c>
       <c r="AA42" s="15" t="n">
-        <v>3425.597528</v>
+        <v>3427.008028</v>
       </c>
       <c r="AB42" s="15" t="n">
-        <v>0.2015057369411765</v>
+        <v>0.2015887075294118</v>
       </c>
       <c r="AC42" s="15" t="n">
-        <v>18.12485464550264</v>
+        <v>18.13231760846561</v>
       </c>
       <c r="AD42" s="15" t="n">
-        <v>218652.10697349</v>
+        <v>218653.51747349</v>
       </c>
       <c r="AE42" s="15" t="n">
-        <v>12.86188864549941</v>
+        <v>12.86197161608765</v>
       </c>
       <c r="AF42" s="15" t="n">
-        <v>1156.88945488619</v>
+        <v>1156.896917849153</v>
       </c>
     </row>
     <row r="43">
@@ -22148,22 +22148,22 @@
         <v>-3.855931507936508</v>
       </c>
       <c r="AA140" s="11" t="n">
-        <v>-20</v>
+        <v>-26.55</v>
       </c>
       <c r="AB140" s="11" t="n">
-        <v>-0.001176470588235294</v>
+        <v>-0.001561764705882353</v>
       </c>
       <c r="AC140" s="11" t="n">
-        <v>-0.1058201058201058</v>
+        <v>-0.1404761904761905</v>
       </c>
       <c r="AD140" s="11" t="n">
-        <v>-748.771055</v>
+        <v>-755.321055</v>
       </c>
       <c r="AE140" s="11" t="n">
-        <v>-0.0440453561764706</v>
+        <v>-0.04443065029411766</v>
       </c>
       <c r="AF140" s="11" t="n">
-        <v>-3.961751613756614</v>
+        <v>-3.996407698412698</v>
       </c>
     </row>
     <row r="141">
@@ -22355,22 +22355,22 @@
         <v>-12.69779923280423</v>
       </c>
       <c r="AA143" s="15" t="n">
-        <v>-20</v>
+        <v>-26.55</v>
       </c>
       <c r="AB143" s="15" t="n">
-        <v>-0.001176470588235294</v>
+        <v>-0.001561764705882353</v>
       </c>
       <c r="AC143" s="15" t="n">
-        <v>-0.1058201058201058</v>
+        <v>-0.1404761904761905</v>
       </c>
       <c r="AD143" s="15" t="n">
-        <v>-2419.884055</v>
+        <v>-2426.434055</v>
       </c>
       <c r="AE143" s="15" t="n">
-        <v>-0.142346120882353</v>
+        <v>-0.142731415</v>
       </c>
       <c r="AF143" s="15" t="n">
-        <v>-12.80361933862434</v>
+        <v>-12.83827542328042</v>
       </c>
     </row>
     <row r="144">
@@ -22489,22 +22489,22 @@
         <v>-0.08716731047619047</v>
       </c>
       <c r="AA145" s="11" t="n">
-        <v>-0.604723</v>
+        <v>-0.607223</v>
       </c>
       <c r="AB145" s="11" t="n">
-        <v>-3.557194117647059e-05</v>
+        <v>-3.571899999999999e-05</v>
       </c>
       <c r="AC145" s="11" t="n">
-        <v>-0.003199592592592593</v>
+        <v>-0.003212820105820106</v>
       </c>
       <c r="AD145" s="11" t="n">
-        <v>-17.07934468</v>
+        <v>-17.08184468</v>
       </c>
       <c r="AE145" s="11" t="n">
-        <v>-0.001004667334117647</v>
+        <v>-0.001004814392941176</v>
       </c>
       <c r="AF145" s="11" t="n">
-        <v>-0.09036690306878306</v>
+        <v>-0.09038013058201058</v>
       </c>
     </row>
     <row r="146">
@@ -22945,22 +22945,22 @@
         <v>-29.99334867783069</v>
       </c>
       <c r="AA151" s="15" t="n">
-        <v>-0.604723</v>
+        <v>-0.607223</v>
       </c>
       <c r="AB151" s="15" t="n">
-        <v>-3.557194117647059e-05</v>
+        <v>-3.571899999999999e-05</v>
       </c>
       <c r="AC151" s="15" t="n">
-        <v>-0.003199592592592593</v>
+        <v>-0.003212820105820106</v>
       </c>
       <c r="AD151" s="15" t="n">
-        <v>-5669.34762311</v>
+        <v>-5669.35012311</v>
       </c>
       <c r="AE151" s="15" t="n">
-        <v>-0.3334910366535295</v>
+        <v>-0.333491183712353</v>
       </c>
       <c r="AF151" s="15" t="n">
-        <v>-29.99654827042328</v>
+        <v>-29.9965614979365</v>
       </c>
     </row>
     <row r="152">
@@ -23042,22 +23042,22 @@
         <v>-1478.868993977989</v>
       </c>
       <c r="AA152" s="19" t="n">
-        <v>-1808.087363</v>
+        <v>-1814.639863</v>
       </c>
       <c r="AB152" s="19" t="n">
-        <v>-0.1063580801764706</v>
+        <v>-0.1067435213529412</v>
       </c>
       <c r="AC152" s="19" t="n">
-        <v>-9.566599804232805</v>
+        <v>-9.601269116402117</v>
       </c>
       <c r="AD152" s="19" t="n">
-        <v>-281314.3272248399</v>
+        <v>-281320.8797248399</v>
       </c>
       <c r="AE152" s="19" t="n">
-        <v>-16.54790160146118</v>
+        <v>-16.54828704263765</v>
       </c>
       <c r="AF152" s="19" t="n">
-        <v>-1488.435593782222</v>
+        <v>-1488.470263094391</v>
       </c>
     </row>
     <row r="153">
@@ -23139,22 +23139,22 @@
         <v>-340.1043937373017</v>
       </c>
       <c r="AA153" s="19" t="n">
-        <v>1617.510165</v>
+        <v>1612.368165</v>
       </c>
       <c r="AB153" s="19" t="n">
-        <v>0.09514765676470588</v>
+        <v>0.0948451861764706</v>
       </c>
       <c r="AC153" s="19" t="n">
-        <v>8.558254841269841</v>
+        <v>8.531048492063492</v>
       </c>
       <c r="AD153" s="19" t="n">
-        <v>-62662.22025135002</v>
+        <v>-62667.36225135002</v>
       </c>
       <c r="AE153" s="19" t="n">
-        <v>-3.686012955961766</v>
+        <v>-3.686315426550001</v>
       </c>
       <c r="AF153" s="19" t="n">
-        <v>-331.5461388960318</v>
+        <v>-331.5733452452382</v>
       </c>
     </row>
     <row r="154">
@@ -23236,22 +23236,22 @@
         <v>16.8991026984656</v>
       </c>
       <c r="AA154" s="7" t="n">
-        <v>4811.44057501</v>
+        <v>4806.29857501</v>
       </c>
       <c r="AB154" s="7" t="n">
-        <v>0.2830259161770588</v>
+        <v>0.2827234455888235</v>
       </c>
       <c r="AC154" s="7" t="n">
-        <v>25.45735753973545</v>
+        <v>25.4301511905291</v>
       </c>
       <c r="AD154" s="7" t="n">
-        <v>4811.44057501</v>
+        <v>4806.29857501</v>
       </c>
       <c r="AE154" s="7" t="n">
-        <v>0.2830259161770588</v>
+        <v>0.2827234455888235</v>
       </c>
       <c r="AF154" s="7" t="n">
-        <v>25.45735753973545</v>
+        <v>25.4301511905291</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh dashboard Thu 08/13/2026 17:04
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CF Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CF Summary (IDR Mio)" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bank - Jan" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bank - Feb" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bank - Mar" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bank - Apr" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bank - May" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bank - Jun" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bank - Jul" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bank - Aug" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="CF Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="CF Summary (IDR Mio)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Bank - Jan" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Bank - Feb" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Bank - Mar" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Bank - Apr" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Bank - May" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Bank - Jun" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Bank - Jul" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Bank - Aug" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -726,7 +726,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 11 Aug 2026 17:18</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 13 Aug 2026 17:04</t>
         </is>
       </c>
     </row>
@@ -794,14 +794,14 @@
       <c r="Z3" s="4" t="n"/>
       <c r="AA3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 11 Aug 2026</t>
+          <t>MTD as of 13 Aug 2026</t>
         </is>
       </c>
       <c r="AB3" s="4" t="n"/>
       <c r="AC3" s="4" t="n"/>
       <c r="AD3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 11 Aug 2026</t>
+          <t>YTD as of 13 Aug 2026</t>
         </is>
       </c>
       <c r="AE3" s="4" t="n"/>
@@ -1173,22 +1173,22 @@
         <v>873088236.8412699</v>
       </c>
       <c r="AA7" s="11" t="n">
-        <v>3417299808</v>
+        <v>3597677676</v>
       </c>
       <c r="AB7" s="11" t="n">
-        <v>201017.6357647059</v>
+        <v>211628.0985882353</v>
       </c>
       <c r="AC7" s="11" t="n">
-        <v>18080951.36507937</v>
+        <v>19035331.61904762</v>
       </c>
       <c r="AD7" s="11" t="n">
-        <v>168430976571</v>
+        <v>168611354439</v>
       </c>
       <c r="AE7" s="11" t="n">
-        <v>9907704.50417647</v>
+        <v>9918314.967</v>
       </c>
       <c r="AF7" s="11" t="n">
-        <v>891169188.2063493</v>
+        <v>892123568.4603175</v>
       </c>
     </row>
     <row r="8">
@@ -1524,17 +1524,23 @@
       <c r="Z11" s="11" t="n">
         <v>38029556.94708995</v>
       </c>
-      <c r="AA11" s="11" t="n"/>
-      <c r="AB11" s="11" t="n"/>
-      <c r="AC11" s="11" t="n"/>
+      <c r="AA11" s="11" t="n">
+        <v>180377868</v>
+      </c>
+      <c r="AB11" s="11" t="n">
+        <v>10610.46282352941</v>
+      </c>
+      <c r="AC11" s="11" t="n">
+        <v>954380.253968254</v>
+      </c>
       <c r="AD11" s="11" t="n">
-        <v>7187586263</v>
+        <v>7367964131</v>
       </c>
       <c r="AE11" s="11" t="n">
-        <v>422799.1919411765</v>
+        <v>433409.6547647059</v>
       </c>
       <c r="AF11" s="11" t="n">
-        <v>38029556.94708995</v>
+        <v>38983937.2010582</v>
       </c>
     </row>
     <row r="12">
@@ -2025,22 +2031,22 @@
         <v>2099643.822698413</v>
       </c>
       <c r="AA19" s="11" t="n">
-        <v>9708220</v>
+        <v>11818180</v>
       </c>
       <c r="AB19" s="11" t="n">
-        <v>571.0717647058824</v>
+        <v>695.1870588235294</v>
       </c>
       <c r="AC19" s="11" t="n">
-        <v>51366.24338624338</v>
+        <v>62530.05291005291</v>
       </c>
       <c r="AD19" s="11" t="n">
-        <v>406540902.49</v>
+        <v>408650862.49</v>
       </c>
       <c r="AE19" s="11" t="n">
-        <v>23914.17073470588</v>
+        <v>24038.28602882353</v>
       </c>
       <c r="AF19" s="11" t="n">
-        <v>2151010.066084656</v>
+        <v>2162173.875608466</v>
       </c>
     </row>
     <row r="20">
@@ -2256,22 +2262,22 @@
         <v>140849.2063492063</v>
       </c>
       <c r="AA22" s="13" t="n">
-        <v>5316500</v>
+        <v>7404500</v>
       </c>
       <c r="AB22" s="13" t="n">
-        <v>312.7352941176471</v>
+        <v>435.5588235294118</v>
       </c>
       <c r="AC22" s="13" t="n">
-        <v>28129.62962962963</v>
+        <v>39177.24867724867</v>
       </c>
       <c r="AD22" s="13" t="n">
-        <v>31937000</v>
+        <v>34025000</v>
       </c>
       <c r="AE22" s="13" t="n">
-        <v>1878.647058823529</v>
+        <v>2001.470588235294</v>
       </c>
       <c r="AF22" s="13" t="n">
-        <v>168978.835978836</v>
+        <v>180026.455026455</v>
       </c>
     </row>
     <row r="23">
@@ -2566,17 +2572,23 @@
       <c r="Z27" s="11" t="n">
         <v>62742.76190476191</v>
       </c>
-      <c r="AA27" s="11" t="n"/>
-      <c r="AB27" s="11" t="n"/>
-      <c r="AC27" s="11" t="n"/>
+      <c r="AA27" s="11" t="n">
+        <v>21960</v>
+      </c>
+      <c r="AB27" s="11" t="n">
+        <v>1.291764705882353</v>
+      </c>
+      <c r="AC27" s="11" t="n">
+        <v>116.1904761904762</v>
+      </c>
       <c r="AD27" s="11" t="n">
-        <v>11858382</v>
+        <v>11880342</v>
       </c>
       <c r="AE27" s="11" t="n">
-        <v>697.5518823529411</v>
+        <v>698.8436470588234</v>
       </c>
       <c r="AF27" s="11" t="n">
-        <v>62742.76190476191</v>
+        <v>62858.95238095238</v>
       </c>
     </row>
     <row r="28">
@@ -3512,22 +3524,22 @@
         <v>1138764600.240688</v>
       </c>
       <c r="AA42" s="15" t="n">
-        <v>3427008028</v>
+        <v>3609495856</v>
       </c>
       <c r="AB42" s="15" t="n">
-        <v>201588.7075294118</v>
+        <v>212323.2856470588</v>
       </c>
       <c r="AC42" s="15" t="n">
-        <v>18132317.60846561</v>
+        <v>19097861.67195767</v>
       </c>
       <c r="AD42" s="15" t="n">
-        <v>218653517473.49</v>
+        <v>218836005301.49</v>
       </c>
       <c r="AE42" s="15" t="n">
-        <v>12861971.61608765</v>
+        <v>12872706.19420529</v>
       </c>
       <c r="AF42" s="15" t="n">
-        <v>1156896917.849154</v>
+        <v>1157862461.912646</v>
       </c>
     </row>
     <row r="43">
@@ -3878,22 +3890,22 @@
         <v>-6710414.91005291</v>
       </c>
       <c r="AA48" s="13" t="n">
-        <v>-175119091</v>
+        <v>-330642699</v>
       </c>
       <c r="AB48" s="13" t="n">
-        <v>-10301.123</v>
+        <v>-19449.57052941177</v>
       </c>
       <c r="AC48" s="13" t="n">
-        <v>-926556.0370370371</v>
+        <v>-1749432.26984127</v>
       </c>
       <c r="AD48" s="13" t="n">
-        <v>-1443387509</v>
+        <v>-1598911117</v>
       </c>
       <c r="AE48" s="13" t="n">
-        <v>-84905.1475882353</v>
+        <v>-94053.59511764706</v>
       </c>
       <c r="AF48" s="13" t="n">
-        <v>-7636970.947089947</v>
+        <v>-8459847.179894179</v>
       </c>
     </row>
     <row r="49">
@@ -4146,22 +4158,22 @@
         <v>-5318351.925925925</v>
       </c>
       <c r="AA52" s="13" t="n">
-        <v>-79714150</v>
+        <v>-196493076</v>
       </c>
       <c r="AB52" s="13" t="n">
-        <v>-4689.067647058823</v>
+        <v>-11558.41623529412</v>
       </c>
       <c r="AC52" s="13" t="n">
-        <v>-421767.9894179894</v>
+        <v>-1039645.904761905</v>
       </c>
       <c r="AD52" s="13" t="n">
-        <v>-1084882664</v>
+        <v>-1201661590</v>
       </c>
       <c r="AE52" s="13" t="n">
-        <v>-63816.62729411765</v>
+        <v>-70685.97588235294</v>
       </c>
       <c r="AF52" s="13" t="n">
-        <v>-5740119.915343915</v>
+        <v>-6357997.83068783</v>
       </c>
     </row>
     <row r="53">
@@ -4370,17 +4382,23 @@
       <c r="Z55" s="11" t="n">
         <v>-981189.5714285715</v>
       </c>
-      <c r="AA55" s="11" t="n"/>
-      <c r="AB55" s="11" t="n"/>
-      <c r="AC55" s="11" t="n"/>
+      <c r="AA55" s="11" t="n">
+        <v>-50750000</v>
+      </c>
+      <c r="AB55" s="11" t="n">
+        <v>-2985.294117647059</v>
+      </c>
+      <c r="AC55" s="11" t="n">
+        <v>-268518.5185185185</v>
+      </c>
       <c r="AD55" s="11" t="n">
-        <v>-185444829</v>
+        <v>-236194829</v>
       </c>
       <c r="AE55" s="11" t="n">
-        <v>-10908.51935294118</v>
+        <v>-13893.81347058824</v>
       </c>
       <c r="AF55" s="11" t="n">
-        <v>-981189.5714285715</v>
+        <v>-1249708.08994709</v>
       </c>
     </row>
     <row r="56">
@@ -4462,22 +4480,22 @@
         <v>-14482685.85121693</v>
       </c>
       <c r="AA56" s="13" t="n">
-        <v>-21932500</v>
+        <v>-197257569</v>
       </c>
       <c r="AB56" s="13" t="n">
-        <v>-1290.14705882353</v>
+        <v>-11603.38641176471</v>
       </c>
       <c r="AC56" s="13" t="n">
-        <v>-116044.9735449735</v>
+        <v>-1043690.841269841</v>
       </c>
       <c r="AD56" s="13" t="n">
-        <v>-2759160125.88</v>
+        <v>-2934485194.88</v>
       </c>
       <c r="AE56" s="13" t="n">
-        <v>-162303.5368164706</v>
+        <v>-172616.7761694118</v>
       </c>
       <c r="AF56" s="13" t="n">
-        <v>-14598730.8247619</v>
+        <v>-15526376.69248677</v>
       </c>
     </row>
     <row r="57">
@@ -4754,22 +4772,22 @@
         <v>-75623143.55492064</v>
       </c>
       <c r="AA60" s="15" t="n">
-        <v>-280761741</v>
+        <v>-779139344</v>
       </c>
       <c r="AB60" s="15" t="n">
-        <v>-16515.39652941177</v>
+        <v>-45831.72611764706</v>
       </c>
       <c r="AC60" s="15" t="n">
-        <v>-1485511.857142857</v>
+        <v>-4122430.391534391</v>
       </c>
       <c r="AD60" s="15" t="n">
-        <v>-14573535872.88</v>
+        <v>-15071913475.88</v>
       </c>
       <c r="AE60" s="15" t="n">
-        <v>-857266.8160517646</v>
+        <v>-886583.1456399999</v>
       </c>
       <c r="AF60" s="15" t="n">
-        <v>-77108655.41206349</v>
+        <v>-79745573.94645503</v>
       </c>
     </row>
     <row r="61">
@@ -5853,22 +5871,22 @@
         <v>-37173938.39968254</v>
       </c>
       <c r="AA79" s="13" t="n">
-        <v>-1025670494</v>
+        <v>-1610498009</v>
       </c>
       <c r="AB79" s="13" t="n">
-        <v>-60333.55847058824</v>
+        <v>-94735.177</v>
       </c>
       <c r="AC79" s="13" t="n">
-        <v>-5426828.01058201</v>
+        <v>-8521153.486772487</v>
       </c>
       <c r="AD79" s="13" t="n">
-        <v>-8051544851.54</v>
+        <v>-8636372366.540001</v>
       </c>
       <c r="AE79" s="13" t="n">
-        <v>-473620.2853847059</v>
+        <v>-508021.9039141176</v>
       </c>
       <c r="AF79" s="13" t="n">
-        <v>-42600766.41026455</v>
+        <v>-45695091.88645503</v>
       </c>
     </row>
     <row r="80">
@@ -6041,22 +6059,22 @@
         <v>-2010421.349206349</v>
       </c>
       <c r="AA81" s="13" t="n">
-        <v>-4350012</v>
+        <v>-7701172</v>
       </c>
       <c r="AB81" s="13" t="n">
-        <v>-255.8830588235294</v>
+        <v>-453.0101176470588</v>
       </c>
       <c r="AC81" s="13" t="n">
-        <v>-23015.93650793651</v>
+        <v>-40746.9417989418</v>
       </c>
       <c r="AD81" s="13" t="n">
-        <v>-384319647</v>
+        <v>-387670807</v>
       </c>
       <c r="AE81" s="13" t="n">
-        <v>-22607.03805882353</v>
+        <v>-22804.16511764706</v>
       </c>
       <c r="AF81" s="13" t="n">
-        <v>-2033437.285714286</v>
+        <v>-2051168.291005291</v>
       </c>
     </row>
     <row r="82">
@@ -6138,22 +6156,22 @@
         <v>-104413128.6271958</v>
       </c>
       <c r="AA82" s="15" t="n">
-        <v>-1030020506</v>
+        <v>-1618199181</v>
       </c>
       <c r="AB82" s="15" t="n">
-        <v>-60589.44152941176</v>
+        <v>-95188.18711764706</v>
       </c>
       <c r="AC82" s="15" t="n">
-        <v>-5449843.947089947</v>
+        <v>-8561900.428571429</v>
       </c>
       <c r="AD82" s="15" t="n">
-        <v>-20764101816.54</v>
+        <v>-21352280491.54</v>
       </c>
       <c r="AE82" s="15" t="n">
-        <v>-1221417.753914118</v>
+        <v>-1256016.499502353</v>
       </c>
       <c r="AF82" s="15" t="n">
-        <v>-109862972.5742857</v>
+        <v>-112975029.0557672</v>
       </c>
     </row>
     <row r="83">
@@ -6601,22 +6619,22 @@
         <v>-516486.5661375662</v>
       </c>
       <c r="AA89" s="11" t="n">
-        <v>-11771650</v>
+        <v>-16662275</v>
       </c>
       <c r="AB89" s="11" t="n">
-        <v>-692.45</v>
+        <v>-980.1338235294118</v>
       </c>
       <c r="AC89" s="11" t="n">
-        <v>-62283.86243386244</v>
+        <v>-88160.18518518518</v>
       </c>
       <c r="AD89" s="11" t="n">
-        <v>-109387611</v>
+        <v>-114278236</v>
       </c>
       <c r="AE89" s="11" t="n">
-        <v>-6434.565352941176</v>
+        <v>-6722.249176470587</v>
       </c>
       <c r="AF89" s="11" t="n">
-        <v>-578770.4285714286</v>
+        <v>-604646.7513227514</v>
       </c>
     </row>
     <row r="90">
@@ -6686,22 +6704,22 @@
         <v>-8792.042328042327</v>
       </c>
       <c r="AA90" s="13" t="n">
-        <v>-222100</v>
+        <v>-266800</v>
       </c>
       <c r="AB90" s="13" t="n">
-        <v>-13.06470588235294</v>
+        <v>-15.69411764705882</v>
       </c>
       <c r="AC90" s="13" t="n">
-        <v>-1175.132275132275</v>
+        <v>-1411.640211640212</v>
       </c>
       <c r="AD90" s="13" t="n">
-        <v>-1883796</v>
+        <v>-1928496</v>
       </c>
       <c r="AE90" s="13" t="n">
-        <v>-110.8115294117647</v>
+        <v>-113.4409411764706</v>
       </c>
       <c r="AF90" s="13" t="n">
-        <v>-9967.174603174602</v>
+        <v>-10203.68253968254</v>
       </c>
     </row>
     <row r="91">
@@ -6783,22 +6801,22 @@
         <v>-1216540.901798942</v>
       </c>
       <c r="AA91" s="15" t="n">
-        <v>-12968230</v>
+        <v>-17903555</v>
       </c>
       <c r="AB91" s="15" t="n">
-        <v>-762.8370588235294</v>
+        <v>-1053.150294117647</v>
       </c>
       <c r="AC91" s="15" t="n">
-        <v>-68614.97354497355</v>
+        <v>-94727.80423280424</v>
       </c>
       <c r="AD91" s="15" t="n">
-        <v>-242894460.44</v>
+        <v>-247829785.44</v>
       </c>
       <c r="AE91" s="15" t="n">
-        <v>-14287.90943764706</v>
+        <v>-14578.22267294118</v>
       </c>
       <c r="AF91" s="15" t="n">
-        <v>-1285155.875343915</v>
+        <v>-1311268.706031746</v>
       </c>
     </row>
     <row r="92">
@@ -7093,22 +7111,22 @@
         <v>-33682338.66910053</v>
       </c>
       <c r="AA95" s="11" t="n">
-        <v>-26144663</v>
+        <v>-95187678</v>
       </c>
       <c r="AB95" s="11" t="n">
-        <v>-1537.921352941177</v>
+        <v>-5599.275176470588</v>
       </c>
       <c r="AC95" s="11" t="n">
-        <v>-138331.5502645503</v>
+        <v>-503638.5079365079</v>
       </c>
       <c r="AD95" s="11" t="n">
-        <v>-6392106671.46</v>
+        <v>-6461149686.46</v>
       </c>
       <c r="AE95" s="11" t="n">
-        <v>-376006.2747917647</v>
+        <v>-380067.6286152941</v>
       </c>
       <c r="AF95" s="11" t="n">
-        <v>-33820670.21936508</v>
+        <v>-34185977.17703704</v>
       </c>
     </row>
     <row r="96">
@@ -7190,22 +7208,22 @@
         <v>-1024866.306878307</v>
       </c>
       <c r="AA96" s="13" t="n">
-        <v>-7718584</v>
+        <v>-51239630</v>
       </c>
       <c r="AB96" s="13" t="n">
-        <v>-454.0343529411765</v>
+        <v>-3014.095882352941</v>
       </c>
       <c r="AC96" s="13" t="n">
-        <v>-40839.06878306878</v>
+        <v>-271109.1534391535</v>
       </c>
       <c r="AD96" s="13" t="n">
-        <v>-201418316</v>
+        <v>-244939362</v>
       </c>
       <c r="AE96" s="13" t="n">
-        <v>-11848.13623529412</v>
+        <v>-14408.19776470588</v>
       </c>
       <c r="AF96" s="13" t="n">
-        <v>-1065705.375661375</v>
+        <v>-1295975.46031746</v>
       </c>
     </row>
     <row r="97">
@@ -7287,22 +7305,22 @@
         <v>-1550969.746031746</v>
       </c>
       <c r="AA97" s="11" t="n">
-        <v>-2281700</v>
+        <v>-21011525</v>
       </c>
       <c r="AB97" s="11" t="n">
-        <v>-134.2176470588235</v>
+        <v>-1235.972058823529</v>
       </c>
       <c r="AC97" s="11" t="n">
-        <v>-12072.48677248677</v>
+        <v>-111172.0899470899</v>
       </c>
       <c r="AD97" s="11" t="n">
-        <v>-295414982</v>
+        <v>-314144807</v>
       </c>
       <c r="AE97" s="11" t="n">
-        <v>-17377.35188235294</v>
+        <v>-18479.10629411765</v>
       </c>
       <c r="AF97" s="11" t="n">
-        <v>-1563042.232804233</v>
+        <v>-1662141.835978836</v>
       </c>
     </row>
     <row r="98">
@@ -7384,22 +7402,22 @@
         <v>-37700914.92835979</v>
       </c>
       <c r="AA98" s="15" t="n">
-        <v>-44301847</v>
+        <v>-175595733</v>
       </c>
       <c r="AB98" s="15" t="n">
-        <v>-2605.991</v>
+        <v>-10329.16076470588</v>
       </c>
       <c r="AC98" s="15" t="n">
-        <v>-234401.3068783069</v>
+        <v>-929077.9523809524</v>
       </c>
       <c r="AD98" s="15" t="n">
-        <v>-7169774768.46</v>
+        <v>-7301068654.46</v>
       </c>
       <c r="AE98" s="15" t="n">
-        <v>-421751.4569682353</v>
+        <v>-429474.6267329411</v>
       </c>
       <c r="AF98" s="15" t="n">
-        <v>-37935316.2352381</v>
+        <v>-38629992.88074075</v>
       </c>
     </row>
     <row r="99">
@@ -7518,22 +7536,22 @@
         <v>-969478.4497354496</v>
       </c>
       <c r="AA100" s="11" t="n">
-        <v>-16550100</v>
+        <v>-16795100</v>
       </c>
       <c r="AB100" s="11" t="n">
-        <v>-973.535294117647</v>
+        <v>-987.9470588235295</v>
       </c>
       <c r="AC100" s="11" t="n">
-        <v>-87566.66666666667</v>
+        <v>-88862.96296296296</v>
       </c>
       <c r="AD100" s="11" t="n">
-        <v>-199781527</v>
+        <v>-200026527</v>
       </c>
       <c r="AE100" s="11" t="n">
-        <v>-11751.85452941176</v>
+        <v>-11766.26629411765</v>
       </c>
       <c r="AF100" s="11" t="n">
-        <v>-1057045.116402116</v>
+        <v>-1058341.412698413</v>
       </c>
     </row>
     <row r="101">
@@ -7615,22 +7633,22 @@
         <v>-848295.1375661377</v>
       </c>
       <c r="AA101" s="13" t="n">
-        <v>-3996850</v>
+        <v>-9791050</v>
       </c>
       <c r="AB101" s="13" t="n">
-        <v>-235.1088235294118</v>
+        <v>-575.9441176470589</v>
       </c>
       <c r="AC101" s="13" t="n">
-        <v>-21147.3544973545</v>
+        <v>-51804.49735449735</v>
       </c>
       <c r="AD101" s="13" t="n">
-        <v>-164324631</v>
+        <v>-170118831</v>
       </c>
       <c r="AE101" s="13" t="n">
-        <v>-9666.154764705883</v>
+        <v>-10006.99005882353</v>
       </c>
       <c r="AF101" s="13" t="n">
-        <v>-869442.4920634922</v>
+        <v>-900099.634920635</v>
       </c>
     </row>
     <row r="102">
@@ -7712,22 +7730,22 @@
         <v>-6305078.687830688</v>
       </c>
       <c r="AA102" s="11" t="n">
-        <v>-71406928</v>
+        <v>-193402912</v>
       </c>
       <c r="AB102" s="11" t="n">
-        <v>-4200.407529411765</v>
+        <v>-11376.64188235294</v>
       </c>
       <c r="AC102" s="11" t="n">
-        <v>-377814.4338624339</v>
+        <v>-1023295.830687831</v>
       </c>
       <c r="AD102" s="11" t="n">
-        <v>-1263066800</v>
+        <v>-1385062784</v>
       </c>
       <c r="AE102" s="11" t="n">
-        <v>-74298.04705882353</v>
+        <v>-81474.28141176471</v>
       </c>
       <c r="AF102" s="11" t="n">
-        <v>-6682893.121693121</v>
+        <v>-7328374.518518519</v>
       </c>
     </row>
     <row r="103">
@@ -7900,22 +7918,22 @@
         <v>-8950173.915343916</v>
       </c>
       <c r="AA104" s="15" t="n">
-        <v>-114617703</v>
+        <v>-242652887</v>
       </c>
       <c r="AB104" s="15" t="n">
-        <v>-6742.217823529411</v>
+        <v>-14273.69923529412</v>
       </c>
       <c r="AC104" s="15" t="n">
-        <v>-606442.873015873</v>
+        <v>-1283877.708994709</v>
       </c>
       <c r="AD104" s="15" t="n">
-        <v>-1806200573</v>
+        <v>-1934235757</v>
       </c>
       <c r="AE104" s="15" t="n">
-        <v>-106247.0925294118</v>
+        <v>-113778.5739411765</v>
       </c>
       <c r="AF104" s="15" t="n">
-        <v>-9556616.788359789</v>
+        <v>-10234051.62433862</v>
       </c>
     </row>
     <row r="105">
@@ -8028,22 +8046,22 @@
         <v>-695585.1851851851</v>
       </c>
       <c r="AA106" s="11" t="n">
-        <v>-4030000</v>
+        <v>-5600000</v>
       </c>
       <c r="AB106" s="11" t="n">
-        <v>-237.0588235294118</v>
+        <v>-329.4117647058824</v>
       </c>
       <c r="AC106" s="11" t="n">
-        <v>-21322.75132275132</v>
+        <v>-29629.62962962963</v>
       </c>
       <c r="AD106" s="11" t="n">
-        <v>-135495600</v>
+        <v>-137065600</v>
       </c>
       <c r="AE106" s="11" t="n">
-        <v>-7970.329411764706</v>
+        <v>-8062.682352941176</v>
       </c>
       <c r="AF106" s="11" t="n">
-        <v>-716907.9365079363</v>
+        <v>-725214.8148148147</v>
       </c>
     </row>
     <row r="107">
@@ -8185,17 +8203,23 @@
       <c r="Z108" s="11" t="n">
         <v>-1935291.592592593</v>
       </c>
-      <c r="AA108" s="11" t="n"/>
-      <c r="AB108" s="11" t="n"/>
-      <c r="AC108" s="11" t="n"/>
+      <c r="AA108" s="11" t="n">
+        <v>-48787500</v>
+      </c>
+      <c r="AB108" s="11" t="n">
+        <v>-2869.852941176471</v>
+      </c>
+      <c r="AC108" s="11" t="n">
+        <v>-258134.9206349206</v>
+      </c>
       <c r="AD108" s="11" t="n">
-        <v>-365770111</v>
+        <v>-414557611</v>
       </c>
       <c r="AE108" s="11" t="n">
-        <v>-21515.88888235294</v>
+        <v>-24385.74182352941</v>
       </c>
       <c r="AF108" s="11" t="n">
-        <v>-1935291.592592593</v>
+        <v>-2193426.513227513</v>
       </c>
     </row>
     <row r="109">
@@ -8277,22 +8301,22 @@
         <v>-2674466.724867725</v>
       </c>
       <c r="AA109" s="15" t="n">
-        <v>-4030000</v>
+        <v>-54387500</v>
       </c>
       <c r="AB109" s="15" t="n">
-        <v>-237.0588235294118</v>
+        <v>-3199.264705882353</v>
       </c>
       <c r="AC109" s="15" t="n">
-        <v>-21322.75132275132</v>
+        <v>-287764.5502645503</v>
       </c>
       <c r="AD109" s="15" t="n">
-        <v>-509504211</v>
+        <v>-559861711</v>
       </c>
       <c r="AE109" s="15" t="n">
-        <v>-29970.83594117647</v>
+        <v>-32933.04182352941</v>
       </c>
       <c r="AF109" s="15" t="n">
-        <v>-2695789.476190476</v>
+        <v>-2962231.275132275</v>
       </c>
     </row>
     <row r="110">
@@ -8654,22 +8678,22 @@
         <v>-2187928.798941799</v>
       </c>
       <c r="AA114" s="13" t="n">
-        <v>-11193285</v>
+        <v>-63669101</v>
       </c>
       <c r="AB114" s="13" t="n">
-        <v>-658.4285294117647</v>
+        <v>-3745.241235294118</v>
       </c>
       <c r="AC114" s="13" t="n">
-        <v>-59223.73015873016</v>
+        <v>-336873.5502645503</v>
       </c>
       <c r="AD114" s="13" t="n">
-        <v>-424711828</v>
+        <v>-477187644</v>
       </c>
       <c r="AE114" s="13" t="n">
-        <v>-24983.04870588236</v>
+        <v>-28069.86141176471</v>
       </c>
       <c r="AF114" s="13" t="n">
-        <v>-2247152.529100529</v>
+        <v>-2524802.349206349</v>
       </c>
     </row>
     <row r="115">
@@ -8751,22 +8775,22 @@
         <v>-4774101.851851852</v>
       </c>
       <c r="AA115" s="15" t="n">
-        <v>-36883285</v>
+        <v>-89359101</v>
       </c>
       <c r="AB115" s="15" t="n">
-        <v>-2169.605</v>
+        <v>-5256.417705882352</v>
       </c>
       <c r="AC115" s="15" t="n">
-        <v>-195149.6560846561</v>
+        <v>-472799.4761904762</v>
       </c>
       <c r="AD115" s="15" t="n">
-        <v>-939188535</v>
+        <v>-991664351</v>
       </c>
       <c r="AE115" s="15" t="n">
-        <v>-55246.38441176471</v>
+        <v>-58333.19711764706</v>
       </c>
       <c r="AF115" s="15" t="n">
-        <v>-4969251.507936507</v>
+        <v>-5246901.328042328</v>
       </c>
     </row>
     <row r="116">
@@ -8885,22 +8909,22 @@
         <v>-24120218.13227513</v>
       </c>
       <c r="AA117" s="11" t="n">
-        <v>-233396828</v>
+        <v>-699168276</v>
       </c>
       <c r="AB117" s="11" t="n">
-        <v>-13729.22517647059</v>
+        <v>-41127.54564705883</v>
       </c>
       <c r="AC117" s="11" t="n">
-        <v>-1234903.851851852</v>
+        <v>-3699303.047619048</v>
       </c>
       <c r="AD117" s="11" t="n">
-        <v>-4792118055</v>
+        <v>-5257889503</v>
       </c>
       <c r="AE117" s="11" t="n">
-        <v>-281889.2973529412</v>
+        <v>-309287.6178235294</v>
       </c>
       <c r="AF117" s="11" t="n">
-        <v>-25355121.98412699</v>
+        <v>-27819521.17989418</v>
       </c>
     </row>
     <row r="118">
@@ -8982,22 +9006,22 @@
         <v>-24120218.13227513</v>
       </c>
       <c r="AA118" s="15" t="n">
-        <v>-233396828</v>
+        <v>-699168276</v>
       </c>
       <c r="AB118" s="15" t="n">
-        <v>-13729.22517647059</v>
+        <v>-41127.54564705883</v>
       </c>
       <c r="AC118" s="15" t="n">
-        <v>-1234903.851851852</v>
+        <v>-3699303.047619048</v>
       </c>
       <c r="AD118" s="15" t="n">
-        <v>-4792118055</v>
+        <v>-5257889503</v>
       </c>
       <c r="AE118" s="15" t="n">
-        <v>-281889.2973529412</v>
+        <v>-309287.6178235294</v>
       </c>
       <c r="AF118" s="15" t="n">
-        <v>-25355121.98412699</v>
+        <v>-27819521.17989418</v>
       </c>
     </row>
     <row r="119">
@@ -9334,17 +9358,23 @@
       <c r="Z123" s="13" t="n">
         <v>-5011963.626507936</v>
       </c>
-      <c r="AA123" s="13" t="n"/>
-      <c r="AB123" s="13" t="n"/>
-      <c r="AC123" s="13" t="n"/>
+      <c r="AA123" s="13" t="n">
+        <v>-3993717</v>
+      </c>
+      <c r="AB123" s="13" t="n">
+        <v>-234.9245294117647</v>
+      </c>
+      <c r="AC123" s="13" t="n">
+        <v>-21130.77777777778</v>
+      </c>
       <c r="AD123" s="13" t="n">
-        <v>-947261125.4100001</v>
+        <v>-951254842.4100001</v>
       </c>
       <c r="AE123" s="13" t="n">
-        <v>-55721.24267117648</v>
+        <v>-55956.16720058824</v>
       </c>
       <c r="AF123" s="13" t="n">
-        <v>-5011963.626507936</v>
+        <v>-5033094.404285714</v>
       </c>
     </row>
     <row r="124">
@@ -9601,17 +9631,23 @@
       <c r="Z126" s="11" t="n">
         <v>-5542077.719576718</v>
       </c>
-      <c r="AA126" s="11" t="n"/>
-      <c r="AB126" s="11" t="n"/>
-      <c r="AC126" s="11" t="n"/>
+      <c r="AA126" s="11" t="n">
+        <v>-62945324</v>
+      </c>
+      <c r="AB126" s="11" t="n">
+        <v>-3702.666117647059</v>
+      </c>
+      <c r="AC126" s="11" t="n">
+        <v>-333044.0423280423</v>
+      </c>
       <c r="AD126" s="11" t="n">
-        <v>-1047452689</v>
+        <v>-1110398013</v>
       </c>
       <c r="AE126" s="11" t="n">
-        <v>-61614.86405882354</v>
+        <v>-65317.53017647059</v>
       </c>
       <c r="AF126" s="11" t="n">
-        <v>-5542077.719576718</v>
+        <v>-5875121.76190476</v>
       </c>
     </row>
     <row r="127">
@@ -9693,22 +9729,22 @@
         <v>-129966981.6476719</v>
       </c>
       <c r="AA127" s="15" t="n">
-        <v>-28138500</v>
+        <v>-95077541</v>
       </c>
       <c r="AB127" s="15" t="n">
-        <v>-1655.205882352941</v>
+        <v>-5592.796529411765</v>
       </c>
       <c r="AC127" s="15" t="n">
-        <v>-148880.9523809524</v>
+        <v>-503055.7724867725</v>
       </c>
       <c r="AD127" s="15" t="n">
-        <v>-24591898031.41</v>
+        <v>-24658837072.41</v>
       </c>
       <c r="AE127" s="15" t="n">
-        <v>-1446582.237141765</v>
+        <v>-1450519.827788824</v>
       </c>
       <c r="AF127" s="15" t="n">
-        <v>-130115862.6000529</v>
+        <v>-130470037.4201587</v>
       </c>
     </row>
     <row r="128">
@@ -9815,22 +9851,22 @@
         <v>-150745.0793650794</v>
       </c>
       <c r="AA129" s="11" t="n">
-        <v>-1966500</v>
+        <v>-2777500</v>
       </c>
       <c r="AB129" s="11" t="n">
-        <v>-115.6764705882353</v>
+        <v>-163.3823529411765</v>
       </c>
       <c r="AC129" s="11" t="n">
-        <v>-10404.7619047619</v>
+        <v>-14695.7671957672</v>
       </c>
       <c r="AD129" s="11" t="n">
-        <v>-30457320</v>
+        <v>-31268320</v>
       </c>
       <c r="AE129" s="11" t="n">
-        <v>-1791.60705882353</v>
+        <v>-1839.312941176471</v>
       </c>
       <c r="AF129" s="11" t="n">
-        <v>-161149.8412698413</v>
+        <v>-165440.8465608466</v>
       </c>
     </row>
     <row r="130">
@@ -10076,22 +10112,22 @@
         <v>-490002.2645502645</v>
       </c>
       <c r="AA132" s="13" t="n">
-        <v>-397500</v>
+        <v>-2945500</v>
       </c>
       <c r="AB132" s="13" t="n">
-        <v>-23.38235294117647</v>
+        <v>-173.2647058823529</v>
       </c>
       <c r="AC132" s="13" t="n">
-        <v>-2103.174603174603</v>
+        <v>-15584.65608465608</v>
       </c>
       <c r="AD132" s="13" t="n">
-        <v>-93007928</v>
+        <v>-95555928</v>
       </c>
       <c r="AE132" s="13" t="n">
-        <v>-5471.054588235294</v>
+        <v>-5620.93694117647</v>
       </c>
       <c r="AF132" s="13" t="n">
-        <v>-492105.4391534391</v>
+        <v>-505586.9206349205</v>
       </c>
     </row>
     <row r="133">
@@ -10319,22 +10355,22 @@
         <v>-3770904.661375661</v>
       </c>
       <c r="AA135" s="15" t="n">
-        <v>-2364000</v>
+        <v>-5723000</v>
       </c>
       <c r="AB135" s="15" t="n">
-        <v>-139.0588235294118</v>
+        <v>-336.6470588235294</v>
       </c>
       <c r="AC135" s="15" t="n">
-        <v>-12507.93650793651</v>
+        <v>-30280.42328042328</v>
       </c>
       <c r="AD135" s="15" t="n">
-        <v>-715064981</v>
+        <v>-718423981</v>
       </c>
       <c r="AE135" s="15" t="n">
-        <v>-42062.64594117647</v>
+        <v>-42260.23417647059</v>
       </c>
       <c r="AF135" s="15" t="n">
-        <v>-3783412.597883598</v>
+        <v>-3801185.084656085</v>
       </c>
     </row>
     <row r="136">
@@ -10416,22 +10452,22 @@
         <v>-213174302.763545</v>
       </c>
       <c r="AA136" s="15" t="n">
-        <v>-476700393</v>
+        <v>-1379867593</v>
       </c>
       <c r="AB136" s="15" t="n">
-        <v>-28041.19958823529</v>
+        <v>-81168.68194117647</v>
       </c>
       <c r="AC136" s="15" t="n">
-        <v>-2522224.301587302</v>
+        <v>-7300886.735449735</v>
       </c>
       <c r="AD136" s="15" t="n">
-        <v>-40766643615.31001</v>
+        <v>-41669810815.31001</v>
       </c>
       <c r="AE136" s="15" t="n">
-        <v>-2398037.859724118</v>
+        <v>-2451165.342077059</v>
       </c>
       <c r="AF136" s="15" t="n">
-        <v>-215696527.0651323</v>
+        <v>-220475189.4989947</v>
       </c>
     </row>
     <row r="137">
@@ -11019,22 +11055,22 @@
         <v>-87167.31047619047</v>
       </c>
       <c r="AA145" s="11" t="n">
-        <v>-607223</v>
+        <v>-633223</v>
       </c>
       <c r="AB145" s="11" t="n">
-        <v>-35.719</v>
+        <v>-37.24841176470589</v>
       </c>
       <c r="AC145" s="11" t="n">
-        <v>-3212.820105820106</v>
+        <v>-3350.386243386243</v>
       </c>
       <c r="AD145" s="11" t="n">
-        <v>-17081844.68</v>
+        <v>-17107844.68</v>
       </c>
       <c r="AE145" s="11" t="n">
-        <v>-1004.814392941176</v>
+        <v>-1006.343804705882</v>
       </c>
       <c r="AF145" s="11" t="n">
-        <v>-90380.13058201058</v>
+        <v>-90517.69671957671</v>
       </c>
     </row>
     <row r="146">
@@ -11249,17 +11285,23 @@
       <c r="Z148" s="13" t="n">
         <v>-21541150.10492063</v>
       </c>
-      <c r="AA148" s="13" t="n"/>
-      <c r="AB148" s="13" t="n"/>
-      <c r="AC148" s="13" t="n"/>
+      <c r="AA148" s="13" t="n">
+        <v>-195109877</v>
+      </c>
+      <c r="AB148" s="13" t="n">
+        <v>-11477.05158823529</v>
+      </c>
+      <c r="AC148" s="13" t="n">
+        <v>-1032327.391534392</v>
+      </c>
       <c r="AD148" s="13" t="n">
-        <v>-4071277369.83</v>
+        <v>-4266387246.83</v>
       </c>
       <c r="AE148" s="13" t="n">
-        <v>-239486.9041076471</v>
+        <v>-250963.9556958824</v>
       </c>
       <c r="AF148" s="13" t="n">
-        <v>-21541150.10492063</v>
+        <v>-22573477.49645502</v>
       </c>
     </row>
     <row r="149">
@@ -11475,22 +11517,22 @@
         <v>-29993348.67783069</v>
       </c>
       <c r="AA151" s="15" t="n">
-        <v>-607223</v>
+        <v>-195743100</v>
       </c>
       <c r="AB151" s="15" t="n">
-        <v>-35.719</v>
+        <v>-11514.3</v>
       </c>
       <c r="AC151" s="15" t="n">
-        <v>-3212.820105820106</v>
+        <v>-1035677.777777778</v>
       </c>
       <c r="AD151" s="15" t="n">
-        <v>-5669350123.110001</v>
+        <v>-5864486000.110001</v>
       </c>
       <c r="AE151" s="15" t="n">
-        <v>-333491.1837123529</v>
+        <v>-344969.7647123529</v>
       </c>
       <c r="AF151" s="15" t="n">
-        <v>-29996561.49793651</v>
+        <v>-31029026.45560846</v>
       </c>
     </row>
     <row r="152">
@@ -11572,22 +11614,22 @@
         <v>-1478868993.977989</v>
       </c>
       <c r="AA152" s="19" t="n">
-        <v>-1814639863</v>
+        <v>-3999499218</v>
       </c>
       <c r="AB152" s="19" t="n">
-        <v>-106743.5213529412</v>
+        <v>-235264.6598823529</v>
       </c>
       <c r="AC152" s="19" t="n">
-        <v>-9601269.116402116</v>
+        <v>-21161371.52380952</v>
       </c>
       <c r="AD152" s="19" t="n">
-        <v>-281320879724.84</v>
+        <v>-283505739079.84</v>
       </c>
       <c r="AE152" s="19" t="n">
-        <v>-16548287.04263764</v>
+        <v>-16676808.18116706</v>
       </c>
       <c r="AF152" s="19" t="n">
-        <v>-1488470263.094392</v>
+        <v>-1500030365.501799</v>
       </c>
     </row>
     <row r="153">
@@ -11669,22 +11711,22 @@
         <v>-340104393.7373017</v>
       </c>
       <c r="AA153" s="19" t="n">
-        <v>1612368165</v>
+        <v>-390003362</v>
       </c>
       <c r="AB153" s="19" t="n">
-        <v>94845.18617647058</v>
+        <v>-22941.37423529412</v>
       </c>
       <c r="AC153" s="19" t="n">
-        <v>8531048.492063493</v>
+        <v>-2063509.851851852</v>
       </c>
       <c r="AD153" s="19" t="n">
-        <v>-62667362251.35001</v>
+        <v>-64669733778.35001</v>
       </c>
       <c r="AE153" s="19" t="n">
-        <v>-3686315.426550001</v>
+        <v>-3804101.986961766</v>
       </c>
       <c r="AF153" s="19" t="n">
-        <v>-331573345.2452382</v>
+        <v>-342167903.5891536</v>
       </c>
     </row>
     <row r="154">
@@ -11766,22 +11808,22 @@
         <v>16899102.6984656</v>
       </c>
       <c r="AA154" s="7" t="n">
-        <v>4806298575.009999</v>
+        <v>2803927048.009999</v>
       </c>
       <c r="AB154" s="7" t="n">
-        <v>282723.4455888235</v>
+        <v>164936.8851770588</v>
       </c>
       <c r="AC154" s="7" t="n">
-        <v>25430151.1905291</v>
+        <v>14835592.84661375</v>
       </c>
       <c r="AD154" s="7" t="n">
-        <v>4806298575.009999</v>
+        <v>2803927048.009999</v>
       </c>
       <c r="AE154" s="7" t="n">
-        <v>282723.4455888235</v>
+        <v>164936.8851770588</v>
       </c>
       <c r="AF154" s="7" t="n">
-        <v>25430151.1905291</v>
+        <v>14835592.84661375</v>
       </c>
     </row>
   </sheetData>
@@ -11908,16 +11950,16 @@
         <v>2698509305</v>
       </c>
       <c r="E6" s="11" t="n">
-        <v>1844867025</v>
+        <v>-1652546696</v>
       </c>
       <c r="F6" s="11" t="n">
-        <v>4543376330</v>
+        <v>1045962609</v>
       </c>
       <c r="G6" s="23" t="n">
-        <v>267257.4311764706</v>
+        <v>61527.21229411765</v>
       </c>
       <c r="H6" s="23" t="n">
-        <v>24039028.2010582</v>
+        <v>5534193.698412699</v>
       </c>
     </row>
     <row r="7">
@@ -11940,16 +11982,16 @@
         <v>337418375</v>
       </c>
       <c r="E7" s="13" t="n">
-        <v>-135002900</v>
+        <v>-149734909</v>
       </c>
       <c r="F7" s="13" t="n">
-        <v>202415475</v>
+        <v>187683466</v>
       </c>
       <c r="G7" s="24" t="n">
-        <v>11906.79264705882</v>
+        <v>11040.20388235294</v>
       </c>
       <c r="H7" s="24" t="n">
-        <v>1070981.349206349</v>
+        <v>993034.2116402116</v>
       </c>
     </row>
     <row r="8">
@@ -12004,16 +12046,16 @@
         <v>44055921.71</v>
       </c>
       <c r="E9" s="13" t="n">
-        <v>-37271637</v>
+        <v>72502566</v>
       </c>
       <c r="F9" s="13" t="n">
-        <v>6784284.710000001</v>
+        <v>116558487.71</v>
       </c>
       <c r="G9" s="24" t="n">
-        <v>399.0755711764706</v>
+        <v>6856.381630000001</v>
       </c>
       <c r="H9" s="24" t="n">
-        <v>35895.6862962963</v>
+        <v>616711.5751851852</v>
       </c>
     </row>
     <row r="10">
@@ -12068,16 +12110,16 @@
         <v>79086482.06</v>
       </c>
       <c r="E11" s="13" t="n">
-        <v>-60249323</v>
+        <v>1339750677</v>
       </c>
       <c r="F11" s="13" t="n">
-        <v>18837159.06</v>
+        <v>1418837159.06</v>
       </c>
       <c r="G11" s="24" t="n">
-        <v>1108.06818</v>
+        <v>83461.00935647059</v>
       </c>
       <c r="H11" s="24" t="n">
-        <v>99667.50825396826</v>
+        <v>7507074.915661375</v>
       </c>
     </row>
     <row r="12">
@@ -12123,13 +12165,13 @@
       <c r="D13" s="26" t="n"/>
       <c r="E13" s="26" t="n"/>
       <c r="F13" s="27" t="n">
-        <v>4806298577.01</v>
+        <v>2803927050.01</v>
       </c>
       <c r="G13" s="28" t="n">
-        <v>282723.4457064706</v>
+        <v>164936.8852947059</v>
       </c>
       <c r="H13" s="28" t="n">
-        <v>25430151.20111111</v>
+        <v>14835592.85719577</v>
       </c>
     </row>
   </sheetData>
@@ -12196,7 +12238,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 11 Aug 2026 17:18 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 13 Aug 2026 17:04 (in IDR Million)</t>
         </is>
       </c>
     </row>
@@ -12264,14 +12306,14 @@
       <c r="Z3" s="4" t="n"/>
       <c r="AA3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 11 Aug 2026</t>
+          <t>MTD as of 13 Aug 2026</t>
         </is>
       </c>
       <c r="AB3" s="4" t="n"/>
       <c r="AC3" s="4" t="n"/>
       <c r="AD3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 11 Aug 2026</t>
+          <t>YTD as of 13 Aug 2026</t>
         </is>
       </c>
       <c r="AE3" s="4" t="n"/>
@@ -12643,22 +12685,22 @@
         <v>873.0882368412699</v>
       </c>
       <c r="AA7" s="11" t="n">
-        <v>3417.299808</v>
+        <v>3597.677676</v>
       </c>
       <c r="AB7" s="11" t="n">
-        <v>0.2010176357647059</v>
+        <v>0.2116280985882353</v>
       </c>
       <c r="AC7" s="11" t="n">
-        <v>18.08095136507936</v>
+        <v>19.03533161904762</v>
       </c>
       <c r="AD7" s="11" t="n">
-        <v>168430.976571</v>
+        <v>168611.354439</v>
       </c>
       <c r="AE7" s="11" t="n">
-        <v>9.907704504176468</v>
+        <v>9.918314966999999</v>
       </c>
       <c r="AF7" s="11" t="n">
-        <v>891.1691882063493</v>
+        <v>892.1235684603175</v>
       </c>
     </row>
     <row r="8">
@@ -12994,17 +13036,23 @@
       <c r="Z11" s="11" t="n">
         <v>38.02955694708995</v>
       </c>
-      <c r="AA11" s="11" t="n"/>
-      <c r="AB11" s="11" t="n"/>
-      <c r="AC11" s="11" t="n"/>
+      <c r="AA11" s="11" t="n">
+        <v>180.377868</v>
+      </c>
+      <c r="AB11" s="11" t="n">
+        <v>0.01061046282352941</v>
+      </c>
+      <c r="AC11" s="11" t="n">
+        <v>0.954380253968254</v>
+      </c>
       <c r="AD11" s="11" t="n">
-        <v>7187.586263000001</v>
+        <v>7367.964131000001</v>
       </c>
       <c r="AE11" s="11" t="n">
-        <v>0.4227991919411765</v>
+        <v>0.4334096547647059</v>
       </c>
       <c r="AF11" s="11" t="n">
-        <v>38.02955694708995</v>
+        <v>38.9839372010582</v>
       </c>
     </row>
     <row r="12">
@@ -13495,22 +13543,22 @@
         <v>2.099643822698413</v>
       </c>
       <c r="AA19" s="11" t="n">
-        <v>9.708220000000001</v>
+        <v>11.81818</v>
       </c>
       <c r="AB19" s="11" t="n">
-        <v>0.0005710717647058824</v>
+        <v>0.0006951870588235294</v>
       </c>
       <c r="AC19" s="11" t="n">
-        <v>0.05136624338624339</v>
+        <v>0.06253005291005291</v>
       </c>
       <c r="AD19" s="11" t="n">
-        <v>406.54090249</v>
+        <v>408.65086249</v>
       </c>
       <c r="AE19" s="11" t="n">
-        <v>0.02391417073470588</v>
+        <v>0.02403828602882353</v>
       </c>
       <c r="AF19" s="11" t="n">
-        <v>2.151010066084656</v>
+        <v>2.162173875608466</v>
       </c>
     </row>
     <row r="20">
@@ -13726,22 +13774,22 @@
         <v>0.1408492063492063</v>
       </c>
       <c r="AA22" s="13" t="n">
-        <v>5.3165</v>
+        <v>7.4045</v>
       </c>
       <c r="AB22" s="13" t="n">
-        <v>0.000312735294117647</v>
+        <v>0.0004355588235294117</v>
       </c>
       <c r="AC22" s="13" t="n">
-        <v>0.02812962962962963</v>
+        <v>0.03917724867724868</v>
       </c>
       <c r="AD22" s="13" t="n">
-        <v>31.937</v>
+        <v>34.025</v>
       </c>
       <c r="AE22" s="13" t="n">
-        <v>0.001878647058823529</v>
+        <v>0.002001470588235294</v>
       </c>
       <c r="AF22" s="13" t="n">
-        <v>0.168978835978836</v>
+        <v>0.180026455026455</v>
       </c>
     </row>
     <row r="23">
@@ -14036,17 +14084,23 @@
       <c r="Z27" s="11" t="n">
         <v>0.0627427619047619</v>
       </c>
-      <c r="AA27" s="11" t="n"/>
-      <c r="AB27" s="11" t="n"/>
-      <c r="AC27" s="11" t="n"/>
+      <c r="AA27" s="11" t="n">
+        <v>0.02196</v>
+      </c>
+      <c r="AB27" s="11" t="n">
+        <v>1.291764705882353e-06</v>
+      </c>
+      <c r="AC27" s="11" t="n">
+        <v>0.0001161904761904762</v>
+      </c>
       <c r="AD27" s="11" t="n">
-        <v>11.858382</v>
+        <v>11.880342</v>
       </c>
       <c r="AE27" s="11" t="n">
-        <v>0.0006975518823529412</v>
+        <v>0.0006988436470588235</v>
       </c>
       <c r="AF27" s="11" t="n">
-        <v>0.0627427619047619</v>
+        <v>0.06285895238095238</v>
       </c>
     </row>
     <row r="28">
@@ -14982,22 +15036,22 @@
         <v>1138.764600240688</v>
       </c>
       <c r="AA42" s="15" t="n">
-        <v>3427.008028</v>
+        <v>3609.495856</v>
       </c>
       <c r="AB42" s="15" t="n">
-        <v>0.2015887075294118</v>
+        <v>0.2123232856470588</v>
       </c>
       <c r="AC42" s="15" t="n">
-        <v>18.13231760846561</v>
+        <v>19.09786167195767</v>
       </c>
       <c r="AD42" s="15" t="n">
-        <v>218653.51747349</v>
+        <v>218836.00530149</v>
       </c>
       <c r="AE42" s="15" t="n">
-        <v>12.86197161608765</v>
+        <v>12.87270619420529</v>
       </c>
       <c r="AF42" s="15" t="n">
-        <v>1156.896917849153</v>
+        <v>1157.862461912645</v>
       </c>
     </row>
     <row r="43">
@@ -15348,22 +15402,22 @@
         <v>-6.71041491005291</v>
       </c>
       <c r="AA48" s="13" t="n">
-        <v>-175.119091</v>
+        <v>-330.642699</v>
       </c>
       <c r="AB48" s="13" t="n">
-        <v>-0.010301123</v>
+        <v>-0.01944957052941176</v>
       </c>
       <c r="AC48" s="13" t="n">
-        <v>-0.926556037037037</v>
+        <v>-1.74943226984127</v>
       </c>
       <c r="AD48" s="13" t="n">
-        <v>-1443.387509</v>
+        <v>-1598.911117</v>
       </c>
       <c r="AE48" s="13" t="n">
-        <v>-0.08490514758823531</v>
+        <v>-0.09405359511764708</v>
       </c>
       <c r="AF48" s="13" t="n">
-        <v>-7.636970947089947</v>
+        <v>-8.459847179894179</v>
       </c>
     </row>
     <row r="49">
@@ -15616,22 +15670,22 @@
         <v>-5.318351925925926</v>
       </c>
       <c r="AA52" s="13" t="n">
-        <v>-79.71415</v>
+        <v>-196.493076</v>
       </c>
       <c r="AB52" s="13" t="n">
-        <v>-0.004689067647058824</v>
+        <v>-0.01155841623529412</v>
       </c>
       <c r="AC52" s="13" t="n">
-        <v>-0.4217679894179894</v>
+        <v>-1.039645904761905</v>
       </c>
       <c r="AD52" s="13" t="n">
-        <v>-1084.882664</v>
+        <v>-1201.66159</v>
       </c>
       <c r="AE52" s="13" t="n">
-        <v>-0.06381662729411765</v>
+        <v>-0.07068597588235294</v>
       </c>
       <c r="AF52" s="13" t="n">
-        <v>-5.740119915343915</v>
+        <v>-6.357997830687831</v>
       </c>
     </row>
     <row r="53">
@@ -15840,17 +15894,23 @@
       <c r="Z55" s="11" t="n">
         <v>-0.9811895714285714</v>
       </c>
-      <c r="AA55" s="11" t="n"/>
-      <c r="AB55" s="11" t="n"/>
-      <c r="AC55" s="11" t="n"/>
+      <c r="AA55" s="11" t="n">
+        <v>-50.75</v>
+      </c>
+      <c r="AB55" s="11" t="n">
+        <v>-0.002985294117647059</v>
+      </c>
+      <c r="AC55" s="11" t="n">
+        <v>-0.2685185185185185</v>
+      </c>
       <c r="AD55" s="11" t="n">
-        <v>-185.444829</v>
+        <v>-236.194829</v>
       </c>
       <c r="AE55" s="11" t="n">
-        <v>-0.01090851935294117</v>
+        <v>-0.01389381347058823</v>
       </c>
       <c r="AF55" s="11" t="n">
-        <v>-0.9811895714285714</v>
+        <v>-1.24970808994709</v>
       </c>
     </row>
     <row r="56">
@@ -15932,22 +15992,22 @@
         <v>-14.48268585121693</v>
       </c>
       <c r="AA56" s="13" t="n">
-        <v>-21.9325</v>
+        <v>-197.257569</v>
       </c>
       <c r="AB56" s="13" t="n">
-        <v>-0.00129014705882353</v>
+        <v>-0.01160338641176471</v>
       </c>
       <c r="AC56" s="13" t="n">
-        <v>-0.1160449735449735</v>
+        <v>-1.043690841269841</v>
       </c>
       <c r="AD56" s="13" t="n">
-        <v>-2759.16012588</v>
+        <v>-2934.48519488</v>
       </c>
       <c r="AE56" s="13" t="n">
-        <v>-0.1623035368164706</v>
+        <v>-0.1726167761694117</v>
       </c>
       <c r="AF56" s="13" t="n">
-        <v>-14.5987308247619</v>
+        <v>-15.52637669248677</v>
       </c>
     </row>
     <row r="57">
@@ -16224,22 +16284,22 @@
         <v>-75.62314355492063</v>
       </c>
       <c r="AA60" s="15" t="n">
-        <v>-280.761741</v>
+        <v>-779.1393440000001</v>
       </c>
       <c r="AB60" s="15" t="n">
-        <v>-0.01651539652941176</v>
+        <v>-0.04583172611764706</v>
       </c>
       <c r="AC60" s="15" t="n">
-        <v>-1.485511857142857</v>
+        <v>-4.122430391534392</v>
       </c>
       <c r="AD60" s="15" t="n">
-        <v>-14573.53587288</v>
+        <v>-15071.91347588</v>
       </c>
       <c r="AE60" s="15" t="n">
-        <v>-0.8572668160517647</v>
+        <v>-0.88658314564</v>
       </c>
       <c r="AF60" s="15" t="n">
-        <v>-77.10865541206348</v>
+        <v>-79.74557394645502</v>
       </c>
     </row>
     <row r="61">
@@ -17323,22 +17383,22 @@
         <v>-37.17393839968254</v>
       </c>
       <c r="AA79" s="13" t="n">
-        <v>-1025.670494</v>
+        <v>-1610.498009</v>
       </c>
       <c r="AB79" s="13" t="n">
-        <v>-0.06033355847058823</v>
+        <v>-0.09473517699999999</v>
       </c>
       <c r="AC79" s="13" t="n">
-        <v>-5.42682801058201</v>
+        <v>-8.521153486772487</v>
       </c>
       <c r="AD79" s="13" t="n">
-        <v>-8051.544851539998</v>
+        <v>-8636.372366539999</v>
       </c>
       <c r="AE79" s="13" t="n">
-        <v>-0.4736202853847059</v>
+        <v>-0.5080219039141176</v>
       </c>
       <c r="AF79" s="13" t="n">
-        <v>-42.60076641026455</v>
+        <v>-45.69509188645503</v>
       </c>
     </row>
     <row r="80">
@@ -17511,22 +17571,22 @@
         <v>-2.010421349206349</v>
       </c>
       <c r="AA81" s="13" t="n">
-        <v>-4.350012</v>
+        <v>-7.701172</v>
       </c>
       <c r="AB81" s="13" t="n">
-        <v>-0.0002558830588235294</v>
+        <v>-0.0004530101176470588</v>
       </c>
       <c r="AC81" s="13" t="n">
-        <v>-0.02301593650793651</v>
+        <v>-0.0407469417989418</v>
       </c>
       <c r="AD81" s="13" t="n">
-        <v>-384.319647</v>
+        <v>-387.670807</v>
       </c>
       <c r="AE81" s="13" t="n">
-        <v>-0.02260703805882353</v>
+        <v>-0.02280416511764706</v>
       </c>
       <c r="AF81" s="13" t="n">
-        <v>-2.033437285714286</v>
+        <v>-2.051168291005291</v>
       </c>
     </row>
     <row r="82">
@@ -17608,22 +17668,22 @@
         <v>-104.4131286271957</v>
       </c>
       <c r="AA82" s="15" t="n">
-        <v>-1030.020506</v>
+        <v>-1618.199181</v>
       </c>
       <c r="AB82" s="15" t="n">
-        <v>-0.06058944152941177</v>
+        <v>-0.09518818711764705</v>
       </c>
       <c r="AC82" s="15" t="n">
-        <v>-5.449843947089947</v>
+        <v>-8.561900428571429</v>
       </c>
       <c r="AD82" s="15" t="n">
-        <v>-20764.10181654</v>
+        <v>-21352.28049154</v>
       </c>
       <c r="AE82" s="15" t="n">
-        <v>-1.221417753914118</v>
+        <v>-1.256016499502353</v>
       </c>
       <c r="AF82" s="15" t="n">
-        <v>-109.8629725742857</v>
+        <v>-112.9750290557672</v>
       </c>
     </row>
     <row r="83">
@@ -18071,22 +18131,22 @@
         <v>-0.5164865661375662</v>
       </c>
       <c r="AA89" s="11" t="n">
-        <v>-11.77165</v>
+        <v>-16.662275</v>
       </c>
       <c r="AB89" s="11" t="n">
-        <v>-0.0006924499999999999</v>
+        <v>-0.0009801338235294118</v>
       </c>
       <c r="AC89" s="11" t="n">
-        <v>-0.06228386243386243</v>
+        <v>-0.08816018518518519</v>
       </c>
       <c r="AD89" s="11" t="n">
-        <v>-109.387611</v>
+        <v>-114.278236</v>
       </c>
       <c r="AE89" s="11" t="n">
-        <v>-0.006434565352941176</v>
+        <v>-0.006722249176470588</v>
       </c>
       <c r="AF89" s="11" t="n">
-        <v>-0.5787704285714286</v>
+        <v>-0.6046467513227514</v>
       </c>
     </row>
     <row r="90">
@@ -18156,22 +18216,22 @@
         <v>-0.008792042328042328</v>
       </c>
       <c r="AA90" s="13" t="n">
-        <v>-0.2221</v>
+        <v>-0.2668</v>
       </c>
       <c r="AB90" s="13" t="n">
-        <v>-1.306470588235294e-05</v>
+        <v>-1.569411764705882e-05</v>
       </c>
       <c r="AC90" s="13" t="n">
-        <v>-0.001175132275132275</v>
+        <v>-0.001411640211640211</v>
       </c>
       <c r="AD90" s="13" t="n">
-        <v>-1.883796</v>
+        <v>-1.928496</v>
       </c>
       <c r="AE90" s="13" t="n">
-        <v>-0.0001108115294117647</v>
+        <v>-0.0001134409411764706</v>
       </c>
       <c r="AF90" s="13" t="n">
-        <v>-0.009967174603174603</v>
+        <v>-0.01020368253968254</v>
       </c>
     </row>
     <row r="91">
@@ -18253,22 +18313,22 @@
         <v>-1.216540901798942</v>
       </c>
       <c r="AA91" s="15" t="n">
-        <v>-12.96823</v>
+        <v>-17.903555</v>
       </c>
       <c r="AB91" s="15" t="n">
-        <v>-0.0007628370588235294</v>
+        <v>-0.001053150294117647</v>
       </c>
       <c r="AC91" s="15" t="n">
-        <v>-0.06861497354497355</v>
+        <v>-0.09472780423280423</v>
       </c>
       <c r="AD91" s="15" t="n">
-        <v>-242.89446044</v>
+        <v>-247.8297854400001</v>
       </c>
       <c r="AE91" s="15" t="n">
-        <v>-0.01428790943764706</v>
+        <v>-0.01457822267294118</v>
       </c>
       <c r="AF91" s="15" t="n">
-        <v>-1.285155875343915</v>
+        <v>-1.311268706031746</v>
       </c>
     </row>
     <row r="92">
@@ -18563,22 +18623,22 @@
         <v>-33.68233866910053</v>
       </c>
       <c r="AA95" s="11" t="n">
-        <v>-26.144663</v>
+        <v>-95.18767800000001</v>
       </c>
       <c r="AB95" s="11" t="n">
-        <v>-0.001537921352941177</v>
+        <v>-0.005599275176470589</v>
       </c>
       <c r="AC95" s="11" t="n">
-        <v>-0.1383315502645503</v>
+        <v>-0.503638507936508</v>
       </c>
       <c r="AD95" s="11" t="n">
-        <v>-6392.10667146</v>
+        <v>-6461.14968646</v>
       </c>
       <c r="AE95" s="11" t="n">
-        <v>-0.3760062747917647</v>
+        <v>-0.3800676286152941</v>
       </c>
       <c r="AF95" s="11" t="n">
-        <v>-33.82067021936508</v>
+        <v>-34.18597717703704</v>
       </c>
     </row>
     <row r="96">
@@ -18660,22 +18720,22 @@
         <v>-1.024866306878307</v>
       </c>
       <c r="AA96" s="13" t="n">
-        <v>-7.718584</v>
+        <v>-51.23963</v>
       </c>
       <c r="AB96" s="13" t="n">
-        <v>-0.0004540343529411765</v>
+        <v>-0.003014095882352941</v>
       </c>
       <c r="AC96" s="13" t="n">
-        <v>-0.04083906878306878</v>
+        <v>-0.2711091534391534</v>
       </c>
       <c r="AD96" s="13" t="n">
-        <v>-201.418316</v>
+        <v>-244.939362</v>
       </c>
       <c r="AE96" s="13" t="n">
-        <v>-0.01184813623529412</v>
+        <v>-0.01440819776470588</v>
       </c>
       <c r="AF96" s="13" t="n">
-        <v>-1.065705375661376</v>
+        <v>-1.29597546031746</v>
       </c>
     </row>
     <row r="97">
@@ -18757,22 +18817,22 @@
         <v>-1.550969746031746</v>
       </c>
       <c r="AA97" s="11" t="n">
-        <v>-2.2817</v>
+        <v>-21.011525</v>
       </c>
       <c r="AB97" s="11" t="n">
-        <v>-0.0001342176470588235</v>
+        <v>-0.001235972058823529</v>
       </c>
       <c r="AC97" s="11" t="n">
-        <v>-0.01207248677248677</v>
+        <v>-0.1111720899470899</v>
       </c>
       <c r="AD97" s="11" t="n">
-        <v>-295.414982</v>
+        <v>-314.144807</v>
       </c>
       <c r="AE97" s="11" t="n">
-        <v>-0.01737735188235294</v>
+        <v>-0.01847910629411765</v>
       </c>
       <c r="AF97" s="11" t="n">
-        <v>-1.563042232804233</v>
+        <v>-1.662141835978836</v>
       </c>
     </row>
     <row r="98">
@@ -18854,22 +18914,22 @@
         <v>-37.70091492835979</v>
       </c>
       <c r="AA98" s="15" t="n">
-        <v>-44.301847</v>
+        <v>-175.595733</v>
       </c>
       <c r="AB98" s="15" t="n">
-        <v>-0.002605991</v>
+        <v>-0.01032916076470588</v>
       </c>
       <c r="AC98" s="15" t="n">
-        <v>-0.2344013068783069</v>
+        <v>-0.9290779523809524</v>
       </c>
       <c r="AD98" s="15" t="n">
-        <v>-7169.77476846</v>
+        <v>-7301.06865446</v>
       </c>
       <c r="AE98" s="15" t="n">
-        <v>-0.4217514569682353</v>
+        <v>-0.4294746267329412</v>
       </c>
       <c r="AF98" s="15" t="n">
-        <v>-37.93531623523809</v>
+        <v>-38.62999288074074</v>
       </c>
     </row>
     <row r="99">
@@ -18988,22 +19048,22 @@
         <v>-0.9694784497354496</v>
       </c>
       <c r="AA100" s="11" t="n">
-        <v>-16.5501</v>
+        <v>-16.7951</v>
       </c>
       <c r="AB100" s="11" t="n">
-        <v>-0.0009735352941176471</v>
+        <v>-0.0009879470588235295</v>
       </c>
       <c r="AC100" s="11" t="n">
-        <v>-0.08756666666666667</v>
+        <v>-0.08886296296296298</v>
       </c>
       <c r="AD100" s="11" t="n">
-        <v>-199.781527</v>
+        <v>-200.026527</v>
       </c>
       <c r="AE100" s="11" t="n">
-        <v>-0.01175185452941176</v>
+        <v>-0.01176626629411765</v>
       </c>
       <c r="AF100" s="11" t="n">
-        <v>-1.057045116402116</v>
+        <v>-1.058341412698413</v>
       </c>
     </row>
     <row r="101">
@@ -19085,22 +19145,22 @@
         <v>-0.8482951375661376</v>
       </c>
       <c r="AA101" s="13" t="n">
-        <v>-3.99685</v>
+        <v>-9.79105</v>
       </c>
       <c r="AB101" s="13" t="n">
-        <v>-0.0002351088235294118</v>
+        <v>-0.0005759441176470589</v>
       </c>
       <c r="AC101" s="13" t="n">
-        <v>-0.02114735449735449</v>
+        <v>-0.05180449735449735</v>
       </c>
       <c r="AD101" s="13" t="n">
-        <v>-164.324631</v>
+        <v>-170.118831</v>
       </c>
       <c r="AE101" s="13" t="n">
-        <v>-0.009666154764705883</v>
+        <v>-0.01000699005882353</v>
       </c>
       <c r="AF101" s="13" t="n">
-        <v>-0.8694424920634921</v>
+        <v>-0.9000996349206349</v>
       </c>
     </row>
     <row r="102">
@@ -19182,22 +19242,22 @@
         <v>-6.305078687830688</v>
       </c>
       <c r="AA102" s="11" t="n">
-        <v>-71.40692799999999</v>
+        <v>-193.402912</v>
       </c>
       <c r="AB102" s="11" t="n">
-        <v>-0.004200407529411764</v>
+        <v>-0.01137664188235294</v>
       </c>
       <c r="AC102" s="11" t="n">
-        <v>-0.3778144338624339</v>
+        <v>-1.023295830687831</v>
       </c>
       <c r="AD102" s="11" t="n">
-        <v>-1263.0668</v>
+        <v>-1385.062784</v>
       </c>
       <c r="AE102" s="11" t="n">
-        <v>-0.07429804705882352</v>
+        <v>-0.08147428141176469</v>
       </c>
       <c r="AF102" s="11" t="n">
-        <v>-6.682893121693122</v>
+        <v>-7.328374518518519</v>
       </c>
     </row>
     <row r="103">
@@ -19370,22 +19430,22 @@
         <v>-8.950173915343914</v>
       </c>
       <c r="AA104" s="15" t="n">
-        <v>-114.617703</v>
+        <v>-242.652887</v>
       </c>
       <c r="AB104" s="15" t="n">
-        <v>-0.006742217823529412</v>
+        <v>-0.01427369923529412</v>
       </c>
       <c r="AC104" s="15" t="n">
-        <v>-0.6064428730158731</v>
+        <v>-1.283877708994709</v>
       </c>
       <c r="AD104" s="15" t="n">
-        <v>-1806.200573</v>
+        <v>-1934.235757</v>
       </c>
       <c r="AE104" s="15" t="n">
-        <v>-0.1062470925294118</v>
+        <v>-0.1137785739411765</v>
       </c>
       <c r="AF104" s="15" t="n">
-        <v>-9.556616788359786</v>
+        <v>-10.23405162433862</v>
       </c>
     </row>
     <row r="105">
@@ -19498,22 +19558,22 @@
         <v>-0.6955851851851852</v>
       </c>
       <c r="AA106" s="11" t="n">
-        <v>-4.03</v>
+        <v>-5.6</v>
       </c>
       <c r="AB106" s="11" t="n">
-        <v>-0.0002370588235294118</v>
+        <v>-0.0003294117647058823</v>
       </c>
       <c r="AC106" s="11" t="n">
-        <v>-0.02132275132275132</v>
+        <v>-0.02962962962962963</v>
       </c>
       <c r="AD106" s="11" t="n">
-        <v>-135.4956</v>
+        <v>-137.0656</v>
       </c>
       <c r="AE106" s="11" t="n">
-        <v>-0.007970329411764706</v>
+        <v>-0.008062682352941176</v>
       </c>
       <c r="AF106" s="11" t="n">
-        <v>-0.7169079365079365</v>
+        <v>-0.7252148148148149</v>
       </c>
     </row>
     <row r="107">
@@ -19655,17 +19715,23 @@
       <c r="Z108" s="11" t="n">
         <v>-1.935291592592593</v>
       </c>
-      <c r="AA108" s="11" t="n"/>
-      <c r="AB108" s="11" t="n"/>
-      <c r="AC108" s="11" t="n"/>
+      <c r="AA108" s="11" t="n">
+        <v>-48.7875</v>
+      </c>
+      <c r="AB108" s="11" t="n">
+        <v>-0.002869852941176471</v>
+      </c>
+      <c r="AC108" s="11" t="n">
+        <v>-0.2581349206349207</v>
+      </c>
       <c r="AD108" s="11" t="n">
-        <v>-365.770111</v>
+        <v>-414.5576110000001</v>
       </c>
       <c r="AE108" s="11" t="n">
-        <v>-0.02151588888235294</v>
+        <v>-0.02438574182352941</v>
       </c>
       <c r="AF108" s="11" t="n">
-        <v>-1.935291592592593</v>
+        <v>-2.193426513227513</v>
       </c>
     </row>
     <row r="109">
@@ -19747,22 +19813,22 @@
         <v>-2.674466724867725</v>
       </c>
       <c r="AA109" s="15" t="n">
-        <v>-4.03</v>
+        <v>-54.3875</v>
       </c>
       <c r="AB109" s="15" t="n">
-        <v>-0.0002370588235294118</v>
+        <v>-0.003199264705882353</v>
       </c>
       <c r="AC109" s="15" t="n">
-        <v>-0.02132275132275132</v>
+        <v>-0.2877645502645503</v>
       </c>
       <c r="AD109" s="15" t="n">
-        <v>-509.5042109999999</v>
+        <v>-559.861711</v>
       </c>
       <c r="AE109" s="15" t="n">
-        <v>-0.02997083594117647</v>
+        <v>-0.03293304182352941</v>
       </c>
       <c r="AF109" s="15" t="n">
-        <v>-2.695789476190476</v>
+        <v>-2.962231275132275</v>
       </c>
     </row>
     <row r="110">
@@ -20124,22 +20190,22 @@
         <v>-2.187928798941799</v>
       </c>
       <c r="AA114" s="13" t="n">
-        <v>-11.193285</v>
+        <v>-63.669101</v>
       </c>
       <c r="AB114" s="13" t="n">
-        <v>-0.0006584285294117647</v>
+        <v>-0.003745241235294117</v>
       </c>
       <c r="AC114" s="13" t="n">
-        <v>-0.05922373015873016</v>
+        <v>-0.3368735502645502</v>
       </c>
       <c r="AD114" s="13" t="n">
-        <v>-424.711828</v>
+        <v>-477.187644</v>
       </c>
       <c r="AE114" s="13" t="n">
-        <v>-0.02498304870588235</v>
+        <v>-0.02806986141176471</v>
       </c>
       <c r="AF114" s="13" t="n">
-        <v>-2.247152529100529</v>
+        <v>-2.524802349206349</v>
       </c>
     </row>
     <row r="115">
@@ -20221,22 +20287,22 @@
         <v>-4.774101851851852</v>
       </c>
       <c r="AA115" s="15" t="n">
-        <v>-36.883285</v>
+        <v>-89.359101</v>
       </c>
       <c r="AB115" s="15" t="n">
-        <v>-0.002169605</v>
+        <v>-0.005256417705882353</v>
       </c>
       <c r="AC115" s="15" t="n">
-        <v>-0.1951496560846561</v>
+        <v>-0.4727994761904762</v>
       </c>
       <c r="AD115" s="15" t="n">
-        <v>-939.188535</v>
+        <v>-991.664351</v>
       </c>
       <c r="AE115" s="15" t="n">
-        <v>-0.05524638441176471</v>
+        <v>-0.05833319711764706</v>
       </c>
       <c r="AF115" s="15" t="n">
-        <v>-4.969251507936508</v>
+        <v>-5.246901328042329</v>
       </c>
     </row>
     <row r="116">
@@ -20355,22 +20421,22 @@
         <v>-24.12021813227513</v>
       </c>
       <c r="AA117" s="11" t="n">
-        <v>-233.396828</v>
+        <v>-699.168276</v>
       </c>
       <c r="AB117" s="11" t="n">
-        <v>-0.01372922517647059</v>
+        <v>-0.04112754564705882</v>
       </c>
       <c r="AC117" s="11" t="n">
-        <v>-1.234903851851852</v>
+        <v>-3.699303047619047</v>
       </c>
       <c r="AD117" s="11" t="n">
-        <v>-4792.118055</v>
+        <v>-5257.889503</v>
       </c>
       <c r="AE117" s="11" t="n">
-        <v>-0.2818892973529412</v>
+        <v>-0.3092876178235294</v>
       </c>
       <c r="AF117" s="11" t="n">
-        <v>-25.35512198412698</v>
+        <v>-27.81952117989418</v>
       </c>
     </row>
     <row r="118">
@@ -20452,22 +20518,22 @@
         <v>-24.12021813227513</v>
       </c>
       <c r="AA118" s="15" t="n">
-        <v>-233.396828</v>
+        <v>-699.168276</v>
       </c>
       <c r="AB118" s="15" t="n">
-        <v>-0.01372922517647059</v>
+        <v>-0.04112754564705882</v>
       </c>
       <c r="AC118" s="15" t="n">
-        <v>-1.234903851851852</v>
+        <v>-3.699303047619047</v>
       </c>
       <c r="AD118" s="15" t="n">
-        <v>-4792.118055</v>
+        <v>-5257.889503</v>
       </c>
       <c r="AE118" s="15" t="n">
-        <v>-0.2818892973529412</v>
+        <v>-0.3092876178235294</v>
       </c>
       <c r="AF118" s="15" t="n">
-        <v>-25.35512198412698</v>
+        <v>-27.81952117989418</v>
       </c>
     </row>
     <row r="119">
@@ -20804,17 +20870,23 @@
       <c r="Z123" s="13" t="n">
         <v>-5.011963626507937</v>
       </c>
-      <c r="AA123" s="13" t="n"/>
-      <c r="AB123" s="13" t="n"/>
-      <c r="AC123" s="13" t="n"/>
+      <c r="AA123" s="13" t="n">
+        <v>-3.993717</v>
+      </c>
+      <c r="AB123" s="13" t="n">
+        <v>-0.0002349245294117647</v>
+      </c>
+      <c r="AC123" s="13" t="n">
+        <v>-0.02113077777777778</v>
+      </c>
       <c r="AD123" s="13" t="n">
-        <v>-947.26112541</v>
+        <v>-951.2548424099999</v>
       </c>
       <c r="AE123" s="13" t="n">
-        <v>-0.05572124267117647</v>
+        <v>-0.05595616720058823</v>
       </c>
       <c r="AF123" s="13" t="n">
-        <v>-5.011963626507937</v>
+        <v>-5.033094404285714</v>
       </c>
     </row>
     <row r="124">
@@ -21071,17 +21143,23 @@
       <c r="Z126" s="11" t="n">
         <v>-5.54207771957672</v>
       </c>
-      <c r="AA126" s="11" t="n"/>
-      <c r="AB126" s="11" t="n"/>
-      <c r="AC126" s="11" t="n"/>
+      <c r="AA126" s="11" t="n">
+        <v>-62.945324</v>
+      </c>
+      <c r="AB126" s="11" t="n">
+        <v>-0.003702666117647059</v>
+      </c>
+      <c r="AC126" s="11" t="n">
+        <v>-0.3330440423280423</v>
+      </c>
       <c r="AD126" s="11" t="n">
-        <v>-1047.452689</v>
+        <v>-1110.398013</v>
       </c>
       <c r="AE126" s="11" t="n">
-        <v>-0.06161486405882353</v>
+        <v>-0.06531753017647059</v>
       </c>
       <c r="AF126" s="11" t="n">
-        <v>-5.54207771957672</v>
+        <v>-5.875121761904762</v>
       </c>
     </row>
     <row r="127">
@@ -21163,22 +21241,22 @@
         <v>-129.966981647672</v>
       </c>
       <c r="AA127" s="15" t="n">
-        <v>-28.1385</v>
+        <v>-95.077541</v>
       </c>
       <c r="AB127" s="15" t="n">
-        <v>-0.001655205882352941</v>
+        <v>-0.005592796529411764</v>
       </c>
       <c r="AC127" s="15" t="n">
-        <v>-0.1488809523809524</v>
+        <v>-0.5030557724867725</v>
       </c>
       <c r="AD127" s="15" t="n">
-        <v>-24591.89803141</v>
+        <v>-24658.83707241</v>
       </c>
       <c r="AE127" s="15" t="n">
-        <v>-1.446582237141765</v>
+        <v>-1.450519827788824</v>
       </c>
       <c r="AF127" s="15" t="n">
-        <v>-130.1158626000529</v>
+        <v>-130.4700374201587</v>
       </c>
     </row>
     <row r="128">
@@ -21285,22 +21363,22 @@
         <v>-0.1507450793650794</v>
       </c>
       <c r="AA129" s="11" t="n">
-        <v>-1.9665</v>
+        <v>-2.7775</v>
       </c>
       <c r="AB129" s="11" t="n">
-        <v>-0.0001156764705882353</v>
+        <v>-0.0001633823529411764</v>
       </c>
       <c r="AC129" s="11" t="n">
-        <v>-0.0104047619047619</v>
+        <v>-0.01469576719576719</v>
       </c>
       <c r="AD129" s="11" t="n">
-        <v>-30.45732</v>
+        <v>-31.26832</v>
       </c>
       <c r="AE129" s="11" t="n">
-        <v>-0.00179160705882353</v>
+        <v>-0.001839312941176471</v>
       </c>
       <c r="AF129" s="11" t="n">
-        <v>-0.1611498412698413</v>
+        <v>-0.1654408465608466</v>
       </c>
     </row>
     <row r="130">
@@ -21546,22 +21624,22 @@
         <v>-0.4900022645502646</v>
       </c>
       <c r="AA132" s="13" t="n">
-        <v>-0.3975</v>
+        <v>-2.9455</v>
       </c>
       <c r="AB132" s="13" t="n">
-        <v>-2.338235294117647e-05</v>
+        <v>-0.0001732647058823529</v>
       </c>
       <c r="AC132" s="13" t="n">
-        <v>-0.002103174603174603</v>
+        <v>-0.01558465608465608</v>
       </c>
       <c r="AD132" s="13" t="n">
-        <v>-93.00792799999999</v>
+        <v>-95.55592799999999</v>
       </c>
       <c r="AE132" s="13" t="n">
-        <v>-0.005471054588235295</v>
+        <v>-0.005620936941176471</v>
       </c>
       <c r="AF132" s="13" t="n">
-        <v>-0.4921054391534392</v>
+        <v>-0.5055869206349206</v>
       </c>
     </row>
     <row r="133">
@@ -21789,22 +21867,22 @@
         <v>-3.770904661375662</v>
       </c>
       <c r="AA135" s="15" t="n">
-        <v>-2.364</v>
+        <v>-5.723</v>
       </c>
       <c r="AB135" s="15" t="n">
-        <v>-0.0001390588235294117</v>
+        <v>-0.0003366470588235294</v>
       </c>
       <c r="AC135" s="15" t="n">
-        <v>-0.01250793650793651</v>
+        <v>-0.03028042328042328</v>
       </c>
       <c r="AD135" s="15" t="n">
-        <v>-715.0649810000001</v>
+        <v>-718.423981</v>
       </c>
       <c r="AE135" s="15" t="n">
-        <v>-0.04206264594117647</v>
+        <v>-0.04226023417647059</v>
       </c>
       <c r="AF135" s="15" t="n">
-        <v>-3.783412597883598</v>
+        <v>-3.801185084656085</v>
       </c>
     </row>
     <row r="136">
@@ -21886,22 +21964,22 @@
         <v>-213.1743027635449</v>
       </c>
       <c r="AA136" s="15" t="n">
-        <v>-476.700393</v>
+        <v>-1379.867593</v>
       </c>
       <c r="AB136" s="15" t="n">
-        <v>-0.0280411995882353</v>
+        <v>-0.08116868194117646</v>
       </c>
       <c r="AC136" s="15" t="n">
-        <v>-2.522224301587302</v>
+        <v>-7.300886735449735</v>
       </c>
       <c r="AD136" s="15" t="n">
-        <v>-40766.64361531</v>
+        <v>-41669.81081531</v>
       </c>
       <c r="AE136" s="15" t="n">
-        <v>-2.398037859724117</v>
+        <v>-2.451165342077058</v>
       </c>
       <c r="AF136" s="15" t="n">
-        <v>-215.6965270651322</v>
+        <v>-220.4751894989947</v>
       </c>
     </row>
     <row r="137">
@@ -22489,22 +22567,22 @@
         <v>-0.08716731047619047</v>
       </c>
       <c r="AA145" s="11" t="n">
-        <v>-0.607223</v>
+        <v>-0.633223</v>
       </c>
       <c r="AB145" s="11" t="n">
-        <v>-3.571899999999999e-05</v>
+        <v>-3.724841176470588e-05</v>
       </c>
       <c r="AC145" s="11" t="n">
-        <v>-0.003212820105820106</v>
+        <v>-0.003350386243386243</v>
       </c>
       <c r="AD145" s="11" t="n">
-        <v>-17.08184468</v>
+        <v>-17.10784468</v>
       </c>
       <c r="AE145" s="11" t="n">
-        <v>-0.001004814392941176</v>
+        <v>-0.001006343804705882</v>
       </c>
       <c r="AF145" s="11" t="n">
-        <v>-0.09038013058201058</v>
+        <v>-0.09051769671957671</v>
       </c>
     </row>
     <row r="146">
@@ -22719,17 +22797,23 @@
       <c r="Z148" s="13" t="n">
         <v>-21.54115010492064</v>
       </c>
-      <c r="AA148" s="13" t="n"/>
-      <c r="AB148" s="13" t="n"/>
-      <c r="AC148" s="13" t="n"/>
+      <c r="AA148" s="13" t="n">
+        <v>-195.109877</v>
+      </c>
+      <c r="AB148" s="13" t="n">
+        <v>-0.01147705158823529</v>
+      </c>
+      <c r="AC148" s="13" t="n">
+        <v>-1.032327391534392</v>
+      </c>
       <c r="AD148" s="13" t="n">
-        <v>-4071.27736983</v>
+        <v>-4266.38724683</v>
       </c>
       <c r="AE148" s="13" t="n">
-        <v>-0.2394869041076471</v>
+        <v>-0.2509639556958824</v>
       </c>
       <c r="AF148" s="13" t="n">
-        <v>-21.54115010492064</v>
+        <v>-22.57347749645503</v>
       </c>
     </row>
     <row r="149">
@@ -22945,22 +23029,22 @@
         <v>-29.99334867783069</v>
       </c>
       <c r="AA151" s="15" t="n">
-        <v>-0.607223</v>
+        <v>-195.7431</v>
       </c>
       <c r="AB151" s="15" t="n">
-        <v>-3.571899999999999e-05</v>
+        <v>-0.0115143</v>
       </c>
       <c r="AC151" s="15" t="n">
-        <v>-0.003212820105820106</v>
+        <v>-1.035677777777778</v>
       </c>
       <c r="AD151" s="15" t="n">
-        <v>-5669.35012311</v>
+        <v>-5864.48600011</v>
       </c>
       <c r="AE151" s="15" t="n">
-        <v>-0.333491183712353</v>
+        <v>-0.344969764712353</v>
       </c>
       <c r="AF151" s="15" t="n">
-        <v>-29.9965614979365</v>
+        <v>-31.02902645560846</v>
       </c>
     </row>
     <row r="152">
@@ -23042,22 +23126,22 @@
         <v>-1478.868993977989</v>
       </c>
       <c r="AA152" s="19" t="n">
-        <v>-1814.639863</v>
+        <v>-3999.499218</v>
       </c>
       <c r="AB152" s="19" t="n">
-        <v>-0.1067435213529412</v>
+        <v>-0.2352646598823529</v>
       </c>
       <c r="AC152" s="19" t="n">
-        <v>-9.601269116402117</v>
+        <v>-21.16137152380952</v>
       </c>
       <c r="AD152" s="19" t="n">
-        <v>-281320.8797248399</v>
+        <v>-283505.7390798399</v>
       </c>
       <c r="AE152" s="19" t="n">
-        <v>-16.54828704263765</v>
+        <v>-16.67680818116706</v>
       </c>
       <c r="AF152" s="19" t="n">
-        <v>-1488.470263094391</v>
+        <v>-1500.030365501799</v>
       </c>
     </row>
     <row r="153">
@@ -23139,22 +23223,22 @@
         <v>-340.1043937373017</v>
       </c>
       <c r="AA153" s="19" t="n">
-        <v>1612.368165</v>
+        <v>-390.003362</v>
       </c>
       <c r="AB153" s="19" t="n">
-        <v>0.0948451861764706</v>
+        <v>-0.02294137423529412</v>
       </c>
       <c r="AC153" s="19" t="n">
-        <v>8.531048492063492</v>
+        <v>-2.063509851851852</v>
       </c>
       <c r="AD153" s="19" t="n">
-        <v>-62667.36225135002</v>
+        <v>-64669.73377835002</v>
       </c>
       <c r="AE153" s="19" t="n">
-        <v>-3.686315426550001</v>
+        <v>-3.804101986961766</v>
       </c>
       <c r="AF153" s="19" t="n">
-        <v>-331.5733452452382</v>
+        <v>-342.1679035891535</v>
       </c>
     </row>
     <row r="154">
@@ -23236,22 +23320,22 @@
         <v>16.8991026984656</v>
       </c>
       <c r="AA154" s="7" t="n">
-        <v>4806.29857501</v>
+        <v>2803.927048009999</v>
       </c>
       <c r="AB154" s="7" t="n">
-        <v>0.2827234455888235</v>
+        <v>0.1649368851770588</v>
       </c>
       <c r="AC154" s="7" t="n">
-        <v>25.4301511905291</v>
+        <v>14.83559284661375</v>
       </c>
       <c r="AD154" s="7" t="n">
-        <v>4806.29857501</v>
+        <v>2803.927048009999</v>
       </c>
       <c r="AE154" s="7" t="n">
-        <v>0.2827234455888235</v>
+        <v>0.1649368851770588</v>
       </c>
       <c r="AF154" s="7" t="n">
-        <v>25.4301511905291</v>
+        <v>14.83559284661375</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh dashboard Thu 08/13/2026 17:07
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -726,7 +726,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 13 Aug 2026 17:04</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 13 Aug 2026 17:07</t>
         </is>
       </c>
     </row>
@@ -12238,7 +12238,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 13 Aug 2026 17:04 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 13 Aug 2026 17:07 (in IDR Million)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh dashboard Fri 08/14/2026 16:36
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -726,7 +726,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 13 Aug 2026 17:07</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 14 Aug 2026 16:36</t>
         </is>
       </c>
     </row>
@@ -794,14 +794,14 @@
       <c r="Z3" s="4" t="n"/>
       <c r="AA3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 13 Aug 2026</t>
+          <t>MTD as of 14 Aug 2026</t>
         </is>
       </c>
       <c r="AB3" s="4" t="n"/>
       <c r="AC3" s="4" t="n"/>
       <c r="AD3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 13 Aug 2026</t>
+          <t>YTD as of 14 Aug 2026</t>
         </is>
       </c>
       <c r="AE3" s="4" t="n"/>
@@ -1173,22 +1173,22 @@
         <v>873088236.8412699</v>
       </c>
       <c r="AA7" s="11" t="n">
-        <v>3597677676</v>
+        <v>3598215705</v>
       </c>
       <c r="AB7" s="11" t="n">
-        <v>211628.0985882353</v>
+        <v>211659.7473529412</v>
       </c>
       <c r="AC7" s="11" t="n">
-        <v>19035331.61904762</v>
+        <v>19038178.33333333</v>
       </c>
       <c r="AD7" s="11" t="n">
-        <v>168611354439</v>
+        <v>168611892468</v>
       </c>
       <c r="AE7" s="11" t="n">
-        <v>9918314.967</v>
+        <v>9918346.615764705</v>
       </c>
       <c r="AF7" s="11" t="n">
-        <v>892123568.4603175</v>
+        <v>892126415.1746032</v>
       </c>
     </row>
     <row r="8">
@@ -1337,22 +1337,22 @@
         <v>168810238.6349206</v>
       </c>
       <c r="AA9" s="11" t="n">
-        <v>1562649989</v>
+        <v>1563188018</v>
       </c>
       <c r="AB9" s="11" t="n">
-        <v>91920.5875882353</v>
+        <v>91952.23635294118</v>
       </c>
       <c r="AC9" s="11" t="n">
-        <v>8267989.35978836</v>
+        <v>8270836.074074074</v>
       </c>
       <c r="AD9" s="11" t="n">
-        <v>33467785091</v>
+        <v>33468323120</v>
       </c>
       <c r="AE9" s="11" t="n">
-        <v>1968693.240647059</v>
+        <v>1968724.889411765</v>
       </c>
       <c r="AF9" s="11" t="n">
-        <v>177078227.994709</v>
+        <v>177081074.7089947</v>
       </c>
     </row>
     <row r="10">
@@ -2031,22 +2031,22 @@
         <v>2099643.822698413</v>
       </c>
       <c r="AA19" s="11" t="n">
-        <v>11818180</v>
+        <v>12175180</v>
       </c>
       <c r="AB19" s="11" t="n">
-        <v>695.1870588235294</v>
+        <v>716.1870588235294</v>
       </c>
       <c r="AC19" s="11" t="n">
-        <v>62530.05291005291</v>
+        <v>64418.9417989418</v>
       </c>
       <c r="AD19" s="11" t="n">
-        <v>408650862.49</v>
+        <v>409007862.49</v>
       </c>
       <c r="AE19" s="11" t="n">
-        <v>24038.28602882353</v>
+        <v>24059.28602882353</v>
       </c>
       <c r="AF19" s="11" t="n">
-        <v>2162173.875608466</v>
+        <v>2164062.764497355</v>
       </c>
     </row>
     <row r="20">
@@ -2262,22 +2262,22 @@
         <v>140849.2063492063</v>
       </c>
       <c r="AA22" s="13" t="n">
-        <v>7404500</v>
+        <v>7761500</v>
       </c>
       <c r="AB22" s="13" t="n">
-        <v>435.5588235294118</v>
+        <v>456.5588235294118</v>
       </c>
       <c r="AC22" s="13" t="n">
-        <v>39177.24867724867</v>
+        <v>41066.13756613756</v>
       </c>
       <c r="AD22" s="13" t="n">
-        <v>34025000</v>
+        <v>34382000</v>
       </c>
       <c r="AE22" s="13" t="n">
-        <v>2001.470588235294</v>
+        <v>2022.470588235294</v>
       </c>
       <c r="AF22" s="13" t="n">
-        <v>180026.455026455</v>
+        <v>181915.3439153439</v>
       </c>
     </row>
     <row r="23">
@@ -3524,22 +3524,22 @@
         <v>1138764600.240688</v>
       </c>
       <c r="AA42" s="15" t="n">
-        <v>3609495856</v>
+        <v>3610390885</v>
       </c>
       <c r="AB42" s="15" t="n">
-        <v>212323.2856470588</v>
+        <v>212375.9344117647</v>
       </c>
       <c r="AC42" s="15" t="n">
-        <v>19097861.67195767</v>
+        <v>19102597.27513228</v>
       </c>
       <c r="AD42" s="15" t="n">
-        <v>218836005301.49</v>
+        <v>218836900330.49</v>
       </c>
       <c r="AE42" s="15" t="n">
-        <v>12872706.19420529</v>
+        <v>12872758.84297</v>
       </c>
       <c r="AF42" s="15" t="n">
-        <v>1157862461.912646</v>
+        <v>1157867197.51582</v>
       </c>
     </row>
     <row r="43">
@@ -10714,22 +10714,22 @@
         <v>-3855931.507936508</v>
       </c>
       <c r="AA140" s="11" t="n">
-        <v>-26550000</v>
+        <v>-33950000</v>
       </c>
       <c r="AB140" s="11" t="n">
-        <v>-1561.764705882353</v>
+        <v>-1997.058823529412</v>
       </c>
       <c r="AC140" s="11" t="n">
-        <v>-140476.1904761905</v>
+        <v>-179629.6296296296</v>
       </c>
       <c r="AD140" s="11" t="n">
-        <v>-755321055</v>
+        <v>-762721055</v>
       </c>
       <c r="AE140" s="11" t="n">
-        <v>-44430.65029411764</v>
+        <v>-44865.94441176471</v>
       </c>
       <c r="AF140" s="11" t="n">
-        <v>-3996407.698412698</v>
+        <v>-4035561.137566138</v>
       </c>
     </row>
     <row r="141">
@@ -10921,22 +10921,22 @@
         <v>-12697799.23280423</v>
       </c>
       <c r="AA143" s="15" t="n">
-        <v>-26550000</v>
+        <v>-33950000</v>
       </c>
       <c r="AB143" s="15" t="n">
-        <v>-1561.764705882353</v>
+        <v>-1997.058823529412</v>
       </c>
       <c r="AC143" s="15" t="n">
-        <v>-140476.1904761905</v>
+        <v>-179629.6296296296</v>
       </c>
       <c r="AD143" s="15" t="n">
-        <v>-2426434055</v>
+        <v>-2433834055</v>
       </c>
       <c r="AE143" s="15" t="n">
-        <v>-142731.415</v>
+        <v>-143166.7091176471</v>
       </c>
       <c r="AF143" s="15" t="n">
-        <v>-12838275.42328042</v>
+        <v>-12877428.86243386</v>
       </c>
     </row>
     <row r="144">
@@ -11055,22 +11055,22 @@
         <v>-87167.31047619047</v>
       </c>
       <c r="AA145" s="11" t="n">
-        <v>-633223</v>
+        <v>-635723</v>
       </c>
       <c r="AB145" s="11" t="n">
-        <v>-37.24841176470589</v>
+        <v>-37.39547058823529</v>
       </c>
       <c r="AC145" s="11" t="n">
-        <v>-3350.386243386243</v>
+        <v>-3363.613756613757</v>
       </c>
       <c r="AD145" s="11" t="n">
-        <v>-17107844.68</v>
+        <v>-17110344.68</v>
       </c>
       <c r="AE145" s="11" t="n">
-        <v>-1006.343804705882</v>
+        <v>-1006.490863529412</v>
       </c>
       <c r="AF145" s="11" t="n">
-        <v>-90517.69671957671</v>
+        <v>-90530.92423280423</v>
       </c>
     </row>
     <row r="146">
@@ -11517,22 +11517,22 @@
         <v>-29993348.67783069</v>
       </c>
       <c r="AA151" s="15" t="n">
-        <v>-195743100</v>
+        <v>-195745600</v>
       </c>
       <c r="AB151" s="15" t="n">
-        <v>-11514.3</v>
+        <v>-11514.44705882353</v>
       </c>
       <c r="AC151" s="15" t="n">
-        <v>-1035677.777777778</v>
+        <v>-1035691.005291005</v>
       </c>
       <c r="AD151" s="15" t="n">
-        <v>-5864486000.110001</v>
+        <v>-5864488500.110001</v>
       </c>
       <c r="AE151" s="15" t="n">
-        <v>-344969.7647123529</v>
+        <v>-344969.9117711764</v>
       </c>
       <c r="AF151" s="15" t="n">
-        <v>-31029026.45560846</v>
+        <v>-31029039.68312169</v>
       </c>
     </row>
     <row r="152">
@@ -11614,22 +11614,22 @@
         <v>-1478868993.977989</v>
       </c>
       <c r="AA152" s="19" t="n">
-        <v>-3999499218</v>
+        <v>-4006901718</v>
       </c>
       <c r="AB152" s="19" t="n">
-        <v>-235264.6598823529</v>
+        <v>-235700.1010588235</v>
       </c>
       <c r="AC152" s="19" t="n">
-        <v>-21161371.52380952</v>
+        <v>-21200538.19047619</v>
       </c>
       <c r="AD152" s="19" t="n">
-        <v>-283505739079.84</v>
+        <v>-283513141579.84</v>
       </c>
       <c r="AE152" s="19" t="n">
-        <v>-16676808.18116706</v>
+        <v>-16677243.62234353</v>
       </c>
       <c r="AF152" s="19" t="n">
-        <v>-1500030365.501799</v>
+        <v>-1500069532.168466</v>
       </c>
     </row>
     <row r="153">
@@ -11711,22 +11711,22 @@
         <v>-340104393.7373017</v>
       </c>
       <c r="AA153" s="19" t="n">
-        <v>-390003362</v>
+        <v>-396510833</v>
       </c>
       <c r="AB153" s="19" t="n">
-        <v>-22941.37423529412</v>
+        <v>-23324.16664705882</v>
       </c>
       <c r="AC153" s="19" t="n">
-        <v>-2063509.851851852</v>
+        <v>-2097940.915343915</v>
       </c>
       <c r="AD153" s="19" t="n">
-        <v>-64669733778.35001</v>
+        <v>-64676241249.35001</v>
       </c>
       <c r="AE153" s="19" t="n">
-        <v>-3804101.986961766</v>
+        <v>-3804484.77937353</v>
       </c>
       <c r="AF153" s="19" t="n">
-        <v>-342167903.5891536</v>
+        <v>-342202334.6526456</v>
       </c>
     </row>
     <row r="154">
@@ -11808,22 +11808,22 @@
         <v>16899102.6984656</v>
       </c>
       <c r="AA154" s="7" t="n">
-        <v>2803927048.009999</v>
+        <v>2797419577.009999</v>
       </c>
       <c r="AB154" s="7" t="n">
-        <v>164936.8851770588</v>
+        <v>164554.0927652941</v>
       </c>
       <c r="AC154" s="7" t="n">
-        <v>14835592.84661375</v>
+        <v>14801161.78312169</v>
       </c>
       <c r="AD154" s="7" t="n">
-        <v>2803927048.009999</v>
+        <v>2797419577.009999</v>
       </c>
       <c r="AE154" s="7" t="n">
-        <v>164936.8851770588</v>
+        <v>164554.0927652941</v>
       </c>
       <c r="AF154" s="7" t="n">
-        <v>14835592.84661375</v>
+        <v>14801161.78312169</v>
       </c>
     </row>
   </sheetData>
@@ -11950,16 +11950,16 @@
         <v>2698509305</v>
       </c>
       <c r="E6" s="11" t="n">
-        <v>-1652546696</v>
+        <v>-1652008667</v>
       </c>
       <c r="F6" s="11" t="n">
-        <v>1045962609</v>
+        <v>1046500638</v>
       </c>
       <c r="G6" s="23" t="n">
-        <v>61527.21229411765</v>
+        <v>61558.86105882353</v>
       </c>
       <c r="H6" s="23" t="n">
-        <v>5534193.698412699</v>
+        <v>5537040.412698412</v>
       </c>
     </row>
     <row r="7">
@@ -12046,16 +12046,16 @@
         <v>44055921.71</v>
       </c>
       <c r="E9" s="13" t="n">
-        <v>72502566</v>
+        <v>65457066</v>
       </c>
       <c r="F9" s="13" t="n">
-        <v>116558487.71</v>
+        <v>109512987.71</v>
       </c>
       <c r="G9" s="24" t="n">
-        <v>6856.381630000001</v>
+        <v>6441.940453529412</v>
       </c>
       <c r="H9" s="24" t="n">
-        <v>616711.5751851852</v>
+        <v>579433.7974074074</v>
       </c>
     </row>
     <row r="10">
@@ -12165,13 +12165,13 @@
       <c r="D13" s="26" t="n"/>
       <c r="E13" s="26" t="n"/>
       <c r="F13" s="27" t="n">
-        <v>2803927050.01</v>
+        <v>2797419579.01</v>
       </c>
       <c r="G13" s="28" t="n">
-        <v>164936.8852947059</v>
+        <v>164554.0928829412</v>
       </c>
       <c r="H13" s="28" t="n">
-        <v>14835592.85719577</v>
+        <v>14801161.79370371</v>
       </c>
     </row>
   </sheetData>
@@ -12238,7 +12238,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 13 Aug 2026 17:07 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 14 Aug 2026 16:36 (in IDR Million)</t>
         </is>
       </c>
     </row>
@@ -12306,14 +12306,14 @@
       <c r="Z3" s="4" t="n"/>
       <c r="AA3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 13 Aug 2026</t>
+          <t>MTD as of 14 Aug 2026</t>
         </is>
       </c>
       <c r="AB3" s="4" t="n"/>
       <c r="AC3" s="4" t="n"/>
       <c r="AD3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 13 Aug 2026</t>
+          <t>YTD as of 14 Aug 2026</t>
         </is>
       </c>
       <c r="AE3" s="4" t="n"/>
@@ -12685,22 +12685,22 @@
         <v>873.0882368412699</v>
       </c>
       <c r="AA7" s="11" t="n">
-        <v>3597.677676</v>
+        <v>3598.215705</v>
       </c>
       <c r="AB7" s="11" t="n">
-        <v>0.2116280985882353</v>
+        <v>0.2116597473529412</v>
       </c>
       <c r="AC7" s="11" t="n">
-        <v>19.03533161904762</v>
+        <v>19.03817833333333</v>
       </c>
       <c r="AD7" s="11" t="n">
-        <v>168611.354439</v>
+        <v>168611.892468</v>
       </c>
       <c r="AE7" s="11" t="n">
-        <v>9.918314966999999</v>
+        <v>9.918346615764705</v>
       </c>
       <c r="AF7" s="11" t="n">
-        <v>892.1235684603175</v>
+        <v>892.1264151746033</v>
       </c>
     </row>
     <row r="8">
@@ -12849,22 +12849,22 @@
         <v>168.8102386349206</v>
       </c>
       <c r="AA9" s="11" t="n">
-        <v>1562.649989</v>
+        <v>1563.188018</v>
       </c>
       <c r="AB9" s="11" t="n">
-        <v>0.09192058758823529</v>
+        <v>0.09195223635294118</v>
       </c>
       <c r="AC9" s="11" t="n">
-        <v>8.267989359788359</v>
+        <v>8.270836074074074</v>
       </c>
       <c r="AD9" s="11" t="n">
-        <v>33467.785091</v>
+        <v>33468.32312</v>
       </c>
       <c r="AE9" s="11" t="n">
-        <v>1.968693240647059</v>
+        <v>1.968724889411765</v>
       </c>
       <c r="AF9" s="11" t="n">
-        <v>177.078227994709</v>
+        <v>177.0810747089947</v>
       </c>
     </row>
     <row r="10">
@@ -13543,22 +13543,22 @@
         <v>2.099643822698413</v>
       </c>
       <c r="AA19" s="11" t="n">
-        <v>11.81818</v>
+        <v>12.17518</v>
       </c>
       <c r="AB19" s="11" t="n">
-        <v>0.0006951870588235294</v>
+        <v>0.0007161870588235293</v>
       </c>
       <c r="AC19" s="11" t="n">
-        <v>0.06253005291005291</v>
+        <v>0.0644189417989418</v>
       </c>
       <c r="AD19" s="11" t="n">
-        <v>408.65086249</v>
+        <v>409.00786249</v>
       </c>
       <c r="AE19" s="11" t="n">
-        <v>0.02403828602882353</v>
+        <v>0.02405928602882353</v>
       </c>
       <c r="AF19" s="11" t="n">
-        <v>2.162173875608466</v>
+        <v>2.164062764497355</v>
       </c>
     </row>
     <row r="20">
@@ -13774,22 +13774,22 @@
         <v>0.1408492063492063</v>
       </c>
       <c r="AA22" s="13" t="n">
-        <v>7.4045</v>
+        <v>7.7615</v>
       </c>
       <c r="AB22" s="13" t="n">
-        <v>0.0004355588235294117</v>
+        <v>0.0004565588235294117</v>
       </c>
       <c r="AC22" s="13" t="n">
-        <v>0.03917724867724868</v>
+        <v>0.04106613756613756</v>
       </c>
       <c r="AD22" s="13" t="n">
-        <v>34.025</v>
+        <v>34.382</v>
       </c>
       <c r="AE22" s="13" t="n">
-        <v>0.002001470588235294</v>
+        <v>0.002022470588235294</v>
       </c>
       <c r="AF22" s="13" t="n">
-        <v>0.180026455026455</v>
+        <v>0.1819153439153439</v>
       </c>
     </row>
     <row r="23">
@@ -15036,22 +15036,22 @@
         <v>1138.764600240688</v>
       </c>
       <c r="AA42" s="15" t="n">
-        <v>3609.495856</v>
+        <v>3610.390885</v>
       </c>
       <c r="AB42" s="15" t="n">
-        <v>0.2123232856470588</v>
+        <v>0.2123759344117647</v>
       </c>
       <c r="AC42" s="15" t="n">
-        <v>19.09786167195767</v>
+        <v>19.10259727513228</v>
       </c>
       <c r="AD42" s="15" t="n">
-        <v>218836.00530149</v>
+        <v>218836.90033049</v>
       </c>
       <c r="AE42" s="15" t="n">
-        <v>12.87270619420529</v>
+        <v>12.87275884297</v>
       </c>
       <c r="AF42" s="15" t="n">
-        <v>1157.862461912645</v>
+        <v>1157.86719751582</v>
       </c>
     </row>
     <row r="43">
@@ -22226,22 +22226,22 @@
         <v>-3.855931507936508</v>
       </c>
       <c r="AA140" s="11" t="n">
-        <v>-26.55</v>
+        <v>-33.95</v>
       </c>
       <c r="AB140" s="11" t="n">
-        <v>-0.001561764705882353</v>
+        <v>-0.001997058823529412</v>
       </c>
       <c r="AC140" s="11" t="n">
-        <v>-0.1404761904761905</v>
+        <v>-0.1796296296296296</v>
       </c>
       <c r="AD140" s="11" t="n">
-        <v>-755.321055</v>
+        <v>-762.7210550000001</v>
       </c>
       <c r="AE140" s="11" t="n">
-        <v>-0.04443065029411766</v>
+        <v>-0.04486594441176472</v>
       </c>
       <c r="AF140" s="11" t="n">
-        <v>-3.996407698412698</v>
+        <v>-4.035561137566138</v>
       </c>
     </row>
     <row r="141">
@@ -22433,22 +22433,22 @@
         <v>-12.69779923280423</v>
       </c>
       <c r="AA143" s="15" t="n">
-        <v>-26.55</v>
+        <v>-33.95</v>
       </c>
       <c r="AB143" s="15" t="n">
-        <v>-0.001561764705882353</v>
+        <v>-0.001997058823529412</v>
       </c>
       <c r="AC143" s="15" t="n">
-        <v>-0.1404761904761905</v>
+        <v>-0.1796296296296296</v>
       </c>
       <c r="AD143" s="15" t="n">
-        <v>-2426.434055</v>
+        <v>-2433.834055</v>
       </c>
       <c r="AE143" s="15" t="n">
-        <v>-0.142731415</v>
+        <v>-0.1431667091176471</v>
       </c>
       <c r="AF143" s="15" t="n">
-        <v>-12.83827542328042</v>
+        <v>-12.87742886243386</v>
       </c>
     </row>
     <row r="144">
@@ -22567,22 +22567,22 @@
         <v>-0.08716731047619047</v>
       </c>
       <c r="AA145" s="11" t="n">
-        <v>-0.633223</v>
+        <v>-0.635723</v>
       </c>
       <c r="AB145" s="11" t="n">
-        <v>-3.724841176470588e-05</v>
+        <v>-3.739547058823529e-05</v>
       </c>
       <c r="AC145" s="11" t="n">
-        <v>-0.003350386243386243</v>
+        <v>-0.003363613756613757</v>
       </c>
       <c r="AD145" s="11" t="n">
-        <v>-17.10784468</v>
+        <v>-17.11034468</v>
       </c>
       <c r="AE145" s="11" t="n">
-        <v>-0.001006343804705882</v>
+        <v>-0.001006490863529412</v>
       </c>
       <c r="AF145" s="11" t="n">
-        <v>-0.09051769671957671</v>
+        <v>-0.09053092423280423</v>
       </c>
     </row>
     <row r="146">
@@ -23029,22 +23029,22 @@
         <v>-29.99334867783069</v>
       </c>
       <c r="AA151" s="15" t="n">
-        <v>-195.7431</v>
+        <v>-195.7456</v>
       </c>
       <c r="AB151" s="15" t="n">
-        <v>-0.0115143</v>
+        <v>-0.01151444705882353</v>
       </c>
       <c r="AC151" s="15" t="n">
-        <v>-1.035677777777778</v>
+        <v>-1.035691005291005</v>
       </c>
       <c r="AD151" s="15" t="n">
-        <v>-5864.48600011</v>
+        <v>-5864.48850011</v>
       </c>
       <c r="AE151" s="15" t="n">
-        <v>-0.344969764712353</v>
+        <v>-0.3449699117711765</v>
       </c>
       <c r="AF151" s="15" t="n">
-        <v>-31.02902645560846</v>
+        <v>-31.02903968312169</v>
       </c>
     </row>
     <row r="152">
@@ -23126,22 +23126,22 @@
         <v>-1478.868993977989</v>
       </c>
       <c r="AA152" s="19" t="n">
-        <v>-3999.499218</v>
+        <v>-4006.901718</v>
       </c>
       <c r="AB152" s="19" t="n">
-        <v>-0.2352646598823529</v>
+        <v>-0.2357001010588235</v>
       </c>
       <c r="AC152" s="19" t="n">
-        <v>-21.16137152380952</v>
+        <v>-21.20053819047619</v>
       </c>
       <c r="AD152" s="19" t="n">
-        <v>-283505.7390798399</v>
+        <v>-283513.1415798399</v>
       </c>
       <c r="AE152" s="19" t="n">
-        <v>-16.67680818116706</v>
+        <v>-16.67724362234353</v>
       </c>
       <c r="AF152" s="19" t="n">
-        <v>-1500.030365501799</v>
+        <v>-1500.069532168465</v>
       </c>
     </row>
     <row r="153">
@@ -23223,22 +23223,22 @@
         <v>-340.1043937373017</v>
       </c>
       <c r="AA153" s="19" t="n">
-        <v>-390.003362</v>
+        <v>-396.510833</v>
       </c>
       <c r="AB153" s="19" t="n">
-        <v>-0.02294137423529412</v>
+        <v>-0.02332416664705882</v>
       </c>
       <c r="AC153" s="19" t="n">
-        <v>-2.063509851851852</v>
+        <v>-2.097940915343915</v>
       </c>
       <c r="AD153" s="19" t="n">
-        <v>-64669.73377835002</v>
+        <v>-64676.24124935002</v>
       </c>
       <c r="AE153" s="19" t="n">
-        <v>-3.804101986961766</v>
+        <v>-3.804484779373531</v>
       </c>
       <c r="AF153" s="19" t="n">
-        <v>-342.1679035891535</v>
+        <v>-342.2023346526456</v>
       </c>
     </row>
     <row r="154">
@@ -23320,22 +23320,22 @@
         <v>16.8991026984656</v>
       </c>
       <c r="AA154" s="7" t="n">
-        <v>2803.927048009999</v>
+        <v>2797.419577009999</v>
       </c>
       <c r="AB154" s="7" t="n">
-        <v>0.1649368851770588</v>
+        <v>0.1645540927652941</v>
       </c>
       <c r="AC154" s="7" t="n">
-        <v>14.83559284661375</v>
+        <v>14.80116178312169</v>
       </c>
       <c r="AD154" s="7" t="n">
-        <v>2803.927048009999</v>
+        <v>2797.419577009999</v>
       </c>
       <c r="AE154" s="7" t="n">
-        <v>0.1649368851770588</v>
+        <v>0.1645540927652941</v>
       </c>
       <c r="AF154" s="7" t="n">
-        <v>14.83559284661375</v>
+        <v>14.80116178312169</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh dashboard Sat 08/15/2026  7:25
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -726,7 +726,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 14 Aug 2026 16:36</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 15 Aug 2026 07:25</t>
         </is>
       </c>
     </row>
@@ -794,14 +794,14 @@
       <c r="Z3" s="4" t="n"/>
       <c r="AA3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 14 Aug 2026</t>
+          <t>MTD as of 15 Aug 2026</t>
         </is>
       </c>
       <c r="AB3" s="4" t="n"/>
       <c r="AC3" s="4" t="n"/>
       <c r="AD3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 14 Aug 2026</t>
+          <t>YTD as of 15 Aug 2026</t>
         </is>
       </c>
       <c r="AE3" s="4" t="n"/>
@@ -12238,7 +12238,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 14 Aug 2026 16:36 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 15 Aug 2026 07:25 (in IDR Million)</t>
         </is>
       </c>
     </row>
@@ -12306,14 +12306,14 @@
       <c r="Z3" s="4" t="n"/>
       <c r="AA3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 14 Aug 2026</t>
+          <t>MTD as of 15 Aug 2026</t>
         </is>
       </c>
       <c r="AB3" s="4" t="n"/>
       <c r="AC3" s="4" t="n"/>
       <c r="AD3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 14 Aug 2026</t>
+          <t>YTD as of 15 Aug 2026</t>
         </is>
       </c>
       <c r="AE3" s="4" t="n"/>

</xml_diff>

<commit_message>
Refresh dashboard Sat 08/15/2026  7:30
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -726,7 +726,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 15 Aug 2026 07:25</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 15 Aug 2026 07:30</t>
         </is>
       </c>
     </row>
@@ -12238,7 +12238,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 15 Aug 2026 07:25 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 15 Aug 2026 07:30 (in IDR Million)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh dashboard Tue 08/18/2026 16:08
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -726,7 +726,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 15 Aug 2026 07:30</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 18 Aug 2026 16:08</t>
         </is>
       </c>
     </row>
@@ -794,14 +794,14 @@
       <c r="Z3" s="4" t="n"/>
       <c r="AA3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 15 Aug 2026</t>
+          <t>MTD as of 18 Aug 2026</t>
         </is>
       </c>
       <c r="AB3" s="4" t="n"/>
       <c r="AC3" s="4" t="n"/>
       <c r="AD3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 15 Aug 2026</t>
+          <t>YTD as of 18 Aug 2026</t>
         </is>
       </c>
       <c r="AE3" s="4" t="n"/>
@@ -1173,22 +1173,22 @@
         <v>873088236.8412699</v>
       </c>
       <c r="AA7" s="11" t="n">
-        <v>3598215705</v>
+        <v>3626295705</v>
       </c>
       <c r="AB7" s="11" t="n">
-        <v>211659.7473529412</v>
+        <v>213311.5120588235</v>
       </c>
       <c r="AC7" s="11" t="n">
-        <v>19038178.33333333</v>
+        <v>19186749.76190476</v>
       </c>
       <c r="AD7" s="11" t="n">
-        <v>168611892468</v>
+        <v>168639972468</v>
       </c>
       <c r="AE7" s="11" t="n">
-        <v>9918346.615764705</v>
+        <v>9919998.380470589</v>
       </c>
       <c r="AF7" s="11" t="n">
-        <v>892126415.1746032</v>
+        <v>892274986.6031746</v>
       </c>
     </row>
     <row r="8">
@@ -1829,17 +1829,23 @@
       <c r="Z16" s="13" t="n">
         <v>41777.77777777778</v>
       </c>
-      <c r="AA16" s="13" t="n"/>
-      <c r="AB16" s="13" t="n"/>
-      <c r="AC16" s="13" t="n"/>
+      <c r="AA16" s="13" t="n">
+        <v>28080000</v>
+      </c>
+      <c r="AB16" s="13" t="n">
+        <v>1651.764705882353</v>
+      </c>
+      <c r="AC16" s="13" t="n">
+        <v>148571.4285714286</v>
+      </c>
       <c r="AD16" s="13" t="n">
-        <v>7896000</v>
+        <v>35976000</v>
       </c>
       <c r="AE16" s="13" t="n">
-        <v>464.4705882352941</v>
+        <v>2116.235294117647</v>
       </c>
       <c r="AF16" s="13" t="n">
-        <v>41777.77777777778</v>
+        <v>190349.2063492064</v>
       </c>
     </row>
     <row r="17">
@@ -2031,22 +2037,22 @@
         <v>2099643.822698413</v>
       </c>
       <c r="AA19" s="11" t="n">
-        <v>12175180</v>
+        <v>13774680</v>
       </c>
       <c r="AB19" s="11" t="n">
-        <v>716.1870588235294</v>
+        <v>810.275294117647</v>
       </c>
       <c r="AC19" s="11" t="n">
-        <v>64418.9417989418</v>
+        <v>72881.90476190476</v>
       </c>
       <c r="AD19" s="11" t="n">
-        <v>409007862.49</v>
+        <v>410607362.49</v>
       </c>
       <c r="AE19" s="11" t="n">
-        <v>24059.28602882353</v>
+        <v>24153.37426411765</v>
       </c>
       <c r="AF19" s="11" t="n">
-        <v>2164062.764497355</v>
+        <v>2172525.727460318</v>
       </c>
     </row>
     <row r="20">
@@ -2262,22 +2268,22 @@
         <v>140849.2063492063</v>
       </c>
       <c r="AA22" s="13" t="n">
-        <v>7761500</v>
+        <v>9361000</v>
       </c>
       <c r="AB22" s="13" t="n">
-        <v>456.5588235294118</v>
+        <v>550.6470588235294</v>
       </c>
       <c r="AC22" s="13" t="n">
-        <v>41066.13756613756</v>
+        <v>49529.10052910053</v>
       </c>
       <c r="AD22" s="13" t="n">
-        <v>34382000</v>
+        <v>35981500</v>
       </c>
       <c r="AE22" s="13" t="n">
-        <v>2022.470588235294</v>
+        <v>2116.558823529412</v>
       </c>
       <c r="AF22" s="13" t="n">
-        <v>181915.3439153439</v>
+        <v>190378.3068783068</v>
       </c>
     </row>
     <row r="23">
@@ -3524,22 +3530,22 @@
         <v>1138764600.240688</v>
       </c>
       <c r="AA42" s="15" t="n">
-        <v>3610390885</v>
+        <v>3640070385</v>
       </c>
       <c r="AB42" s="15" t="n">
-        <v>212375.9344117647</v>
+        <v>214121.7873529412</v>
       </c>
       <c r="AC42" s="15" t="n">
-        <v>19102597.27513228</v>
+        <v>19259631.66666667</v>
       </c>
       <c r="AD42" s="15" t="n">
-        <v>218836900330.49</v>
+        <v>218866579830.49</v>
       </c>
       <c r="AE42" s="15" t="n">
-        <v>12872758.84297</v>
+        <v>12874504.69591118</v>
       </c>
       <c r="AF42" s="15" t="n">
-        <v>1157867197.51582</v>
+        <v>1158024231.907355</v>
       </c>
     </row>
     <row r="43">
@@ -11711,22 +11717,22 @@
         <v>-340104393.7373017</v>
       </c>
       <c r="AA153" s="19" t="n">
-        <v>-396510833</v>
+        <v>-366831333</v>
       </c>
       <c r="AB153" s="19" t="n">
-        <v>-23324.16664705882</v>
+        <v>-21578.31370588235</v>
       </c>
       <c r="AC153" s="19" t="n">
-        <v>-2097940.915343915</v>
+        <v>-1940906.523809524</v>
       </c>
       <c r="AD153" s="19" t="n">
-        <v>-64676241249.35001</v>
+        <v>-64646561749.35001</v>
       </c>
       <c r="AE153" s="19" t="n">
-        <v>-3804484.77937353</v>
+        <v>-3802738.926432354</v>
       </c>
       <c r="AF153" s="19" t="n">
-        <v>-342202334.6526456</v>
+        <v>-342045300.2611113</v>
       </c>
     </row>
     <row r="154">
@@ -11808,22 +11814,22 @@
         <v>16899102.6984656</v>
       </c>
       <c r="AA154" s="7" t="n">
-        <v>2797419577.009999</v>
+        <v>2827099077.009999</v>
       </c>
       <c r="AB154" s="7" t="n">
-        <v>164554.0927652941</v>
+        <v>166299.9457064705</v>
       </c>
       <c r="AC154" s="7" t="n">
-        <v>14801161.78312169</v>
+        <v>14958196.17465608</v>
       </c>
       <c r="AD154" s="7" t="n">
-        <v>2797419577.009999</v>
+        <v>2827099077.009999</v>
       </c>
       <c r="AE154" s="7" t="n">
-        <v>164554.0927652941</v>
+        <v>166299.9457064705</v>
       </c>
       <c r="AF154" s="7" t="n">
-        <v>14801161.78312169</v>
+        <v>14958196.17465608</v>
       </c>
     </row>
   </sheetData>
@@ -12046,16 +12052,16 @@
         <v>44055921.71</v>
       </c>
       <c r="E9" s="13" t="n">
-        <v>65457066</v>
+        <v>67056566</v>
       </c>
       <c r="F9" s="13" t="n">
-        <v>109512987.71</v>
+        <v>111112487.71</v>
       </c>
       <c r="G9" s="24" t="n">
-        <v>6441.940453529412</v>
+        <v>6536.02868882353</v>
       </c>
       <c r="H9" s="24" t="n">
-        <v>579433.7974074074</v>
+        <v>587896.7603703705</v>
       </c>
     </row>
     <row r="10">
@@ -12110,16 +12116,16 @@
         <v>79086482.06</v>
       </c>
       <c r="E11" s="13" t="n">
-        <v>1339750677</v>
+        <v>1367830677</v>
       </c>
       <c r="F11" s="13" t="n">
-        <v>1418837159.06</v>
+        <v>1446917159.06</v>
       </c>
       <c r="G11" s="24" t="n">
-        <v>83461.00935647059</v>
+        <v>85112.77406235294</v>
       </c>
       <c r="H11" s="24" t="n">
-        <v>7507074.915661375</v>
+        <v>7655646.344232804</v>
       </c>
     </row>
     <row r="12">
@@ -12165,13 +12171,13 @@
       <c r="D13" s="26" t="n"/>
       <c r="E13" s="26" t="n"/>
       <c r="F13" s="27" t="n">
-        <v>2797419579.01</v>
+        <v>2827099079.01</v>
       </c>
       <c r="G13" s="28" t="n">
-        <v>164554.0928829412</v>
+        <v>166299.9458241177</v>
       </c>
       <c r="H13" s="28" t="n">
-        <v>14801161.79370371</v>
+        <v>14958196.1852381</v>
       </c>
     </row>
   </sheetData>
@@ -12238,7 +12244,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 15 Aug 2026 07:30 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 18 Aug 2026 16:08 (in IDR Million)</t>
         </is>
       </c>
     </row>
@@ -12306,14 +12312,14 @@
       <c r="Z3" s="4" t="n"/>
       <c r="AA3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 15 Aug 2026</t>
+          <t>MTD as of 18 Aug 2026</t>
         </is>
       </c>
       <c r="AB3" s="4" t="n"/>
       <c r="AC3" s="4" t="n"/>
       <c r="AD3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 15 Aug 2026</t>
+          <t>YTD as of 18 Aug 2026</t>
         </is>
       </c>
       <c r="AE3" s="4" t="n"/>
@@ -12685,22 +12691,22 @@
         <v>873.0882368412699</v>
       </c>
       <c r="AA7" s="11" t="n">
-        <v>3598.215705</v>
+        <v>3626.295705</v>
       </c>
       <c r="AB7" s="11" t="n">
-        <v>0.2116597473529412</v>
+        <v>0.2133115120588235</v>
       </c>
       <c r="AC7" s="11" t="n">
-        <v>19.03817833333333</v>
+        <v>19.18674976190476</v>
       </c>
       <c r="AD7" s="11" t="n">
-        <v>168611.892468</v>
+        <v>168639.972468</v>
       </c>
       <c r="AE7" s="11" t="n">
-        <v>9.918346615764705</v>
+        <v>9.919998380470586</v>
       </c>
       <c r="AF7" s="11" t="n">
-        <v>892.1264151746033</v>
+        <v>892.2749866031746</v>
       </c>
     </row>
     <row r="8">
@@ -13341,17 +13347,23 @@
       <c r="Z16" s="13" t="n">
         <v>0.04177777777777777</v>
       </c>
-      <c r="AA16" s="13" t="n"/>
-      <c r="AB16" s="13" t="n"/>
-      <c r="AC16" s="13" t="n"/>
+      <c r="AA16" s="13" t="n">
+        <v>28.08</v>
+      </c>
+      <c r="AB16" s="13" t="n">
+        <v>0.001651764705882353</v>
+      </c>
+      <c r="AC16" s="13" t="n">
+        <v>0.1485714285714285</v>
+      </c>
       <c r="AD16" s="13" t="n">
-        <v>7.896</v>
+        <v>35.976</v>
       </c>
       <c r="AE16" s="13" t="n">
-        <v>0.0004644705882352941</v>
+        <v>0.002116235294117647</v>
       </c>
       <c r="AF16" s="13" t="n">
-        <v>0.04177777777777777</v>
+        <v>0.1903492063492063</v>
       </c>
     </row>
     <row r="17">
@@ -13543,22 +13555,22 @@
         <v>2.099643822698413</v>
       </c>
       <c r="AA19" s="11" t="n">
-        <v>12.17518</v>
+        <v>13.77468</v>
       </c>
       <c r="AB19" s="11" t="n">
-        <v>0.0007161870588235293</v>
+        <v>0.0008102752941176471</v>
       </c>
       <c r="AC19" s="11" t="n">
-        <v>0.0644189417989418</v>
+        <v>0.07288190476190476</v>
       </c>
       <c r="AD19" s="11" t="n">
-        <v>409.00786249</v>
+        <v>410.60736249</v>
       </c>
       <c r="AE19" s="11" t="n">
-        <v>0.02405928602882353</v>
+        <v>0.02415337426411765</v>
       </c>
       <c r="AF19" s="11" t="n">
-        <v>2.164062764497355</v>
+        <v>2.172525727460318</v>
       </c>
     </row>
     <row r="20">
@@ -13774,22 +13786,22 @@
         <v>0.1408492063492063</v>
       </c>
       <c r="AA22" s="13" t="n">
-        <v>7.7615</v>
+        <v>9.361000000000001</v>
       </c>
       <c r="AB22" s="13" t="n">
-        <v>0.0004565588235294117</v>
+        <v>0.0005506470588235294</v>
       </c>
       <c r="AC22" s="13" t="n">
-        <v>0.04106613756613756</v>
+        <v>0.04952910052910053</v>
       </c>
       <c r="AD22" s="13" t="n">
-        <v>34.382</v>
+        <v>35.9815</v>
       </c>
       <c r="AE22" s="13" t="n">
-        <v>0.002022470588235294</v>
+        <v>0.002116558823529411</v>
       </c>
       <c r="AF22" s="13" t="n">
-        <v>0.1819153439153439</v>
+        <v>0.1903783068783069</v>
       </c>
     </row>
     <row r="23">
@@ -15036,22 +15048,22 @@
         <v>1138.764600240688</v>
       </c>
       <c r="AA42" s="15" t="n">
-        <v>3610.390885</v>
+        <v>3640.070385</v>
       </c>
       <c r="AB42" s="15" t="n">
-        <v>0.2123759344117647</v>
+        <v>0.2141217873529412</v>
       </c>
       <c r="AC42" s="15" t="n">
-        <v>19.10259727513228</v>
+        <v>19.25963166666667</v>
       </c>
       <c r="AD42" s="15" t="n">
-        <v>218836.90033049</v>
+        <v>218866.57983049</v>
       </c>
       <c r="AE42" s="15" t="n">
-        <v>12.87275884297</v>
+        <v>12.87450469591117</v>
       </c>
       <c r="AF42" s="15" t="n">
-        <v>1157.86719751582</v>
+        <v>1158.024231907354</v>
       </c>
     </row>
     <row r="43">
@@ -23223,22 +23235,22 @@
         <v>-340.1043937373017</v>
       </c>
       <c r="AA153" s="19" t="n">
-        <v>-396.510833</v>
+        <v>-366.831333</v>
       </c>
       <c r="AB153" s="19" t="n">
-        <v>-0.02332416664705882</v>
+        <v>-0.02157831370588235</v>
       </c>
       <c r="AC153" s="19" t="n">
-        <v>-2.097940915343915</v>
+        <v>-1.940906523809524</v>
       </c>
       <c r="AD153" s="19" t="n">
-        <v>-64676.24124935002</v>
+        <v>-64646.56174935002</v>
       </c>
       <c r="AE153" s="19" t="n">
-        <v>-3.804484779373531</v>
+        <v>-3.802738926432354</v>
       </c>
       <c r="AF153" s="19" t="n">
-        <v>-342.2023346526456</v>
+        <v>-342.0453002611112</v>
       </c>
     </row>
     <row r="154">
@@ -23320,22 +23332,22 @@
         <v>16.8991026984656</v>
       </c>
       <c r="AA154" s="7" t="n">
-        <v>2797.419577009999</v>
+        <v>2827.099077009999</v>
       </c>
       <c r="AB154" s="7" t="n">
-        <v>0.1645540927652941</v>
+        <v>0.1662999457064706</v>
       </c>
       <c r="AC154" s="7" t="n">
-        <v>14.80116178312169</v>
+        <v>14.95819617465608</v>
       </c>
       <c r="AD154" s="7" t="n">
-        <v>2797.419577009999</v>
+        <v>2827.099077009999</v>
       </c>
       <c r="AE154" s="7" t="n">
-        <v>0.1645540927652941</v>
+        <v>0.1662999457064706</v>
       </c>
       <c r="AF154" s="7" t="n">
-        <v>14.80116178312169</v>
+        <v>14.95819617465608</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh dashboard Wed 08/19/2026 16:32
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -726,7 +726,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 18 Aug 2026 16:08</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 19 Aug 2026 16:32</t>
         </is>
       </c>
     </row>
@@ -794,14 +794,14 @@
       <c r="Z3" s="4" t="n"/>
       <c r="AA3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 18 Aug 2026</t>
+          <t>MTD as of 19 Aug 2026</t>
         </is>
       </c>
       <c r="AB3" s="4" t="n"/>
       <c r="AC3" s="4" t="n"/>
       <c r="AD3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 18 Aug 2026</t>
+          <t>YTD as of 19 Aug 2026</t>
         </is>
       </c>
       <c r="AE3" s="4" t="n"/>
@@ -2037,22 +2037,22 @@
         <v>2099643.822698413</v>
       </c>
       <c r="AA19" s="11" t="n">
-        <v>13774680</v>
+        <v>15067680</v>
       </c>
       <c r="AB19" s="11" t="n">
-        <v>810.275294117647</v>
+        <v>886.3341176470589</v>
       </c>
       <c r="AC19" s="11" t="n">
-        <v>72881.90476190476</v>
+        <v>79723.1746031746</v>
       </c>
       <c r="AD19" s="11" t="n">
-        <v>410607362.49</v>
+        <v>411900362.49</v>
       </c>
       <c r="AE19" s="11" t="n">
-        <v>24153.37426411765</v>
+        <v>24229.43308764706</v>
       </c>
       <c r="AF19" s="11" t="n">
-        <v>2172525.727460318</v>
+        <v>2179366.997301587</v>
       </c>
     </row>
     <row r="20">
@@ -2268,22 +2268,22 @@
         <v>140849.2063492063</v>
       </c>
       <c r="AA22" s="13" t="n">
-        <v>9361000</v>
+        <v>10654000</v>
       </c>
       <c r="AB22" s="13" t="n">
-        <v>550.6470588235294</v>
+        <v>626.7058823529412</v>
       </c>
       <c r="AC22" s="13" t="n">
-        <v>49529.10052910053</v>
+        <v>56370.37037037037</v>
       </c>
       <c r="AD22" s="13" t="n">
-        <v>35981500</v>
+        <v>37274500</v>
       </c>
       <c r="AE22" s="13" t="n">
-        <v>2116.558823529412</v>
+        <v>2192.617647058823</v>
       </c>
       <c r="AF22" s="13" t="n">
-        <v>190378.3068783068</v>
+        <v>197219.5767195767</v>
       </c>
     </row>
     <row r="23">
@@ -3530,22 +3530,22 @@
         <v>1138764600.240688</v>
       </c>
       <c r="AA42" s="15" t="n">
-        <v>3640070385</v>
+        <v>3641363385</v>
       </c>
       <c r="AB42" s="15" t="n">
-        <v>214121.7873529412</v>
+        <v>214197.8461764706</v>
       </c>
       <c r="AC42" s="15" t="n">
-        <v>19259631.66666667</v>
+        <v>19266472.93650794</v>
       </c>
       <c r="AD42" s="15" t="n">
-        <v>218866579830.49</v>
+        <v>218867872830.49</v>
       </c>
       <c r="AE42" s="15" t="n">
-        <v>12874504.69591118</v>
+        <v>12874580.7547347</v>
       </c>
       <c r="AF42" s="15" t="n">
-        <v>1158024231.907355</v>
+        <v>1158031073.177196</v>
       </c>
     </row>
     <row r="43">
@@ -5973,17 +5973,23 @@
       <c r="Z80" s="11" t="n">
         <v>-33054126.4021164</v>
       </c>
-      <c r="AA80" s="11" t="n"/>
-      <c r="AB80" s="11" t="n"/>
-      <c r="AC80" s="11" t="n"/>
+      <c r="AA80" s="11" t="n">
+        <v>-1375836654</v>
+      </c>
+      <c r="AB80" s="11" t="n">
+        <v>-80931.56788235295</v>
+      </c>
+      <c r="AC80" s="11" t="n">
+        <v>-7279559.015873016</v>
+      </c>
       <c r="AD80" s="11" t="n">
-        <v>-6247229890</v>
+        <v>-7623066544</v>
       </c>
       <c r="AE80" s="11" t="n">
-        <v>-367484.1111764705</v>
+        <v>-448415.6790588235</v>
       </c>
       <c r="AF80" s="11" t="n">
-        <v>-33054126.4021164</v>
+        <v>-40333685.41798942</v>
       </c>
     </row>
     <row r="81">
@@ -6162,22 +6168,22 @@
         <v>-104413128.6271958</v>
       </c>
       <c r="AA82" s="15" t="n">
-        <v>-1618199181</v>
+        <v>-2994035835</v>
       </c>
       <c r="AB82" s="15" t="n">
-        <v>-95188.18711764706</v>
+        <v>-176119.755</v>
       </c>
       <c r="AC82" s="15" t="n">
-        <v>-8561900.428571429</v>
+        <v>-15841459.44444444</v>
       </c>
       <c r="AD82" s="15" t="n">
-        <v>-21352280491.54</v>
+        <v>-22728117145.54</v>
       </c>
       <c r="AE82" s="15" t="n">
-        <v>-1256016.499502353</v>
+        <v>-1336948.067384706</v>
       </c>
       <c r="AF82" s="15" t="n">
-        <v>-112975029.0557672</v>
+        <v>-120254588.0716402</v>
       </c>
     </row>
     <row r="83">
@@ -6333,22 +6339,22 @@
         <v>-627244.4497354499</v>
       </c>
       <c r="AA85" s="11" t="n">
-        <v>-902480</v>
+        <v>-1378670</v>
       </c>
       <c r="AB85" s="11" t="n">
-        <v>-53.08705882352941</v>
+        <v>-81.09823529411764</v>
       </c>
       <c r="AC85" s="11" t="n">
-        <v>-4775.026455026455</v>
+        <v>-7294.550264550265</v>
       </c>
       <c r="AD85" s="11" t="n">
-        <v>-119451681</v>
+        <v>-119927871</v>
       </c>
       <c r="AE85" s="11" t="n">
-        <v>-7026.569470588236</v>
+        <v>-7054.580647058824</v>
       </c>
       <c r="AF85" s="11" t="n">
-        <v>-632019.4761904763</v>
+        <v>-634539.0000000001</v>
       </c>
     </row>
     <row r="86">
@@ -6807,22 +6813,22 @@
         <v>-1216540.901798942</v>
       </c>
       <c r="AA91" s="15" t="n">
-        <v>-17903555</v>
+        <v>-18379745</v>
       </c>
       <c r="AB91" s="15" t="n">
-        <v>-1053.150294117647</v>
+        <v>-1081.161470588235</v>
       </c>
       <c r="AC91" s="15" t="n">
-        <v>-94727.80423280424</v>
+        <v>-97247.32804232804</v>
       </c>
       <c r="AD91" s="15" t="n">
-        <v>-247829785.44</v>
+        <v>-248305975.44</v>
       </c>
       <c r="AE91" s="15" t="n">
-        <v>-14578.22267294118</v>
+        <v>-14606.23384941176</v>
       </c>
       <c r="AF91" s="15" t="n">
-        <v>-1311268.706031746</v>
+        <v>-1313788.22984127</v>
       </c>
     </row>
     <row r="92">
@@ -8897,40 +8903,40 @@
         <v>-8604999.264550265</v>
       </c>
       <c r="U117" s="11" t="n">
-        <v>-678095650</v>
+        <v>-678093650</v>
       </c>
       <c r="V117" s="11" t="n">
-        <v>-39887.9794117647</v>
+        <v>-39887.86176470589</v>
       </c>
       <c r="W117" s="11" t="n">
-        <v>-3587807.671957672</v>
+        <v>-3587797.08994709</v>
       </c>
       <c r="X117" s="11" t="n">
-        <v>-4558721227</v>
+        <v>-4558719227</v>
       </c>
       <c r="Y117" s="11" t="n">
-        <v>-268160.0721764706</v>
+        <v>-268159.9545294117</v>
       </c>
       <c r="Z117" s="11" t="n">
-        <v>-24120218.13227513</v>
+        <v>-24120207.55026455</v>
       </c>
       <c r="AA117" s="11" t="n">
-        <v>-699168276</v>
+        <v>-757339866</v>
       </c>
       <c r="AB117" s="11" t="n">
-        <v>-41127.54564705883</v>
+        <v>-44549.40388235294</v>
       </c>
       <c r="AC117" s="11" t="n">
-        <v>-3699303.047619048</v>
+        <v>-4007089.238095238</v>
       </c>
       <c r="AD117" s="11" t="n">
-        <v>-5257889503</v>
+        <v>-5316059093</v>
       </c>
       <c r="AE117" s="11" t="n">
-        <v>-309287.6178235294</v>
+        <v>-312709.3584117647</v>
       </c>
       <c r="AF117" s="11" t="n">
-        <v>-27819521.17989418</v>
+        <v>-28127296.78835979</v>
       </c>
     </row>
     <row r="118">
@@ -8994,40 +9000,40 @@
         <v>-8604999.264550265</v>
       </c>
       <c r="U118" s="15" t="n">
-        <v>-678095650</v>
+        <v>-678093650</v>
       </c>
       <c r="V118" s="15" t="n">
-        <v>-39887.9794117647</v>
+        <v>-39887.86176470589</v>
       </c>
       <c r="W118" s="15" t="n">
-        <v>-3587807.671957672</v>
+        <v>-3587797.08994709</v>
       </c>
       <c r="X118" s="15" t="n">
-        <v>-4558721227</v>
+        <v>-4558719227</v>
       </c>
       <c r="Y118" s="15" t="n">
-        <v>-268160.0721764706</v>
+        <v>-268159.9545294117</v>
       </c>
       <c r="Z118" s="15" t="n">
-        <v>-24120218.13227513</v>
+        <v>-24120207.55026455</v>
       </c>
       <c r="AA118" s="15" t="n">
-        <v>-699168276</v>
+        <v>-757339866</v>
       </c>
       <c r="AB118" s="15" t="n">
-        <v>-41127.54564705883</v>
+        <v>-44549.40388235294</v>
       </c>
       <c r="AC118" s="15" t="n">
-        <v>-3699303.047619048</v>
+        <v>-4007089.238095238</v>
       </c>
       <c r="AD118" s="15" t="n">
-        <v>-5257889503</v>
+        <v>-5316059093</v>
       </c>
       <c r="AE118" s="15" t="n">
-        <v>-309287.6178235294</v>
+        <v>-312709.3584117647</v>
       </c>
       <c r="AF118" s="15" t="n">
-        <v>-27819521.17989418</v>
+        <v>-28127296.78835979</v>
       </c>
     </row>
     <row r="119">
@@ -9450,22 +9456,22 @@
         <v>-1586642.857142857</v>
       </c>
       <c r="AA124" s="11" t="n">
-        <v>-28138500</v>
+        <v>-28238500</v>
       </c>
       <c r="AB124" s="11" t="n">
-        <v>-1655.205882352941</v>
+        <v>-1661.088235294118</v>
       </c>
       <c r="AC124" s="11" t="n">
-        <v>-148880.9523809524</v>
+        <v>-149410.0529100529</v>
       </c>
       <c r="AD124" s="11" t="n">
-        <v>-328014000</v>
+        <v>-328114000</v>
       </c>
       <c r="AE124" s="11" t="n">
-        <v>-19294.94117647059</v>
+        <v>-19300.82352941177</v>
       </c>
       <c r="AF124" s="11" t="n">
-        <v>-1735523.80952381</v>
+        <v>-1736052.91005291</v>
       </c>
     </row>
     <row r="125">
@@ -9546,17 +9552,23 @@
       <c r="Z125" s="13" t="n">
         <v>-73717938.56084655</v>
       </c>
-      <c r="AA125" s="13" t="n"/>
-      <c r="AB125" s="13" t="n"/>
-      <c r="AC125" s="13" t="n"/>
+      <c r="AA125" s="13" t="n">
+        <v>-1309164</v>
+      </c>
+      <c r="AB125" s="13" t="n">
+        <v>-77.00964705882353</v>
+      </c>
+      <c r="AC125" s="13" t="n">
+        <v>-6926.793650793651</v>
+      </c>
       <c r="AD125" s="13" t="n">
-        <v>-13932690388</v>
+        <v>-13933999552</v>
       </c>
       <c r="AE125" s="13" t="n">
-        <v>-819570.0228235294</v>
+        <v>-819647.0324705882</v>
       </c>
       <c r="AF125" s="13" t="n">
-        <v>-73717938.56084655</v>
+        <v>-73724865.35449734</v>
       </c>
     </row>
     <row r="126">
@@ -9735,22 +9747,22 @@
         <v>-129966981.6476719</v>
       </c>
       <c r="AA127" s="15" t="n">
-        <v>-95077541</v>
+        <v>-96486705</v>
       </c>
       <c r="AB127" s="15" t="n">
-        <v>-5592.796529411765</v>
+        <v>-5675.688529411765</v>
       </c>
       <c r="AC127" s="15" t="n">
-        <v>-503055.7724867725</v>
+        <v>-510511.6666666667</v>
       </c>
       <c r="AD127" s="15" t="n">
-        <v>-24658837072.41</v>
+        <v>-24660246236.41</v>
       </c>
       <c r="AE127" s="15" t="n">
-        <v>-1450519.827788824</v>
+        <v>-1450602.719788824</v>
       </c>
       <c r="AF127" s="15" t="n">
-        <v>-130470037.4201587</v>
+        <v>-130477493.3143386</v>
       </c>
     </row>
     <row r="128">
@@ -10440,40 +10452,40 @@
         <v>-18308852.74497355</v>
       </c>
       <c r="U136" s="15" t="n">
-        <v>-4043272117.94</v>
+        <v>-4043270117.94</v>
       </c>
       <c r="V136" s="15" t="n">
-        <v>-237839.5363494118</v>
+        <v>-237839.4187023529</v>
       </c>
       <c r="W136" s="15" t="n">
-        <v>-21392974.16899471</v>
+        <v>-21392963.58698413</v>
       </c>
       <c r="X136" s="15" t="n">
-        <v>-40289943222.31001</v>
+        <v>-40289941222.31001</v>
       </c>
       <c r="Y136" s="15" t="n">
-        <v>-2369996.660135882</v>
+        <v>-2369996.542488824</v>
       </c>
       <c r="Z136" s="15" t="n">
-        <v>-213174302.763545</v>
+        <v>-213174292.1815344</v>
       </c>
       <c r="AA136" s="15" t="n">
-        <v>-1379867593</v>
+        <v>-1439924537</v>
       </c>
       <c r="AB136" s="15" t="n">
-        <v>-81168.68194117647</v>
+        <v>-84701.44335294118</v>
       </c>
       <c r="AC136" s="15" t="n">
-        <v>-7300886.735449735</v>
+        <v>-7618648.343915344</v>
       </c>
       <c r="AD136" s="15" t="n">
-        <v>-41669810815.31001</v>
+        <v>-41729865759.31001</v>
       </c>
       <c r="AE136" s="15" t="n">
-        <v>-2451165.342077059</v>
+        <v>-2454697.985841765</v>
       </c>
       <c r="AF136" s="15" t="n">
-        <v>-220475189.4989947</v>
+        <v>-220792940.5254497</v>
       </c>
     </row>
     <row r="137">
@@ -11043,40 +11055,40 @@
         <v>-7794.830687830688</v>
       </c>
       <c r="U145" s="11" t="n">
-        <v>-2281144</v>
+        <v>-2283144</v>
       </c>
       <c r="V145" s="11" t="n">
-        <v>-134.1849411764706</v>
+        <v>-134.3025882352941</v>
       </c>
       <c r="W145" s="11" t="n">
-        <v>-12069.54497354497</v>
+        <v>-12080.12698412698</v>
       </c>
       <c r="X145" s="11" t="n">
-        <v>-16474621.68</v>
+        <v>-16476621.68</v>
       </c>
       <c r="Y145" s="11" t="n">
-        <v>-969.0953929411764</v>
+        <v>-969.21304</v>
       </c>
       <c r="Z145" s="11" t="n">
-        <v>-87167.31047619047</v>
+        <v>-87177.89248677247</v>
       </c>
       <c r="AA145" s="11" t="n">
-        <v>-635723</v>
+        <v>-1310261</v>
       </c>
       <c r="AB145" s="11" t="n">
-        <v>-37.39547058823529</v>
+        <v>-77.07417647058824</v>
       </c>
       <c r="AC145" s="11" t="n">
-        <v>-3363.613756613757</v>
+        <v>-6932.597883597884</v>
       </c>
       <c r="AD145" s="11" t="n">
-        <v>-17110344.68</v>
+        <v>-17786882.68</v>
       </c>
       <c r="AE145" s="11" t="n">
-        <v>-1006.490863529412</v>
+        <v>-1046.287216470588</v>
       </c>
       <c r="AF145" s="11" t="n">
-        <v>-90530.92423280423</v>
+        <v>-94110.49037037036</v>
       </c>
     </row>
     <row r="146">
@@ -11505,40 +11517,40 @@
         <v>-1768715.506190476</v>
       </c>
       <c r="U151" s="15" t="n">
-        <v>-296977086.26</v>
+        <v>-296979086.26</v>
       </c>
       <c r="V151" s="15" t="n">
-        <v>-17469.24036823529</v>
+        <v>-17469.35801529412</v>
       </c>
       <c r="W151" s="15" t="n">
-        <v>-1571307.334708995</v>
+        <v>-1571317.916719577</v>
       </c>
       <c r="X151" s="15" t="n">
-        <v>-5668742900.110001</v>
+        <v>-5668744900.110001</v>
       </c>
       <c r="Y151" s="15" t="n">
-        <v>-333455.4647123529</v>
+        <v>-333455.5823594118</v>
       </c>
       <c r="Z151" s="15" t="n">
-        <v>-29993348.67783069</v>
+        <v>-29993359.25984127</v>
       </c>
       <c r="AA151" s="15" t="n">
-        <v>-195745600</v>
+        <v>-196420138</v>
       </c>
       <c r="AB151" s="15" t="n">
-        <v>-11514.44705882353</v>
+        <v>-11554.12576470588</v>
       </c>
       <c r="AC151" s="15" t="n">
-        <v>-1035691.005291005</v>
+        <v>-1039259.989417989</v>
       </c>
       <c r="AD151" s="15" t="n">
-        <v>-5864488500.110001</v>
+        <v>-5865165038.110001</v>
       </c>
       <c r="AE151" s="15" t="n">
-        <v>-344969.9117711764</v>
+        <v>-345009.7081241176</v>
       </c>
       <c r="AF151" s="15" t="n">
-        <v>-31029039.68312169</v>
+        <v>-31032619.24925926</v>
       </c>
     </row>
     <row r="152">
@@ -11620,22 +11632,22 @@
         <v>-1478868993.977989</v>
       </c>
       <c r="AA152" s="19" t="n">
-        <v>-4006901718</v>
+        <v>-5443469854</v>
       </c>
       <c r="AB152" s="19" t="n">
-        <v>-235700.1010588235</v>
+        <v>-320204.1090588236</v>
       </c>
       <c r="AC152" s="19" t="n">
-        <v>-21200538.19047619</v>
+        <v>-28801427.7989418</v>
       </c>
       <c r="AD152" s="19" t="n">
-        <v>-283513141579.84</v>
+        <v>-284949709715.84</v>
       </c>
       <c r="AE152" s="19" t="n">
-        <v>-16677243.62234353</v>
+        <v>-16761747.63034353</v>
       </c>
       <c r="AF152" s="19" t="n">
-        <v>-1500069532.168466</v>
+        <v>-1507670421.776931</v>
       </c>
     </row>
     <row r="153">
@@ -11717,22 +11729,22 @@
         <v>-340104393.7373017</v>
       </c>
       <c r="AA153" s="19" t="n">
-        <v>-366831333</v>
+        <v>-1802106469</v>
       </c>
       <c r="AB153" s="19" t="n">
-        <v>-21578.31370588235</v>
+        <v>-106006.2628823529</v>
       </c>
       <c r="AC153" s="19" t="n">
-        <v>-1940906.523809524</v>
+        <v>-9534954.862433862</v>
       </c>
       <c r="AD153" s="19" t="n">
-        <v>-64646561749.35001</v>
+        <v>-66081836885.35001</v>
       </c>
       <c r="AE153" s="19" t="n">
-        <v>-3802738.926432354</v>
+        <v>-3887166.875608824</v>
       </c>
       <c r="AF153" s="19" t="n">
-        <v>-342045300.2611113</v>
+        <v>-349639348.5997356</v>
       </c>
     </row>
     <row r="154">
@@ -11814,22 +11826,22 @@
         <v>16899102.6984656</v>
       </c>
       <c r="AA154" s="7" t="n">
-        <v>2827099077.009999</v>
+        <v>1391823941.009999</v>
       </c>
       <c r="AB154" s="7" t="n">
-        <v>166299.9457064705</v>
+        <v>81871.99652999996</v>
       </c>
       <c r="AC154" s="7" t="n">
-        <v>14958196.17465608</v>
+        <v>7364147.836031742</v>
       </c>
       <c r="AD154" s="7" t="n">
-        <v>2827099077.009999</v>
+        <v>1391823941.009999</v>
       </c>
       <c r="AE154" s="7" t="n">
-        <v>166299.9457064705</v>
+        <v>81871.99652999996</v>
       </c>
       <c r="AF154" s="7" t="n">
-        <v>14958196.17465608</v>
+        <v>7364147.836031742</v>
       </c>
     </row>
   </sheetData>
@@ -11988,16 +12000,16 @@
         <v>337418375</v>
       </c>
       <c r="E7" s="13" t="n">
-        <v>-149734909</v>
+        <v>-329734909</v>
       </c>
       <c r="F7" s="13" t="n">
-        <v>187683466</v>
+        <v>7683466</v>
       </c>
       <c r="G7" s="24" t="n">
-        <v>11040.20388235294</v>
+        <v>451.9685882352941</v>
       </c>
       <c r="H7" s="24" t="n">
-        <v>993034.2116402116</v>
+        <v>40653.25925925926</v>
       </c>
     </row>
     <row r="8">
@@ -12052,16 +12064,16 @@
         <v>44055921.71</v>
       </c>
       <c r="E9" s="13" t="n">
-        <v>67056566</v>
+        <v>246940402</v>
       </c>
       <c r="F9" s="13" t="n">
-        <v>111112487.71</v>
+        <v>290996323.71</v>
       </c>
       <c r="G9" s="24" t="n">
-        <v>6536.02868882353</v>
+        <v>17117.43080647059</v>
       </c>
       <c r="H9" s="24" t="n">
-        <v>587896.7603703705</v>
+        <v>1539663.088412698</v>
       </c>
     </row>
     <row r="10">
@@ -12116,16 +12128,16 @@
         <v>79086482.06</v>
       </c>
       <c r="E11" s="13" t="n">
-        <v>1367830677</v>
+        <v>-67328295</v>
       </c>
       <c r="F11" s="13" t="n">
-        <v>1446917159.06</v>
+        <v>11758187.06</v>
       </c>
       <c r="G11" s="24" t="n">
-        <v>85112.77406235294</v>
+        <v>691.6580623529413</v>
       </c>
       <c r="H11" s="24" t="n">
-        <v>7655646.344232804</v>
+        <v>62212.62994708996</v>
       </c>
     </row>
     <row r="12">
@@ -12171,13 +12183,13 @@
       <c r="D13" s="26" t="n"/>
       <c r="E13" s="26" t="n"/>
       <c r="F13" s="27" t="n">
-        <v>2827099079.01</v>
+        <v>1391823943.01</v>
       </c>
       <c r="G13" s="28" t="n">
-        <v>166299.9458241177</v>
+        <v>81871.99664764706</v>
       </c>
       <c r="H13" s="28" t="n">
-        <v>14958196.1852381</v>
+        <v>7364147.846613756</v>
       </c>
     </row>
   </sheetData>
@@ -12244,7 +12256,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 18 Aug 2026 16:08 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 19 Aug 2026 16:32 (in IDR Million)</t>
         </is>
       </c>
     </row>
@@ -12312,14 +12324,14 @@
       <c r="Z3" s="4" t="n"/>
       <c r="AA3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 18 Aug 2026</t>
+          <t>MTD as of 19 Aug 2026</t>
         </is>
       </c>
       <c r="AB3" s="4" t="n"/>
       <c r="AC3" s="4" t="n"/>
       <c r="AD3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 18 Aug 2026</t>
+          <t>YTD as of 19 Aug 2026</t>
         </is>
       </c>
       <c r="AE3" s="4" t="n"/>
@@ -13555,22 +13567,22 @@
         <v>2.099643822698413</v>
       </c>
       <c r="AA19" s="11" t="n">
-        <v>13.77468</v>
+        <v>15.06768</v>
       </c>
       <c r="AB19" s="11" t="n">
-        <v>0.0008102752941176471</v>
+        <v>0.0008863341176470588</v>
       </c>
       <c r="AC19" s="11" t="n">
-        <v>0.07288190476190476</v>
+        <v>0.0797231746031746</v>
       </c>
       <c r="AD19" s="11" t="n">
-        <v>410.60736249</v>
+        <v>411.90036249</v>
       </c>
       <c r="AE19" s="11" t="n">
-        <v>0.02415337426411765</v>
+        <v>0.02422943308764706</v>
       </c>
       <c r="AF19" s="11" t="n">
-        <v>2.172525727460318</v>
+        <v>2.179366997301587</v>
       </c>
     </row>
     <row r="20">
@@ -13786,22 +13798,22 @@
         <v>0.1408492063492063</v>
       </c>
       <c r="AA22" s="13" t="n">
-        <v>9.361000000000001</v>
+        <v>10.654</v>
       </c>
       <c r="AB22" s="13" t="n">
-        <v>0.0005506470588235294</v>
+        <v>0.0006267058823529412</v>
       </c>
       <c r="AC22" s="13" t="n">
-        <v>0.04952910052910053</v>
+        <v>0.05637037037037037</v>
       </c>
       <c r="AD22" s="13" t="n">
-        <v>35.9815</v>
+        <v>37.2745</v>
       </c>
       <c r="AE22" s="13" t="n">
-        <v>0.002116558823529411</v>
+        <v>0.002192617647058824</v>
       </c>
       <c r="AF22" s="13" t="n">
-        <v>0.1903783068783069</v>
+        <v>0.1972195767195767</v>
       </c>
     </row>
     <row r="23">
@@ -15048,22 +15060,22 @@
         <v>1138.764600240688</v>
       </c>
       <c r="AA42" s="15" t="n">
-        <v>3640.070385</v>
+        <v>3641.363385</v>
       </c>
       <c r="AB42" s="15" t="n">
-        <v>0.2141217873529412</v>
+        <v>0.2141978461764706</v>
       </c>
       <c r="AC42" s="15" t="n">
-        <v>19.25963166666667</v>
+        <v>19.26647293650794</v>
       </c>
       <c r="AD42" s="15" t="n">
-        <v>218866.57983049</v>
+        <v>218867.87283049</v>
       </c>
       <c r="AE42" s="15" t="n">
-        <v>12.87450469591117</v>
+        <v>12.8745807547347</v>
       </c>
       <c r="AF42" s="15" t="n">
-        <v>1158.024231907354</v>
+        <v>1158.031073177196</v>
       </c>
     </row>
     <row r="43">
@@ -17491,17 +17503,23 @@
       <c r="Z80" s="11" t="n">
         <v>-33.0541264021164</v>
       </c>
-      <c r="AA80" s="11" t="n"/>
-      <c r="AB80" s="11" t="n"/>
-      <c r="AC80" s="11" t="n"/>
+      <c r="AA80" s="11" t="n">
+        <v>-1375.836654</v>
+      </c>
+      <c r="AB80" s="11" t="n">
+        <v>-0.08093156788235294</v>
+      </c>
+      <c r="AC80" s="11" t="n">
+        <v>-7.279559015873016</v>
+      </c>
       <c r="AD80" s="11" t="n">
-        <v>-6247.229889999999</v>
+        <v>-7623.066543999998</v>
       </c>
       <c r="AE80" s="11" t="n">
-        <v>-0.3674841111764706</v>
+        <v>-0.4484156790588235</v>
       </c>
       <c r="AF80" s="11" t="n">
-        <v>-33.0541264021164</v>
+        <v>-40.33368541798941</v>
       </c>
     </row>
     <row r="81">
@@ -17680,22 +17698,22 @@
         <v>-104.4131286271957</v>
       </c>
       <c r="AA82" s="15" t="n">
-        <v>-1618.199181</v>
+        <v>-2994.035835</v>
       </c>
       <c r="AB82" s="15" t="n">
-        <v>-0.09518818711764705</v>
+        <v>-0.176119755</v>
       </c>
       <c r="AC82" s="15" t="n">
-        <v>-8.561900428571429</v>
+        <v>-15.84145944444444</v>
       </c>
       <c r="AD82" s="15" t="n">
-        <v>-21352.28049154</v>
+        <v>-22728.11714554</v>
       </c>
       <c r="AE82" s="15" t="n">
-        <v>-1.256016499502353</v>
+        <v>-1.336948067384706</v>
       </c>
       <c r="AF82" s="15" t="n">
-        <v>-112.9750290557672</v>
+        <v>-120.2545880716402</v>
       </c>
     </row>
     <row r="83">
@@ -17851,22 +17869,22 @@
         <v>-0.6272444497354498</v>
       </c>
       <c r="AA85" s="11" t="n">
-        <v>-0.9024799999999999</v>
+        <v>-1.37867</v>
       </c>
       <c r="AB85" s="11" t="n">
-        <v>-5.308705882352941e-05</v>
+        <v>-8.109823529411765e-05</v>
       </c>
       <c r="AC85" s="11" t="n">
-        <v>-0.004775026455026455</v>
+        <v>-0.007294550264550265</v>
       </c>
       <c r="AD85" s="11" t="n">
-        <v>-119.451681</v>
+        <v>-119.927871</v>
       </c>
       <c r="AE85" s="11" t="n">
-        <v>-0.007026569470588236</v>
+        <v>-0.007054580647058824</v>
       </c>
       <c r="AF85" s="11" t="n">
-        <v>-0.6320194761904763</v>
+        <v>-0.6345390000000001</v>
       </c>
     </row>
     <row r="86">
@@ -18325,22 +18343,22 @@
         <v>-1.216540901798942</v>
       </c>
       <c r="AA91" s="15" t="n">
-        <v>-17.903555</v>
+        <v>-18.379745</v>
       </c>
       <c r="AB91" s="15" t="n">
-        <v>-0.001053150294117647</v>
+        <v>-0.001081161470588235</v>
       </c>
       <c r="AC91" s="15" t="n">
-        <v>-0.09472780423280423</v>
+        <v>-0.09724732804232804</v>
       </c>
       <c r="AD91" s="15" t="n">
-        <v>-247.8297854400001</v>
+        <v>-248.3059754400001</v>
       </c>
       <c r="AE91" s="15" t="n">
-        <v>-0.01457822267294118</v>
+        <v>-0.01460623384941176</v>
       </c>
       <c r="AF91" s="15" t="n">
-        <v>-1.311268706031746</v>
+        <v>-1.31378822984127</v>
       </c>
     </row>
     <row r="92">
@@ -20415,40 +20433,40 @@
         <v>-8.604999264550266</v>
       </c>
       <c r="U117" s="11" t="n">
-        <v>-678.09565</v>
+        <v>-678.09365</v>
       </c>
       <c r="V117" s="11" t="n">
-        <v>-0.0398879794117647</v>
+        <v>-0.03988786176470589</v>
       </c>
       <c r="W117" s="11" t="n">
-        <v>-3.587807671957672</v>
+        <v>-3.58779708994709</v>
       </c>
       <c r="X117" s="11" t="n">
-        <v>-4558.721227</v>
+        <v>-4558.719227</v>
       </c>
       <c r="Y117" s="11" t="n">
-        <v>-0.2681600721764706</v>
+        <v>-0.2681599545294118</v>
       </c>
       <c r="Z117" s="11" t="n">
-        <v>-24.12021813227513</v>
+        <v>-24.12020755026455</v>
       </c>
       <c r="AA117" s="11" t="n">
-        <v>-699.168276</v>
+        <v>-757.339866</v>
       </c>
       <c r="AB117" s="11" t="n">
-        <v>-0.04112754564705882</v>
+        <v>-0.04454940388235294</v>
       </c>
       <c r="AC117" s="11" t="n">
-        <v>-3.699303047619047</v>
+        <v>-4.007089238095238</v>
       </c>
       <c r="AD117" s="11" t="n">
-        <v>-5257.889503</v>
+        <v>-5316.059093</v>
       </c>
       <c r="AE117" s="11" t="n">
-        <v>-0.3092876178235294</v>
+        <v>-0.3127093584117647</v>
       </c>
       <c r="AF117" s="11" t="n">
-        <v>-27.81952117989418</v>
+        <v>-28.12729678835979</v>
       </c>
     </row>
     <row r="118">
@@ -20512,40 +20530,40 @@
         <v>-8.604999264550266</v>
       </c>
       <c r="U118" s="15" t="n">
-        <v>-678.09565</v>
+        <v>-678.09365</v>
       </c>
       <c r="V118" s="15" t="n">
-        <v>-0.0398879794117647</v>
+        <v>-0.03988786176470589</v>
       </c>
       <c r="W118" s="15" t="n">
-        <v>-3.587807671957672</v>
+        <v>-3.58779708994709</v>
       </c>
       <c r="X118" s="15" t="n">
-        <v>-4558.721227</v>
+        <v>-4558.719227</v>
       </c>
       <c r="Y118" s="15" t="n">
-        <v>-0.2681600721764706</v>
+        <v>-0.2681599545294118</v>
       </c>
       <c r="Z118" s="15" t="n">
-        <v>-24.12021813227513</v>
+        <v>-24.12020755026455</v>
       </c>
       <c r="AA118" s="15" t="n">
-        <v>-699.168276</v>
+        <v>-757.339866</v>
       </c>
       <c r="AB118" s="15" t="n">
-        <v>-0.04112754564705882</v>
+        <v>-0.04454940388235294</v>
       </c>
       <c r="AC118" s="15" t="n">
-        <v>-3.699303047619047</v>
+        <v>-4.007089238095238</v>
       </c>
       <c r="AD118" s="15" t="n">
-        <v>-5257.889503</v>
+        <v>-5316.059093</v>
       </c>
       <c r="AE118" s="15" t="n">
-        <v>-0.3092876178235294</v>
+        <v>-0.3127093584117647</v>
       </c>
       <c r="AF118" s="15" t="n">
-        <v>-27.81952117989418</v>
+        <v>-28.12729678835979</v>
       </c>
     </row>
     <row r="119">
@@ -20968,22 +20986,22 @@
         <v>-1.586642857142857</v>
       </c>
       <c r="AA124" s="11" t="n">
-        <v>-28.1385</v>
+        <v>-28.2385</v>
       </c>
       <c r="AB124" s="11" t="n">
-        <v>-0.001655205882352941</v>
+        <v>-0.001661088235294118</v>
       </c>
       <c r="AC124" s="11" t="n">
-        <v>-0.1488809523809524</v>
+        <v>-0.1494100529100529</v>
       </c>
       <c r="AD124" s="11" t="n">
-        <v>-328.014</v>
+        <v>-328.114</v>
       </c>
       <c r="AE124" s="11" t="n">
-        <v>-0.01929494117647059</v>
+        <v>-0.01930082352941177</v>
       </c>
       <c r="AF124" s="11" t="n">
-        <v>-1.735523809523809</v>
+        <v>-1.73605291005291</v>
       </c>
     </row>
     <row r="125">
@@ -21064,17 +21082,23 @@
       <c r="Z125" s="13" t="n">
         <v>-73.71793856084655</v>
       </c>
-      <c r="AA125" s="13" t="n"/>
-      <c r="AB125" s="13" t="n"/>
-      <c r="AC125" s="13" t="n"/>
+      <c r="AA125" s="13" t="n">
+        <v>-1.309164</v>
+      </c>
+      <c r="AB125" s="13" t="n">
+        <v>-7.700964705882354e-05</v>
+      </c>
+      <c r="AC125" s="13" t="n">
+        <v>-0.00692679365079365</v>
+      </c>
       <c r="AD125" s="13" t="n">
-        <v>-13932.690388</v>
+        <v>-13933.999552</v>
       </c>
       <c r="AE125" s="13" t="n">
-        <v>-0.8195700228235293</v>
+        <v>-0.8196470324705881</v>
       </c>
       <c r="AF125" s="13" t="n">
-        <v>-73.71793856084655</v>
+        <v>-73.72486535449734</v>
       </c>
     </row>
     <row r="126">
@@ -21253,22 +21277,22 @@
         <v>-129.966981647672</v>
       </c>
       <c r="AA127" s="15" t="n">
-        <v>-95.077541</v>
+        <v>-96.486705</v>
       </c>
       <c r="AB127" s="15" t="n">
-        <v>-0.005592796529411764</v>
+        <v>-0.005675688529411764</v>
       </c>
       <c r="AC127" s="15" t="n">
-        <v>-0.5030557724867725</v>
+        <v>-0.5105116666666667</v>
       </c>
       <c r="AD127" s="15" t="n">
-        <v>-24658.83707241</v>
+        <v>-24660.24623641</v>
       </c>
       <c r="AE127" s="15" t="n">
-        <v>-1.450519827788824</v>
+        <v>-1.450602719788824</v>
       </c>
       <c r="AF127" s="15" t="n">
-        <v>-130.4700374201587</v>
+        <v>-130.4774933143386</v>
       </c>
     </row>
     <row r="128">
@@ -21958,40 +21982,40 @@
         <v>-18.30885274497355</v>
       </c>
       <c r="U136" s="15" t="n">
-        <v>-4043.27211794</v>
+        <v>-4043.27011794</v>
       </c>
       <c r="V136" s="15" t="n">
-        <v>-0.2378395363494118</v>
+        <v>-0.237839418702353</v>
       </c>
       <c r="W136" s="15" t="n">
-        <v>-21.39297416899471</v>
+        <v>-21.39296358698413</v>
       </c>
       <c r="X136" s="15" t="n">
-        <v>-40289.94322231</v>
+        <v>-40289.94122231</v>
       </c>
       <c r="Y136" s="15" t="n">
-        <v>-2.369996660135882</v>
+        <v>-2.369996542488823</v>
       </c>
       <c r="Z136" s="15" t="n">
-        <v>-213.1743027635449</v>
+        <v>-213.1742921815344</v>
       </c>
       <c r="AA136" s="15" t="n">
-        <v>-1379.867593</v>
+        <v>-1439.924537</v>
       </c>
       <c r="AB136" s="15" t="n">
-        <v>-0.08116868194117646</v>
+        <v>-0.08470144335294118</v>
       </c>
       <c r="AC136" s="15" t="n">
-        <v>-7.300886735449735</v>
+        <v>-7.618648343915345</v>
       </c>
       <c r="AD136" s="15" t="n">
-        <v>-41669.81081531</v>
+        <v>-41729.86575931</v>
       </c>
       <c r="AE136" s="15" t="n">
-        <v>-2.451165342077058</v>
+        <v>-2.454697985841765</v>
       </c>
       <c r="AF136" s="15" t="n">
-        <v>-220.4751894989947</v>
+        <v>-220.7929405254497</v>
       </c>
     </row>
     <row r="137">
@@ -22561,40 +22585,40 @@
         <v>-0.007794830687830687</v>
       </c>
       <c r="U145" s="11" t="n">
-        <v>-2.281144</v>
+        <v>-2.283144</v>
       </c>
       <c r="V145" s="11" t="n">
-        <v>-0.0001341849411764706</v>
+        <v>-0.0001343025882352941</v>
       </c>
       <c r="W145" s="11" t="n">
-        <v>-0.01206954497354497</v>
+        <v>-0.01208012698412698</v>
       </c>
       <c r="X145" s="11" t="n">
-        <v>-16.47462168</v>
+        <v>-16.47662168</v>
       </c>
       <c r="Y145" s="11" t="n">
-        <v>-0.0009690953929411766</v>
+        <v>-0.0009692130400000001</v>
       </c>
       <c r="Z145" s="11" t="n">
-        <v>-0.08716731047619047</v>
+        <v>-0.08717789248677249</v>
       </c>
       <c r="AA145" s="11" t="n">
-        <v>-0.635723</v>
+        <v>-1.310261</v>
       </c>
       <c r="AB145" s="11" t="n">
-        <v>-3.739547058823529e-05</v>
+        <v>-7.707417647058822e-05</v>
       </c>
       <c r="AC145" s="11" t="n">
-        <v>-0.003363613756613757</v>
+        <v>-0.006932597883597883</v>
       </c>
       <c r="AD145" s="11" t="n">
-        <v>-17.11034468</v>
+        <v>-17.78688268</v>
       </c>
       <c r="AE145" s="11" t="n">
-        <v>-0.001006490863529412</v>
+        <v>-0.001046287216470588</v>
       </c>
       <c r="AF145" s="11" t="n">
-        <v>-0.09053092423280423</v>
+        <v>-0.09411049037037038</v>
       </c>
     </row>
     <row r="146">
@@ -23023,40 +23047,40 @@
         <v>-1.768715506190476</v>
       </c>
       <c r="U151" s="15" t="n">
-        <v>-296.97708626</v>
+        <v>-296.97908626</v>
       </c>
       <c r="V151" s="15" t="n">
-        <v>-0.01746924036823529</v>
+        <v>-0.01746935801529412</v>
       </c>
       <c r="W151" s="15" t="n">
-        <v>-1.571307334708995</v>
+        <v>-1.571317916719577</v>
       </c>
       <c r="X151" s="15" t="n">
-        <v>-5668.74290011</v>
+        <v>-5668.74490011</v>
       </c>
       <c r="Y151" s="15" t="n">
-        <v>-0.333455464712353</v>
+        <v>-0.3334555823594119</v>
       </c>
       <c r="Z151" s="15" t="n">
-        <v>-29.99334867783069</v>
+        <v>-29.99335925984127</v>
       </c>
       <c r="AA151" s="15" t="n">
-        <v>-195.7456</v>
+        <v>-196.420138</v>
       </c>
       <c r="AB151" s="15" t="n">
-        <v>-0.01151444705882353</v>
+        <v>-0.01155412576470588</v>
       </c>
       <c r="AC151" s="15" t="n">
-        <v>-1.035691005291005</v>
+        <v>-1.039259989417989</v>
       </c>
       <c r="AD151" s="15" t="n">
-        <v>-5864.48850011</v>
+        <v>-5865.165038110001</v>
       </c>
       <c r="AE151" s="15" t="n">
-        <v>-0.3449699117711765</v>
+        <v>-0.3450097081241177</v>
       </c>
       <c r="AF151" s="15" t="n">
-        <v>-31.02903968312169</v>
+        <v>-31.03261924925926</v>
       </c>
     </row>
     <row r="152">
@@ -23138,22 +23162,22 @@
         <v>-1478.868993977989</v>
       </c>
       <c r="AA152" s="19" t="n">
-        <v>-4006.901718</v>
+        <v>-5443.469854</v>
       </c>
       <c r="AB152" s="19" t="n">
-        <v>-0.2357001010588235</v>
+        <v>-0.3202041090588235</v>
       </c>
       <c r="AC152" s="19" t="n">
-        <v>-21.20053819047619</v>
+        <v>-28.8014277989418</v>
       </c>
       <c r="AD152" s="19" t="n">
-        <v>-283513.1415798399</v>
+        <v>-284949.7097158399</v>
       </c>
       <c r="AE152" s="19" t="n">
-        <v>-16.67724362234353</v>
+        <v>-16.76174763034353</v>
       </c>
       <c r="AF152" s="19" t="n">
-        <v>-1500.069532168465</v>
+        <v>-1507.670421776931</v>
       </c>
     </row>
     <row r="153">
@@ -23235,22 +23259,22 @@
         <v>-340.1043937373017</v>
       </c>
       <c r="AA153" s="19" t="n">
-        <v>-366.831333</v>
+        <v>-1802.106469</v>
       </c>
       <c r="AB153" s="19" t="n">
-        <v>-0.02157831370588235</v>
+        <v>-0.1060062628823529</v>
       </c>
       <c r="AC153" s="19" t="n">
-        <v>-1.940906523809524</v>
+        <v>-9.534954862433862</v>
       </c>
       <c r="AD153" s="19" t="n">
-        <v>-64646.56174935002</v>
+        <v>-66081.83688535001</v>
       </c>
       <c r="AE153" s="19" t="n">
-        <v>-3.802738926432354</v>
+        <v>-3.887166875608825</v>
       </c>
       <c r="AF153" s="19" t="n">
-        <v>-342.0453002611112</v>
+        <v>-349.6393485997355</v>
       </c>
     </row>
     <row r="154">
@@ -23332,22 +23356,22 @@
         <v>16.8991026984656</v>
       </c>
       <c r="AA154" s="7" t="n">
-        <v>2827.099077009999</v>
+        <v>1391.823941009999</v>
       </c>
       <c r="AB154" s="7" t="n">
-        <v>0.1662999457064706</v>
+        <v>0.08187199652999996</v>
       </c>
       <c r="AC154" s="7" t="n">
-        <v>14.95819617465608</v>
+        <v>7.364147836031743</v>
       </c>
       <c r="AD154" s="7" t="n">
-        <v>2827.099077009999</v>
+        <v>1391.823941009999</v>
       </c>
       <c r="AE154" s="7" t="n">
-        <v>0.1662999457064706</v>
+        <v>0.08187199652999996</v>
       </c>
       <c r="AF154" s="7" t="n">
-        <v>14.95819617465608</v>
+        <v>7.364147836031743</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh dashboard Thu 08/20/2026 10:49
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -726,7 +726,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 19 Aug 2026 16:32</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 20 Aug 2026 10:49</t>
         </is>
       </c>
     </row>
@@ -794,14 +794,14 @@
       <c r="Z3" s="4" t="n"/>
       <c r="AA3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 19 Aug 2026</t>
+          <t>MTD as of 20 Aug 2026</t>
         </is>
       </c>
       <c r="AB3" s="4" t="n"/>
       <c r="AC3" s="4" t="n"/>
       <c r="AD3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 19 Aug 2026</t>
+          <t>YTD as of 20 Aug 2026</t>
         </is>
       </c>
       <c r="AE3" s="4" t="n"/>
@@ -12256,7 +12256,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 19 Aug 2026 16:32 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 20 Aug 2026 10:49 (in IDR Million)</t>
         </is>
       </c>
     </row>
@@ -12324,14 +12324,14 @@
       <c r="Z3" s="4" t="n"/>
       <c r="AA3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 19 Aug 2026</t>
+          <t>MTD as of 20 Aug 2026</t>
         </is>
       </c>
       <c r="AB3" s="4" t="n"/>
       <c r="AC3" s="4" t="n"/>
       <c r="AD3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 19 Aug 2026</t>
+          <t>YTD as of 20 Aug 2026</t>
         </is>
       </c>
       <c r="AE3" s="4" t="n"/>

</xml_diff>

<commit_message>
Refresh dashboard Thu 08/20/2026 11:23
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -726,7 +726,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 20 Aug 2026 10:49</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 20 Aug 2026 11:23</t>
         </is>
       </c>
     </row>
@@ -12256,7 +12256,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 20 Aug 2026 10:49 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 20 Aug 2026 11:23 (in IDR Million)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh dashboard Thu 08/20/2026 11:27
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -726,7 +726,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 20 Aug 2026 11:23</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 20 Aug 2026 11:27</t>
         </is>
       </c>
     </row>
@@ -12256,7 +12256,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 20 Aug 2026 11:23 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 20 Aug 2026 11:27 (in IDR Million)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh dashboard Thu 08/20/2026 13:10
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -726,7 +726,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 20 Aug 2026 11:27</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 20 Aug 2026 13:10</t>
         </is>
       </c>
     </row>
@@ -12256,7 +12256,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 20 Aug 2026 11:27 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 20 Aug 2026 13:10 (in IDR Million)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh dashboard Fri 08/21/2026 10:48
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -726,7 +726,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 20 Aug 2026 16:05</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 21 Aug 2026 10:48</t>
         </is>
       </c>
     </row>
@@ -794,14 +794,14 @@
       <c r="Z3" s="4" t="n"/>
       <c r="AA3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 20 Aug 2026</t>
+          <t>MTD as of 21 Aug 2026</t>
         </is>
       </c>
       <c r="AB3" s="4" t="n"/>
       <c r="AC3" s="4" t="n"/>
       <c r="AD3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 20 Aug 2026</t>
+          <t>YTD as of 21 Aug 2026</t>
         </is>
       </c>
       <c r="AE3" s="4" t="n"/>
@@ -12317,7 +12317,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 20 Aug 2026 16:05 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 21 Aug 2026 10:48 (in IDR Million)</t>
         </is>
       </c>
     </row>
@@ -12385,14 +12385,14 @@
       <c r="Z3" s="4" t="n"/>
       <c r="AA3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 20 Aug 2026</t>
+          <t>MTD as of 21 Aug 2026</t>
         </is>
       </c>
       <c r="AB3" s="4" t="n"/>
       <c r="AC3" s="4" t="n"/>
       <c r="AD3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 20 Aug 2026</t>
+          <t>YTD as of 21 Aug 2026</t>
         </is>
       </c>
       <c r="AE3" s="4" t="n"/>

</xml_diff>

<commit_message>
Refresh dashboard Fri 08/21/2026 10:52
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -726,7 +726,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 21 Aug 2026 10:48</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 21 Aug 2026 10:52</t>
         </is>
       </c>
     </row>
@@ -12317,7 +12317,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 21 Aug 2026 10:48 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 21 Aug 2026 10:52 (in IDR Million)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh dashboard Fri 08/21/2026 16:44
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -726,7 +726,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 21 Aug 2026 10:52</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 21 Aug 2026 16:44</t>
         </is>
       </c>
     </row>
@@ -2086,22 +2086,22 @@
         <v>2099643.822698413</v>
       </c>
       <c r="AA20" s="13" t="n">
-        <v>15592680</v>
+        <v>18193180</v>
       </c>
       <c r="AB20" s="13" t="n">
-        <v>917.2164705882353</v>
+        <v>1070.187058823529</v>
       </c>
       <c r="AC20" s="13" t="n">
-        <v>82500.95238095238</v>
+        <v>96260.21164021164</v>
       </c>
       <c r="AD20" s="13" t="n">
-        <v>412425362.49</v>
+        <v>415025862.49</v>
       </c>
       <c r="AE20" s="13" t="n">
-        <v>24260.31544058823</v>
+        <v>24413.28602882353</v>
       </c>
       <c r="AF20" s="13" t="n">
-        <v>2182144.775079365</v>
+        <v>2195904.034338625</v>
       </c>
     </row>
     <row r="21">
@@ -2317,22 +2317,22 @@
         <v>140849.2063492063</v>
       </c>
       <c r="AA23" s="11" t="n">
-        <v>11179000</v>
+        <v>13779500</v>
       </c>
       <c r="AB23" s="11" t="n">
-        <v>657.5882352941177</v>
+        <v>810.5588235294117</v>
       </c>
       <c r="AC23" s="11" t="n">
-        <v>59148.14814814815</v>
+        <v>72907.4074074074</v>
       </c>
       <c r="AD23" s="11" t="n">
-        <v>37799500</v>
+        <v>40400000</v>
       </c>
       <c r="AE23" s="11" t="n">
-        <v>2223.5</v>
+        <v>2376.470588235294</v>
       </c>
       <c r="AF23" s="11" t="n">
-        <v>199997.3544973545</v>
+        <v>213756.6137566137</v>
       </c>
     </row>
     <row r="24">
@@ -3579,22 +3579,22 @@
         <v>1138764600.240688</v>
       </c>
       <c r="AA43" s="15" t="n">
-        <v>5055117184</v>
+        <v>5057717684</v>
       </c>
       <c r="AB43" s="15" t="n">
-        <v>297359.8343529412</v>
+        <v>297512.8049411765</v>
       </c>
       <c r="AC43" s="15" t="n">
-        <v>26746651.76719577</v>
+        <v>26760411.02645503</v>
       </c>
       <c r="AD43" s="15" t="n">
-        <v>220281626629.49</v>
+        <v>220284227129.49</v>
       </c>
       <c r="AE43" s="15" t="n">
-        <v>12957742.74291117</v>
+        <v>12957895.71349941</v>
       </c>
       <c r="AF43" s="15" t="n">
-        <v>1165511252.007884</v>
+        <v>1165525011.267143</v>
       </c>
     </row>
     <row r="44">
@@ -10793,22 +10793,22 @@
         <v>-3855931.507936508</v>
       </c>
       <c r="AA141" s="11" t="n">
-        <v>-98781360</v>
+        <v>-102281360</v>
       </c>
       <c r="AB141" s="11" t="n">
-        <v>-5810.668235294118</v>
+        <v>-6016.550588235295</v>
       </c>
       <c r="AC141" s="11" t="n">
-        <v>-522652.6984126984</v>
+        <v>-541171.2169312169</v>
       </c>
       <c r="AD141" s="11" t="n">
-        <v>-827552415</v>
+        <v>-831052415</v>
       </c>
       <c r="AE141" s="11" t="n">
-        <v>-48679.55382352942</v>
+        <v>-48885.43617647059</v>
       </c>
       <c r="AF141" s="11" t="n">
-        <v>-4378584.206349206</v>
+        <v>-4397102.724867725</v>
       </c>
     </row>
     <row r="142">
@@ -11000,22 +11000,22 @@
         <v>-12697799.23280423</v>
       </c>
       <c r="AA144" s="15" t="n">
-        <v>-98781360</v>
+        <v>-102281360</v>
       </c>
       <c r="AB144" s="15" t="n">
-        <v>-5810.668235294118</v>
+        <v>-6016.550588235295</v>
       </c>
       <c r="AC144" s="15" t="n">
-        <v>-522652.6984126984</v>
+        <v>-541171.2169312169</v>
       </c>
       <c r="AD144" s="15" t="n">
-        <v>-2498665415</v>
+        <v>-2502165415</v>
       </c>
       <c r="AE144" s="15" t="n">
-        <v>-146980.3185294118</v>
+        <v>-147186.2008823529</v>
       </c>
       <c r="AF144" s="15" t="n">
-        <v>-13220451.93121693</v>
+        <v>-13238970.44973545</v>
       </c>
     </row>
     <row r="145">
@@ -11693,22 +11693,22 @@
         <v>-1478868993.977989</v>
       </c>
       <c r="AA153" s="19" t="n">
-        <v>-5806014857</v>
+        <v>-5809514857</v>
       </c>
       <c r="AB153" s="19" t="n">
-        <v>-341530.2857058824</v>
+        <v>-341736.1680588235</v>
       </c>
       <c r="AC153" s="19" t="n">
-        <v>-30719655.32804233</v>
+        <v>-30738173.84656085</v>
       </c>
       <c r="AD153" s="19" t="n">
-        <v>-285312254718.84</v>
+        <v>-285315754718.84</v>
       </c>
       <c r="AE153" s="19" t="n">
-        <v>-16783073.80699059</v>
+        <v>-16783279.68934353</v>
       </c>
       <c r="AF153" s="19" t="n">
-        <v>-1509588649.306032</v>
+        <v>-1509607167.82455</v>
       </c>
     </row>
     <row r="154">
@@ -11790,22 +11790,22 @@
         <v>-340104393.7373017</v>
       </c>
       <c r="AA154" s="19" t="n">
-        <v>-750897673</v>
+        <v>-751797173</v>
       </c>
       <c r="AB154" s="19" t="n">
-        <v>-44170.45135294118</v>
+        <v>-44223.36311764706</v>
       </c>
       <c r="AC154" s="19" t="n">
-        <v>-3973003.560846561</v>
+        <v>-3977762.82010582</v>
       </c>
       <c r="AD154" s="19" t="n">
-        <v>-65030628089.35001</v>
+        <v>-65031527589.35001</v>
       </c>
       <c r="AE154" s="19" t="n">
-        <v>-3825331.064079413</v>
+        <v>-3825383.975844118</v>
       </c>
       <c r="AF154" s="19" t="n">
-        <v>-344077397.2981483</v>
+        <v>-344082156.5574075</v>
       </c>
     </row>
     <row r="155">
@@ -11887,22 +11887,22 @@
         <v>16899102.6984656</v>
       </c>
       <c r="AA155" s="7" t="n">
-        <v>2443032737.009999</v>
+        <v>2442133237.009999</v>
       </c>
       <c r="AB155" s="7" t="n">
-        <v>143707.8080594117</v>
+        <v>143654.8962947058</v>
       </c>
       <c r="AC155" s="7" t="n">
-        <v>12926099.13761904</v>
+        <v>12921339.87835979</v>
       </c>
       <c r="AD155" s="7" t="n">
-        <v>2443032737.009999</v>
+        <v>2442133237.009999</v>
       </c>
       <c r="AE155" s="7" t="n">
-        <v>143707.8080594117</v>
+        <v>143654.8962947058</v>
       </c>
       <c r="AF155" s="7" t="n">
-        <v>12926099.13761904</v>
+        <v>12921339.87835979</v>
       </c>
     </row>
   </sheetData>
@@ -12125,16 +12125,16 @@
         <v>44055921.71</v>
       </c>
       <c r="E9" s="13" t="n">
-        <v>247465402</v>
+        <v>246565902</v>
       </c>
       <c r="F9" s="13" t="n">
-        <v>291521323.71</v>
+        <v>290621823.71</v>
       </c>
       <c r="G9" s="24" t="n">
-        <v>17148.31315941176</v>
+        <v>17095.40139470588</v>
       </c>
       <c r="H9" s="24" t="n">
-        <v>1542440.866190476</v>
+        <v>1537681.606931217</v>
       </c>
     </row>
     <row r="10">
@@ -12244,13 +12244,13 @@
       <c r="D13" s="26" t="n"/>
       <c r="E13" s="26" t="n"/>
       <c r="F13" s="27" t="n">
-        <v>2443032739.01</v>
+        <v>2442133239.01</v>
       </c>
       <c r="G13" s="28" t="n">
-        <v>143707.8081770588</v>
+        <v>143654.8964123529</v>
       </c>
       <c r="H13" s="28" t="n">
-        <v>12926099.14820106</v>
+        <v>12921339.8889418</v>
       </c>
     </row>
   </sheetData>
@@ -12317,7 +12317,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 21 Aug 2026 10:52 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 21 Aug 2026 16:44 (in IDR Million)</t>
         </is>
       </c>
     </row>
@@ -13677,22 +13677,22 @@
         <v>2.099643822698413</v>
       </c>
       <c r="AA20" s="13" t="n">
-        <v>15.59268</v>
+        <v>18.19318</v>
       </c>
       <c r="AB20" s="13" t="n">
-        <v>0.0009172164705882353</v>
+        <v>0.00107018705882353</v>
       </c>
       <c r="AC20" s="13" t="n">
-        <v>0.08250095238095238</v>
+        <v>0.09626021164021165</v>
       </c>
       <c r="AD20" s="13" t="n">
-        <v>412.4253624899999</v>
+        <v>415.02586249</v>
       </c>
       <c r="AE20" s="13" t="n">
-        <v>0.02426031544058824</v>
+        <v>0.02441328602882353</v>
       </c>
       <c r="AF20" s="13" t="n">
-        <v>2.182144775079365</v>
+        <v>2.195904034338624</v>
       </c>
     </row>
     <row r="21">
@@ -13908,22 +13908,22 @@
         <v>0.1408492063492063</v>
       </c>
       <c r="AA23" s="11" t="n">
-        <v>11.179</v>
+        <v>13.7795</v>
       </c>
       <c r="AB23" s="11" t="n">
-        <v>0.0006575882352941177</v>
+        <v>0.0008105588235294118</v>
       </c>
       <c r="AC23" s="11" t="n">
-        <v>0.05914814814814815</v>
+        <v>0.07290740740740741</v>
       </c>
       <c r="AD23" s="11" t="n">
-        <v>37.7995</v>
+        <v>40.4</v>
       </c>
       <c r="AE23" s="11" t="n">
-        <v>0.0022235</v>
+        <v>0.002376470588235294</v>
       </c>
       <c r="AF23" s="11" t="n">
-        <v>0.1999973544973545</v>
+        <v>0.2137566137566138</v>
       </c>
     </row>
     <row r="24">
@@ -15170,22 +15170,22 @@
         <v>1138.764600240688</v>
       </c>
       <c r="AA43" s="15" t="n">
-        <v>5055.117184</v>
+        <v>5057.717684</v>
       </c>
       <c r="AB43" s="15" t="n">
-        <v>0.2973598343529412</v>
+        <v>0.2975128049411765</v>
       </c>
       <c r="AC43" s="15" t="n">
-        <v>26.74665176719576</v>
+        <v>26.76041102645503</v>
       </c>
       <c r="AD43" s="15" t="n">
-        <v>220281.62662949</v>
+        <v>220284.22712949</v>
       </c>
       <c r="AE43" s="15" t="n">
-        <v>12.95774274291117</v>
+        <v>12.95789571349941</v>
       </c>
       <c r="AF43" s="15" t="n">
-        <v>1165.511252007884</v>
+        <v>1165.525011267143</v>
       </c>
     </row>
     <row r="44">
@@ -22384,22 +22384,22 @@
         <v>-3.855931507936508</v>
       </c>
       <c r="AA141" s="11" t="n">
-        <v>-98.78136000000001</v>
+        <v>-102.28136</v>
       </c>
       <c r="AB141" s="11" t="n">
-        <v>-0.005810668235294118</v>
+        <v>-0.006016550588235295</v>
       </c>
       <c r="AC141" s="11" t="n">
-        <v>-0.5226526984126985</v>
+        <v>-0.5411712169312169</v>
       </c>
       <c r="AD141" s="11" t="n">
-        <v>-827.5524150000001</v>
+        <v>-831.0524150000001</v>
       </c>
       <c r="AE141" s="11" t="n">
-        <v>-0.04867955382352942</v>
+        <v>-0.0488854361764706</v>
       </c>
       <c r="AF141" s="11" t="n">
-        <v>-4.378584206349206</v>
+        <v>-4.397102724867725</v>
       </c>
     </row>
     <row r="142">
@@ -22591,22 +22591,22 @@
         <v>-12.69779923280423</v>
       </c>
       <c r="AA144" s="15" t="n">
-        <v>-98.78136000000001</v>
+        <v>-102.28136</v>
       </c>
       <c r="AB144" s="15" t="n">
-        <v>-0.005810668235294118</v>
+        <v>-0.006016550588235295</v>
       </c>
       <c r="AC144" s="15" t="n">
-        <v>-0.5226526984126985</v>
+        <v>-0.5411712169312169</v>
       </c>
       <c r="AD144" s="15" t="n">
-        <v>-2498.665415</v>
+        <v>-2502.165415</v>
       </c>
       <c r="AE144" s="15" t="n">
-        <v>-0.1469803185294118</v>
+        <v>-0.147186200882353</v>
       </c>
       <c r="AF144" s="15" t="n">
-        <v>-13.22045193121693</v>
+        <v>-13.23897044973545</v>
       </c>
     </row>
     <row r="145">
@@ -23284,22 +23284,22 @@
         <v>-1478.868993977989</v>
       </c>
       <c r="AA153" s="19" t="n">
-        <v>-5806.014857</v>
+        <v>-5809.514857</v>
       </c>
       <c r="AB153" s="19" t="n">
-        <v>-0.3415302857058823</v>
+        <v>-0.3417361680588236</v>
       </c>
       <c r="AC153" s="19" t="n">
-        <v>-30.71965532804233</v>
+        <v>-30.73817384656085</v>
       </c>
       <c r="AD153" s="19" t="n">
-        <v>-285312.2547188399</v>
+        <v>-285315.7547188399</v>
       </c>
       <c r="AE153" s="19" t="n">
-        <v>-16.78307380699059</v>
+        <v>-16.78327968934353</v>
       </c>
       <c r="AF153" s="19" t="n">
-        <v>-1509.588649306032</v>
+        <v>-1509.60716782455</v>
       </c>
     </row>
     <row r="154">
@@ -23381,22 +23381,22 @@
         <v>-340.1043937373017</v>
       </c>
       <c r="AA154" s="19" t="n">
-        <v>-750.8976730000001</v>
+        <v>-751.797173</v>
       </c>
       <c r="AB154" s="19" t="n">
-        <v>-0.04417045135294118</v>
+        <v>-0.04422336311764706</v>
       </c>
       <c r="AC154" s="19" t="n">
-        <v>-3.973003560846561</v>
+        <v>-3.97776282010582</v>
       </c>
       <c r="AD154" s="19" t="n">
-        <v>-65030.62808935002</v>
+        <v>-65031.52758935001</v>
       </c>
       <c r="AE154" s="19" t="n">
-        <v>-3.825331064079413</v>
+        <v>-3.825383975844119</v>
       </c>
       <c r="AF154" s="19" t="n">
-        <v>-344.0773972981482</v>
+        <v>-344.0821565574075</v>
       </c>
     </row>
     <row r="155">
@@ -23478,22 +23478,22 @@
         <v>16.8991026984656</v>
       </c>
       <c r="AA155" s="7" t="n">
-        <v>2443.032737009999</v>
+        <v>2442.133237009999</v>
       </c>
       <c r="AB155" s="7" t="n">
-        <v>0.1437078080594117</v>
+        <v>0.1436548962947058</v>
       </c>
       <c r="AC155" s="7" t="n">
-        <v>12.92609913761904</v>
+        <v>12.92133987835978</v>
       </c>
       <c r="AD155" s="7" t="n">
-        <v>2443.032737009999</v>
+        <v>2442.133237009999</v>
       </c>
       <c r="AE155" s="7" t="n">
-        <v>0.1437078080594117</v>
+        <v>0.1436548962947058</v>
       </c>
       <c r="AF155" s="7" t="n">
-        <v>12.92609913761904</v>
+        <v>12.92133987835978</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh dashboard Mon 08/31/2026 16:27
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -726,7 +726,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 28 Aug 2026 14:40</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 31 Aug 2026 16:27</t>
         </is>
       </c>
     </row>
@@ -794,14 +794,14 @@
       <c r="Z3" s="4" t="n"/>
       <c r="AA3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 28 Aug 2026</t>
+          <t>MTD as of 31 Aug 2026</t>
         </is>
       </c>
       <c r="AB3" s="4" t="n"/>
       <c r="AC3" s="4" t="n"/>
       <c r="AD3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 28 Aug 2026</t>
+          <t>YTD as of 31 Aug 2026</t>
         </is>
       </c>
       <c r="AE3" s="4" t="n"/>
@@ -1173,22 +1173,22 @@
         <v>873088236.8412699</v>
       </c>
       <c r="AA7" s="11" t="n">
-        <v>7735236564</v>
+        <v>7793312564</v>
       </c>
       <c r="AB7" s="11" t="n">
-        <v>455013.9155294118</v>
+        <v>458430.1508235294</v>
       </c>
       <c r="AC7" s="11" t="n">
-        <v>40927177.58730159</v>
+        <v>41234458.01058201</v>
       </c>
       <c r="AD7" s="11" t="n">
-        <v>172748913327</v>
+        <v>172806989327</v>
       </c>
       <c r="AE7" s="11" t="n">
-        <v>10161700.78394118</v>
+        <v>10165117.01923529</v>
       </c>
       <c r="AF7" s="11" t="n">
-        <v>914015414.4285715</v>
+        <v>914322694.8518518</v>
       </c>
     </row>
     <row r="8">
@@ -1827,7 +1827,7 @@
     <row r="17">
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">        Kariono</t>
+          <t xml:space="preserve">        CV Permata Abadi Nusantara</t>
         </is>
       </c>
       <c r="C17" s="11" t="n"/>
@@ -1842,53 +1842,53 @@
       <c r="L17" s="11" t="n"/>
       <c r="M17" s="11" t="n"/>
       <c r="N17" s="11" t="n"/>
-      <c r="O17" s="11" t="n">
-        <v>28188000</v>
-      </c>
-      <c r="P17" s="11" t="n">
-        <v>1658.117647058823</v>
-      </c>
-      <c r="Q17" s="11" t="n">
-        <v>149142.8571428571</v>
-      </c>
+      <c r="O17" s="11" t="n"/>
+      <c r="P17" s="11" t="n"/>
+      <c r="Q17" s="11" t="n"/>
       <c r="R17" s="11" t="n"/>
       <c r="S17" s="11" t="n"/>
       <c r="T17" s="11" t="n"/>
       <c r="U17" s="11" t="n">
-        <v>12720000</v>
+        <v>7896000</v>
       </c>
       <c r="V17" s="11" t="n">
-        <v>748.2352941176471</v>
+        <v>464.4705882352941</v>
       </c>
       <c r="W17" s="11" t="n">
-        <v>67301.58730158731</v>
+        <v>41777.77777777778</v>
       </c>
       <c r="X17" s="11" t="n">
-        <v>40908000</v>
+        <v>7896000</v>
       </c>
       <c r="Y17" s="11" t="n">
-        <v>2406.35294117647</v>
+        <v>464.4705882352941</v>
       </c>
       <c r="Z17" s="11" t="n">
-        <v>216444.4444444444</v>
-      </c>
-      <c r="AA17" s="11" t="n"/>
-      <c r="AB17" s="11" t="n"/>
-      <c r="AC17" s="11" t="n"/>
+        <v>41777.77777777778</v>
+      </c>
+      <c r="AA17" s="11" t="n">
+        <v>86156000</v>
+      </c>
+      <c r="AB17" s="11" t="n">
+        <v>5068</v>
+      </c>
+      <c r="AC17" s="11" t="n">
+        <v>455851.8518518519</v>
+      </c>
       <c r="AD17" s="11" t="n">
-        <v>40908000</v>
+        <v>94052000</v>
       </c>
       <c r="AE17" s="11" t="n">
-        <v>2406.35294117647</v>
+        <v>5532.470588235294</v>
       </c>
       <c r="AF17" s="11" t="n">
-        <v>216444.4444444444</v>
+        <v>497629.6296296297</v>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">        CV Permata Abadi Nusantara</t>
+          <t xml:space="preserve">        Kariono</t>
         </is>
       </c>
       <c r="C18" s="13" t="n"/>
@@ -1903,47 +1903,47 @@
       <c r="L18" s="13" t="n"/>
       <c r="M18" s="13" t="n"/>
       <c r="N18" s="13" t="n"/>
-      <c r="O18" s="13" t="n"/>
-      <c r="P18" s="13" t="n"/>
-      <c r="Q18" s="13" t="n"/>
+      <c r="O18" s="13" t="n">
+        <v>28188000</v>
+      </c>
+      <c r="P18" s="13" t="n">
+        <v>1658.117647058823</v>
+      </c>
+      <c r="Q18" s="13" t="n">
+        <v>149142.8571428571</v>
+      </c>
       <c r="R18" s="13" t="n"/>
       <c r="S18" s="13" t="n"/>
       <c r="T18" s="13" t="n"/>
       <c r="U18" s="13" t="n">
-        <v>7896000</v>
+        <v>12720000</v>
       </c>
       <c r="V18" s="13" t="n">
-        <v>464.4705882352941</v>
+        <v>748.2352941176471</v>
       </c>
       <c r="W18" s="13" t="n">
-        <v>41777.77777777778</v>
+        <v>67301.58730158731</v>
       </c>
       <c r="X18" s="13" t="n">
-        <v>7896000</v>
+        <v>40908000</v>
       </c>
       <c r="Y18" s="13" t="n">
-        <v>464.4705882352941</v>
+        <v>2406.35294117647</v>
       </c>
       <c r="Z18" s="13" t="n">
-        <v>41777.77777777778</v>
-      </c>
-      <c r="AA18" s="13" t="n">
-        <v>28080000</v>
-      </c>
-      <c r="AB18" s="13" t="n">
-        <v>1651.764705882353</v>
-      </c>
-      <c r="AC18" s="13" t="n">
-        <v>148571.4285714286</v>
-      </c>
+        <v>216444.4444444444</v>
+      </c>
+      <c r="AA18" s="13" t="n"/>
+      <c r="AB18" s="13" t="n"/>
+      <c r="AC18" s="13" t="n"/>
       <c r="AD18" s="13" t="n">
-        <v>35976000</v>
+        <v>40908000</v>
       </c>
       <c r="AE18" s="13" t="n">
-        <v>2116.235294117647</v>
+        <v>2406.35294117647</v>
       </c>
       <c r="AF18" s="13" t="n">
-        <v>190349.2063492064</v>
+        <v>216444.4444444444</v>
       </c>
     </row>
     <row r="19">
@@ -2184,22 +2184,22 @@
         <v>2099643.822698413</v>
       </c>
       <c r="AA22" s="13" t="n">
-        <v>36555180</v>
+        <v>39539680</v>
       </c>
       <c r="AB22" s="13" t="n">
-        <v>2150.304705882353</v>
+        <v>2325.863529411765</v>
       </c>
       <c r="AC22" s="13" t="n">
-        <v>193413.6507936508</v>
+        <v>209204.6560846561</v>
       </c>
       <c r="AD22" s="13" t="n">
-        <v>433387862.49</v>
+        <v>436372362.49</v>
       </c>
       <c r="AE22" s="13" t="n">
-        <v>25493.40367588235</v>
+        <v>25668.96249941176</v>
       </c>
       <c r="AF22" s="13" t="n">
-        <v>2293057.473492064</v>
+        <v>2308848.478783069</v>
       </c>
     </row>
     <row r="23">
@@ -2415,22 +2415,22 @@
         <v>140849.2063492063</v>
       </c>
       <c r="AA25" s="11" t="n">
-        <v>31398500</v>
+        <v>34383000</v>
       </c>
       <c r="AB25" s="11" t="n">
-        <v>1846.970588235294</v>
+        <v>2022.529411764706</v>
       </c>
       <c r="AC25" s="11" t="n">
-        <v>166129.6296296296</v>
+        <v>181920.6349206349</v>
       </c>
       <c r="AD25" s="11" t="n">
-        <v>58019000</v>
+        <v>61003500</v>
       </c>
       <c r="AE25" s="11" t="n">
-        <v>3412.882352941177</v>
+        <v>3588.441176470588</v>
       </c>
       <c r="AF25" s="11" t="n">
-        <v>306978.8359788359</v>
+        <v>322769.8412698412</v>
       </c>
     </row>
     <row r="26">
@@ -3726,22 +3726,22 @@
         <v>1138764600.240688</v>
       </c>
       <c r="AA46" s="15" t="n">
-        <v>7771791744</v>
+        <v>7832852244</v>
       </c>
       <c r="AB46" s="15" t="n">
-        <v>457164.2202352941</v>
+        <v>460756.0143529412</v>
       </c>
       <c r="AC46" s="15" t="n">
-        <v>41120591.23809524</v>
+        <v>41443662.66666666</v>
       </c>
       <c r="AD46" s="15" t="n">
-        <v>222998301189.49</v>
+        <v>223059361689.49</v>
       </c>
       <c r="AE46" s="15" t="n">
-        <v>13117547.12879353</v>
+        <v>13121138.92291118</v>
       </c>
       <c r="AF46" s="15" t="n">
-        <v>1179885191.478783</v>
+        <v>1180208262.907355</v>
       </c>
     </row>
     <row r="47">
@@ -11767,17 +11767,23 @@
       <c r="Z156" s="11" t="n">
         <v>-3945265.031746032</v>
       </c>
-      <c r="AA156" s="11" t="n"/>
-      <c r="AB156" s="11" t="n"/>
-      <c r="AC156" s="11" t="n"/>
+      <c r="AA156" s="11" t="n">
+        <v>-103034108</v>
+      </c>
+      <c r="AB156" s="11" t="n">
+        <v>-6060.829882352941</v>
+      </c>
+      <c r="AC156" s="11" t="n">
+        <v>-545154.0105820106</v>
+      </c>
       <c r="AD156" s="11" t="n">
-        <v>-745655091</v>
+        <v>-848689199</v>
       </c>
       <c r="AE156" s="11" t="n">
-        <v>-43862.06417647059</v>
+        <v>-49922.89405882353</v>
       </c>
       <c r="AF156" s="11" t="n">
-        <v>-3945265.031746032</v>
+        <v>-4490419.042328042</v>
       </c>
     </row>
     <row r="157">
@@ -11914,22 +11920,22 @@
         <v>-29993359.25984127</v>
       </c>
       <c r="AA158" s="15" t="n">
-        <v>-197252238</v>
+        <v>-300286346</v>
       </c>
       <c r="AB158" s="15" t="n">
-        <v>-11603.07282352941</v>
+        <v>-17663.90270588235</v>
       </c>
       <c r="AC158" s="15" t="n">
-        <v>-1043662.634920635</v>
+        <v>-1588816.645502646</v>
       </c>
       <c r="AD158" s="15" t="n">
-        <v>-5865997138.110001</v>
+        <v>-5969031246.110001</v>
       </c>
       <c r="AE158" s="15" t="n">
-        <v>-345058.6551829412</v>
+        <v>-351119.4850652941</v>
       </c>
       <c r="AF158" s="15" t="n">
-        <v>-31037021.89476191</v>
+        <v>-31582175.90534392</v>
       </c>
     </row>
     <row r="159">
@@ -12011,22 +12017,22 @@
         <v>-1478868993.977989</v>
       </c>
       <c r="AA159" s="19" t="n">
-        <v>-9451783249</v>
+        <v>-9554817357</v>
       </c>
       <c r="AB159" s="19" t="n">
-        <v>-555987.2499411765</v>
+        <v>-562048.0798235295</v>
       </c>
       <c r="AC159" s="19" t="n">
-        <v>-50009435.17989418</v>
+        <v>-50554589.19047619</v>
       </c>
       <c r="AD159" s="19" t="n">
-        <v>-288958023110.84</v>
+        <v>-289061057218.84</v>
       </c>
       <c r="AE159" s="19" t="n">
-        <v>-16997530.77122588</v>
+        <v>-17003591.60110823</v>
       </c>
       <c r="AF159" s="19" t="n">
-        <v>-1528878429.157884</v>
+        <v>-1529423583.168466</v>
       </c>
     </row>
     <row r="160">
@@ -12108,22 +12114,22 @@
         <v>-340104393.7373017</v>
       </c>
       <c r="AA160" s="19" t="n">
-        <v>-1679991505</v>
+        <v>-1721965113</v>
       </c>
       <c r="AB160" s="19" t="n">
-        <v>-98823.02970588235</v>
+        <v>-101292.0654705882</v>
       </c>
       <c r="AC160" s="19" t="n">
-        <v>-8888843.941798942</v>
+        <v>-9110926.523809524</v>
       </c>
       <c r="AD160" s="19" t="n">
-        <v>-65959721921.35001</v>
+        <v>-66001695529.35001</v>
       </c>
       <c r="AE160" s="19" t="n">
-        <v>-3879983.642432354</v>
+        <v>-3882452.67819706</v>
       </c>
       <c r="AF160" s="19" t="n">
-        <v>-348993237.6791006</v>
+        <v>-349215320.2611113</v>
       </c>
     </row>
     <row r="161">
@@ -12205,22 +12211,22 @@
         <v>16899102.6984656</v>
       </c>
       <c r="AA161" s="7" t="n">
-        <v>1513938905.009998</v>
+        <v>1471965297.009998</v>
       </c>
       <c r="AB161" s="7" t="n">
-        <v>89055.22970647049</v>
+        <v>86586.19394176461</v>
       </c>
       <c r="AC161" s="7" t="n">
-        <v>8010258.756666658</v>
+        <v>7788176.174656075</v>
       </c>
       <c r="AD161" s="7" t="n">
-        <v>1513938905.009998</v>
+        <v>1471965297.009998</v>
       </c>
       <c r="AE161" s="7" t="n">
-        <v>89055.22970647049</v>
+        <v>86586.19394176461</v>
       </c>
       <c r="AF161" s="7" t="n">
-        <v>8010258.756666658</v>
+        <v>7788176.174656075</v>
       </c>
     </row>
   </sheetData>
@@ -12347,16 +12353,16 @@
         <v>2698509305</v>
       </c>
       <c r="E6" s="11" t="n">
-        <v>-1458798493</v>
+        <v>-1561832601</v>
       </c>
       <c r="F6" s="11" t="n">
-        <v>1239710812</v>
+        <v>1136676704</v>
       </c>
       <c r="G6" s="23" t="n">
-        <v>72924.16541176471</v>
+        <v>66863.33552941176</v>
       </c>
       <c r="H6" s="23" t="n">
-        <v>6559316.465608465</v>
+        <v>6014162.455026455</v>
       </c>
     </row>
     <row r="7">
@@ -12443,16 +12449,16 @@
         <v>44055921.71</v>
       </c>
       <c r="E9" s="13" t="n">
-        <v>134057832</v>
+        <v>137042332</v>
       </c>
       <c r="F9" s="13" t="n">
-        <v>178113753.71</v>
+        <v>181098253.71</v>
       </c>
       <c r="G9" s="24" t="n">
-        <v>10477.27963</v>
+        <v>10652.83845352941</v>
       </c>
       <c r="H9" s="24" t="n">
-        <v>942400.8132804233</v>
+        <v>958191.8185714287</v>
       </c>
     </row>
     <row r="10">
@@ -12507,16 +12513,16 @@
         <v>79086482.06</v>
       </c>
       <c r="E11" s="13" t="n">
-        <v>-25540935</v>
+        <v>32535065</v>
       </c>
       <c r="F11" s="13" t="n">
-        <v>53545547.06</v>
+        <v>111621547.06</v>
       </c>
       <c r="G11" s="24" t="n">
-        <v>3149.738062352941</v>
+        <v>6565.973356470588</v>
       </c>
       <c r="H11" s="24" t="n">
-        <v>283309.7728042328</v>
+        <v>590590.1960846561</v>
       </c>
     </row>
     <row r="12">
@@ -12562,13 +12568,13 @@
       <c r="D13" s="26" t="n"/>
       <c r="E13" s="26" t="n"/>
       <c r="F13" s="27" t="n">
-        <v>1513938907.01</v>
+        <v>1471965299.01</v>
       </c>
       <c r="G13" s="28" t="n">
-        <v>89055.22982411765</v>
+        <v>86586.19405941176</v>
       </c>
       <c r="H13" s="28" t="n">
-        <v>8010258.767248677</v>
+        <v>7788176.185238095</v>
       </c>
     </row>
   </sheetData>
@@ -12635,7 +12641,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 28 Aug 2026 14:40 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 31 Aug 2026 16:27 (in IDR Million)</t>
         </is>
       </c>
     </row>
@@ -12703,14 +12709,14 @@
       <c r="Z3" s="4" t="n"/>
       <c r="AA3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 28 Aug 2026</t>
+          <t>MTD as of 31 Aug 2026</t>
         </is>
       </c>
       <c r="AB3" s="4" t="n"/>
       <c r="AC3" s="4" t="n"/>
       <c r="AD3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 28 Aug 2026</t>
+          <t>YTD as of 31 Aug 2026</t>
         </is>
       </c>
       <c r="AE3" s="4" t="n"/>
@@ -13082,22 +13088,22 @@
         <v>873.0882368412699</v>
       </c>
       <c r="AA7" s="11" t="n">
-        <v>7735.236564</v>
+        <v>7793.312564</v>
       </c>
       <c r="AB7" s="11" t="n">
-        <v>0.4550139155294117</v>
+        <v>0.4584301508235294</v>
       </c>
       <c r="AC7" s="11" t="n">
-        <v>40.92717758730159</v>
+        <v>41.23445801058201</v>
       </c>
       <c r="AD7" s="11" t="n">
-        <v>172748.913327</v>
+        <v>172806.989327</v>
       </c>
       <c r="AE7" s="11" t="n">
-        <v>10.16170078394117</v>
+        <v>10.16511701923529</v>
       </c>
       <c r="AF7" s="11" t="n">
-        <v>914.0154144285715</v>
+        <v>914.3226948518519</v>
       </c>
     </row>
     <row r="8">
@@ -13736,7 +13742,7 @@
     <row r="17">
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">        Kariono</t>
+          <t xml:space="preserve">        CV Permata Abadi Nusantara</t>
         </is>
       </c>
       <c r="C17" s="11" t="n"/>
@@ -13751,53 +13757,53 @@
       <c r="L17" s="11" t="n"/>
       <c r="M17" s="11" t="n"/>
       <c r="N17" s="11" t="n"/>
-      <c r="O17" s="11" t="n">
-        <v>28.188</v>
-      </c>
-      <c r="P17" s="11" t="n">
-        <v>0.001658117647058823</v>
-      </c>
-      <c r="Q17" s="11" t="n">
-        <v>0.1491428571428571</v>
-      </c>
+      <c r="O17" s="11" t="n"/>
+      <c r="P17" s="11" t="n"/>
+      <c r="Q17" s="11" t="n"/>
       <c r="R17" s="11" t="n"/>
       <c r="S17" s="11" t="n"/>
       <c r="T17" s="11" t="n"/>
       <c r="U17" s="11" t="n">
-        <v>12.72</v>
+        <v>7.896</v>
       </c>
       <c r="V17" s="11" t="n">
-        <v>0.0007482352941176471</v>
+        <v>0.0004644705882352941</v>
       </c>
       <c r="W17" s="11" t="n">
-        <v>0.06730158730158731</v>
+        <v>0.04177777777777777</v>
       </c>
       <c r="X17" s="11" t="n">
-        <v>40.908</v>
+        <v>7.896</v>
       </c>
       <c r="Y17" s="11" t="n">
-        <v>0.002406352941176471</v>
+        <v>0.0004644705882352941</v>
       </c>
       <c r="Z17" s="11" t="n">
-        <v>0.2164444444444444</v>
-      </c>
-      <c r="AA17" s="11" t="n"/>
-      <c r="AB17" s="11" t="n"/>
-      <c r="AC17" s="11" t="n"/>
+        <v>0.04177777777777777</v>
+      </c>
+      <c r="AA17" s="11" t="n">
+        <v>86.15600000000001</v>
+      </c>
+      <c r="AB17" s="11" t="n">
+        <v>0.005068</v>
+      </c>
+      <c r="AC17" s="11" t="n">
+        <v>0.4558518518518519</v>
+      </c>
       <c r="AD17" s="11" t="n">
-        <v>40.908</v>
+        <v>94.05200000000001</v>
       </c>
       <c r="AE17" s="11" t="n">
-        <v>0.002406352941176471</v>
+        <v>0.005532470588235295</v>
       </c>
       <c r="AF17" s="11" t="n">
-        <v>0.2164444444444444</v>
+        <v>0.4976296296296296</v>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">        CV Permata Abadi Nusantara</t>
+          <t xml:space="preserve">        Kariono</t>
         </is>
       </c>
       <c r="C18" s="13" t="n"/>
@@ -13812,47 +13818,47 @@
       <c r="L18" s="13" t="n"/>
       <c r="M18" s="13" t="n"/>
       <c r="N18" s="13" t="n"/>
-      <c r="O18" s="13" t="n"/>
-      <c r="P18" s="13" t="n"/>
-      <c r="Q18" s="13" t="n"/>
+      <c r="O18" s="13" t="n">
+        <v>28.188</v>
+      </c>
+      <c r="P18" s="13" t="n">
+        <v>0.001658117647058823</v>
+      </c>
+      <c r="Q18" s="13" t="n">
+        <v>0.1491428571428571</v>
+      </c>
       <c r="R18" s="13" t="n"/>
       <c r="S18" s="13" t="n"/>
       <c r="T18" s="13" t="n"/>
       <c r="U18" s="13" t="n">
-        <v>7.896</v>
+        <v>12.72</v>
       </c>
       <c r="V18" s="13" t="n">
-        <v>0.0004644705882352941</v>
+        <v>0.0007482352941176471</v>
       </c>
       <c r="W18" s="13" t="n">
-        <v>0.04177777777777777</v>
+        <v>0.06730158730158731</v>
       </c>
       <c r="X18" s="13" t="n">
-        <v>7.896</v>
+        <v>40.908</v>
       </c>
       <c r="Y18" s="13" t="n">
-        <v>0.0004644705882352941</v>
+        <v>0.002406352941176471</v>
       </c>
       <c r="Z18" s="13" t="n">
-        <v>0.04177777777777777</v>
-      </c>
-      <c r="AA18" s="13" t="n">
-        <v>28.08</v>
-      </c>
-      <c r="AB18" s="13" t="n">
-        <v>0.001651764705882353</v>
-      </c>
-      <c r="AC18" s="13" t="n">
-        <v>0.1485714285714285</v>
-      </c>
+        <v>0.2164444444444444</v>
+      </c>
+      <c r="AA18" s="13" t="n"/>
+      <c r="AB18" s="13" t="n"/>
+      <c r="AC18" s="13" t="n"/>
       <c r="AD18" s="13" t="n">
-        <v>35.976</v>
+        <v>40.908</v>
       </c>
       <c r="AE18" s="13" t="n">
-        <v>0.002116235294117647</v>
+        <v>0.002406352941176471</v>
       </c>
       <c r="AF18" s="13" t="n">
-        <v>0.1903492063492063</v>
+        <v>0.2164444444444444</v>
       </c>
     </row>
     <row r="19">
@@ -14093,22 +14099,22 @@
         <v>2.099643822698413</v>
       </c>
       <c r="AA22" s="13" t="n">
-        <v>36.55518</v>
+        <v>39.53968</v>
       </c>
       <c r="AB22" s="13" t="n">
-        <v>0.002150304705882353</v>
+        <v>0.002325863529411764</v>
       </c>
       <c r="AC22" s="13" t="n">
-        <v>0.1934136507936508</v>
+        <v>0.2092046560846561</v>
       </c>
       <c r="AD22" s="13" t="n">
-        <v>433.38786249</v>
+        <v>436.3723624899999</v>
       </c>
       <c r="AE22" s="13" t="n">
-        <v>0.02549340367588235</v>
+        <v>0.02566896249941177</v>
       </c>
       <c r="AF22" s="13" t="n">
-        <v>2.293057473492063</v>
+        <v>2.308848478783069</v>
       </c>
     </row>
     <row r="23">
@@ -14324,22 +14330,22 @@
         <v>0.1408492063492063</v>
       </c>
       <c r="AA25" s="11" t="n">
-        <v>31.3985</v>
+        <v>34.383</v>
       </c>
       <c r="AB25" s="11" t="n">
-        <v>0.001846970588235294</v>
+        <v>0.002022529411764706</v>
       </c>
       <c r="AC25" s="11" t="n">
-        <v>0.1661296296296296</v>
+        <v>0.1819206349206349</v>
       </c>
       <c r="AD25" s="11" t="n">
-        <v>58.019</v>
+        <v>61.0035</v>
       </c>
       <c r="AE25" s="11" t="n">
-        <v>0.003412882352941176</v>
+        <v>0.003588441176470589</v>
       </c>
       <c r="AF25" s="11" t="n">
-        <v>0.306978835978836</v>
+        <v>0.3227698412698413</v>
       </c>
     </row>
     <row r="26">
@@ -15635,22 +15641,22 @@
         <v>1138.764600240688</v>
       </c>
       <c r="AA46" s="15" t="n">
-        <v>7771.791744</v>
+        <v>7832.852244</v>
       </c>
       <c r="AB46" s="15" t="n">
-        <v>0.4571642202352941</v>
+        <v>0.4607560143529412</v>
       </c>
       <c r="AC46" s="15" t="n">
-        <v>41.12059123809524</v>
+        <v>41.44366266666667</v>
       </c>
       <c r="AD46" s="15" t="n">
-        <v>222998.30118949</v>
+        <v>223059.36168949</v>
       </c>
       <c r="AE46" s="15" t="n">
-        <v>13.11754712879353</v>
+        <v>13.12113892291118</v>
       </c>
       <c r="AF46" s="15" t="n">
-        <v>1179.885191478783</v>
+        <v>1180.208262907354</v>
       </c>
     </row>
     <row r="47">
@@ -23676,17 +23682,23 @@
       <c r="Z156" s="11" t="n">
         <v>-3.945265031746032</v>
       </c>
-      <c r="AA156" s="11" t="n"/>
-      <c r="AB156" s="11" t="n"/>
-      <c r="AC156" s="11" t="n"/>
+      <c r="AA156" s="11" t="n">
+        <v>-103.034108</v>
+      </c>
+      <c r="AB156" s="11" t="n">
+        <v>-0.006060829882352942</v>
+      </c>
+      <c r="AC156" s="11" t="n">
+        <v>-0.5451540105820106</v>
+      </c>
       <c r="AD156" s="11" t="n">
-        <v>-745.6550910000001</v>
+        <v>-848.6891990000001</v>
       </c>
       <c r="AE156" s="11" t="n">
-        <v>-0.04386206417647059</v>
+        <v>-0.04992289405882353</v>
       </c>
       <c r="AF156" s="11" t="n">
-        <v>-3.945265031746032</v>
+        <v>-4.490419042328043</v>
       </c>
     </row>
     <row r="157">
@@ -23823,22 +23835,22 @@
         <v>-29.99335925984127</v>
       </c>
       <c r="AA158" s="15" t="n">
-        <v>-197.252238</v>
+        <v>-300.286346</v>
       </c>
       <c r="AB158" s="15" t="n">
-        <v>-0.01160307282352941</v>
+        <v>-0.01766390270588235</v>
       </c>
       <c r="AC158" s="15" t="n">
-        <v>-1.043662634920635</v>
+        <v>-1.588816645502645</v>
       </c>
       <c r="AD158" s="15" t="n">
-        <v>-5865.99713811</v>
+        <v>-5969.03124611</v>
       </c>
       <c r="AE158" s="15" t="n">
-        <v>-0.3450586551829413</v>
+        <v>-0.3511194850652942</v>
       </c>
       <c r="AF158" s="15" t="n">
-        <v>-31.0370218947619</v>
+        <v>-31.58217590534391</v>
       </c>
     </row>
     <row r="159">
@@ -23920,22 +23932,22 @@
         <v>-1478.868993977989</v>
       </c>
       <c r="AA159" s="19" t="n">
-        <v>-9451.783249</v>
+        <v>-9554.817357</v>
       </c>
       <c r="AB159" s="19" t="n">
-        <v>-0.5559872499411764</v>
+        <v>-0.5620480798235294</v>
       </c>
       <c r="AC159" s="19" t="n">
-        <v>-50.00943517989418</v>
+        <v>-50.55458919047619</v>
       </c>
       <c r="AD159" s="19" t="n">
-        <v>-288958.0231108399</v>
+        <v>-289061.0572188399</v>
       </c>
       <c r="AE159" s="19" t="n">
-        <v>-16.99753077122588</v>
+        <v>-17.00359160110824</v>
       </c>
       <c r="AF159" s="19" t="n">
-        <v>-1528.878429157883</v>
+        <v>-1529.423583168465</v>
       </c>
     </row>
     <row r="160">
@@ -24017,22 +24029,22 @@
         <v>-340.1043937373017</v>
       </c>
       <c r="AA160" s="19" t="n">
-        <v>-1679.991505</v>
+        <v>-1721.965113</v>
       </c>
       <c r="AB160" s="19" t="n">
-        <v>-0.09882302970588235</v>
+        <v>-0.1012920654705882</v>
       </c>
       <c r="AC160" s="19" t="n">
-        <v>-8.888843941798942</v>
+        <v>-9.110926523809523</v>
       </c>
       <c r="AD160" s="19" t="n">
-        <v>-65959.72192135002</v>
+        <v>-66001.69552935002</v>
       </c>
       <c r="AE160" s="19" t="n">
-        <v>-3.879983642432354</v>
+        <v>-3.88245267819706</v>
       </c>
       <c r="AF160" s="19" t="n">
-        <v>-348.9932376791006</v>
+        <v>-349.2153202611112</v>
       </c>
     </row>
     <row r="161">
@@ -24114,22 +24126,22 @@
         <v>16.8991026984656</v>
       </c>
       <c r="AA161" s="7" t="n">
-        <v>1513.938905009998</v>
+        <v>1471.965297009998</v>
       </c>
       <c r="AB161" s="7" t="n">
-        <v>0.08905522970647049</v>
+        <v>0.0865861939417646</v>
       </c>
       <c r="AC161" s="7" t="n">
-        <v>8.010258756666657</v>
+        <v>7.788176174656075</v>
       </c>
       <c r="AD161" s="7" t="n">
-        <v>1513.938905009998</v>
+        <v>1471.965297009998</v>
       </c>
       <c r="AE161" s="7" t="n">
-        <v>0.08905522970647049</v>
+        <v>0.0865861939417646</v>
       </c>
       <c r="AF161" s="7" t="n">
-        <v>8.010258756666657</v>
+        <v>7.788176174656075</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh dashboard Tue 09/01/2026 16:45
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -723,7 +723,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 01 Sep 2026 16:07</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 01 Sep 2026 16:45</t>
         </is>
       </c>
     </row>
@@ -11361,7 +11361,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 01 Sep 2026 16:07 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 01 Sep 2026 16:45 (in IDR Million)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh dashboard Thu 09/03/2026 17:09
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -730,7 +730,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 01 Sep 2026 16:46</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 03 Sep 2026 17:09</t>
         </is>
       </c>
     </row>
@@ -805,14 +805,14 @@
       <c r="AC3" s="4" t="n"/>
       <c r="AD3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 01 Sep 2026</t>
+          <t>MTD as of 03 Sep 2026</t>
         </is>
       </c>
       <c r="AE3" s="4" t="n"/>
       <c r="AF3" s="4" t="n"/>
       <c r="AG3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 01 Sep 2026</t>
+          <t>YTD as of 03 Sep 2026</t>
         </is>
       </c>
       <c r="AH3" s="4" t="n"/>
@@ -2357,17 +2357,23 @@
       <c r="AC23" s="11" t="n">
         <v>2321849.073439153</v>
       </c>
-      <c r="AD23" s="11" t="n"/>
-      <c r="AE23" s="11" t="n"/>
-      <c r="AF23" s="11" t="n"/>
+      <c r="AD23" s="11" t="n">
+        <v>3528000</v>
+      </c>
+      <c r="AE23" s="11" t="n">
+        <v>207.5294117647059</v>
+      </c>
+      <c r="AF23" s="11" t="n">
+        <v>18666.66666666667</v>
+      </c>
       <c r="AG23" s="11" t="n">
-        <v>438829474.88</v>
+        <v>442357474.88</v>
       </c>
       <c r="AH23" s="11" t="n">
-        <v>25813.49852235294</v>
+        <v>26021.02793411765</v>
       </c>
       <c r="AI23" s="11" t="n">
-        <v>2321849.073439153</v>
+        <v>2340515.74010582</v>
       </c>
     </row>
     <row r="24">
@@ -2603,17 +2609,23 @@
       <c r="AC26" s="13" t="n">
         <v>332547.6190476191</v>
       </c>
-      <c r="AD26" s="13" t="n"/>
-      <c r="AE26" s="13" t="n"/>
-      <c r="AF26" s="13" t="n"/>
+      <c r="AD26" s="13" t="n">
+        <v>3528000</v>
+      </c>
+      <c r="AE26" s="13" t="n">
+        <v>207.5294117647059</v>
+      </c>
+      <c r="AF26" s="13" t="n">
+        <v>18666.66666666667</v>
+      </c>
       <c r="AG26" s="13" t="n">
-        <v>62851500</v>
+        <v>66379500</v>
       </c>
       <c r="AH26" s="13" t="n">
-        <v>3697.147058823529</v>
+        <v>3904.676470588235</v>
       </c>
       <c r="AI26" s="13" t="n">
-        <v>332547.6190476191</v>
+        <v>351214.2857142857</v>
       </c>
     </row>
     <row r="27">
@@ -3984,22 +3996,22 @@
         <v>1180222393.205714</v>
       </c>
       <c r="AD47" s="15" t="n">
-        <v>75379454</v>
+        <v>78907454</v>
       </c>
       <c r="AE47" s="15" t="n">
-        <v>4434.085529411765</v>
+        <v>4641.614941176471</v>
       </c>
       <c r="AF47" s="15" t="n">
-        <v>398833.08994709</v>
+        <v>417499.7566137566</v>
       </c>
       <c r="AG47" s="15" t="n">
-        <v>223137411769.88</v>
+        <v>223140939769.88</v>
       </c>
       <c r="AH47" s="15" t="n">
-        <v>13125730.10411059</v>
+        <v>13125937.63352235</v>
       </c>
       <c r="AI47" s="15" t="n">
-        <v>1180621226.295661</v>
+        <v>1180639892.962328</v>
       </c>
     </row>
     <row r="48">
@@ -11725,17 +11737,23 @@
       <c r="AC148" s="11" t="n">
         <v>-4894589.497354497</v>
       </c>
-      <c r="AD148" s="11" t="n"/>
-      <c r="AE148" s="11" t="n"/>
-      <c r="AF148" s="11" t="n"/>
+      <c r="AD148" s="11" t="n">
+        <v>-1000000</v>
+      </c>
+      <c r="AE148" s="11" t="n">
+        <v>-58.8235294117647</v>
+      </c>
+      <c r="AF148" s="11" t="n">
+        <v>-5291.005291005291</v>
+      </c>
       <c r="AG148" s="11" t="n">
-        <v>-925077415</v>
+        <v>-926077415</v>
       </c>
       <c r="AH148" s="11" t="n">
-        <v>-54416.31852941176</v>
+        <v>-54475.14205882353</v>
       </c>
       <c r="AI148" s="11" t="n">
-        <v>-4894589.497354497</v>
+        <v>-4899880.502645503</v>
       </c>
     </row>
     <row r="149">
@@ -11941,17 +11959,23 @@
       <c r="AC151" s="15" t="n">
         <v>-13736457.22222222</v>
       </c>
-      <c r="AD151" s="15" t="n"/>
-      <c r="AE151" s="15" t="n"/>
-      <c r="AF151" s="15" t="n"/>
+      <c r="AD151" s="15" t="n">
+        <v>-1000000</v>
+      </c>
+      <c r="AE151" s="15" t="n">
+        <v>-58.8235294117647</v>
+      </c>
+      <c r="AF151" s="15" t="n">
+        <v>-5291.005291005291</v>
+      </c>
       <c r="AG151" s="15" t="n">
-        <v>-2596190415</v>
+        <v>-2597190415</v>
       </c>
       <c r="AH151" s="15" t="n">
-        <v>-152717.0832352941</v>
+        <v>-152775.9067647059</v>
       </c>
       <c r="AI151" s="15" t="n">
-        <v>-13736457.22222222</v>
+        <v>-13741748.22751323</v>
       </c>
     </row>
     <row r="152">
@@ -12081,17 +12105,23 @@
       <c r="AC153" s="11" t="n">
         <v>-99449.19407407405</v>
       </c>
-      <c r="AD153" s="11" t="n"/>
-      <c r="AE153" s="11" t="n"/>
-      <c r="AF153" s="11" t="n"/>
+      <c r="AD153" s="11" t="n">
+        <v>-2500</v>
+      </c>
+      <c r="AE153" s="11" t="n">
+        <v>-0.1470588235294118</v>
+      </c>
+      <c r="AF153" s="11" t="n">
+        <v>-13.22751322751323</v>
+      </c>
       <c r="AG153" s="11" t="n">
-        <v>-18795897.68</v>
+        <v>-18798397.68</v>
       </c>
       <c r="AH153" s="11" t="n">
-        <v>-1105.64104</v>
+        <v>-1105.788098823529</v>
       </c>
       <c r="AI153" s="11" t="n">
-        <v>-99449.19407407405</v>
+        <v>-99462.42158730156</v>
       </c>
     </row>
     <row r="154">
@@ -12567,17 +12597,23 @@
       <c r="AC159" s="15" t="n">
         <v>-31583868.07253968</v>
       </c>
-      <c r="AD159" s="15" t="n"/>
-      <c r="AE159" s="15" t="n"/>
-      <c r="AF159" s="15" t="n"/>
+      <c r="AD159" s="15" t="n">
+        <v>-2500</v>
+      </c>
+      <c r="AE159" s="15" t="n">
+        <v>-0.1470588235294118</v>
+      </c>
+      <c r="AF159" s="15" t="n">
+        <v>-13.22751322751323</v>
+      </c>
       <c r="AG159" s="15" t="n">
-        <v>-5969351065.710001</v>
+        <v>-5969353565.710001</v>
       </c>
       <c r="AH159" s="15" t="n">
-        <v>-351138.2979829411</v>
+        <v>-351138.4450417647</v>
       </c>
       <c r="AI159" s="15" t="n">
-        <v>-31583868.07253968</v>
+        <v>-31583881.30005291</v>
       </c>
     </row>
     <row r="160">
@@ -12668,22 +12704,22 @@
         <v>-1529478500.653757</v>
       </c>
       <c r="AD160" s="19" t="n">
-        <v>-11312300</v>
+        <v>-12314800</v>
       </c>
       <c r="AE160" s="19" t="n">
-        <v>-665.4294117647058</v>
+        <v>-724.4</v>
       </c>
       <c r="AF160" s="19" t="n">
-        <v>-59853.43915343915</v>
+        <v>-65157.67195767196</v>
       </c>
       <c r="AG160" s="19" t="n">
-        <v>-289082748923.5599</v>
+        <v>-289083751423.5599</v>
       </c>
       <c r="AH160" s="19" t="n">
-        <v>-17004867.58373882</v>
+        <v>-17004926.55432706</v>
       </c>
       <c r="AI160" s="19" t="n">
-        <v>-1529538354.09291</v>
+        <v>-1529543658.325714</v>
       </c>
     </row>
     <row r="161">
@@ -12774,22 +12810,22 @@
         <v>-349256107.4480425</v>
       </c>
       <c r="AD161" s="19" t="n">
-        <v>64067154</v>
+        <v>66592654</v>
       </c>
       <c r="AE161" s="19" t="n">
-        <v>3768.656117647059</v>
+        <v>3917.214941176471</v>
       </c>
       <c r="AF161" s="19" t="n">
-        <v>338979.6507936508</v>
+        <v>352342.0846560847</v>
       </c>
       <c r="AG161" s="19" t="n">
-        <v>-65945337153.68</v>
+        <v>-65942811653.68</v>
       </c>
       <c r="AH161" s="19" t="n">
-        <v>-3879137.479628236</v>
+        <v>-3878988.920804706</v>
       </c>
       <c r="AI161" s="19" t="n">
-        <v>-348917127.7972488</v>
+        <v>-348903765.3633864</v>
       </c>
     </row>
     <row r="162">
@@ -12880,22 +12916,22 @@
         <v>7747388.987724859</v>
       </c>
       <c r="AD162" s="7" t="n">
-        <v>1528323672.679998</v>
+        <v>1530849172.679998</v>
       </c>
       <c r="AE162" s="7" t="n">
-        <v>89901.39251058814</v>
+        <v>90049.95133411755</v>
       </c>
       <c r="AF162" s="7" t="n">
-        <v>8086368.63851851</v>
+        <v>8099731.072380944</v>
       </c>
       <c r="AG162" s="7" t="n">
-        <v>1528323672.679998</v>
+        <v>1530849172.679998</v>
       </c>
       <c r="AH162" s="7" t="n">
-        <v>89901.39251058814</v>
+        <v>90049.95133411755</v>
       </c>
       <c r="AI162" s="7" t="n">
-        <v>8086368.63851851</v>
+        <v>8099731.072380944</v>
       </c>
     </row>
   </sheetData>
@@ -13424,16 +13460,16 @@
         <v>1975000</v>
       </c>
       <c r="E8" s="11" t="n">
-        <v>0</v>
+        <v>25000</v>
       </c>
       <c r="F8" s="11" t="n">
-        <v>1975000</v>
+        <v>2000000</v>
       </c>
       <c r="G8" s="23" t="n">
-        <v>116.1764705882353</v>
+        <v>117.6470588235294</v>
       </c>
       <c r="H8" s="23" t="n">
-        <v>10449.73544973545</v>
+        <v>10582.01058201058</v>
       </c>
     </row>
     <row r="9">
@@ -13456,16 +13492,16 @@
         <v>172976399.24</v>
       </c>
       <c r="E9" s="13" t="n">
-        <v>-11312300</v>
+        <v>-8811800</v>
       </c>
       <c r="F9" s="13" t="n">
-        <v>161664099.24</v>
+        <v>164164599.24</v>
       </c>
       <c r="G9" s="24" t="n">
-        <v>9509.652896470589</v>
+        <v>9656.741131764706</v>
       </c>
       <c r="H9" s="24" t="n">
-        <v>855365.6044444445</v>
+        <v>868595.7631746032</v>
       </c>
     </row>
     <row r="10">
@@ -13575,13 +13611,13 @@
       <c r="D13" s="26" t="n"/>
       <c r="E13" s="26" t="n"/>
       <c r="F13" s="27" t="n">
-        <v>1528323674.68</v>
+        <v>1530849174.68</v>
       </c>
       <c r="G13" s="28" t="n">
-        <v>89901.39262823529</v>
+        <v>90049.9514517647</v>
       </c>
       <c r="H13" s="28" t="n">
-        <v>8086368.649100529</v>
+        <v>8099731.082962964</v>
       </c>
     </row>
   </sheetData>
@@ -13651,7 +13687,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 01 Sep 2026 16:46 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 03 Sep 2026 17:09 (in IDR Million)</t>
         </is>
       </c>
     </row>
@@ -13726,14 +13762,14 @@
       <c r="AC3" s="4" t="n"/>
       <c r="AD3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 01 Sep 2026</t>
+          <t>MTD as of 03 Sep 2026</t>
         </is>
       </c>
       <c r="AE3" s="4" t="n"/>
       <c r="AF3" s="4" t="n"/>
       <c r="AG3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 01 Sep 2026</t>
+          <t>YTD as of 03 Sep 2026</t>
         </is>
       </c>
       <c r="AH3" s="4" t="n"/>
@@ -15278,17 +15314,23 @@
       <c r="AC23" s="11" t="n">
         <v>2.321849073439154</v>
       </c>
-      <c r="AD23" s="11" t="n"/>
-      <c r="AE23" s="11" t="n"/>
-      <c r="AF23" s="11" t="n"/>
+      <c r="AD23" s="11" t="n">
+        <v>3.528</v>
+      </c>
+      <c r="AE23" s="11" t="n">
+        <v>0.0002075294117647059</v>
+      </c>
+      <c r="AF23" s="11" t="n">
+        <v>0.01866666666666667</v>
+      </c>
       <c r="AG23" s="11" t="n">
-        <v>438.82947488</v>
+        <v>442.35747488</v>
       </c>
       <c r="AH23" s="11" t="n">
-        <v>0.02581349852235294</v>
+        <v>0.02602102793411765</v>
       </c>
       <c r="AI23" s="11" t="n">
-        <v>2.321849073439154</v>
+        <v>2.340515740105821</v>
       </c>
     </row>
     <row r="24">
@@ -15524,17 +15566,23 @@
       <c r="AC26" s="13" t="n">
         <v>0.332547619047619</v>
       </c>
-      <c r="AD26" s="13" t="n"/>
-      <c r="AE26" s="13" t="n"/>
-      <c r="AF26" s="13" t="n"/>
+      <c r="AD26" s="13" t="n">
+        <v>3.528</v>
+      </c>
+      <c r="AE26" s="13" t="n">
+        <v>0.0002075294117647059</v>
+      </c>
+      <c r="AF26" s="13" t="n">
+        <v>0.01866666666666667</v>
+      </c>
       <c r="AG26" s="13" t="n">
-        <v>62.8515</v>
+        <v>66.37950000000001</v>
       </c>
       <c r="AH26" s="13" t="n">
-        <v>0.00369714705882353</v>
+        <v>0.003904676470588236</v>
       </c>
       <c r="AI26" s="13" t="n">
-        <v>0.332547619047619</v>
+        <v>0.3512142857142857</v>
       </c>
     </row>
     <row r="27">
@@ -16905,22 +16953,22 @@
         <v>1180.222393205714</v>
       </c>
       <c r="AD47" s="15" t="n">
-        <v>75.379454</v>
+        <v>78.907454</v>
       </c>
       <c r="AE47" s="15" t="n">
-        <v>0.004434085529411764</v>
+        <v>0.004641614941176471</v>
       </c>
       <c r="AF47" s="15" t="n">
-        <v>0.3988330899470899</v>
+        <v>0.4174997566137566</v>
       </c>
       <c r="AG47" s="15" t="n">
-        <v>223137.41176988</v>
+        <v>223140.93976988</v>
       </c>
       <c r="AH47" s="15" t="n">
-        <v>13.12573010411059</v>
+        <v>13.12593763352235</v>
       </c>
       <c r="AI47" s="15" t="n">
-        <v>1180.621226295661</v>
+        <v>1180.639892962328</v>
       </c>
     </row>
     <row r="48">
@@ -24646,17 +24694,23 @@
       <c r="AC148" s="11" t="n">
         <v>-4.894589497354497</v>
       </c>
-      <c r="AD148" s="11" t="n"/>
-      <c r="AE148" s="11" t="n"/>
-      <c r="AF148" s="11" t="n"/>
+      <c r="AD148" s="11" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AE148" s="11" t="n">
+        <v>-5.882352941176471e-05</v>
+      </c>
+      <c r="AF148" s="11" t="n">
+        <v>-0.005291005291005291</v>
+      </c>
       <c r="AG148" s="11" t="n">
-        <v>-925.0774150000001</v>
+        <v>-926.0774150000001</v>
       </c>
       <c r="AH148" s="11" t="n">
-        <v>-0.05441631852941178</v>
+        <v>-0.05447514205882354</v>
       </c>
       <c r="AI148" s="11" t="n">
-        <v>-4.894589497354497</v>
+        <v>-4.899880502645503</v>
       </c>
     </row>
     <row r="149">
@@ -24862,17 +24916,23 @@
       <c r="AC151" s="15" t="n">
         <v>-13.73645722222222</v>
       </c>
-      <c r="AD151" s="15" t="n"/>
-      <c r="AE151" s="15" t="n"/>
-      <c r="AF151" s="15" t="n"/>
+      <c r="AD151" s="15" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AE151" s="15" t="n">
+        <v>-5.882352941176471e-05</v>
+      </c>
+      <c r="AF151" s="15" t="n">
+        <v>-0.005291005291005291</v>
+      </c>
       <c r="AG151" s="15" t="n">
-        <v>-2596.190415</v>
+        <v>-2597.190415</v>
       </c>
       <c r="AH151" s="15" t="n">
-        <v>-0.1527170832352941</v>
+        <v>-0.1527759067647059</v>
       </c>
       <c r="AI151" s="15" t="n">
-        <v>-13.73645722222222</v>
+        <v>-13.74174822751323</v>
       </c>
     </row>
     <row r="152">
@@ -25002,17 +25062,23 @@
       <c r="AC153" s="11" t="n">
         <v>-0.09944919407407407</v>
       </c>
-      <c r="AD153" s="11" t="n"/>
-      <c r="AE153" s="11" t="n"/>
-      <c r="AF153" s="11" t="n"/>
+      <c r="AD153" s="11" t="n">
+        <v>-0.0025</v>
+      </c>
+      <c r="AE153" s="11" t="n">
+        <v>-1.470588235294118e-07</v>
+      </c>
+      <c r="AF153" s="11" t="n">
+        <v>-1.322751322751323e-05</v>
+      </c>
       <c r="AG153" s="11" t="n">
-        <v>-18.79589768</v>
+        <v>-18.79839768</v>
       </c>
       <c r="AH153" s="11" t="n">
-        <v>-0.00110564104</v>
+        <v>-0.00110578809882353</v>
       </c>
       <c r="AI153" s="11" t="n">
-        <v>-0.09944919407407407</v>
+        <v>-0.09946242158730158</v>
       </c>
     </row>
     <row r="154">
@@ -25488,17 +25554,23 @@
       <c r="AC159" s="15" t="n">
         <v>-31.58386807253968</v>
       </c>
-      <c r="AD159" s="15" t="n"/>
-      <c r="AE159" s="15" t="n"/>
-      <c r="AF159" s="15" t="n"/>
+      <c r="AD159" s="15" t="n">
+        <v>-0.0025</v>
+      </c>
+      <c r="AE159" s="15" t="n">
+        <v>-1.470588235294118e-07</v>
+      </c>
+      <c r="AF159" s="15" t="n">
+        <v>-1.322751322751323e-05</v>
+      </c>
       <c r="AG159" s="15" t="n">
-        <v>-5969.351065710001</v>
+        <v>-5969.35356571</v>
       </c>
       <c r="AH159" s="15" t="n">
-        <v>-0.3511382979829413</v>
+        <v>-0.3511384450417648</v>
       </c>
       <c r="AI159" s="15" t="n">
-        <v>-31.58386807253968</v>
+        <v>-31.58388130005291</v>
       </c>
     </row>
     <row r="160">
@@ -25589,22 +25661,22 @@
         <v>-1529.478500653756</v>
       </c>
       <c r="AD160" s="19" t="n">
-        <v>-11.3123</v>
+        <v>-12.3148</v>
       </c>
       <c r="AE160" s="19" t="n">
-        <v>-0.0006654294117647059</v>
+        <v>-0.0007244</v>
       </c>
       <c r="AF160" s="19" t="n">
-        <v>-0.05985343915343916</v>
+        <v>-0.06515767195767196</v>
       </c>
       <c r="AG160" s="19" t="n">
-        <v>-289082.7489235599</v>
+        <v>-289083.7514235599</v>
       </c>
       <c r="AH160" s="19" t="n">
-        <v>-17.00486758373883</v>
+        <v>-17.00492655432706</v>
       </c>
       <c r="AI160" s="19" t="n">
-        <v>-1529.53835409291</v>
+        <v>-1529.543658325714</v>
       </c>
     </row>
     <row r="161">
@@ -25695,22 +25767,22 @@
         <v>-349.2561074480424</v>
       </c>
       <c r="AD161" s="19" t="n">
-        <v>64.067154</v>
+        <v>66.592654</v>
       </c>
       <c r="AE161" s="19" t="n">
-        <v>0.003768656117647059</v>
+        <v>0.003917214941176471</v>
       </c>
       <c r="AF161" s="19" t="n">
-        <v>0.3389796507936508</v>
+        <v>0.3523420846560846</v>
       </c>
       <c r="AG161" s="19" t="n">
-        <v>-65945.33715368001</v>
+        <v>-65942.81165368002</v>
       </c>
       <c r="AH161" s="19" t="n">
-        <v>-3.879137479628236</v>
+        <v>-3.878988920804707</v>
       </c>
       <c r="AI161" s="19" t="n">
-        <v>-348.9171277972488</v>
+        <v>-348.9037653633864</v>
       </c>
     </row>
     <row r="162">
@@ -25801,22 +25873,22 @@
         <v>7.747388987724859</v>
       </c>
       <c r="AD162" s="7" t="n">
-        <v>1528.323672679998</v>
+        <v>1530.849172679998</v>
       </c>
       <c r="AE162" s="7" t="n">
-        <v>0.08990139251058815</v>
+        <v>0.09004995133411756</v>
       </c>
       <c r="AF162" s="7" t="n">
-        <v>8.086368638518511</v>
+        <v>8.099731072380944</v>
       </c>
       <c r="AG162" s="7" t="n">
-        <v>1528.323672679998</v>
+        <v>1530.849172679998</v>
       </c>
       <c r="AH162" s="7" t="n">
-        <v>0.08990139251058815</v>
+        <v>0.09004995133411756</v>
       </c>
       <c r="AI162" s="7" t="n">
-        <v>8.086368638518511</v>
+        <v>8.099731072380944</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh dashboard Fri 09/04/2026 13:53
</commit_message>
<xml_diff>
--- a/public/PSI Cash Flow Report.xlsx
+++ b/public/PSI Cash Flow Report.xlsx
@@ -730,7 +730,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 03 Sep 2026 17:09</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 04 Sep 2026 13:53</t>
         </is>
       </c>
     </row>
@@ -805,14 +805,14 @@
       <c r="AC3" s="4" t="n"/>
       <c r="AD3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 03 Sep 2026</t>
+          <t>MTD as of 04 Sep 2026</t>
         </is>
       </c>
       <c r="AE3" s="4" t="n"/>
       <c r="AF3" s="4" t="n"/>
       <c r="AG3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 03 Sep 2026</t>
+          <t>YTD as of 04 Sep 2026</t>
         </is>
       </c>
       <c r="AH3" s="4" t="n"/>
@@ -13687,7 +13687,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 03 Sep 2026 17:09 (in IDR Million)</t>
+          <t>Cash Flow Statement   |   USD = Rp 17,000   |   INR = Rp 189   |   Generated: 04 Sep 2026 13:53 (in IDR Million)</t>
         </is>
       </c>
     </row>
@@ -13762,14 +13762,14 @@
       <c r="AC3" s="4" t="n"/>
       <c r="AD3" s="3" t="inlineStr">
         <is>
-          <t>MTD as of 03 Sep 2026</t>
+          <t>MTD as of 04 Sep 2026</t>
         </is>
       </c>
       <c r="AE3" s="4" t="n"/>
       <c r="AF3" s="4" t="n"/>
       <c r="AG3" s="3" t="inlineStr">
         <is>
-          <t>YTD as of 03 Sep 2026</t>
+          <t>YTD as of 04 Sep 2026</t>
         </is>
       </c>
       <c r="AH3" s="4" t="n"/>

</xml_diff>